<commit_message>
Update berita 2026-08-10 18:46 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-11.xlsx
+++ b/data/berita_2026-08-11.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1091,8 +1091,102 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Gempa magnitudo 5,1 guncang Bengkulu tak berpotensi tsunami</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 00:48:12 +0700</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Gempa magnitudo 5,1 mengguncang Kecamatan Enggano, Kabupaten Bengkulu Utara, pada Selasa dini hari sekitar pukul 00.08 ...</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688380/gempa-magnitudo-51-guncang-bengkulu-tak-berpotensi-tsunami</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG_20260811_003935.jpg</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Viral KDMP Berdiri di Tengah Pasar Papahan Karanganyar, Ternyata Ini Alasan Lokasinya Dipilih</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 00:52:07 +0700</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Viral Koperasi Desa Merah Putih (KDMP) berdiri di dalam area Pasar Desa Papahan, Kecamatan Tasikmadu, Kabupaten Karanganyar, Jawa Tengah.</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7866579/viral-kdmp-berdiri-di-tengah-pasar-papahan-karanganyar-ternyata-ini-alasan-lokasinya-dipilih</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/HeE3ln7veTR03JkbSYojXYqN5XA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Viral-KDMP-Berdiri-di-Tengah-Pasar-Papahan-Karanganyar-Ternyata-Ini-Alasan-Lokasinya-Dipilih.jpg</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I14"/>
+  <autoFilter ref="A1:I16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-10 20:36 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-11.xlsx
+++ b/data/berita_2026-08-11.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1467,8 +1467,149 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Sahroni Apresiasi BNN Bongkar Penyelundupan 1,3 Ton Ketamin: Mengerikan</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 03:17:55 +0700</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Matius Alfons Hutajulu</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Wakil Ketua Komisi III DPR Sahroni apresiasi BNN dan Polri atas penggagalan penyelundupan 1,3 ton ketamin. Ia dorong larangan vape untuk lindungi generasi muda.</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8613006/sahroni-apresiasi-bnn-bongkar-penyelundupan-1-3-ton-ketamin-mengerikan</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/02/20/wakil-ketua-komisi-iii-dpr-ri-ahmad-sahroni-1771531633340_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Presiden Kolombia Sebut Setidaknya 111 Orang Tewas dalam Gempa Magnitudo 7,4</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 03:15:00 +0700</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>"Per pukul 12.30 (waktu setempat), korban tewas mencapai 111 orang dan 87 orang luka-luka, dengan 1.575 rumah rusak,"</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7866582/presiden-kolombia-sebut-setidaknya-111-orang-tewas-dalam-gempa-magnitudo-74</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/URaiCze4k2TRjD74O4lopRgG6kY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/PRESIDEN-KOLOMBIA-Presiden-Kolombia-yang-baru-dilantik-Abelardo-de-la-Espriella.jpg</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Trump Klaim Perang Iran Segera Berakhir, Teheran Pasang Syarat Buka Hormuz, Pakar: Strategi Tekan AS</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 02:54:27 +0700</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Trump yakin perang Iran segera berakhir, tetapi Teheran masih mensyaratkan sejumlah hal untuk membuka kembali Selat Hormuz.</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7866581/trump-klaim-perang-iran-segera-berakhir-teheran-pasang-syarat-buka-hormuz-pakar-strategi-tekan-as</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/pd58Lh0QZkuUPrM04LfPl7UxG4o=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/residen-AS-Donald-Trump-Senin-27-Juli-2026-Foto-Res.jpg</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I22"/>
+  <autoFilter ref="A1:I25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-10 22:28 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-11.xlsx
+++ b/data/berita_2026-08-11.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,13 +419,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="33" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -1655,8 +1655,384 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Tottenham Hotspur perpanjang kontrak Micky van de Ven</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 04:42:06 +0700</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Tottenham Hotspur resmi memperpanjang kontrak bek tengah asal Belanda, Micky van de Ven di bursa transfer musim panas ...</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688399/tottenham-hotspur-perpanjang-kontrak-micky-van-de-ven</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1000044029.jpg</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Federasi sepak bola AS dan Kanada dukung kritik terhadap Infantino</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 04:37:43 +0700</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Federasi sepak bola Amerika Serikat (US Soccer) dan Kanada (Canada Soccer) mendukung pernyataan tiga konfederasi yang ...</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688395/federasi-sepak-bola-as-dan-kanada-dukung-kritik-terhadap-infantino</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2020/06/12/Fifa.jpg</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Menhut Sebut Prabowo Dukung Penuh Upaya Restorasi Ekosistem di Indonesia</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 05:08:09 +0700</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Menhut Raja Juli Antoni mengungkapkan dukungan Presiden Prabowo untuk restorasi ekosistem di Indonesia, menargetkan pemulihan lahan kritis 12 juta hektare.</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8613011/menhut-sebut-prabowo-dukung-penuh-upaya-restorasi-ekosistem-di-indonesia</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/03/12/raja-juli-antoni-1773304564547_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Bigmo 2 Kali Dipolisikan Gegara Konten: Sangat Kapok!</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 05:10:01 +0700</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Febryantino Nur Pratama</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Bigmo mengaku kapok dua kali dipolisikan karena konten. Bigmo ngaku kapok, benar atau hanya ucapan di mulut saja?</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8612978/bigmo-2-kali-dipolisikan-gegara-konten-sangat-kapok</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/10/youtuber-bigmo-tengah-meminta-maaf-soal-konten-promosi-vape-ajak-anak-in-frame-saat-siaran-langsung-1786363802068_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Trump Geser Strategi Hadapi Iran, Serangan Militer Diganti Tekanan Ekonomi, Pakar: AS Makin Terdesak</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 04:43:52 +0700</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Trump menggeser strategi menghadapi Iran ke tekanan ekonomi. Namun, Iran menjadikan Selat Hormuz sebagai kartu tawar untuk menekan balik AS.</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7866583/trump-geser-strategi-hadapi-iran-serangan-militer-diganti-tekanan-ekonomi-pakar-as-makin-terdesak</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ehJMjfAn9SH0LhD96-yXjyWtw7o=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Presiden-AS-Donald-Trump-berbicara-deF.jpg</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>4 Tersangka Bank BJB Ditahan, KPK Ungkap Nasib Ridwan Kamil</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 05:17:47 +0700</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>KPK membuka peluang kembali memeriksa Ridwan Kamil untuk melengkapi penyidikan kasus dugaan korupsi pengadaan iklan Bank BJB.</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266664/4-tersangka-bank-bjb-ditahan-kpk-ungkap-nasib-ridwan-kamil</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/neDfj15bxZKgfagFGEEQHaZsWWE=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/5430010/original/078632300_1764649557-Ridwan_Kamil_penuhi_panggilan_KPK.jpg</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Gempa Magnitudo 5,1 Guncang Bengkulu, Tak Berpotensi Tsunami</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 04:32:42 +0700</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Gempa yang mengguncang Kabupaten Bengkulu Utara, Provinsi Bengkulu itu berlokasi di titik koordinat 5.89 LS dan 102.43 BT.</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266665/gempa-magnitudo-51-guncang-bengkulu-tak-berpotensi-tsunami</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/ruRqc-lTqT-XvDVyvgHjqgAm-Lk=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9320778/original/021979200_1786397556-Jepretan_Layar_2025-08-11_pukul_04.31.35.jpg</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Imbas Kebakaran Gudang Limbah di Brebes, PMI: Warga Sekitar Mulai Keluhkan Sesak Napas</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 05:28:31 +0700</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Kebakaran gudang limbah di Brebes memasuki hari ketiga, menyebabkan 17 warga terdampak asap pekat. PMI imbau penggunaan masker.</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/08/10/220954978/imbas-kebakaran-gudang-limbah-di-brebes-pmi-warga-sekitar-mulai-keluhkan</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/D8y5Ijxhx87jJp8_zZsHGbAAgmc=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/10/6a79e553413c6.jpg</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I26"/>
+  <autoFilter ref="A1:I34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-10 23:28 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-11.xlsx
+++ b/data/berita_2026-08-11.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$61</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2031,8 +2031,1277 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Kenapa panjat pinang jadi tradisi 17 Agustus? Ini sejarahnya</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 06:23:51 +0700</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Panjat pinang menjadi salah satu perlombaan yang identik dengan perayaan Hari Ulang Tahun (HUT) Kemerdekaan Republik ...</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688427/kenapa-panjat-pinang-jadi-tradisi-17-agustus-ini-sejarahnya</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/28/Perayaan-Hut-ke-80-Bhayangkara-di-Balikpapan-280626-AP-9.jpg</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Selasa, Jakarta diperkirakan cerah berawan sepanjang hari</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 06:21:33 +0700</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) memprakirakan seluruh wilayah DKI Jakarta cerah berawan sepanjang ...</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688423/selasa-jakarta-diperkirakan-cerah-berawan-sepanjang-hari</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/26/cerah-berawan.jpg</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Baru mulai lari? Hindari 5 kesalahan ini agar tak mudah cedera</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 06:20:45 +0700</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Lari menjadi salah satu olahraga yang cukup mudah untuk dimulai. Tidak perlu banyak peralatan, bisa dilakukan di ...</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688421/baru-mulai-lari-hindari-5-kesalahan-ini-agar-tak-mudah-cedera</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/12/4a857c34-57d4-49c7-902f-a2db84fd3474.jpeg</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>BMKG prakirakan cuaca di sebagian besar RI berawan tebal pada Selasa</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 06:20:26 +0700</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) memprakirakan cuaca hari ini, Selasa, di sebagian besar wilayah ...</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688417/bmkg-prakirakan-cuaca-di-sebagian-besar-ri-berawan-tebal-pada-selasa</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/IMG_20260727_000432.jpg</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Kenapa lari makin populer di kota? Ini 8 alasannya</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 06:17:48 +0700</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Lari kini bukan lagi sekadar aktivitas olahraga yang dilakukan oleh atlet atau mereka yang sedang mempersiapkan diri ...</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688415/kenapa-lari-makin-populer-di-kota-ini-8-alasannya</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/lomba-lari-lila-wangsa-run-di-lhokseumawe-2837668.jpg</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>DKI kemarin, persiapan HUT RI hingga transportasi Kepulauan Seribu</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 06:16:56 +0700</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Sejumlah berita seputar DKI Jakarta yang terjadi pada Senin (10/8), mulai dari persiapan HUT ke-81 RI hingga ...</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688412/dki-kemarin-persiapan-hut-ri-hingga-transportasi-kepulauan-seribu</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/02/07/antarafoto-aktivitas-penyeberangan-kapal-kepulauan-seribu-070224-bay-7.jpg</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Lari 30 menit setiap hari, ini 7 manfaatnya bagi kesehatan</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 06:13:32 +0700</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Di tengah rutinitas yang semakin padat, olahraga tidak selalu harus dilakukan berjam-jam di pusat kebugaran. Salah satu ...</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688411/lari-30-menit-setiap-hari-ini-7-manfaatnya-bagi-kesehatan</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/IMG_7942.jpg</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Flowdesk Mendapatkan Lisensi VARA Penuh untuk Layanan Broker-Dealer</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 06:06:20 +0700</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>- Flowdesk merupakan penyedia likuiditas global sekaligus perusahaan teknologi perdagangan aset virtual dan hari ini ...</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688407/flowdesk-mendapatkan-lisensi-vara-penuh-untuk-layanan-broker-dealer</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2020/03/23/Logo-BusinessWire-800x600.jpg</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Rp4 triliun BOS madrasah mulai disalurkan</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 06:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Kementerian Agama (Kemenag) menyalurkan dana Bantuan Operasional Sekolah (BOS) tahap II dengan total nilai lebih dari ...</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/infografik/5688175/rp4-triliun-bos-madrasah-mulai-disalurkan</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/20260810-Rp4-triliun-BOS-madrasah-mulai-disalurkan.jpg</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Kriminal kemarin, ekshumasi Sutrimo hingga pemeriksaan Bigmo</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 05:59:42 +0700</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Sejumlah peristiwa berkaitan dengan keamanan menghiasi Jakarta yang terjadi pada Senin (10/8) kemarin, mulai dari ...</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688403/kriminal-kemarin-ekshumasi-sutrimo-hingga-pemeriksaan-bigmo</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1000912256.jpg</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Penjelasan DJP soal Pajak Rumah Kontrakan</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 05:55:37 +0700</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Retno Ayuningrum</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Direktorat Jenderal Pajak (DJP) Kementerian Keuangan menjelaskan rencana pemungutan pajak kepada pemilik rumah kontrakan pada 2027.</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8612434/penjelasan-djp-soal-pajak-rumah-kontrakan</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2014/10/01/aba994a2-34ed-467e-b236-0838b109f70c_169.jpg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Jessica Mila Klarifikasi Tudingan ke Pulau Padar saat Pelayaran Ditutup</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 06:02:46 +0700</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>wes</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Selebritias Jessica Mila klarifikasi tudingan ke Pulau Padar dan Komodo saat pelayaran ditutup.</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8613015/jessica-mila-klarifikasi-tudingan-ke-pulau-padar-saat-pelayaran-ditutup</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/05/08/jessica-mila-dan-suami-1778209378388_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Keluarga Nyalakan Lilin di Lokasi Tragedi Drag Race Maut Kotamobagu</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 05:59:34 +0700</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Momen duka keluarga korban Drag Race maut Kotamobagu pasang lilin di lokasi tewasnya keluarga mereka usai ditabrak mobil pembalap Tian Ngantung.</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7866593/keluarga-nyalakan-lilin-di-lokasi-tragedi-drag-race-maut-kotamobagu</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/5T63MMdtg-gtQnuc0Xo9vVmIECU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/kolase-2-bakar-lilin-di-drag-race-kotamobagu.jpg</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Viral Promo Miras Pakai Hafalan Alquran di Festival Musik, MUI Kecam Keras : Ini Bentuk Perendahan</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 05:51:28 +0700</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>MUI mengecam keras aksi promosi minuman keras (miras) berkedok tantangan hafalan Alquran yang mendadak viral di media sosial.</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866592/viral-promo-miras-pakai-hafalan-alquran-di-festival-musik-mui-kecam-keras-ini-bentuk-perendahan</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/-2d59XXwfIYkLuE0Rz5s5WSaLms=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-minuman-beralkohol-76t8.jpg</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Drama Pramusim Barcelona di 3 Negara, Penjualan Tiket Lawan Basel Berubah Kekacauan</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 05:46:40 +0700</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Barcelona kembali hadapi drama di pramusim. Setelah beberapa laga uji coba dibatalkan, laga lawan Basel justru membuat server penjualan klub eror.</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7866591/drama-pramusim-barcelona-di-3-negara-penjualan-tiket-lawan-basel-berubah-kekacauan</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/um9v51_Smi_Af51A3wMXpv34uos=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Barcelona-Copa-del-Rey-161.jpg</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Quartararo Tak Anggap MotoGP 2026 Aneh, Aprilia Cocok di Silverstone dan Ducati Dinanti di Aragon</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 05:41:20 +0700</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Fabio Quartararo tidak menganggap persaingan MotoGP 2026 aneh setelah Aprilia tampil dominan di Silverstone dan Ducati kesulitan.</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7866590/quartararo-tak-anggap-motogp-2026-aneh-aprilia-cocok-di-silverstone-dan-ducati-dinanti-di-aragon</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/iq8q0RqjkDf00LiB-ZCYSDyQ6mM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/fabio-quartararo-berbicara-kepada-media-setelah-latihan-bebas-kedua.jpg</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Prakiraan Cuaca Sulawesi Barat Selasa, 11 Agustus 2026: Semua Cerah</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 05:33:48 +0700</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>BMKG melaporkan prakiraan cuaca untuk wilayah Sulawesi Barat (Sulbar), Selasa (11/8/2026). Semua wilayah akan cerah.</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7866589/prakiraan-cuaca-sulawesi-barat-selasa-11-agustus-2026-semua-cerah</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/zuUaADQ8yitcRX5Zk0F6srdEnKw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Prakiraan-Cuaca-Sulawesi-Barat-Selasa-10-Maret-2026Waspada-Hujan-Lebat-di-Wilayah-Ini.jpg</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>5 Populer Regional: Drag Race Maut di Kotamobagu - Sosok 2 Tersangka Perampokan Candra Waskito</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 05:32:13 +0700</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Drag race Kotamobagu menewaskan 7 orang, sementara dua tersangka pembunuhan bos Royal Phone Ambarawa ditangkap polisi.</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7866588/5-populer-regional-drag-race-maut-di-kotamobagu-sosok-2-tersangka-perampokan-candra-waskito</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/AXdgAr9Iw3PgL4auFlOtiwlS1HI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/kecelakaan-Drag-Race-dan-Drag-Bike-di-kotamobagu.jpg</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Ambil Tawaran Sinetron, Betrand Peto Kini Belajar Lebih Luas Lagi soal Dunia Entertain</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 05:30:32 +0700</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Penyanyi Betrand Peto belajar lebih luas lagi soal dunia entertain lewat debut aktingnya di sinetron Ternyata Ini Cinta.</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7866587/ambil-tawaran-sinetron-betrand-peto-kini-belajar-lebih-luas-lagi-soal-dunia-entertain</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/WmDEz8uVI8MheqYNv2eV8ii5aV4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Betrand-Peto-nangis-melihat-video-Sarwendah-viral.jpg</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Hampir Setahun Cerai dari Ahmad Assegaf, Tasya Farasya Curhat soal Sisi Rapuh</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 05:28:18 +0700</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Hampir setahun bercerai ari Ahmad Assegaf, Tasya Farasya kepergok curhat membahas tentang sisi rapuh.</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7866586/hampir-setahun-cerai-dari-ahmad-assegaf-tasya-farasya-curhat-soal-sisi-rapuh</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/myn8Dx3mai8z5-ojphGgM9LQRgY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/beauty-influencer-tasya-farasya.jpg</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Ada Peran Sahabat Lionel Messi di Balik Kepindahan Ronald Araujo ke Liverpool, Pesan Khusus Terkirim</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 05:23:37 +0700</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Ronald Araujo mendapatkan pesan spesial dari Luis Suarez setelah resmi membuka lembaran baru bersama Liverpool sebagai pemain pinjaman Barcelona.</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7866585/ada-peran-sahabat-lionel-messi-di-balik-kepindahan-ronald-araujo-ke-liverpool-pesan-khusus-terkirim</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/MTQ-ST3HxsLdctGDaIeNGoHJwD8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Pemain-pinjaman-Barcelona-Ronald-Araujo-saat-diperkenalkan.jpg</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Kini Gandeng Kekasih Baru, Dahlia Poland Bantah Dicomblangin Dicky SMASH</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 05:22:54 +0700</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Dahlia Poland kini gandeng pacar baru, konten kreator Rangga Azies usai bercerai dengan aktor Fandy Christian. Ia membantah dicomblangin Dicky SMASH.</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7866584/kini-gandeng-kekasih-baru-dahlia-poland-bantah-dicomblangin-dicky-smash</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ESge_XkWLJJAmaVL-NgpugssHB8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Dahlia-Poland-ketika-ditemui-di-kawasan-Tendean-Jakarta-Selatan.jpg</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>KPK Ungkap Dugaan Pengondisian Audit BPK dalam Kasus Korupsi Bank BJB</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 06:17:42 +0700</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>KPK menduga uang nonbujeter dari pengadaan iklan Bank BJB digunakan untuk mengurus temuan audit BPK.</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266666/kpk-ungkap-dugaan-pengondisian-audit-bpk-dalam-kasus-korupsi-bank-bjb</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/JwVem3lzYNfwyZ1ITqmvAg88XZg=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9320689/original/081405900_1786367086-71944.jpg</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Penjelasan KPK soal Sisa Uang Amplop Bupati Kuansing untuk Menhut</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 06:06:52 +0700</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>KPK terus menelusuri sisa uang SGD 2.000 dari total SGD 14.000 dalam kasus dugaan suap Bupati Kuansing dan Kemenhut.</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266678/penjelasan-kpk-soal-sisa-uang-amplop-bupati-kuansing-untuk-menhut</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/HhURMajvSW7aquQf9I_ex0-2LQg=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/7618978/original/014714900_1780405596-IMG_2704.jpg</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>KPK Telusuri Aliran Uang Kasus Bank BJB ke Lisa Mariana Lewat Nomine</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 05:45:50 +0700</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>KPK tengah menelusuri dugaan aliran uang kasus Bank BJB ke Lisa Mariana yang disebut melalui pihak lain atau nomine.</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266660/kpk-telusuri-aliran-uang-kasus-bank-bjb-ke-lisa-mariana-lewat-nomine</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/rUdL_iF94kLXxYVrzb1n0DNLu4A=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/5324168/original/096678300_1755843657-20250822-Lisa_M-HEL_9.jpg</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Bigmo Minta Maaf Usai Diperiksa Polisi, Akui Kontennya Tak Pantas</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 05:31:18 +0700</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>YouTuber Bigmo Mengaku Kapok dan Minta Maaf Usai Diperiksa Polisi Terkait Konten Live Streaming</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266658/bigmo-minta-maaf-usai-diperiksa-polisi-akui-kontennya-tak-pantas</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/RuQNgz1b2xdlesPvESyGkeIiBiw=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9320772/original/046943600_1786395707-Bigmo__1_.jpg</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>MBG Tetap Jalan, Komisi XI Minta Tata Kelola Diperketat</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 06:16:16 +0700</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Mitra SPPG diminta mengikuti standardisasi dan pembenahan tata kelola MBG agar penggunaan APBN semakin transparan dan akuntabel.</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266670/mbg-tetap-jalan-komisi-xi-minta-tata-kelola-diperketat</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/CSIKMS1zrLfH-SxfmCKYABQjZXw=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9295136/original/006741400_1783915651-mbg2.jpg</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I34"/>
+  <autoFilter ref="A1:I61"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-11 05:48 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-11.xlsx
+++ b/data/berita_2026-08-11.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$335</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$439</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I335"/>
+  <dimension ref="A1:I439"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -16179,8 +16179,4898 @@
         </is>
       </c>
     </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>Mendikti: Pendidikan psikologi harus jadi instrumen tekan masalah jiwa</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:44:08 +0700</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>Menteri Pendidikan Tinggi, Sains, dan Teknologi (Mendiktisaintek) Brian Yuliarto menekankan pendidikan psikologi harus ...</t>
+        </is>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G336" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688816/mendikti-pendidikan-psikologi-harus-jadi-instrumen-tekan-masalah-jiwa</t>
+        </is>
+      </c>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/WhatsApp-Image-2026-08-03-at-18.27.21.jpeg</t>
+        </is>
+      </c>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Peking University siap perluas kerja sama riset dengan Kementrans</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:41:36 +0700</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>Perguruan tinggi riset publik di Beijing, China, Institute of South-South Cooperation and ...</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G337" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688812/peking-university-siap-perluas-kerja-sama-riset-dengan-kementrans</t>
+        </is>
+      </c>
+      <c r="H337" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1000179540.jpg</t>
+        </is>
+      </c>
+      <c r="I337" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Mentan apresiasi capaian Unhas pertahankan gelar Pimnas</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:40:14 +0700</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>Menteri Pertanian Andi Amran Sulaiman memberikan apresiasi atas capaian Universitas Hasanuddin (Unhas) yang mampu ...</t>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G338" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688811/mentan-apresiasi-capaian-unhas-pertahankan-gelar-pimnas</t>
+        </is>
+      </c>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG_20260811_085244.jpg</t>
+        </is>
+      </c>
+      <c r="I338" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Ekonom Danamon proyeksikan ekonomi RI tumbuh 5,2 persen pada 2026</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:39:43 +0700</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>Ekonom PT Bank Danamon Indonesia Tbk memproyeksikan ekonomi Indonesia tumbuh 5,2 persen pada 2026, dengan momentum ...</t>
+        </is>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G339" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688807/ekonom-danamon-proyeksikan-ekonomi-ri-tumbuh-52-persen-pada-2026</t>
+        </is>
+      </c>
+      <c r="H339" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/14/1000169493.jpg</t>
+        </is>
+      </c>
+      <c r="I339" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Komisi III minta provokator hoaks dikategorikan sebagai musuh negara</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:34:28 +0700</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>Wakil Ketua Komisi III DPR RI Ahmad Sahroni meminta provokator hoaks di media sosial dikategorikan sebagai musuh negara ...</t>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G340" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688805/komisi-iii-minta-provokator-hoaks-dikategorikan-sebagai-musuh-negara</t>
+        </is>
+      </c>
+      <c r="H340" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/30/raker-komisi-iii-dpr-dengan-kpk-dan-bnn-2807117.jpg</t>
+        </is>
+      </c>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>Airlangga sebut ETF Emas perkuat posisi Indonesia di investasi global</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:32:42 +0700</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>Menteri Koordinator Bidang Perekonomian Airlangga Hartarto mengatakan Exchange Traded Fund (ETF) Emas memperkuat posisi ...</t>
+        </is>
+      </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G341" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688804/airlangga-sebut-etf-emas-perkuat-posisi-indonesia-di-investasi-global</t>
+        </is>
+      </c>
+      <c r="H341" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/B7A00464-D39A-42DE-804D-457E77F33FB2.jpeg</t>
+        </is>
+      </c>
+      <c r="I341" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>OJK tempatkan penguatan ekosistem UMKM sebagai program utama</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:31:42 +0700</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>Ketua Dewan Komisioner Otoritas Jasa Keuangan (DK OJK) Friderica Widyasari Dewi menyatakan pihaknya menempatkan ...</t>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G342" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688801/ojk-tempatkan-penguatan-ekosistem-umkm-sebagai-program-utama</t>
+        </is>
+      </c>
+      <c r="H342" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/WhatsApp-Image-2026-08-11-at-12.24.49.jpeg</t>
+        </is>
+      </c>
+      <c r="I342" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>BRImo beri diskon hingga Rp100 ribu untuk tiket Gaia Music Festival 2026</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:27:21 +0700</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>Bagi pencinta festival musik, Gaia Music Festival 2026 menjadi salah satu agenda hiburan yang patut dinantikan. ...</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G343" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688797/brimo-beri-diskon-hingga-rp100-ribu-untuk-tiket-gaia-music-festival-2026</t>
+        </is>
+      </c>
+      <c r="H343" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/Gaia-Music-Festival-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I343" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>Wamendag: Ekspor F&amp;B masuk lima besar ASEAN</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:26:51 +0700</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>Wakil Menteri Perdagangan (Wamendag) Dyah Roro Esti menyebut ekspor produk makanan dan minuman (food and ...</t>
+        </is>
+      </c>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G344" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688796/wamendag-ekspor-fb-masuk-lima-besar-asean</t>
+        </is>
+      </c>
+      <c r="H344" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG_3743.jpeg</t>
+        </is>
+      </c>
+      <c r="I344" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>PP Pesti siapkan tujuh atlet menuju Asian Games 2026</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:20:56 +0700</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>Pengurus Pusat Persatuan Soft Tennis Indonesia (PP Pesti) menyiapkan tujuh atlet putra dan putri untuk lolos ...</t>
+        </is>
+      </c>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G345" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688793/pp-pesti-siapkan-tujuh-atlet-menuju-asian-games-2026</t>
+        </is>
+      </c>
+      <c r="H345" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/d3f241c9-ca8b-4e11-b845-b8543dd7f9b3.jpeg</t>
+        </is>
+      </c>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Bea Cukai gagalkan penyelundupan 2,7 juta rokok ilegal di Kubu Raya</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:20:10 +0700</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>Kanwil Ditjen Bea dan Cukai Kalimantan Bagian Barat (Kanwil DJBC Kalbagbar) berhasil menggagalkan upaya penyelundupan ...</t>
+        </is>
+      </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G346" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688789/bea-cukai-gagalkan-penyelundupan-27-juta-rokok-ilegal-di-kubu-raya</t>
+        </is>
+      </c>
+      <c r="H346" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/28/1001382866.jpg</t>
+        </is>
+      </c>
+      <c r="I346" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>Bapanas salurkan 610,3 ribu ton beras SPHP hingga 8 Agustus 2026</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:17:59 +0700</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>Badan Pangan Nasional (Bapanas) menyebut penyaluran beras program Stabilisasi Pasokan dan Harga Pangan (SPHP) hingga 8 ...</t>
+        </is>
+      </c>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G347" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688785/bapanas-salurkan-6103-ribu-ton-beras-sphp-hingga-8-agustus-2026</t>
+        </is>
+      </c>
+      <c r="H347" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/E9A3406D-1197-4E14-93E3-ED73348EFD19.jpeg</t>
+        </is>
+      </c>
+      <c r="I347" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Komnas HAM dorong penguatan bantuan bagi pengungsi Papua Tengah</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:16:22 +0700</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>Komisi Nasional Hak Asasi Manusia (Komnas HAM) mendorong penguatan kolaborasi lintas kementerian, pemerintah daerah, ...</t>
+        </is>
+      </c>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G348" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688783/komnas-ham-dorong-penguatan-bantuan-bagi-pengungsi-papua-tengah</t>
+        </is>
+      </c>
+      <c r="H348" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/08/WhatsApp-Image-2026-04-08-at-5.53.23-PM_1.jpeg</t>
+        </is>
+      </c>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Visa Indonesia pegang hak penamaan stasiun MRT Blok A</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:16:03 +0700</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>Visa Indonesia memegang hak penamaan (naming rights) stasiun MRT Blok A sebagai upaya memperluas akses pembayaran ...</t>
+        </is>
+      </c>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G349" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688779/visa-indonesia-pegang-hak-penamaan-stasiun-mrt-blok-a</t>
+        </is>
+      </c>
+      <c r="H349" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1001022419.jpg</t>
+        </is>
+      </c>
+      <c r="I349" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Plus minus penggunaan AI untuk produksi film menurut Brad Pitt</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:13:56 +0700</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>Aktor Hollywood, Brad Pitt menyoroti penggunaan kecerdasan artifisial (AI) untuk film yang dinilainya dapat membantu ...</t>
+        </is>
+      </c>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G350" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688776/plus-minus-penggunaan-ai-untuk-produksi-film-menurut-brad-pitt</t>
+        </is>
+      </c>
+      <c r="H350" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/04/29/Brad.jpeg</t>
+        </is>
+      </c>
+      <c r="I350" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>KPPPA: Sistem terpadu penanganan korban kekerasan butuh kolaborasi K/L</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:10:04 +0700</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>Wakil Menteri Pemberdayaan Perempuan dan Perlindungan Anak Veronica Tan mengatakan kebijakan dan sistem yang terpadu ...</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688772/kpppa-sistem-terpadu-penanganan-korban-kekerasan-butuh-kolaborasi-k-l</t>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/WhatsApp-Image-2026-08-11-at-10.32.14.jpeg</t>
+        </is>
+      </c>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>Mazda konfirmasi CX-3 generasi terbaru akan diproduksi pada 2027</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:07:19 +0700</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>Mazda mengonfirmasi bahwa generasi terbaru dari crossover CX-3 akan mulai diproduksi pada 2027 mendatang.
+Dilansir ...</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5688765/mazda-konfirmasi-cx-3-generasi-terbaru-akan-diproduksi-pada-2027</t>
+        </is>
+      </c>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/29/IMG_1246.jpeg</t>
+        </is>
+      </c>
+      <c r="I352" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>Gulkarmat DKI ingatkan personel jaga keselamatan saat bertugas</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:04:54 +0700</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>Kepala Dinas Penanggulangan Kebakaran dan Penyelamatan (Gulkarmat) DKI Jakarta, Bayu Meghantara meminta para personel ...</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688764/gulkarmat-dki-ingatkan-personel-jaga-keselamatan-saat-bertugas</t>
+        </is>
+      </c>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1000319297.jpg</t>
+        </is>
+      </c>
+      <c r="I353" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Polda Jatim perkuat kesiapan personel hadapi karhutla</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:03:12 +0700</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>Kepolisian Daerah Jawa Timur memperkuat kesiapan personel dan peralatan menghadapi ancaman kebakaran hutan dan lahan ...</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G354" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688760/polda-jatim-perkuat-kesiapan-personel-hadapi-karhutla</t>
+        </is>
+      </c>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1346126.jpg</t>
+        </is>
+      </c>
+      <c r="I354" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Kemlu terus pantau 7 ABK WNI di Kapal MV Star Janet di perairan China</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:01:30 +0700</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>Kementerian Luar Negeri RI terus memantau perkembangan kasus tujuh anak buah kapal (ABK) warga negara Indonesia (WNI) ...</t>
+        </is>
+      </c>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G355" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688756/kemlu-terus-pantau-7-abk-wni-di-kapal-mv-star-janet-di-perairan-china</t>
+        </is>
+      </c>
+      <c r="H355" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/01/WhatsApp-Image-2026-07-01-at-6.44.26-PM.jpeg</t>
+        </is>
+      </c>
+      <c r="I355" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Akselerasi revitalisasi sekolah dan madrasah</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>Pemerintah berupaya mengakselerasi revitalisasi sekolah dan madrasah pada 2026 dengan target lebih dari 70 ribu unit ...</t>
+        </is>
+      </c>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G356" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/infografik/5688743/akselerasi-revitalisasi-sekolah-dan-madrasah</t>
+        </is>
+      </c>
+      <c r="H356" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/20260811-Akselerasi-revitalisasi-sekolah-dan-madrasah.jpg</t>
+        </is>
+      </c>
+      <c r="I356" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>Pemprov Lampung perbaiki akses jalan percepat pembangunan PSEL</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:58:45 +0700</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>Pemerintah Provinsi (Pemprov) Lampung perbaiki akses jalan serta memastikan kesiapan lahan untuk mendukung percepatan ...</t>
+        </is>
+      </c>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G357" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688752/pemprov-lampung-perbaiki-akses-jalan-percepat-pembangunan-psel</t>
+        </is>
+      </c>
+      <c r="H357" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG-20260810-WA0039-1.jpg</t>
+        </is>
+      </c>
+      <c r="I357" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Aksi percobaan pembobolan kotak amal di Tambora terekam CCTV</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:58:26 +0700</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>Seorang pria terekam kamera pengawas (CCTV) diduga mencoba membobol kotak amal di Musala Al-Ikhlas, Jalan Siaga III, RT ...</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G358" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688748/aksi-percobaan-pembobolan-kotak-amal-di-tambora-terekam-cctv</t>
+        </is>
+      </c>
+      <c r="H358" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/03/01/IMG-20260301-WA0014_1.jpg</t>
+        </is>
+      </c>
+      <c r="I358" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Cahaya dari Bukit Menoreh</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:57:57 +0700</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>Pembangunan infrastruktur di Kulon Progo, Yogyakarta, melaju pesat sejak awal 2000-an. Kawasan hortikultura di pantai ...</t>
+        </is>
+      </c>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688745/cahaya-dari-bukit-menoreh</t>
+        </is>
+      </c>
+      <c r="H359" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/25/RHD_6567.jpg.jpeg</t>
+        </is>
+      </c>
+      <c r="I359" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>Israel simpan 1.700 jenazah warga Palestina, kompromi tukar tawanan</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:54:19 +0700</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>Israel menahan jenazah sekitar 1.700 warga Palestina untuk digunakan sebagai alat kompromi pertukaran tawanan ke ...</t>
+        </is>
+      </c>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G360" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688739/israel-simpan-1700-jenazah-warga-palestina-kompromi-tukar-tawanan</t>
+        </is>
+      </c>
+      <c r="H360" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/13/thumbs_b_ddc255f068d62800412e647c5948659a.jpg</t>
+        </is>
+      </c>
+      <c r="I360" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>Pemuda di Jakut diajak sulap sampah jadi barang bernilai ekonomis</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:53:33 +0700</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>Anggota DPRD DKI Jakarta, Bebizie Sri Mulyati mengajak pemuda di Jakarta Utara menyulap sampah menjadi barang yang ...</t>
+        </is>
+      </c>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688737/pemuda-di-jakut-diajak-sulap-sampah-jadi-barang-bernilai-ekonomis</t>
+        </is>
+      </c>
+      <c r="H361" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/ad47cbd6-b89d-467a-a6cc-f440cfa15d4e.jpeg</t>
+        </is>
+      </c>
+      <c r="I361" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>Memotret ekonomi Indonesia dari Kepri</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:51:53 +0700</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>Suatu pagi di pekan ketiga Juni 2026, kediaman pribadi Gubernur Kepulauan Riau (Kepri) Ansar Ahmad di Jalan Peralatan, ...</t>
+        </is>
+      </c>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688733/memotret-ekonomi-indonesia-dari-kepri</t>
+        </is>
+      </c>
+      <c r="H362" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/Facebook_creation_F39777D3-5B89-4505-9238-16B524314731.jpeg</t>
+        </is>
+      </c>
+      <c r="I362" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Dubes Palestina: Korban tewas di Jalur Gaza lampaui 75.000 orang</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:49:15 +0700</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>Duta Besar Palestina untuk Rusia Abdel Hafiz Nofal mengatakan jumlah korban tewas di Jalur Gaza telah melampaui 75.000 ...</t>
+        </is>
+      </c>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G363" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688731/dubes-palestina-korban-tewas-di-jalur-gaza-lampaui-75000-orang</t>
+        </is>
+      </c>
+      <c r="H363" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/thumbs_b_b39e1a6a973e661feeb3926a2ec52632.jpg</t>
+        </is>
+      </c>
+      <c r="I363" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>Program Cicilan BRI Kartu Kredit hadir dengan bunga mulai 0% dan tenor hingga 36 bulan</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:49:04 +0700</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>Di tengah berbagai kebutuhan dan gaya hidup yang semakin dinamis, kemampuan mengatur pengeluaran menjadi salah satu ...</t>
+        </is>
+      </c>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G364" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688727/program-cicilan-bri-kartu-kredit-hadir-dengan-bunga-mulai-0-dan-tenor-hingga-36-bulan</t>
+        </is>
+      </c>
+      <c r="H364" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2022/11/01/pexels-karolina-grabowska-5239804.jpg</t>
+        </is>
+      </c>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>Wamentrans: China dapat jadi referensi pengembangan transmigrasi RI</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:46:14 +0700</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>Wakil Menteri Transmigrasi (Wamentrans) Viva Yoga Mauladi mengatakan pengalaman China dalam pembangunan sumber daya ...</t>
+        </is>
+      </c>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G365" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688724/wamentrans-china-dapat-jadi-referensi-pengembangan-transmigrasi-ri</t>
+        </is>
+      </c>
+      <c r="H365" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1000179538.jpg</t>
+        </is>
+      </c>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>Anggota DPD dukung Pemprov DKI terbitkan obligasi daerah</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:44:21 +0700</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>Anggota Dewan Perwakilan Daerah (DPD) RI dari Daerah Pemilihan (Dapil) DKI Jakarta, Dailami Firdaus mendukung rencana ...</t>
+        </is>
+      </c>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G366" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688721/anggota-dpd-dukung-pemprov-dki-terbitkan-obligasi-daerah</t>
+        </is>
+      </c>
+      <c r="H366" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2022/05/19/WhatsApp-Image-2022-05-19-at-10.45.33.jpeg</t>
+        </is>
+      </c>
+      <c r="I366" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>E-football jadi nomor esports teramai pada Asian Games 2026</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:41:26 +0700</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>E-football menjadi nomor pertandingan esports dengan jumlah peserta negara terbanyak pada Asian Games 2026 Aichi-Nagoya ...</t>
+        </is>
+      </c>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G367" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688719/e-football-jadi-nomor-esports-teramai-pada-asian-games-2026</t>
+        </is>
+      </c>
+      <c r="H367" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2021/04/01/img-6989-_x600.jpg</t>
+        </is>
+      </c>
+      <c r="I367" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>Trump diam-diam ganti pesawat saat di Turkiye di tengah ancaman Iran</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:39:00 +0700</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>Presiden Amerika Serikat (AS) Donald Trump diam-diam meninggalkan Turkiye dengan pesawat militer bulan lalu di ...</t>
+        </is>
+      </c>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G368" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688717/trump-diam-diam-ganti-pesawat-saat-di-turkiye-di-tengah-ancaman-iran</t>
+        </is>
+      </c>
+      <c r="H368" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/thumbs_b_c_0faf781db807e5288836e40ddc754e72.jpg</t>
+        </is>
+      </c>
+      <c r="I368" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Gempa Kolombia beri pemahaman risikonya pada struktur bangunan kota</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:38:38 +0700</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>Pakar dari Ikatan Ahli Kebencanaan Indonesia (IABI) Daryono menyatakan fenomena seismotektonik pada gempa bumi ...</t>
+        </is>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688713/gempa-kolombia-beri-pemahaman-risikonya-pada-struktur-bangunan-kota</t>
+        </is>
+      </c>
+      <c r="H369" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/thumbs_b_c_e726e95b76c6f0cd719dcf122fc06d02.jpg</t>
+        </is>
+      </c>
+      <c r="I369" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Hampir 22 ribu rumah rusak akibat gempa Kumamoto</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:36:52 +0700</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>Otoritas Prefektur Kumamoto, Jepang, mencatat hampir 22.000 rumah mengalami kerusakan akibat gempa bumi ...</t>
+        </is>
+      </c>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G370" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688711/hampir-22-ribu-rumah-rusak-akibat-gempa-kumamoto</t>
+        </is>
+      </c>
+      <c r="H370" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/30/thumbs_b_c_c0a1b3ae6f28b99cdb4f19b3d325f6dc-1.jpg</t>
+        </is>
+      </c>
+      <c r="I370" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>PBB: Krisis kemanusiaan di Sudan kian memburuk akibat konflik</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:36:35 +0700</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>Konflik yang berkelanjutan, pengungsian, dan kekurangan dana terus memperdalam kebutuhan kemanusiaan di seluruh Sudan, ...</t>
+        </is>
+      </c>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G371" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688707/pbb-krisis-kemanusiaan-di-sudan-kian-memburuk-akibat-konflik</t>
+        </is>
+      </c>
+      <c r="H371" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/CjkinzN000009_20260811_CBMFN0A001.jpeg</t>
+        </is>
+      </c>
+      <c r="I371" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>BPBD Sulteng tangani 33 karhutla selama Januari-Agustus 2026</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:34:40 +0700</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>Badan Penanggulangan Bencana Daerah (BPBD) Sulawesi Tengah (Sulteng) telah menangani 33 kejadian kebakaran hutan dan ...</t>
+        </is>
+      </c>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G372" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688703/bpbd-sulteng-tangani-33-karhutla-selama-januari-agustus-2026</t>
+        </is>
+      </c>
+      <c r="H372" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG-20260808-WA0026.jpg</t>
+        </is>
+      </c>
+      <c r="I372" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>Bakamla RI latihan bersama "coast guard" Malaysia - Singapura di Kepri</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:33:31 +0700</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>Badan Keamanan Laut (Bakamla) RI menggelar latihan bersama penjaga pantai (coast guard) Malaysia dan Singapura dalam ...</t>
+        </is>
+      </c>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G373" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688700/bakamla-ri-latihan-bersama-coast-guard-malaysia-singapura-di-kepri</t>
+        </is>
+      </c>
+      <c r="H373" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG_1754.jpeg</t>
+        </is>
+      </c>
+      <c r="I373" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>Cara Jakarta menekan pengangguran dari akar rumput</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:32:13 +0700</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>Dua puluh warga Pasar Rebo tidak perlu mendatangi balai pelatihan kerja untuk belajar meracik kopi atau mengedit video. ...</t>
+        </is>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688699/cara-jakarta-menekan-pengangguran-dari-akar-rumput</t>
+        </is>
+      </c>
+      <c r="H374" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/target-rasio-kewirausahaan-nasional-2834312.jpg</t>
+        </is>
+      </c>
+      <c r="I374" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>Swiatek bertemu Svitolina pada semifinal WTA 1000 Toronto</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:31:15 +0700</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>Iga Swiatek akan menghadapi Elina Svitolina pada semifinal National Bank Open 2026 di Toronto setelah kedua petenis ...</t>
+        </is>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688696/swiatek-bertemu-svitolina-pada-semifinal-wta-1000-toronto</t>
+        </is>
+      </c>
+      <c r="H375" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG_0161.jpeg</t>
+        </is>
+      </c>
+      <c r="I375" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>AS mediasi Israel-Suriah sepakati IAEA evakuasi material nuklir</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:30:33 +0700</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>Amerika Serikat telah menengahi kesepakatan antara Suriah dan Israel untuk membiarkan Badan Energi Atom Internasional ...</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688692/as-mediasi-israel-suriah-sepakati-iaea-evakuasi-material-nuklir</t>
+        </is>
+      </c>
+      <c r="H376" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/03/03/IAEA.jpg</t>
+        </is>
+      </c>
+      <c r="I376" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>Baznas dan Ika Unpad perkuat pemberdayaan mahasiswa berbasis masjid</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:30:22 +0700</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>Badan Amil Zakat Nasional (Baznas) bersama Unit Pengumpulan Zakat (UPZ) Ikatan Alumni Universitas Padjadjaran (IKA ...</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688688/baznas-dan-ika-unpad-perkuat-pemberdayaan-mahasiswa-berbasis-masjid</t>
+        </is>
+      </c>
+      <c r="H377" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG_20260811_091056.jpg.jpeg</t>
+        </is>
+      </c>
+      <c r="I377" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>Semeru delapan kali erupsi dengan tinggi letusan capai 700 meter</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:27:34 +0700</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>Gunung Semeru di perbatasan Kabupaten Lumajang dan Malang, Jawa Timur mengalami delapan kali erupsi dengan tinggi ...</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688685/semeru-delapan-kali-erupsi-dengan-tinggi-letusan-capai-700-meter</t>
+        </is>
+      </c>
+      <c r="H378" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/WhatsApp-Image-2026-08-11-at-10.54.07.jpeg</t>
+        </is>
+      </c>
+      <c r="I378" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Kemensos benahi kedisiplinan pegawai termasuk praktik judol</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:23:40 +0700</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>Kementerian Sosial membenahi kedisiplinan internal seluruh jajarannya, termasuk menskrining oknum pegawai kementerian ...</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G379" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688683/kemensos-benahi-kedisiplinan-pegawai-termasuk-praktik-judol</t>
+        </is>
+      </c>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG20260811094952_103356_1.jpg</t>
+        </is>
+      </c>
+      <c r="I379" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>Sayap pemuda Golkar BMK 1957 ajak kader perkuat konsolidasi nasional</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:23:39 +0700</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>Ketua Umum sayap pemuda Partai Golkar, Barisan Muda Kosgoro (BMK) 1957 Rizky Maulana mengajak seluruh jajaran pengurus ...</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688681/sayap-pemuda-golkar-bmk-1957-ajak-kader-perkuat-konsolidasi-nasional</t>
+        </is>
+      </c>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1000480475_1.jpg</t>
+        </is>
+      </c>
+      <c r="I380" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>KKP dalami dugaan pelanggaran kapal tuna di Benoa</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:17:12 +0700</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>Kementerian Kelautan dan Perikanan (KKP) mengatakan tengah mendalami dugaan pelanggaran yang melibatkan sejumlah kapal ...</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688677/kkp-dalami-dugaan-pelanggaran-kapal-tuna-di-benoa</t>
+        </is>
+      </c>
+      <c r="H381" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2023/05/25/IMG_20230510_112049.jpg</t>
+        </is>
+      </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>Kemenpar-BI gelar pelatihan guna perkuat wisata ramah muslim</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:16:28 +0700</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>Kementerian Pariwisata dan Departemen Ekonomi dan Keuangan Syariah (DEKS) Bank Indonesia (BI) menggelar pelatihan ...</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G382" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688676/kemenpar-bi-gelar-pelatihan-guna-perkuat-wisata-ramah-muslim</t>
+        </is>
+      </c>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/26/wisatawan-kapal-pesiar-kunjungi-masjid-raya-baiturrahman-aceh-111124-apls-4.jpg</t>
+        </is>
+      </c>
+      <c r="I382" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>Uni Eropa siapkan jaringan listrik hadapi gerhana matahari</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:15:46 +0700</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>Operator jaringan listrik Eropa telah mengambil sejumlah langkah tambahan untuk memastikan kelancaran operasi sistem ...</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688673/uni-eropa-siapkan-jaringan-listrik-hadapi-gerhana-matahari</t>
+        </is>
+      </c>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/09/20/antarafoto-gerhana-matahari-sebagian-di-bekasi-20042023-par-2.jpg</t>
+        </is>
+      </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>Jelang Sidang Bersama, Karpet hingga Ornamen Merah Putih Mulai Terpasang</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:21:59 +0700</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>Dwi Rahmawati</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>Persiapan sidang tahunan MPR dan sidang bersama DPR-DPD pada 14 Agustus 2026 terus dilakukan. Rapat protokol dengan pihak kementerian berlangsung pagi ini.</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8613416/jelang-sidang-bersama-karpet-hingga-ornamen-merah-putih-mulai-terpasang</t>
+        </is>
+      </c>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/persiapan-jelang-sidang-tahunan-mpr-dan-sidang-bersama-dpr-dpd-1786425599808_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>Pembalap Drag Race Maut di Kotamobagu Berpotensi Jadi Tersangka</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:21:50 +0700</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>Fistel Mukuan</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>Pembalap bernama Tian Ngantung yang mengemudikan mobil maut itu berpotensi menjadi tersangka.</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G385" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8613415/pembalap-drag-race-maut-di-kotamobagu-berpotensi-jadi-tersangka</t>
+        </is>
+      </c>
+      <c r="H385" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/10/mobil-peserta-drag-race-kotamobagu-tabrak-penonton-hingga-8-orang-meninggal-1786343760891_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I385" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>Polisi Reka Ulang Kasus Mutilasi Pria di Depok, Saepul Dihadirkan</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:02:19 +0700</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>Devi Puspitasari</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>Polisi menggelar reka ulang kasus pembunuhan dan mutilasi pria K di Depok. Tersangka Saepul dijerat pasal pembunuhan berencana dengan ancaman hukuman mati.</t>
+        </is>
+      </c>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8613381/polisi-reka-ulang-kasus-mutilasi-pria-di-depok-saepul-dihadirkan</t>
+        </is>
+      </c>
+      <c r="H386" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/polisi-menggelar-reka-ulang-kasus-mutilasi-pria-di-depok-tersangka-saepul-ikut-dihadirkan-1786424451846_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I386" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>Sopir Travel Pembunuh Wanita di Sulsel Gasak Duit Korban Rp 62 Juta</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:01:45 +0700</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>Agung Pramono</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>Sopir mobil travel bernama Alber alias Latu (37) pelaku pembunuhan Mita (26) di Morowali, Sulawesi Tengah (Sulteng) juga menggasak uang korban.</t>
+        </is>
+      </c>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G387" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8613379/sopir-travel-pembunuh-wanita-di-sulsel-gasak-duit-korban-rp-62-juta</t>
+        </is>
+      </c>
+      <c r="H387" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/11/24/gadis-asal-wajo-paramitha-titania-anggelica-alias-mita-26-sudah-4-bulan-hilang_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I387" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>Gerakan ASRI, Brimob Polda Metro Bersihkan Sampah di Pesisir Pantai Kaligaga</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:53:58 +0700</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>Wildan Noviansah</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>Brimob Polda Metro Jaya laksanakan gerakan ASRI di Pantai Kaligaga, Jakut. Sebanyak 25 personel membereskan sampah untuk lingkungan yang lebih sehat dan nyaman.</t>
+        </is>
+      </c>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8613369/gerakan-asri-brimob-polda-metro-bersihkan-sampah-di-pesisir-pantai-kaligaga</t>
+        </is>
+      </c>
+      <c r="H388" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/brimob-polda-metro-bersihkan-sampah-di-pesisir-pantai-kaligaga-jakarta-utara-1786423926521_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>Mobil yang Ditumpangi Ditabrak Truk, Begini Kondisi Kiai Anwar Zahid</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:34:55 +0700</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>Ainur Rofiq</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>Kiai Anwar Zahid terlibat kecelakaan di Bojonegoro saat menunggu antrean. Kiai Anwar dan sopirnya selamat usai mobilnya ditabrak truk.</t>
+        </is>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G389" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8613339/mobil-yang-ditumpangi-ditabrak-truk-begini-kondisi-kiai-anwar-zahid</t>
+        </is>
+      </c>
+      <c r="H389" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/kiai-anwar-zahid-kecelakaan-di-bojonegoro-1786415552422_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I389" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>Fahira Idris Dukung Rencana TransJ Kelola Transportasi ke Kepulauan Seribu</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:33:45 +0700</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>Annisa Sekar Melati</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>Fahira Idris dukung pengalihan pengelolaan transportasi ke TransJakarta untuk Kepulauan Seribu. Dia soroti pentingnya integrasi dan keselamatan layanan.</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8613323/fahira-idris-dukung-rencana-transj-kelola-transportasi-ke-kepulauan-seribu</t>
+        </is>
+      </c>
+      <c r="H390" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/fahira-idris-puji-rencana-transj-kelola-transportasi-ke-kepulauan-seribu-1786422621769_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>Polisi Selidiki Challenge Hafalan Qur'an demi Miras Saat Konser di Jakut</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:33:17 +0700</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>Wildan Noviansah</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>Viral aksi promosi miras dengan tantangan hafalan Al-Qur'an di konser The Sounds Project. Polisi menyelidiki kejadian tersebut.</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8613322/polisi-selidiki-challenge-hafalan-quran-demi-miras-saat-konser-di-jakut</t>
+        </is>
+      </c>
+      <c r="H391" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/1144667396-1786419072166_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>Dedi Congor Jadi Tersangka Gratifikasi yang Diusut Kortas Tipikor Polri</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:20:56 +0700</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>Kortas Tipikor Polri telah menetapkan Ahmad Dedi alias Dedi Congor sebagai tersangka penerima gratifikasi berdasarkan penyidikan sejak 2023.</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8613308/dedi-congor-jadi-tersangka-gratifikasi-yang-diusut-kortas-tipikor-polri</t>
+        </is>
+      </c>
+      <c r="H392" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/07/kabag-ops-kortas-tipikor-polri-kombes-ahmad-yusuf-afandi-1783415868317_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>Jaksa KPK: Korupsi Kuota Haji Memperkaya Yaqut Rp 4,8 Miliar</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:19:22 +0700</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>Mulia Budi</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>Jaksa menyakini perkara korupsi kuota haji memperkaya Yaqut sebesar USD 271.500 atau jika dikonversi dengan kurs saat ini yakni sekitar Rp 4,8 miliar.</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G393" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8613306/jaksa-kpk-korupsi-kuota-haji-memperkaya-yaqut-rp-4-8-miliar</t>
+        </is>
+      </c>
+      <c r="H393" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/mantan-menag-yaqut-cholil-qoumas-1786417604158_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I393" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>Bukan Bunker, Ruangan di Sekolah Jaksel TKP Temuan Senjata Basemen</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:04:56 +0700</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>Wildan Noviansah</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>Polisi mengungkap isi basemen di sekolah swasta Jakarta, tempat ratusan senjata ditemukan. Penemuan ini terkait konflik internal yayasan.</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8613292/bukan-bunker-ruangan-di-sekolah-jaksel-tkp-temuan-senjata-basemen</t>
+        </is>
+      </c>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/temuan-ratusan-pucuk-senjata-di-sekolah-swasta-di-pondok-pinang-jakarta-selatan-1786014363566_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>KPK Ungkap Selisih SGD 2.000 di Amplop Bupati Kuansing untuk Menhut</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 10:19:20 +0700</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>KPK menyelidiki selisih uang SGD 2 ribu dalam amplop dari Bupati Kuansing Suhardiman Amby untuk Menteri Kehutanan Raja Juli Antoni</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8613216/kpk-ungkap-selisih-sgd-2-000-di-amplop-bupati-kuansing-untuk-menhut</t>
+        </is>
+      </c>
+      <c r="H395" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/22/jumpa-pers-kpk-1784716930554_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>Siap-siap! Magang Nasional Batch 2 Dibuka Bulan Depan</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:32:37 +0700</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>Ilyas Fadilah</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>Pemerintah akan membuka program magang nasional batch 2 tahun 2026 pada September.</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8613433/siap-siap-magang-nasional-batch-2-dibuka-bulan-depan</t>
+        </is>
+      </c>
+      <c r="H396" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/20/tampilan-siapkerja-untuk-program-magang-nasional-2026-1784528861950_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>Mendagri Siapkan 3 Skema Bayar Gaji PPPK di Daerah</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:23:59 +0700</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>Herdi Alif Al Hikam</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>Tiga skema disiapkan untuk mendukung pemerintah daerah (Pemda) dalam memenuhi pembayaran gaji Pegawai Pemerintah dengan Perjanjian Kerja (PPPK).</t>
+        </is>
+      </c>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G397" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8613419/mendagri-siapkan-3-skema-bayar-gaji-pppk-di-daerah</t>
+        </is>
+      </c>
+      <c r="H397" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/mendagri-wanti-wanti-kepala-daerah-jaga-integritas-demi-cegah-korupsi-1785894664987_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>Airlangga Kasih PR ke Maman: Kredit UMKM Harus Tembus Rp 2.000 T</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:11:51 +0700</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>Ignacio Geordi Oswaldo</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>Menteri Koordinator Perekonomian Airlangga Hartarto memberikan tugas ke Menteri UMKM untuk meningkatkan penyaluran kredit UMKM hingga Rp 2.000 triliun.</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G398" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8613404/airlangga-kasih-pr-ke-maman-kredit-umkm-harus-tembus-rp-2-000-t</t>
+        </is>
+      </c>
+      <c r="H398" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/10/menteri-koordinator-bidang-perekonomian-airlangga-hartarto-1783665254890_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I398" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>Destry Jadi Calon Tunggal Gubernur BI, 3 Pejabat Ekonomi Kompak Dukung</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:55:34 +0700</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>Heri Purnomo</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>Menteri Koordinator Perekonomian dan pejabat lainnya dukung Destry Damayanti sebagai calon Gubernur BI. Destry dinilai berpengalaman dan respons pasar positif.</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G399" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8613372/destry-jadi-calon-tunggal-gubernur-bi-3-pejabat-ekonomi-kompak-dukung</t>
+        </is>
+      </c>
+      <c r="H399" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/01/26/btn-economic-outlook-2024-1_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>Kemnaker Sebut Peserta Magang Nasional Lebih Banyak di Luar Jawa</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:53:23 +0700</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>Ilyas Fadilah</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>Kementerian Ketenagakerjaan (Kemnaker) mengungkap sebaran peserta Program Pemagangan Nasional 2026 batch 1 angkatan kedua lebih merata.</t>
+        </is>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G400" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8613368/kemnaker-sebut-peserta-magang-nasional-lebih-banyak-di-luar-jawa</t>
+        </is>
+      </c>
+      <c r="H400" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/04/14/program-magang-1776135871755_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>BPK Temukan Kelebihan Pembayaran di BSSN Meski Raih WTP</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:35:43 +0700</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>Ignacio Geordi Oswaldo</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>BPK memberikan opini WTP untuk laporan keuangan BSSN 2025, meski ditemukan kelebihan pembayaran dan rekomendasi untuk optimalisasi aset.</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G401" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8613390/bpk-temukan-kelebihan-pembayaran-di-bssn-meski-raih-wtp</t>
+        </is>
+      </c>
+      <c r="H401" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2017/05/26/0dadd724-78e9-4380-9aed-8a12fc2c4c57_169.jpg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>Gemas! Ikut Mahalini Nyanyi, Selina Joget Gak Sabar Lari ke Atas Panggung</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:30:58 +0700</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>Desi Puspasari</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>Selina, putri Mahalini dan Rizky Febian bikin gemas. Ikut Mahalini nyanyi, Selina gak bisa diam ikut joget dan mau lari ke depan penonton.</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G402" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8613331/gemas-ikut-mahalini-nyanyi-selina-joget-gak-sabar-lari-ke-atas-panggung</t>
+        </is>
+      </c>
+      <c r="H402" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/mahalini-1786422380970_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>Lesti Kejora dan Asila Maisa Jalani Pemeriksaan di Polda Metro</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:09:24 +0700</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>Febryantino Nur Pratama</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>Rizky Billar, Lesti Kejora, dan Asila Maisa diperiksa di Polda Metro Jaya terkait laporan fitnah. Mereka memberikan keterangan tambahan untuk penyidik.</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8613394/lesti-kejora-dan-asila-maisa-jalani-pemeriksaan-di-polda-metro</t>
+        </is>
+      </c>
+      <c r="H403" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/rizky-billar-lesti-kejora-dan-asilla-1786424585636_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I403" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>Poppy Sovia Idap Bipolar, Kehadiran Anak Bikin Merasa Lebih Berharga</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:25:33 +0700</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>Desi Puspasari</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>Poppy Sovia didiagnosis bipolar tipe 1 dan menemukan kekuatan hidup melalui anaknya. Dia berbagi pengalaman dan motivasi untuk yang mengalami masalah mental.</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G404" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8613085/poppy-sovia-idap-bipolar-kehadiran-anak-bikin-merasa-lebih-berharga</t>
+        </is>
+      </c>
+      <c r="H404" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/poppy-sovia-1786088545842_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I404" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>Reza Gladys Respons Berita Hoaks soal Dirinya Laporkan Suami dan Dhena Devanka atas Dugaan Perzinaan</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:32:02 +0700</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>Reza Gladys memberikan respons terkait dengan berita hoaks soal dirinya melaporkan suami dan Dhena Devanka atas dugaan perzinaan.</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7866790/reza-gladys-respons-berita-hoaks-soal-dirinya-laporkan-suami-dan-dhena-devanka-atas-dugaan-perzinaan</t>
+        </is>
+      </c>
+      <c r="H405" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/3EXsvrumltalnPf2ipCrcZrZzU4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Momen-Reza-Gladys-dan-suami-datangi-Polda-Metro-Jakarta-Selatan.jpg</t>
+        </is>
+      </c>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>Kunci Jawaban IPS Kelas 10 SMA Kurikulum Merdeka Halaman 172 Edisi Revisi: Aktivitas 3.10</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:31:20 +0700</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>Berikut ini kunci jawaban IPS kelas 10 SMA Kurikulum Merdeka Halaman  172 Edisi Revisi: Aktivitas 3.10.</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G406" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/pendidikan/7866789/kunci-jawaban-ips-kelas-10-sma-kurikulum-merdeka-halaman-172-edisi-revisi-aktivitas-310</t>
+        </is>
+      </c>
+      <c r="H406" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/DSga7wM08_0kQh0WIsFqhAjs6F8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Simak-kunci-jawaban-Informatika-Kelas-5-Halaman-139.jpg</t>
+        </is>
+      </c>
+      <c r="I406" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>Denny Sumargo Heran Agama hingga Etnisnya jadi Sasaran Hujat Gara-gara Undang Sarwendah di Podcast</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:30:02 +0700</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>Denny Sumargo kecewa agama dan etnisnya ikut disentil lantaran mengundang Sarwendah di podcastnya.</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G407" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7866788/denny-sumargo-heran-agama-hingga-etnisnya-jadi-sasaran-hujat-gara-gara-undang-sarwendah-di-podcast</t>
+        </is>
+      </c>
+      <c r="H407" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ik23waLzTdDpWPovuqWu3mZdce4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Denny-Sumargo-1-03082026.jpg</t>
+        </is>
+      </c>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>Terjemahan Lirik Lagu Bring Your Love - Madonna dan Sabrina Carpenter: Don’t Comment on My Ideas</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:28:43 +0700</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>Simak lirik dan terjemahan lagu Bring Your Love yang dibawakan oleh Madonna bersama Sabrina Carpenter.</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/musik/7866787/terjemahan-lirik-lagu-bring-your-love-madonna-sabrina-carpenter-dont-comment-on-my-ideas</t>
+        </is>
+      </c>
+      <c r="H408" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/zLN77GXG_MWcQ27NDqNvGgp-QJs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-musik-ilustrasi-lirik-ilustrasi-terjemahan-lirik-lagu.jpg</t>
+        </is>
+      </c>
+      <c r="I408" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>Trump Media Tekor 238 Juta Dolar AS, Pendapatan Cuma 1,7 Juta Dolar AS, Saham Anjlok 8 Persen</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:28:42 +0700</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>Trump Media milik Donald Trump rugi 238 juta dolar AS pada kuartal II 2026,  pendapatan hanya 1,7 juta dolar AS, saham anjlok 8 persen.</t>
+        </is>
+      </c>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G409" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7866786/trump-media-tekor-238-juta-dolar-as-pendapatan-cuma-17-juta-dolar-as-saham-anjlok-8-persen</t>
+        </is>
+      </c>
+      <c r="H409" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/pd58Lh0QZkuUPrM04LfPl7UxG4o=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/residen-AS-Donald-Trump-Senin-27-Juli-2026-Foto-Res.jpg</t>
+        </is>
+      </c>
+      <c r="I409" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>Ada Daya Pikat Legenda AC Milan, Federico Barba Ceritakan Alasannya Tinggalkan Persib</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:27:31 +0700</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>Federico Barba menyebut legenda AC Milan Pippo Inzaghi di balik keputusannya gabung Palermo dan tinggalkan Persib Bandung</t>
+        </is>
+      </c>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G410" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7866785/ada-daya-pikat-legenda-ac-milan-federico-barba-ceritakan-alasannya-tinggalkan-persib</t>
+        </is>
+      </c>
+      <c r="H410" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/5s4Zz2yN9CDSsT-6PRNcPWWt6k8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Aksi-bek-Persib-Bandung-Federico-Barba-berduel-dengan-penyerang-Madura-United-Lulinha.jpg</t>
+        </is>
+      </c>
+      <c r="I410" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>Jelang Sidang Tahunan 2026, Plt Sekjen DPR Ungkap Persiapan hingga Jadwal Acara</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:26:19 +0700</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>MPR, DPR, dan DPD, telah melakukan koordinasi untuk memastikan seluruh rangkaian kegiatan berjalan sesuai agenda.</t>
+        </is>
+      </c>
+      <c r="F411" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G411" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866784/jelang-sidang-tahunan-2026-plt-sekjen-dpr-ungkap-persiapan-hingga-jadwal-acara</t>
+        </is>
+      </c>
+      <c r="H411" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Qsn1R3WnhXiTZM5tZiOuW_dEYUI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Paripurna-DPR-RI-pada-14-Agustus.jpg</t>
+        </is>
+      </c>
+      <c r="I411" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>Doa agar Hati dan Lisan Selalu Jujur dalam Perkataan dan Perbuatan</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:23:53 +0700</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>Hati dan lisan seorang Muslim sebaiknya selalu jujur dalam perkataan dan perbuatan. Berikut doa yang dapat dibaca untuk menjaga kejujuran.</t>
+        </is>
+      </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/lifestyle/7866783/doa-agar-hati-dan-lisan-selalu-jujur-dalam-perkataan-dan-perbuatan</t>
+        </is>
+      </c>
+      <c r="H412" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/U11q51q-CJ66-8lRNT5oRv2mai4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/DOA-AGAR-JUJUR-435634543TR.jpg</t>
+        </is>
+      </c>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>Rizky Billar Santai jadi Saksi Penyebaran Hoaks Selingkuh dengan Asila Maisa, Sempat Goda Wartawan</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:23:47 +0700</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>Rizky Billar terlihat santai saat hadir di Polda Metro Jaya untuk diperiksa sebagai saksi laporan penyebaran hoaks.</t>
+        </is>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G413" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7866782/rizky-billar-santai-jadi-saksi-penyebaran-hoaks-selingkuh-dengan-asila-maisa-sempat-goda-wartawan</t>
+        </is>
+      </c>
+      <c r="H413" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/78EbReGI5C4Aj-1k0Orok3S4lnk=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Rizky-Billar-1-31072026.jpg</t>
+        </is>
+      </c>
+      <c r="I413" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>Gempa M 7,4 Porak-porandakan Kolombia, Darurat Nasional Diberlakukan, Korban Tewas Tembus 110 Jiwa</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:23:03 +0700</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>Gempa M 7,4 guncang Kolombia, menewaskan lebih dari 110 orang. Presiden tetapkan darurat nasional, sementara bantuan internasional mulai berdatangan.</t>
+        </is>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G414" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7866781/gempa-m-74-porak-porandakan-kolombia-darurat-nasional-diberlakukan-korban-tewas-tembus-110-jiwa</t>
+        </is>
+      </c>
+      <c r="H414" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/URaiCze4k2TRjD74O4lopRgG6kY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/PRESIDEN-KOLOMBIA-Presiden-Kolombia-yang-baru-dilantik-Abelardo-de-la-Espriella.jpg</t>
+        </is>
+      </c>
+      <c r="I414" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>Jadwal Acara TV Rabu, 12 Agustus 2026: FYP TRANS 7 dan Cipung Abubu Mentari TV</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:22:39 +0700</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>Simak jadwal acara TV besok Rabu 12 Agustus 2026 terdapat tayangan FYP di TRANS 7 dan Cipung Abubu di Mentari TV.</t>
+        </is>
+      </c>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G415" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7866780/jadwal-acara-tv-rabu-12-agustus-2026-fyp-trans-7-dan-cipung-abubu-mentari-tv</t>
+        </is>
+      </c>
+      <c r="H415" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/H5aLayjCy83MjA-P9TOjSo-_9Qw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ILUSTRASI-TELEVISI-3.jpg</t>
+        </is>
+      </c>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>Seskab Teddy Klaim 30–40 Persen Peserta MagangHub Langsung Kerja, Bagaimana Nasib 60 Persen Lainnya?</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:22:04 +0700</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>Perusahaan cenderung memilih merekrut peserta magang karena mereka telah dibekali keterampilan spesifik selama program berlangsung.</t>
+        </is>
+      </c>
+      <c r="F416" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G416" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866779/seskab-teddy-klaim-3040-persen-peserta-maganghub-langsung-kerja-bagaimana-nasib-60-persen-lainnya</t>
+        </is>
+      </c>
+      <c r="H416" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/monSidTVNgFKT-jHJHuzX_ZIV8c=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/maganghub-klaim-seskab.jpg</t>
+        </is>
+      </c>
+      <c r="I416" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>Yaqut Berjabat Tangan dengan Dua Terdakwa Kasus Korupsi Kuota Haji di Persidangan</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:20:56 +0700</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>Yaqut Cholil Qoumas menjalani sidang dakwaan kasus dugaan korupsi kuota haji, di Pengadilan Tipikor Jakarta Pusat, Selasa (11/8/2026).</t>
+        </is>
+      </c>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G417" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866778/yaqut-berjabat-tangan-dengan-dua-terdakwa-kasus-korupsi-kuota-haji-di-persidangan</t>
+        </is>
+      </c>
+      <c r="H417" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/U3akHItL4FpftqwfKv77oXWMCOk=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/kasus-tersebut-di-Pengadilan-Tipi.jpg</t>
+        </is>
+      </c>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>Mengenal Definisi Hantavirus, Perhatikan Gejala dan Faktor Penularannya</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:20:49 +0700</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>Hantavirus menjadi perhatian karena dapat menular melalui paparan hewan pengerat seperti tikus, berikut gejala, resiko hingga faktor penularannya.</t>
+        </is>
+      </c>
+      <c r="F418" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G418" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7866777/mengenal-definisi-hantavirus-perhatikan-gejala-dan-faktor-penularannya</t>
+        </is>
+      </c>
+      <c r="H418" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/XGOK4B92fWuE_P0GM7lWTImkJRU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/CEK-KESEHATAN-Warga-lansia-di-Kelurahan-Purwantoro.jpg</t>
+        </is>
+      </c>
+      <c r="I418" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>Kunci Jawaban IPS Kelas 10 SMA Kurikulum Merdeka Halaman 167 Edisi Revisi: Aktivitas 3.9</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:17:48 +0700</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>Berikut ini kunci jawaban IPS kelas 10 SMA Kurikulum Merdeka Halaman 167 Edisi Revisi: Aktivitas 3.9.</t>
+        </is>
+      </c>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G419" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/pendidikan/7866776/kunci-jawaban-ips-kelas-10-sma-kurikulum-merdeka-halaman-167-edisi-revisi-aktivitas-39</t>
+        </is>
+      </c>
+      <c r="H419" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/U9U0Ezm2sPloSaaCbS7kqX3m2cw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/suasana-hari-pertama-pembelajaran-tatap-muka-ptm-terbatas-di-kota-bogor-senin-18102021.jpg</t>
+        </is>
+      </c>
+      <c r="I419" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>Edarkan Ribuan Butir Tramadol dan Eximer, Tiga Pria di Kelapa Dua Tangerang Ditangkap Polisi</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:17:27 +0700</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>Polsek Kelapa Dua ringkus tiga pria edarkan obat keras daftar G tanpa resep, ribuan butir tramadol dan eximer disita.</t>
+        </is>
+      </c>
+      <c r="F420" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G420" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7866775/edarkan-ribuan-butir-tramadol-dan-eximer-tiga-pria-di-kelapa-dua-tangerang-ditangkap-polisi</t>
+        </is>
+      </c>
+      <c r="H420" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/v9i6ibfO1bPc8YJ_o5Lf68tR8ys=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Sejumlah-barang-bukti-berupa-ribuan-butir-obat-keras-daftar-G-jenis-Tramadol-dan-Eximer.jpg</t>
+        </is>
+      </c>
+      <c r="I420" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>Sidang Korupsi Kuota Haji, Eks Menag Yaqut Didakwa Memperkaya Diri USD 271.500</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:15:48 +0700</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>Yaqut Cholil Qoumas didakwa memperkaya diri sejumlah USD 271.500 atas pengisian kuota haji khusus tambahan periode tahun 2023 dan 2024.</t>
+        </is>
+      </c>
+      <c r="F421" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G421" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866774/sidang-korupsi-kuota-haji-eks-menag-yaqut-didakwa-memperkaya-diri-usd-271500</t>
+        </is>
+      </c>
+      <c r="H421" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/0ngnyDDP7c9zEA8b30Lkx2Qud2o=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Yaqut-Cholil-Qoumas-DIDAKWA-RUGIKAN-NEGARA-622-miliar.jpg</t>
+        </is>
+      </c>
+      <c r="I421" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>Awal Mula Kasus Penyekapan Berujung Tewasnya Handi, 4 Lokasi Kejadian hingga 8 Orang Jadi Tersangka</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:15:32 +0700</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>Saat ditemukan, Handi berada dalam kondisi kaki terikat menggunakan kawat dan mengalami sejumlah luka.</t>
+        </is>
+      </c>
+      <c r="F422" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G422" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7866773/awal-mula-kasus-penyekapan-berujung-tewasnya-handi-4-lokasi-kejadian-hingga-8-orang-jadi-tersangka</t>
+        </is>
+      </c>
+      <c r="H422" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/A1YYPLRilH3I4xpPq3AfPCEpo4M=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/PENYEKAPAN-sumedang.jpg</t>
+        </is>
+      </c>
+      <c r="I422" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>Beda Sikap dengan US Soccer, Trump Bela Infantino: Ganti Presiden FIFA Kesalahan Besar</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:10:59 +0700</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>Presiden Amerika Serikat Donal Trump memberi pembelaan terhadap Gianni Infantino yang mendapat desakan untuk mundur dari jabatan Presiden FIFA.</t>
+        </is>
+      </c>
+      <c r="F423" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G423" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7866772/beda-sikap-dengan-us-soccer-trump-bela-infantino-ganti-presiden-fifa-kesalahan-besar</t>
+        </is>
+      </c>
+      <c r="H423" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/jJtKQdQXUic7dMeq4jn1wIzwv74=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Gianni-Infantino-bersama-dengan-Donald-Trump.jpg</t>
+        </is>
+      </c>
+      <c r="I423" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>Andrey Santos Siap Gantikan Casemiro di Manchester United: Saya Bisa Lakukan Seperti Dia</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:10:36 +0700</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>Andrey Santos siap menjadi penerus Casemiro di Manchester United. Tampil impresif di pramusim, bertekad bertahan lama di Old Trafford.</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7866771/andrey-santos-siap-gantikan-casemiro-di-manchester-united-saya-bisa-lakukan-seperti-dia</t>
+        </is>
+      </c>
+      <c r="H424" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/AlltmgB8FC-kPtqdF1B1kPc6drs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Aksi-gelandang-anyar-Manchester-United-Andrey-Santos-saat-melawan-PSG.jpg</t>
+        </is>
+      </c>
+      <c r="I424" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>Bisnis</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>Kemenko Polkam, BSSN, dan Telkom Perkuat Kolaborasi Hadapi Ancaman Era Komputasi Kuantum</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:44:15 +0700</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>Ferry kisihandi</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- Pemerintah mulai mempercepat langkah antisipasi menghadapi potensi ancaman keamanan siber seiring perkembangan teknologi komputasi kuantum. 
+Melalui Rapat Koordinasi Urgensi Penyusunan Kebijakan Menghadapi Post-Quantum Computing (PQC), Kamis...</t>
+        </is>
+      </c>
+      <c r="F425" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G425" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjl95r472/kemenko-polkam-bssn-dan-telkom-perkuat-kolaborasi-hadapi-ancaman-era-komputasi-kuantum</t>
+        </is>
+      </c>
+      <c r="H425" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/upaya-memperkuar-sinergi-untuk-menyiapkan-diri-menghadapi-era-pascakuantum_260811114246-855.jpeg</t>
+        </is>
+      </c>
+      <c r="I425" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>Finansial</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>Rupiah Dibuka Melemah 40 Poin Jadi Rp 17.795 per Dolar AS</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:26:38 +0700</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>Gita Amanda</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- Analis mata uang Doo Financial Futures Lukman Leong mengatakan rupiah melemah seiring ketidakpastian geopolitik di Timur Tengah (Timteng). Nilai tukar rupiah terhadap dolar Amerika Serikat (AS) pada pembukaan...</t>
+        </is>
+      </c>
+      <c r="F426" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G426" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjl8ce423/rupiah-dibuka-melemah-40-poin-jadi-rp-17795-per-dolar-as</t>
+        </is>
+      </c>
+      <c r="H426" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/011418000-1780675525-830-556.jpg</t>
+        </is>
+      </c>
+      <c r="I426" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>Infografis Guncang Gempa Kolombia Terkuat Abad Ini</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:44:59 +0700</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>Gempa M7,4 mengguncang Kolombia dan terasa hingga Ekuador.</t>
+        </is>
+      </c>
+      <c r="F427" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G427" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266944/infografis-guncang-gempa-kolombia-terkuat-abad-ini</t>
+        </is>
+      </c>
+      <c r="H427" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/nHHr6ML2g-DBv-fwJmf1AcPgM6U=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9321075/original/010300900_1786426972-45b224e2-a441-426f-bc27-2b77c0ef6b28.jpg</t>
+        </is>
+      </c>
+      <c r="I427" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>Istri Eks Menag Yaqut Hadiri Sidang, Bawa Bantal untuk Suami</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:43:00 +0700</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>Istri mantan Menteri Agama (Menag) Yaqut Cholil Qoumas, Eny Retno turut hadir dalam sidang perdana.</t>
+        </is>
+      </c>
+      <c r="F428" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G428" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266943/istri-eks-menag-yaqut-hadiri-sidang-bawa-bantal-untuk-suami</t>
+        </is>
+      </c>
+      <c r="H428" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/r2EHAFjxKLsUOBdFY3Xr4BeVjMs=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9321074/original/094101400_1786426954-IMG_20260811_094900_510.jpg</t>
+        </is>
+      </c>
+      <c r="I428" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>Terungkap Isi Ruangan yang Disebut Bunker Sekolah Jaksel</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:43:30 +0700</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>Ruangan itu dipastikan bukan bunker, hanya basement yang terhubung dengan sejumlah ruangan.</t>
+        </is>
+      </c>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G429" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266939/terungkap-isi-ruangan-yang-disebut-bunker-sekolah-jaksel</t>
+        </is>
+      </c>
+      <c r="H429" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/DZ4ufKYVxSrVZgr_zDmvYxBWPZc=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9321073/original/094190400_1786426911-WhatsApp_Image_2026-08-11_at_12.40.02.jpeg</t>
+        </is>
+      </c>
+      <c r="I429" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>Viral Challenge Hafalan Al-Qur'an Berhadiah Miras, Polisi Mulai Selidiki</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:20:59 +0700</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>Video dugaan challenge hafalan Al-Qur'an berhadiah minuman keras di booth sponsor The Sounds Project viral dan menuai kecaman. Polisi kini menyelidikinya.</t>
+        </is>
+      </c>
+      <c r="F430" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G430" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266923/viral-challenge-hafalan-al-quran-berhadiah-miras-polisi-mulai-selidiki</t>
+        </is>
+      </c>
+      <c r="H430" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/Fp5iC-vppn7dJSzwqGEBlrLz0gY=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9321055/original/059736500_1786425649-Jepretan_Layar_2025-08-11_pukul_12.15.34.jpg</t>
+        </is>
+      </c>
+      <c r="I430" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>Di Depan Hakim, Yaqut Ungkap Kondisi Kesehatannya Pascaoperasi</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:13:30 +0700</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>Yaqut sempat dibantarkan karena ada masalah kesehatan di pencernaan.</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266912/di-depan-hakim-yaqut-ungkap-kondisi-kesehatannya-pascaoperasi</t>
+        </is>
+      </c>
+      <c r="H431" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/nWrXsW3scvrby34Pqt9_kl75l98=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9320896/original/035022100_1786418319-IMG-20260811-WA0012.jpg</t>
+        </is>
+      </c>
+      <c r="I431" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>Polisi Cari Jejak di Balik 30 Item Senjata di Sekolah Jaksel</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:08:18 +0700</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>Puslabfor mengambil sampel DNA untuk menelusuri jejak orang di lokasi.</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G432" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266907/polisi-cari-jejak-di-balik-30-item-senjata-di-sekolah-jaksel</t>
+        </is>
+      </c>
+      <c r="H432" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/Fl_NzWIZKKZEWAlAQ_ZHoXsZU5g=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9317547/original/022307300_1786020542-WhatsApp_Image_2026-08-06_at_19.28.11.jpeg</t>
+        </is>
+      </c>
+      <c r="I432" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>Warga Teriak Saat Mobil Bupati Lampung Selatan Terjebak Jalan Rusak, 'Jangan Janji Saja'</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:03:32 +0700</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>Bupati Egi mengaku tak menyangka jalanan di Lampung Selatan rusak separah itu.</t>
+        </is>
+      </c>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G433" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266901/warga-teriak-saat-mobil-bupati-lampung-selatan-terjebak-jalan-rusak-jangan-janji-saja</t>
+        </is>
+      </c>
+      <c r="H433" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/mm_wGjwpk26oXordrwSB0W3gYec=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9321037/original/009420000_1786424605-1001541253.jpg</t>
+        </is>
+      </c>
+      <c r="I433" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>Yaqut Didakwa Rugikan Negara Rp 662 Miliar</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:48:46 +0700</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>Yaqut disebut melakukan pelanggaran hukum secara bersama-sama dengan pihak lain.</t>
+        </is>
+      </c>
+      <c r="F434" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G434" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266885/yaqut-didakwa-rugikan-negara-rp-662-miliar</t>
+        </is>
+      </c>
+      <c r="H434" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/eYPEhafi5n-DU_gVv0slO1l2gbc=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9321012/original/036331400_1786423717-IMG-20260811-WA0043.jpg</t>
+        </is>
+      </c>
+      <c r="I434" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>Eks Kepala Bea Cukai Marunda Jadi Tersangka Gratifikasi</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:25:31 +0700</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>Ahmad Dedi diduga menerima hadiah atau janji dalam periode 2008 hingga 2016.</t>
+        </is>
+      </c>
+      <c r="F435" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G435" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266862/eks-kepala-bea-cukai-marunda-jadi-tersangka-gratifikasi</t>
+        </is>
+      </c>
+      <c r="H435" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/2qXbWmSS5nvoujQVDkZ55lzxOSI=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9320991/original/042546300_1786422321-WhatsApp_Image_2026-08-11_at_11.24.27.jpeg</t>
+        </is>
+      </c>
+      <c r="I435" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>Puslabfor Kembali Periksa Sekolah di Jaksel, 30 Barang Dibawa</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:09:09 +0700</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>Pemeriksaan ulang Puslabfor mengungkap puluhan item terkait senjata di sekolah.</t>
+        </is>
+      </c>
+      <c r="F436" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G436" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8266793/puslabfor-kembali-periksa-sekolah-di-jaksel-30-barang-dibawa</t>
+        </is>
+      </c>
+      <c r="H436" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/CtM5XDTHJfKJmDzpcb6YMTVMeWI=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9317273/original/093250400_1786008225-1001014569.jpg</t>
+        </is>
+      </c>
+      <c r="I436" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>Daftar 28 Nama yang Diperkaya dalam Kasus Kuota Haji: Yaqut hingga 313 PIHK</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:48:20 +0700</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>Akibat perbuatan Yaqut dalam kasus korupsi kuota haji khusus, jaksa menyebut negara mengalami kerugian sebesar Rp 622.090.207.166,41.</t>
+        </is>
+      </c>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G437" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/08/11/12475941/daftar-28-nama-yang-diperkaya-dalam-kasus-kuota-haji-yaqut-hingga-313-pihk</t>
+        </is>
+      </c>
+      <c r="H437" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/bDSWiJQj25iIcI4EcSynE7cq6Eo=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/11/6a7a8ccf063f1.jpg</t>
+        </is>
+      </c>
+      <c r="I437" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>Tercatat Ada 1.070 Hotspot Selama 2026, Polda Lampung Siaga Karhutla dan Kekeringan</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:48:20 +0700</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>Polda Lampung memperkuat kesiapsiagaan menghadapi karhutla serta dampak kekeringan di musim kemarau.</t>
+        </is>
+      </c>
+      <c r="F438" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G438" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/08/11/123113378/tercatat-ada-1070-hotspot-selama-2026-polda-lampung-siaga-karhutla-dan</t>
+        </is>
+      </c>
+      <c r="H438" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/mzFOfTGi1fZ7KOFZqTqHfk_pY1s=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/11/6a7a99376603c.jpg</t>
+        </is>
+      </c>
+      <c r="I438" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>Sepekan Jelang HUT RI, Semarak Pernak-pernik Kemerdekaan Penuhi Pasar Jatinegara Jaktim</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:48:20 +0700</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>Di Pasar Jatinegara, sejumlah pembeli terlihat mencari perlengkapan untuk kegiatan kemerdekaan, mulai dari ibu-ibu, anggota PKK, hingga karyawan.</t>
+        </is>
+      </c>
+      <c r="F439" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G439" t="inlineStr">
+        <is>
+          <t>https://megapolitan.kompas.com/read/2026/08/11/12110571/sepekan-jelang-hut-ri-semarak-pernak-pernik-kemerdekaan-penuhi-pasar</t>
+        </is>
+      </c>
+      <c r="H439" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/6ffdo7dCnX1i0lTqKS39TsPlH8M=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/11/6a7a8f1d70649.jpeg</t>
+        </is>
+      </c>
+      <c r="I439" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I335"/>
+  <autoFilter ref="A1:I439"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-11 08:06 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-11.xlsx
+++ b/data/berita_2026-08-11.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$581</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$685</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I581"/>
+  <dimension ref="A1:I685"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -27743,8 +27743,4898 @@
         </is>
       </c>
     </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>Bulog Sumut pastikan penyaluran bantuan pangan 1,73 juta KPM pekan ini</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 15:01:20 +0700</t>
+        </is>
+      </c>
+      <c r="D582" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E582" t="inlineStr">
+        <is>
+          <t>Perum Bulog Kantor Wilayah Sumatera Utara memastikan penyaluran bantuan pangan berupa beras kepada 1,73 juta keluarga ...</t>
+        </is>
+      </c>
+      <c r="F582" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G582" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689076/bulog-sumut-pastikan-penyaluran-bantuan-pangan-173-juta-kpm-pekan-ini</t>
+        </is>
+      </c>
+      <c r="H582" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG-20260811-WA0104.jpg</t>
+        </is>
+      </c>
+      <c r="I582" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>Bagaimana olahraga bisa membantu mengurangi stres?</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 15:00:53 +0700</t>
+        </is>
+      </c>
+      <c r="D583" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E583" t="inlineStr">
+        <is>
+          <t>Stres menjadi bagian yang cukup umum dalam kehidupan sehari-hari. Tuntutan pekerjaan, tugas sekolah, masalah keluarga, ...</t>
+        </is>
+      </c>
+      <c r="F583" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G583" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689075/bagaimana-olahraga-bisa-membantu-mengurangi-stres</t>
+        </is>
+      </c>
+      <c r="H583" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/05/27/pexels-marcus-aurelius-6787161.jpg</t>
+        </is>
+      </c>
+      <c r="I583" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>BI: Industri pengolahan jadi penopang ekonomi Jateng</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:59:29 +0700</t>
+        </is>
+      </c>
+      <c r="D584" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E584" t="inlineStr">
+        <is>
+          <t>Kantor Perwakilan Bank Indonesia Provinsi Jawa Tengah menyebutkan bahwa industri pengolahan dan perdagangan menjadi ...</t>
+        </is>
+      </c>
+      <c r="F584" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G584" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689073/bi-industri-pengolahan-jadi-penopang-ekonomi-jateng</t>
+        </is>
+      </c>
+      <c r="H584" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1001967856.jpg</t>
+        </is>
+      </c>
+      <c r="I584" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>OJK tanggapi wacana Masjid Istiqlal masuk Bursa lewat wakaf produktif</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:58:28 +0700</t>
+        </is>
+      </c>
+      <c r="D585" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E585" t="inlineStr">
+        <is>
+          <t>Kepala Eksekutif Pengawas Pasar Modal, Keuangan Derivatif, dan Bursa Karbon Otoritas Jasa Keuangan (OJK) Hasan Fawzi ...</t>
+        </is>
+      </c>
+      <c r="F585" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G585" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689071/ojk-tanggapi-wacana-masjid-istiqlal-masuk-bursa-lewat-wakaf-produktif</t>
+        </is>
+      </c>
+      <c r="H585" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/WhatsApp-Image-2026-08-11-at-13.30.14_1.jpeg</t>
+        </is>
+      </c>
+      <c r="I585" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>Pemkab Situbondo bikin terobosan KSP Wisata Bahari Pasir Putih</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:58:25 +0700</t>
+        </is>
+      </c>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E586" t="inlineStr">
+        <is>
+          <t>Pemerintah Kabupaten Situbondo, Jawa Timur, membuat terobosan baru yakni Kerja Sama Pemanfaatan (KSP) Wisata Bahari ...</t>
+        </is>
+      </c>
+      <c r="F586" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G586" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689068/pemkab-situbondo-bikin-terobosan-ksp-wisata-bahari-pasir-putih</t>
+        </is>
+      </c>
+      <c r="H586" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/MG_9998.jpg</t>
+        </is>
+      </c>
+      <c r="I586" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>DPR gelar rapat dengan pemerintah-KPA bahas konflik agraria mendesak</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:58:10 +0700</t>
+        </is>
+      </c>
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E587" t="inlineStr">
+        <is>
+          <t>Pimpinan DPR RI menggelar rapat koordinasi dengan lintas kementerian dari pemerintah bersama Konsorsium Pembaruan ...</t>
+        </is>
+      </c>
+      <c r="F587" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G587" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689065/dpr-gelar-rapat-dengan-pemerintah-kpa-bahas-konflik-agraria-mendesak</t>
+        </is>
+      </c>
+      <c r="H587" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1001303394.jpg</t>
+        </is>
+      </c>
+      <c r="I587" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>Conor Benn yakin bungkam Garcia untuk rebut sabuk kelas welter WBC</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:58:05 +0700</t>
+        </is>
+      </c>
+      <c r="D588" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E588" t="inlineStr">
+        <is>
+          <t>Petinju Conor Benn optimistis membungkam Ryan Garcia untuk merebut sabuk juara dunia kelas welter (66,7 kg) World ...</t>
+        </is>
+      </c>
+      <c r="F588" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G588" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689064/conor-benn-yakin-bungkam-garcia-untuk-rebut-sabuk-kelas-welter-wbc</t>
+        </is>
+      </c>
+      <c r="H588" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/00f43e67-8d28-4e2a-a624-edb8baf90f74.jpeg</t>
+        </is>
+      </c>
+      <c r="I588" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>Musim Mas dan Pemkab Deli Serdang Resmikan Alun-Alun Percut Sei Tuan, Hadirkan Ruang Publik untuk Masyarakat dan UMKM</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:57:08 +0700</t>
+        </is>
+      </c>
+      <c r="D589" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E589" t="inlineStr">
+        <is>
+          <t>Masyarakat Kecamatan Percut Sei Tuan kini memiliki ruang publik baru yang dapat dimanfaatkan sebagai tempat ...</t>
+        </is>
+      </c>
+      <c r="F589" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G589" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689060/musim-mas-dan-pemkab-deli-serdang-resmikan-alun-alun-percut-sei-tuan-hadirkan-ruang-publik-untuk-masyarakat-dan-umkm</t>
+        </is>
+      </c>
+      <c r="H589" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/Musim-Mas-dan-Pemerintah-Deli-Serdang.jpg</t>
+        </is>
+      </c>
+      <c r="I589" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>Undangan HUT RI mulai dikirim ke mantan presiden dan wapres</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:57:01 +0700</t>
+        </is>
+      </c>
+      <c r="D590" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E590" t="inlineStr">
+        <is>
+          <t>Menteri Sekretaris Negara Prasetyo Hadi mengatakan panitia HUT Ke-81 Kemerdekaan Republik Indonesia mulai mengantarkan ...</t>
+        </is>
+      </c>
+      <c r="F590" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G590" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689056/undangan-hut-ri-mulai-dikirim-ke-mantan-presiden-dan-wapres</t>
+        </is>
+      </c>
+      <c r="H590" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG_3748.jpeg</t>
+        </is>
+      </c>
+      <c r="I590" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>Kolombia tetapkan status bencana nasional usai gempa magnitudo 7,4</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:55:53 +0700</t>
+        </is>
+      </c>
+      <c r="D591" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E591" t="inlineStr">
+        <is>
+          <t>Otoritas Kolombia menetapkan status bencana nasional menyusul gempa dahsyat yang mengguncang negara tersebut pada Senin ...</t>
+        </is>
+      </c>
+      <c r="F591" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G591" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689052/kolombia-tetapkan-status-bencana-nasional-usai-gempa-magnitudo-74</t>
+        </is>
+      </c>
+      <c r="H591" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/thumbs_b_c_e726e95b76c6f0cd719dcf122fc06d02.jpg</t>
+        </is>
+      </c>
+      <c r="I591" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>DeTect Dapatkan Kontrak Untuk Memasok MERLIN™ True3D® Bird Detection Radar ke Bandara Soekarno-Hatta Jakarta</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:54:35 +0700</t>
+        </is>
+      </c>
+      <c r="D592" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E592" t="inlineStr">
+        <is>
+          <t>DeTect, Inc. mendapatkan kontrak untuk memasok MERLIN 7360 True3D Bird Detection Radar ke Bandara Soekarno-Hatta ...</t>
+        </is>
+      </c>
+      <c r="F592" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G592" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689051/detect-dapatkan-kontrak-untuk-memasok-merlin-true3d-bird-detection-radar-ke-bandara-soekarno-hatta-jakarta</t>
+        </is>
+      </c>
+      <c r="H592" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/MERLIN-True3D-Bird-Detection.jpg</t>
+        </is>
+      </c>
+      <c r="I592" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>Tips memulai "running routine" untuk Anda yang pekerja kantoran</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:54:16 +0700</t>
+        </is>
+      </c>
+      <c r="D593" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E593" t="inlineStr">
+        <is>
+          <t>Kesibukan bekerja dari pagi hingga sore sering membuat aktivitas fisik menjadi hal yang mudah ditunda. Duduk berjam-jam ...</t>
+        </is>
+      </c>
+      <c r="F593" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G593" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689047/tips-memulai-running-routine-untuk-anda-yang-pekerja-kantoran</t>
+        </is>
+      </c>
+      <c r="H593" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2022/04/07/running-gefdf2d723_1280.jpg</t>
+        </is>
+      </c>
+      <c r="I593" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>Danantara targetkan groundbreaking PSEL di Yogyakarta pada akhir 2026</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:53:14 +0700</t>
+        </is>
+      </c>
+      <c r="D594" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E594" t="inlineStr">
+        <is>
+          <t>Badan Pengelola Investasi Daya Anagata Nusantara (Danantara) menargetkan peletakan batu pertama atau groundbreaking ...</t>
+        </is>
+      </c>
+      <c r="F594" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G594" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689045/danantara-targetkan-groundbreaking-psel-di-yogyakarta-pada-akhir-2026</t>
+        </is>
+      </c>
+      <c r="H594" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG_20260811_135515.jpg</t>
+        </is>
+      </c>
+      <c r="I594" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>Tim gabungan Bea Cukai Langsa gagalkan penyelundupan sepeda motor</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:52:58 +0700</t>
+        </is>
+      </c>
+      <c r="D595" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E595" t="inlineStr">
+        <is>
+          <t>Tim gabungan Bea Cukai Langsa bersama Bea Cukai Medan menggagalkan penyelundupan sepeda motor besar atau moge beserta ...</t>
+        </is>
+      </c>
+      <c r="F595" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G595" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689044/tim-gabungan-bea-cukai-langsa-gagalkan-penyelundupan-sepeda-motor</t>
+        </is>
+      </c>
+      <c r="H595" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/sepeda-motor-selundupan.jpg</t>
+        </is>
+      </c>
+      <c r="I595" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>DPR minta pemerintah siapkan pelatihan bagi pengemudi ojol</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:52:39 +0700</t>
+        </is>
+      </c>
+      <c r="D596" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E596" t="inlineStr">
+        <is>
+          <t>Wakil Ketua Komisi VII DPR RI Chusnunia meminta pemerintah menindaklanjuti penetapan pengemudi ojek daring (ojek ...</t>
+        </is>
+      </c>
+      <c r="F596" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G596" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689040/dpr-minta-pemerintah-siapkan-pelatihan-bagi-pengemudi-ojol</t>
+        </is>
+      </c>
+      <c r="H596" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/25/1003229188.jpg</t>
+        </is>
+      </c>
+      <c r="I596" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>Yaqut didakwa rugikan negara Rp622 miliar di kasus korupsi kuota haji</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:51:21 +0700</t>
+        </is>
+      </c>
+      <c r="D597" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E597" t="inlineStr">
+        <is>
+          <t>Menteri Agama periode 2020-2024 Yaqut Cholil Qoumas didakwa merugikan keuangan negara senilai Rp622,09 miliar terkait ...</t>
+        </is>
+      </c>
+      <c r="F597" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G597" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689037/yaqut-didakwa-rugikan-negara-rp622-miliar-di-kasus-korupsi-kuota-haji</t>
+        </is>
+      </c>
+      <c r="H597" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/sidang-dakwaan-yaqut-110826-bay-4A.jpg</t>
+        </is>
+      </c>
+      <c r="I597" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>Wamenekraf: Masuknya gim global buka peluang kembangkan talenta lokal</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:50:17 +0700</t>
+        </is>
+      </c>
+      <c r="D598" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E598" t="inlineStr">
+        <is>
+          <t>Wakil Menteri Ekonomi Kreatif Irene Umar mengatakan kehadiran perusahaan gim global resmi di pasar gim Indonesia ...</t>
+        </is>
+      </c>
+      <c r="F598" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G598" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689033/wamenekraf-masuknya-gim-global-buka-peluang-kembangkan-talenta-lokal</t>
+        </is>
+      </c>
+      <c r="H598" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1000457405.jpg</t>
+        </is>
+      </c>
+      <c r="I598" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>PKK Cilegon beri pendampingan door to door ke UMKM agar naik kelas</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:49:42 +0700</t>
+        </is>
+      </c>
+      <c r="D599" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E599" t="inlineStr">
+        <is>
+          <t>ANTARA - Ketua Tim Penggerak Pemberdayaan Kesejahteraan Keluarga (PKK) Kota Cilegon, Alfi Rizki Aghnia Robinsar bersama ...</t>
+        </is>
+      </c>
+      <c r="F599" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G599" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5688977/pkk-cilegon-beri-pendampingan-door-to-door-ke-umkm-agar-naik-kelas</t>
+        </is>
+      </c>
+      <c r="H599" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Screenshot-2026-08-11-142520.jpg</t>
+        </is>
+      </c>
+      <c r="I599" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>Seskab Teddy tegaskan dukungan Presiden Prabowo pada Magang Nasional</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:49:34 +0700</t>
+        </is>
+      </c>
+      <c r="D600" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E600" t="inlineStr">
+        <is>
+          <t>Sekretaris Kabinet Teddy Indra Wijaya menegaskan dukungan Presiden Prabowo Subianto kepada Program Magang ...</t>
+        </is>
+      </c>
+      <c r="F600" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G600" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689032/seskab-teddy-tegaskan-dukungan-presiden-prabowo-pada-magang-nasional</t>
+        </is>
+      </c>
+      <c r="H600" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG_7901.jpg</t>
+        </is>
+      </c>
+      <c r="I600" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>Tiket Eras Tour Swift sempat jadi sandera uang tebusan oleh peretas</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:49:08 +0700</t>
+        </is>
+      </c>
+      <c r="D601" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E601" t="inlineStr">
+        <is>
+          <t>Tiket "Eras Tour" bintang pop dunia Taylor Swift sempat menjadi sandera untuk uang tebusan operasi kejahatan ...</t>
+        </is>
+      </c>
+      <c r="F601" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G601" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689031/tiket-eras-tour-swift-sempat-jadi-sandera-uang-tebusan-oleh-peretas</t>
+        </is>
+      </c>
+      <c r="H601" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/06/01/taylor-swift-1a.jpg</t>
+        </is>
+      </c>
+      <c r="I601" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>Kapan waktu yang tepat untuk mengganti pakaian?</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:48:55 +0700</t>
+        </is>
+      </c>
+      <c r="D602" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E602" t="inlineStr">
+        <is>
+          <t>Mengganti pakaian secara rutin penting untuk menjaga kebersihan tubuh dan kesehatan kulit. Namun, frekuensinya tidak ...</t>
+        </is>
+      </c>
+      <c r="F602" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G602" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689028/kapan-waktu-yang-tepat-untuk-mengganti-pakaian</t>
+        </is>
+      </c>
+      <c r="H602" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/01/24/cuci.jpg</t>
+        </is>
+      </c>
+      <c r="I602" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>Jorge Martin tak peduli gelar juara dunia</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:48:43 +0700</t>
+        </is>
+      </c>
+      <c r="D603" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E603" t="inlineStr">
+        <is>
+          <t>Pembalap Aprilia Racing Jorge Martin tidak peduli dengan gelar juara dunia MotoGP.
+"Saya sudah menjadi ...</t>
+        </is>
+      </c>
+      <c r="F603" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G603" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689025/jorge-martin-tak-peduli-gelar-juara-dunia</t>
+        </is>
+      </c>
+      <c r="H603" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/12/Report-MGP-GP-FR.jpeg</t>
+        </is>
+      </c>
+      <c r="I603" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>Komisi II sambut baik kebijakan pemerintah cegah PPPK dirumahkan</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:45:50 +0700</t>
+        </is>
+      </c>
+      <c r="D604" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E604" t="inlineStr">
+        <is>
+          <t>Ketua Komisi II DPR RI Rifqinizamy Karsayuda menyambut baik kebijakan pemerintah untuk mencegah Pegawai Pemerintah ...</t>
+        </is>
+      </c>
+      <c r="F604" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G604" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689024/komisi-ii-sambut-baik-kebijakan-pemerintah-cegah-pppk-dirumahkan</t>
+        </is>
+      </c>
+      <c r="H604" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/15/raker-komisi-ii-dpr-dengan-pemerintah-2821844.jpg</t>
+        </is>
+      </c>
+      <c r="I604" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>Temuan senjata di sekolah, polisi cocokkan data dan barang bukti</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:45:48 +0700</t>
+        </is>
+      </c>
+      <c r="D605" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E605" t="inlineStr">
+        <is>
+          <t>Pihak kepolisian telah melakukan pengecekan tambahan, yakni pencocokan data dan barang bukti senjata di sebuah sekolah ...</t>
+        </is>
+      </c>
+      <c r="F605" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G605" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689021/temuan-senjata-di-sekolah-polisi-cocokkan-data-dan-barang-bukti</t>
+        </is>
+      </c>
+      <c r="H605" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG_20260630_094425.jpg</t>
+        </is>
+      </c>
+      <c r="I605" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>Pemerintah finalisasi Pepres tentang ojol, lengkapi sejumlah formula</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:45:44 +0700</t>
+        </is>
+      </c>
+      <c r="D606" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E606" t="inlineStr">
+        <is>
+          <t>Pemerintah tengah melakukan finalisasi Peraturan Presiden (perpres) yang mengatur ekosistem transportasi daring terkait ...</t>
+        </is>
+      </c>
+      <c r="F606" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G606" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689020/pemerintah-finalisasi-pepres-tentang-ojol-lengkapi-sejumlah-formula</t>
+        </is>
+      </c>
+      <c r="H606" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/6b504038-1fa7-4906-a931-30e468891c23.jpg</t>
+        </is>
+      </c>
+      <c r="I606" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>Polisi tangkap dua begal yang serang anggota Polda Sumsel</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:45:35 +0700</t>
+        </is>
+      </c>
+      <c r="D607" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E607" t="inlineStr">
+        <is>
+          <t>Polrestabes Palembang, Sumatera Selatan, menangkap dua tersangka pencurian dengan kekerasan (curas) terhadap seorang ...</t>
+        </is>
+      </c>
+      <c r="F607" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G607" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689016/polisi-tangkap-dua-begal-yang-serang-anggota-polda-sumsel</t>
+        </is>
+      </c>
+      <c r="H607" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1001554933.jpg</t>
+        </is>
+      </c>
+      <c r="I607" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>BNPB: Karhutla di Magetan dan Jombang padam kurang dari 24 jam</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:43:44 +0700</t>
+        </is>
+      </c>
+      <c r="D608" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E608" t="inlineStr">
+        <is>
+          <t>Badan Nasional Penanggulangan Bencana (BNPB) menyatakan peristiwa kebakaran hutan dan lahan (karhutla) di Kabupaten ...</t>
+        </is>
+      </c>
+      <c r="F608" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G608" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689013/bnpb-karhutla-di-magetan-dan-jombang-padam-kurang-dari-24-jam</t>
+        </is>
+      </c>
+      <c r="H608" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG-20260811-WA0000.jpg</t>
+        </is>
+      </c>
+      <c r="I608" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>Bapenda Batam dekatkan layanan pajak ke mal setiap pekan</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:42:08 +0700</t>
+        </is>
+      </c>
+      <c r="D609" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E609" t="inlineStr">
+        <is>
+          <t>Badan Pendapatan Daerah (Bapenda) Kota Batam, Kepulauan Riau (Kepri) memperluas dan mendekatkan layanan perpajakan ...</t>
+        </is>
+      </c>
+      <c r="F609" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G609" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689009/bapenda-batam-dekatkan-layanan-pajak-ke-mal-setiap-pekan</t>
+        </is>
+      </c>
+      <c r="H609" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/236f1b15-68e2-49dc-a26f-e7b0fde92ad1.jpeg</t>
+        </is>
+      </c>
+      <c r="I609" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>Hasil Studi Global yang Dipublikasikan di Aesthetic Surgery Journal Open Forum Ungkap Kaitan antara Kepercayaan Diri dan Estetika</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:41:46 +0700</t>
+        </is>
+      </c>
+      <c r="D610" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E610" t="inlineStr">
+        <is>
+          <t>Aesthetic Surgery Journal Open Forum (ASJ Open Forum) pada bulan ini menerbitkan hasil studi global Merz ...</t>
+        </is>
+      </c>
+      <c r="F610" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G610" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689007/hasil-studi-global-yang-dipublikasikan-di-aesthetic-surgery-journal-open-forum-ungkap-kaitan-antara-kepercayaan-diri-dan-estetika</t>
+        </is>
+      </c>
+      <c r="H610" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/Aesthetics-and-Self-Affirmation.jpg</t>
+        </is>
+      </c>
+      <c r="I610" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>Conscious living: Cara jalani hidup lebih sadar tanpa ikut-ikutan</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:40:41 +0700</t>
+        </is>
+      </c>
+      <c r="D611" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E611" t="inlineStr">
+        <is>
+          <t>Di tengah kehidupan yang serba cepat, mengikuti apa yang sedang populer rasanya sudah menjadi hal yang sulit dihindari. ...</t>
+        </is>
+      </c>
+      <c r="F611" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G611" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689004/conscious-living-cara-jalani-hidup-lebih-sadar-tanpa-ikut-ikutan</t>
+        </is>
+      </c>
+      <c r="H611" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2023/09/27/IMG-20230927-WA0031_2.jpg</t>
+        </is>
+      </c>
+      <c r="I611" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>Sudin SDA Jakpus normalisai saluran di Cempaka Putih Tengah XXII</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:40:01 +0700</t>
+        </is>
+      </c>
+      <c r="D612" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E612" t="inlineStr">
+        <is>
+          <t>Suku Dinas Sumber Daya Air (SDA) Jakarta Pusat menormalisasi saluran air sepanjang 273 meter di Jalan Cempaka Putih ...</t>
+        </is>
+      </c>
+      <c r="F612" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G612" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689000/sudin-sda-jakpus-normalisai-saluran-di-cempaka-putih-tengah-xxii</t>
+        </is>
+      </c>
+      <c r="H612" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/01/10/InShot_20250110_075904218.jpg</t>
+        </is>
+      </c>
+      <c r="I612" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>Kemenag susun pedoman pesantren ramah anak, panduan cegah kekerasan</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:39:06 +0700</t>
+        </is>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>Kementerian Agama tengah menyusun pedoman Pesantren Ramah Anak Tahun 2026 yang akan menjadi panduan bersama dalam ...</t>
+        </is>
+      </c>
+      <c r="F613" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G613" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688996/kemenag-susun-pedoman-pesantren-ramah-anak-panduan-cegah-kekerasan</t>
+        </is>
+      </c>
+      <c r="H613" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1000177468.jpg</t>
+        </is>
+      </c>
+      <c r="I613" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>Pramono: Kenaikan jumlah penumpang transportasi umum bisa tekan polusi</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:38:24 +0700</t>
+        </is>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E614" t="inlineStr">
+        <is>
+          <t>Gubernur DKI Jakarta Pramono Anung Wibowo meyakini peningkatan jumlah pengguna transportasi umum dapat menekan ...</t>
+        </is>
+      </c>
+      <c r="F614" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G614" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688993/pramono-kenaikan-jumlah-penumpang-transportasi-umum-bisa-tekan-polusi</t>
+        </is>
+      </c>
+      <c r="H614" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG_6800.jpeg</t>
+        </is>
+      </c>
+      <c r="I614" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>Pelindo Multi Terminal Catat Kinerja Positif pada Semester I 2026</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:38:13 +0700</t>
+        </is>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>Jakarta (ANTARA) – PT Pelindo Multi Terminal, anak usaha PT Pelabuhan Indonesia (Persero) yang bergerak dalam ...</t>
+        </is>
+      </c>
+      <c r="F615" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G615" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688989/pelindo-multi-terminal-catat-kinerja-positif-pada-semester-i-2026</t>
+        </is>
+      </c>
+      <c r="H615" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/WhatsApp-Image-2026-08-11-at-13.25.21.jpeg</t>
+        </is>
+      </c>
+      <c r="I615" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>Imigrasi Tanjungpinang hadirkan layanan antar paspor IDEPAS</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:38:04 +0700</t>
+        </is>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>Kantor Imigrasi Kelas I TPI Tanjungpinang bekerja sama dengan PT Pos Indonesia (Persero) Cabang Tanjungpinang, ...</t>
+        </is>
+      </c>
+      <c r="F616" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G616" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688987/imigrasi-tanjungpinang-hadirkan-layanan-antar-paspor-idepas</t>
+        </is>
+      </c>
+      <c r="H616" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/20260811_142335.jpg</t>
+        </is>
+      </c>
+      <c r="I616" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>POJK Demutualisasi tidak batasi kepemilikan atas BEI dengan syarat</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:37:53 +0700</t>
+        </is>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>Otoritas Jasa Keuangan (OJK) tengah mengkaji suatu konsep terkait pembatasan kepemilikan maksimum atas PT Bursa Efek ...</t>
+        </is>
+      </c>
+      <c r="F617" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G617" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688984/pojk-demutualisasi-tidak-batasi-kepemilikan-atas-bei-dengan-syarat</t>
+        </is>
+      </c>
+      <c r="H617" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/WhatsApp-Image-2026-08-11-at-13.30.14.jpeg</t>
+        </is>
+      </c>
+      <c r="I617" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>Jaksa Agung lantik kajati dan pejabat eselon II Kejagung</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:36:19 +0700</t>
+        </is>
+      </c>
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E618" t="inlineStr">
+        <is>
+          <t>Jaksa Agung ST Burhanuddin melantik para kepala Kejaksaan Tinggi (kajati) dan pejabat eselon II di lingkungan Kejaksaan ...</t>
+        </is>
+      </c>
+      <c r="F618" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G618" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688981/jaksa-agung-lantik-kajati-dan-pejabat-eselon-ii-kejagung</t>
+        </is>
+      </c>
+      <c r="H618" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1000087642.jpg</t>
+        </is>
+      </c>
+      <c r="I618" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>WBA perpanjang negosiasi perebutan juara dunia Schofield lawan Bahdi</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:36:12 +0700</t>
+        </is>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>World Boxing Association (WBA) memperpanjang masa negosiasi pertarungan perebutan gelar juara dunia kelas ringan (61,2 ...</t>
+        </is>
+      </c>
+      <c r="F619" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G619" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688980/wba-perpanjang-negosiasi-perebutan-juara-dunia-schofield-lawan-bahdi</t>
+        </is>
+      </c>
+      <c r="H619" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/d3a64113-0099-4ae6-8c0a-8f62335d756c_1.jpeg</t>
+        </is>
+      </c>
+      <c r="I619" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>10 aktivitas selain nongkrong yang bisa dilakukan di akhir pekan</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:35:35 +0700</t>
+        </is>
+      </c>
+      <c r="D620" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E620" t="inlineStr">
+        <is>
+          <t>Akhir pekan biasanya menjadi waktu yang paling ditunggu setelah disibukkan oleh rutinitas harian. Tidak sedikit orang ...</t>
+        </is>
+      </c>
+      <c r="F620" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G620" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688979/10-aktivitas-selain-nongkrong-yang-bisa-dilakukan-di-akhir-pekan</t>
+        </is>
+      </c>
+      <c r="H620" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2022/08/08/pexels-august-de-richelieu-4259140.jpg</t>
+        </is>
+      </c>
+      <c r="I620" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>Mensesneg cek latihan gabungan Paskibraka bersama TNI-Polri di Istana</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:32:47 +0700</t>
+        </is>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>ANTARA - Menteri Sekretaris Negara (Mensesneg) Prasetyo Hadi, Selasa (11/8), meninjau langsung latihan gabungan ...</t>
+        </is>
+      </c>
+      <c r="F621" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G621" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5688931/mensesneg-cek-latihan-gabungan-paskibraka-bersama-tni-polri-di-istana</t>
+        </is>
+      </c>
+      <c r="H621" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/MENSESNEG-CEK-LATIHAN-GABUNGAN-PASKIBRAKA-BERSAMA-TNI-POLRI-DI-ISTANA.jpg</t>
+        </is>
+      </c>
+      <c r="I621" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>Utang rental Rp600 ribu berujung maut delapan orang jadi tersangka</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:32:00 +0700</t>
+        </is>
+      </c>
+      <c r="D622" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E622" t="inlineStr">
+        <is>
+          <t>Polres Sumedang, Jawa Barat, menetapkan delapan tersangka dalam kasus dugaan penyekapan dan penganiayaan seorang pria ...</t>
+        </is>
+      </c>
+      <c r="F622" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G622" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688975/utang-rental-rp600-ribu-berujung-maut-delapan-orang-jadi-tersangka</t>
+        </is>
+      </c>
+      <c r="H622" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/491570.jpg</t>
+        </is>
+      </c>
+      <c r="I622" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>Menhan RI perkuat kerja sama dengan Amerika Serikat</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:31:26 +0700</t>
+        </is>
+      </c>
+      <c r="D623" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>Menteri Pertahanan RI Sjafrie Sjamsoeddin berupaya mempererat hubungan bilateral dengan pemerintah Amerika Serikat agar ...</t>
+        </is>
+      </c>
+      <c r="F623" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G623" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688971/menhan-ri-perkuat-kerja-sama-dengan-amerika-serikat</t>
+        </is>
+      </c>
+      <c r="H623" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1001569672.jpg</t>
+        </is>
+      </c>
+      <c r="I623" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>Dari dapur SPPG ke sekolah, MBG jangkau 375 ribu penerima di Sulbar</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:26:04 +0700</t>
+        </is>
+      </c>
+      <c r="D624" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>Sejumlah pekerja membawa ompreng Program Makan Bergizi Gratis (MBG) menggunakan gerobak untuk disalurkan ke sekolah di ...</t>
+        </is>
+      </c>
+      <c r="F624" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G624" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5688969/dari-dapur-sppg-ke-sekolah-mbg-jangkau-375-ribu-penerima-di-sulbar</t>
+        </is>
+      </c>
+      <c r="H624" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/Capaian-realisasi-program-MBG-di-Sulawesi-Barat-110826-At-1A.jpg</t>
+        </is>
+      </c>
+      <c r="I624" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>Demokrat ungkap SBY sedang cek kesehatan di AS, tak akan hadiri HUT RI</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:25:45 +0700</t>
+        </is>
+      </c>
+      <c r="D625" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>Wakil Ketua Umum Partai Demokrat Benny K. Harman mengungkapkan Presiden Ke-6 RI Susilo Bambang Yudhoyono ...</t>
+        </is>
+      </c>
+      <c r="F625" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G625" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688965/demokrat-ungkap-sby-sedang-cek-kesehatan-di-as-tak-akan-hadiri-hut-ri</t>
+        </is>
+      </c>
+      <c r="H625" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/04/Pidato-politik-SBY-070224-fah-2.jpg</t>
+        </is>
+      </c>
+      <c r="I625" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>Pemerintah Yaman ancam balas serangan Houthi yang kian intensif</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:25:32 +0700</t>
+        </is>
+      </c>
+      <c r="D626" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>Pemerintah Yaman, yang diakui secara internasional, pada Senin menyatakan akan merespons serangan berkelanjutan dari ...</t>
+        </is>
+      </c>
+      <c r="F626" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G626" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688964/pemerintah-yaman-ancam-balas-serangan-houthi-yang-kian-intensif</t>
+        </is>
+      </c>
+      <c r="H626" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/08/Tentara-Yaman.jpg</t>
+        </is>
+      </c>
+      <c r="I626" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>Gubernur: Pembebasan lahan Tol Jambi-Rengat tuntas Desember 2026</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:21:03 +0700</t>
+        </is>
+      </c>
+      <c r="D627" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E627" t="inlineStr">
+        <is>
+          <t>Gubernur Jambi Al Haris memastikan seluruh proses penetapan lokasi (penlok) hingga pendataan ganti rugi lahan ...</t>
+        </is>
+      </c>
+      <c r="F627" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G627" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688961/gubernur-pembebasan-lahan-tol-jambi-rengat-tuntasdesember-2026</t>
+        </is>
+      </c>
+      <c r="H627" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/575577.jpg</t>
+        </is>
+      </c>
+      <c r="I627" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>Mensesneg: Pemerintah fokus tangani karhutla di sejumlah wilayah</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:20:47 +0700</t>
+        </is>
+      </c>
+      <c r="D628" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>Menteri Sekretaris Negara (Mensesneg) Prasetyo Hadi memastikan pemerintah saat ini tengah fokus menangani kebakaran ...</t>
+        </is>
+      </c>
+      <c r="F628" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G628" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688957/mensesneg-pemerintah-fokus-tangani-karhutla-di-sejumlah-wilayah</t>
+        </is>
+      </c>
+      <c r="H628" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/cceb30b0-6d5e-4bd4-a740-126ce8224881.jpg</t>
+        </is>
+      </c>
+      <c r="I628" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>TNI AU kaji Tol Probolinggo-Banyuwangi jadi landasan pesawat</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:19:47 +0700</t>
+        </is>
+      </c>
+      <c r="D629" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E629" t="inlineStr">
+        <is>
+          <t>TNI Angkatan Udara mengkaji penggunaan ruas jalan tol di Jawa Timur sebagai landasan alternatif pesawat untuk mendukung ...</t>
+        </is>
+      </c>
+      <c r="F629" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G629" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688956/tni-au-kaji-tol-probolinggo-banyuwangi-jadi-landasan-pesawat</t>
+        </is>
+      </c>
+      <c r="H629" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/03/09/uji-coba-pendaratan-pesawat-tempur-di-jalan-tol-terpeka-1mgau-dom.jpg</t>
+        </is>
+      </c>
+      <c r="I629" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>Pertamina Patra Niaga rampungkan proses docking 12 unit kapal</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:16:40 +0700</t>
+        </is>
+      </c>
+      <c r="D630" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E630" t="inlineStr">
+        <is>
+          <t>PT Pertamina Patra Niaga merampungkan proses docking terhadap 12 unit kapal pada periode Februari 2026 hingga Juli 2026 ...</t>
+        </is>
+      </c>
+      <c r="F630" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G630" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688944/pertamina-patra-niaga-rampungkan-proses-docking-12-unit-kapal</t>
+        </is>
+      </c>
+      <c r="H630" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1000407478.jpg</t>
+        </is>
+      </c>
+      <c r="I630" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>Istana minta maaf persiapan HUT Ke-81 RI ganggu lalu lintas</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:16:27 +0700</t>
+        </is>
+      </c>
+      <c r="D631" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E631" t="inlineStr">
+        <is>
+          <t>Menteri Sekretaris Negara (Mensesneg) Prasetyo Hadi menyampaikan permohonan maaf kepada masyarakat atas penyesuaian dan ...</t>
+        </is>
+      </c>
+      <c r="F631" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G631" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5688940/istana-minta-maaf-persiapan-hut-ke-81-ri-ganggu-lalu-lintas</t>
+        </is>
+      </c>
+      <c r="H631" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG_3746.jpeg</t>
+        </is>
+      </c>
+      <c r="I631" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>AHY Soroti Birokrasi yang Bikin Investor Susah Investasi: Jangan Dipingpong</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:42:52 +0700</t>
+        </is>
+      </c>
+      <c r="D632" t="inlineStr">
+        <is>
+          <t>Brigitta Belia Permata Sari</t>
+        </is>
+      </c>
+      <c r="E632" t="inlineStr">
+        <is>
+          <t>Menteri AHY soroti birokrasi yang menyulitkan investor di Indonesia. Ia minta pemerintah ciptakan kepastian dan kemudahan dalam perizinan investasi.</t>
+        </is>
+      </c>
+      <c r="F632" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G632" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8613682/ahy-soroti-birokrasi-yang-bikin-investor-susah-investasi-jangan-dipingpong</t>
+        </is>
+      </c>
+      <c r="H632" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/menko-ahy-brigitta-beliadetikcom-1786434144294_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I632" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>Digitalisasi Akta Kelahiran Diluncurkan, Layanan Publik Kian Terintegrasi</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:42:34 +0700</t>
+        </is>
+      </c>
+      <c r="D633" t="inlineStr">
+        <is>
+          <t>Inkana Putri</t>
+        </is>
+      </c>
+      <c r="E633" t="inlineStr">
+        <is>
+          <t>Pemerintah luncurkan digitalisasi akta kelahiran terintegrasi dengan layanan kesehatan. Proses penerbitan akta kini lebih cepat dan efisien bagi masyarakat.</t>
+        </is>
+      </c>
+      <c r="F633" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G633" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8613681/digitalisasi-akta-kelahiran-diluncurkan-layanan-publik-kian-terintegrasi</t>
+        </is>
+      </c>
+      <c r="H633" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/digitalisasi-akta-kelahiran-diluncurkan-layanan-publik-kian-terintegrasi-1786434114981.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I633" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>Jaksa Agung Lantik 15 Kajati, Minta Beri Perhatian Khusus Setiap Kasus Besar</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:41:11 +0700</t>
+        </is>
+      </c>
+      <c r="D634" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E634" t="inlineStr">
+        <is>
+          <t>Jaksa Agung ST Burhanuddin melantik pejabat baru di Kejaksaan Agung. Pelantikan ini bertujuan memperkuat manajemen karier dan meningkatkan kinerja institusi.</t>
+        </is>
+      </c>
+      <c r="F634" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G634" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8613679/jaksa-agung-lantik-15-kajati-minta-beri-perhatian-khusus-setiap-kasus-besar</t>
+        </is>
+      </c>
+      <c r="H634" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/jaksa-agung-republik-indonesia-st-burhanuddin-1786434039773_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I634" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>Terungkap di Dakwaan, Ini Hitungan Kerugian Negara Korupsi Kuota Haji Rp 622 M</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:35:38 +0700</t>
+        </is>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>Mulia Budi</t>
+        </is>
+      </c>
+      <c r="E635" t="inlineStr">
+        <is>
+          <t>Hitung-hitungan kerugian negara Rp 622 miliar akibat kasus korupsi kuota haji terungkap di persidangan.</t>
+        </is>
+      </c>
+      <c r="F635" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G635" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8613657/terungkap-di-dakwaan-ini-hitungan-kerugian-negara-korupsi-kuota-haji-rp-622-m</t>
+        </is>
+      </c>
+      <c r="H635" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/eks-menag-yaqut-didakwa-perkara-kuota-haji-negara-disebut-rugi-rp622-miliar-1786428544309_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I635" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>Dikira Bunuh Diri, Wanita di Tangerang Ternyata Tewas Dibunuh Pacar</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:24:27 +0700</t>
+        </is>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>Arief Ikhsanudin</t>
+        </is>
+      </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>Seorang wanita ditemukan tewas tergantung di Tangerang. Penyelidikan mengungkap bahwa pacarnya, pria berinisial A, adalah pelaku pembunuhan.</t>
+        </is>
+      </c>
+      <c r="F636" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G636" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8613647/dikira-bunuh-diri-wanita-di-tangerang-ternyata-tewas-dibunuh-pacar</t>
+        </is>
+      </c>
+      <c r="H636" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2021/04/01/ilustrasi-garis-polisi_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I636" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>Viral Sejumlah Pemuda Sweeping Waria di Alun-alun Kota Rangkasbitung</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:24:24 +0700</t>
+        </is>
+      </c>
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>Aris Rivaldo</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>Sejumlah pemuda melakukan sweeping keberadaan wanita-pria (waria) di Alun-alun Kota Rangkasbitung, Lebak, Banten. Video sweeping waria itu viral di medsos.</t>
+        </is>
+      </c>
+      <c r="F637" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G637" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8613649/viral-sejumlah-pemuda-sweeping-waria-di-alun-alun-kota-rangkasbitung</t>
+        </is>
+      </c>
+      <c r="H637" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/01/10/ilustrasi-media-sosial_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I637" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>Bawa Kabur Motor Teman, Pria Bogor Ditangkap di Kaki Gunung Merbabu</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:21:07 +0700</t>
+        </is>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>Rizky Adha Mahendra</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>Polisi menangkap pria berinisial T (34) di kaki Gunung Merbabu. T ditangkap usai diduga membawa kabur motor temannya dari wilayah Gunung Putri, Bogor.</t>
+        </is>
+      </c>
+      <c r="F638" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G638" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8613641/bawa-kabur-motor-teman-pria-bogor-ditangkap-di-kaki-gunung-merbabu</t>
+        </is>
+      </c>
+      <c r="H638" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/pria-di-bogor-ditangkap-di-kaki-gunung-merbabu-usai-membawa-kabur-motor-temannya-1786432519401_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I638" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>Mensos Ajak Jajaran Jadikan Momentum HUT RI untuk Berbenah-Berprestasi</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:13:09 +0700</t>
+        </is>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>Hana Nushratu</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr">
+        <is>
+          <t>Menteri Sosial Gus Ipul mengajak jajaran Kemensos refleksi dan berbenah saat HUT RI ke-81. Ia menekankan integritas dan keterbukaan untuk meningkatkan layanan.</t>
+        </is>
+      </c>
+      <c r="F639" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G639" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8613622/mensos-ajak-jajaran-jadikan-momentum-hut-ri-untuk-berbenah-berprestasi</t>
+        </is>
+      </c>
+      <c r="H639" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/mensos-ajak-jajaran-jadikan-momentum-hut-ri-untuk-berbenah-berprestasi-1786432327429_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I639" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>Siswa Sekolah Rakyat Bacakan Puisi 'Kamipun Ingin Merdeka' di Kemensos</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:05:39 +0700</t>
+        </is>
+      </c>
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>Hana Nushratu</t>
+        </is>
+      </c>
+      <c r="E640" t="inlineStr">
+        <is>
+          <t>Peringatan HUT RI ke-81 di Kemensos diwarnai penampilan puisi oleh siswa Sekolah Rakyat. Gus Ipul menekankan pentingnya integritas dalam pelayanan.</t>
+        </is>
+      </c>
+      <c r="F640" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G640" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8613605/siswa-sekolah-rakyat-bacakan-puisi-kamipun-ingin-merdeka-di-kemensos</t>
+        </is>
+      </c>
+      <c r="H640" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/kamipun-ingin-merdeka-puisi-anak-sekolah-rakyat-saat-tampil-di-kemensos-1786431674236.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I640" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>Rapat di DPR, Pakar Usul RUU Perampasan Aset Diubah Jadi RUU Melindungi Aset</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:02:58 +0700</t>
+        </is>
+      </c>
+      <c r="D641" t="inlineStr">
+        <is>
+          <t>Dwi Rahmawati</t>
+        </is>
+      </c>
+      <c r="E641" t="inlineStr">
+        <is>
+          <t>Bambang Harymurti mengusulkan nama RUU Perampasan Aset jadi RUU Melindungi Aset. Ia tak ingin UU ini nantinya melegalisir upaya pencurian aset secara legal.</t>
+        </is>
+      </c>
+      <c r="F641" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G641" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8613597/rapat-di-dpr-pakar-usul-ruu-perampasan-aset-diubah-jadi-ruu-melindungi-aset</t>
+        </is>
+      </c>
+      <c r="H641" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/rapat-dengar-pendapat-umum-komisi-iii-dpr-bersama-sejumlah-pakar-di-gedung-dpr-senayan-jakarta-selasa-1182026-1786431721843_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I641" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>Aiptu Asep Gugur Jadi Korban Tabrak Lari di Bandung, Keluarga Berduka</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 13:55:48 +0700</t>
+        </is>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>Tim detikJabar</t>
+        </is>
+      </c>
+      <c r="E642" t="inlineStr">
+        <is>
+          <t>Aiptu Asep Suhara, anggota Polrestabes Bandung, gugur akibat tabrak lari saat bertugas. Keluarga berduka, dan kasus ini sedang ditangani polisi.</t>
+        </is>
+      </c>
+      <c r="F642" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G642" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8613578/aiptu-asep-gugur-jadi-korban-tabrak-lari-di-bandung-keluarga-berduka</t>
+        </is>
+      </c>
+      <c r="H642" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/10/istri-dan-anak-aiptu-asep-suhara-polisi-korban-tabrak-lari-di-bandung-1786332714961_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I642" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>Mensesneg Minta Maaf Jl Veteran-Merdeka Utara Ditutup Imbas Latihan HUT RI</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 13:52:33 +0700</t>
+        </is>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>Firda Cynthia Anggrainy</t>
+        </is>
+      </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>Mensesneg Prasetyo Hadi minta maaf atas penutupan Jalan Veteran III dan Medan Merdeka Utara untuk latihan HUT RI</t>
+        </is>
+      </c>
+      <c r="F643" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G643" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8613571/mensesneg-minta-maaf-jl-veteran-merdeka-utara-ditutup-imbas-latihan-hut-ri</t>
+        </is>
+      </c>
+      <c r="H643" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/mensesneg-dan-seskab-cek-gladi-parsial-upacara-hut-ri-di-istana-1786426651660_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I643" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>Polisi Tetapkan 8 Tersangka Kasus Tewasnya Handi di Sumedang</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 13:38:13 +0700</t>
+        </is>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>Dwiky Maulana Vellayati</t>
+        </is>
+      </c>
+      <c r="E644" t="inlineStr">
+        <is>
+          <t>Polisi pun menetapkan delapan tersangka dalam kasus ini.</t>
+        </is>
+      </c>
+      <c r="F644" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G644" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8613545/polisi-tetapkan-8-tersangka-kasus-tewasnya-handi-di-sumedang</t>
+        </is>
+      </c>
+      <c r="H644" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/polisi-tetapkan-8-orang-menjadi-tersangka-penyekapan-di-sumedang-1786423710480_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I644" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>Jaksa: Surat Keputusan Yaqut Terkait Kuota Haji Tambahan Dibuat Backdated</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 13:35:15 +0700</t>
+        </is>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>Mulia Budi</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr">
+        <is>
+          <t>Jaksa KPK ungkap dugaan korupsi kuota haji oleh mantan Menteri Agama Yaqut, termasuk penandatanganan SK yang backdated</t>
+        </is>
+      </c>
+      <c r="F645" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G645" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8613540/jaksa-surat-keputusan-yaqut-terkait-kuota-haji-tambahan-dibuat-backdated</t>
+        </is>
+      </c>
+      <c r="H645" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/eks-menag-yaqut-didakwa-perkara-kuota-haji-negara-disebut-rugi-rp622-miliar-1786428544180_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I645" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>Soal Senjata di Sekolah Jaksel, Polisi Sebut Ada Kerja Sama Olahraga Menembak</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 13:32:11 +0700</t>
+        </is>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>Wildan Noviansah</t>
+        </is>
+      </c>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>Polisi mengungkap ratusan senjata di sekolah swasta Jakarta, terkait kerja sama olahraga menembak. Legalitas senjata masih didalami. Temukan juga narkotika.</t>
+        </is>
+      </c>
+      <c r="F646" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G646" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8613528/soal-senjata-di-sekolah-jaksel-polisi-sebut-ada-kerja-sama-olahraga-menembak</t>
+        </is>
+      </c>
+      <c r="H646" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/kabid-humas-polda-metro-jaya-kombes-budi-hermanto-1786089469648_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I646" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>Dana Wakaf Masjid Istiqlal Bakal Masuk Pasar Modal, Begini Skemanya</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:57:39 +0700</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>Heri Purnomo</t>
+        </is>
+      </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>Bursa Efek Indonesia rencanakan Masjid Istiqlal masuk ekosistem pasar modal melalui dana wakaf produktif, dikelola profesional oleh manajer investasi.</t>
+        </is>
+      </c>
+      <c r="F647" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G647" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8613719/dana-wakaf-masjid-istiqlal-bakal-masuk-pasar-modal-begini-skemanya</t>
+        </is>
+      </c>
+      <c r="H647" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/06/04/penjabat-sementara-pjs-direktur-utama-bei-jeffrey-hendrik-1780560925234_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I647" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>Naik Kereta Ekonomi Diskon 17%, LRT Jabodebek Cuma Bayar Rp 8</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:48:03 +0700</t>
+        </is>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>Herdi Alif Al Hikam</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>Promo spesial disediakan PT Kereta Api Indonesia (Persero) untuk memperingati Hari Kemerdekaan ke-81 Republik Indonesia.</t>
+        </is>
+      </c>
+      <c r="F648" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G648" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8613698/naik-kereta-ekonomi-diskon-17-lrt-jabodebek-cuma-bayar-rp-8</t>
+        </is>
+      </c>
+      <c r="H648" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/05/19/lrt-jabodebek-makin-jadi-andalan-transum-warga-1779203242481_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I648" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>Suara Istana untuk Destry Damayanti</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:44:25 +0700</t>
+        </is>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>20detik Signature</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>Sejauh mana Destry dapat memberikan perubahan di sisi moneter Indonesia?</t>
+        </is>
+      </c>
+      <c r="F649" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G649" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8613637/suara-istana-untuk-destry-damayanti</t>
+        </is>
+      </c>
+      <c r="H649" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/detiksore-11-agustus-2026-1786432519241_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I649" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>12 Kapal Pertamina Selesai Docking, Distribusi Dipastikan Aman</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 13:41:38 +0700</t>
+        </is>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>Heri Purnomo</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>PT Pertamina Patra Niaga rampungkan docking 12 kapal untuk pemeliharaan armada. Ini memastikan distribusi energi nasional tetap aman dan andal.</t>
+        </is>
+      </c>
+      <c r="F650" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G650" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8613549/12-kapal-pertamina-selesai-docking-distribusi-dipastikan-aman</t>
+        </is>
+      </c>
+      <c r="H650" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/patra-niaga-1786430381337_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I650" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>Peringatan Dini Hujan di Indonesia Rabu, 12 Agustus 2026: Aceh dan Sumatra Utara Waspada</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:52:51 +0700</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>BMKG keluarkan peringatan dini cuaca Rabu, 12 Agustus 2026. Aceh dan Sumatra Utara masuk kategori Waspada.</t>
+        </is>
+      </c>
+      <c r="F651" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G651" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7866893/peringatan-dini-hujan-di-indonesia-rabu-12-agustus-2026-aceh-dan-sumatra-utara-waspada</t>
+        </is>
+      </c>
+      <c r="H651" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/otmRvhuUu5tHTOcJr1Dtcz93LKI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Hujan-deras-di-Bogor565.jpg</t>
+        </is>
+      </c>
+      <c r="I651" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>30 Puisi Maulid Nabi Muhammad SAW yang Menyentuh Hati, Penuh Cinta dan Kerinduan</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:51:38 +0700</t>
+        </is>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr">
+        <is>
+          <t>Peringatan Maulid Nabi Muhammad SAW pada tahun 2026 jatuh pada Selasa, 25 Agustus. Inilah 30 puisi Maulid Nabi Muhammad SAW dapat menjadi inspirasi.</t>
+        </is>
+      </c>
+      <c r="F652" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G652" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866892/30-puisi-maulid-nabi-muhammad-saw-yang-menyentuh-hati-penuh-cinta-dan-kerinduan</t>
+        </is>
+      </c>
+      <c r="H652" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/OgXugpB4daFlVGoTnMGvRC4ZyOM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/perayaan-maulid-nabi-di-kapung-kali-pasir-kota-tangerang_20211020_235657.jpg</t>
+        </is>
+      </c>
+      <c r="I652" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>Terseret Kasus Hukum Buntut Aduan Icel, Karier Akting Anrez Adelio Hancur Berantakan?</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:51:18 +0700</t>
+        </is>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>Jadwal kerja Anrez yang sudah tersusun rapi, berantakan akibat keputusan pihak televisi dan rumah produksi yang memilih menunda keterlibatannya.</t>
+        </is>
+      </c>
+      <c r="F653" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G653" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7866891/terseret-kasus-hukum-buntut-aduan-icel-karier-akting-anrez-adelio-hancur-berantakan</t>
+        </is>
+      </c>
+      <c r="H653" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Dc65IpfbpvxFFlsbdabCUd0thdA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ANREZ-HAMILI-ICEL.jpg</t>
+        </is>
+      </c>
+      <c r="I653" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>Prakiraan Cuaca Madura Jawa Timur Rabu, 12 Agustus 2026: Cerah Berawan di Arjasa dan Kangayan</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:51:05 +0700</t>
+        </is>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E654" t="inlineStr">
+        <is>
+          <t>Pantauan prakiraan cuaca lengkap BMKG untuk wilayah Pulau Madura, Jawa Timur, pada Rabu (12/8/2026) langit cerah berawan</t>
+        </is>
+      </c>
+      <c r="F654" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G654" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7866890/prakiraan-cuaca-madura-jawa-timur-rabu-12-agustus-2026-cerah-berawan-di-arjasa-dan-kangayan</t>
+        </is>
+      </c>
+      <c r="H654" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/5fNbv8oJSiEcLybciut8NHRHy6Y=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/tim-basarnas-saat-lakukan-pencarian-korban-di-perairan-sumenep-rabu-1962019.jpg</t>
+        </is>
+      </c>
+      <c r="I654" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>Nasib Pilu Paramitha Titania, Ditemukan Tinggal Tengkorak usai 2 Tahun Hilang, Dibunuh Sopir Travel</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:50:00 +0700</t>
+        </is>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>Paramitha Titania ditemukan tinggal tengkorak setelah dibunuh sopir travel Alber yang sakit hati dan membuang jasadnya ke jurang.</t>
+        </is>
+      </c>
+      <c r="F655" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G655" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7866889/nasib-pilu-paramitha-titania-ditemukan-tinggal-tengkorak-usai-2-tahun-hilang-dibunuh-sopir-travel</t>
+        </is>
+      </c>
+      <c r="H655" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/BbzHBa9Bq4R9l1GSGNqJ_X8jvC4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Nasib-Pilu-Paramitha-Titania-Ditemukan-Tinggal-Tengkorak-usai-2-Tahun-Hilang-Dibunuh-Sopir-Travel.jpg</t>
+        </is>
+      </c>
+      <c r="I655" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>Jadwal Kick-off Super League, Championship dan Liga Putri 2026/2027, Catat Tanggalnya</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:49:52 +0700</t>
+        </is>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E656" t="inlineStr">
+        <is>
+          <t>Jadwal kompetisi Liga Indonesia 2026/2027 telah ditetapkan. Super League, Championship, hingga Liga Putri siap kembali bergulir.</t>
+        </is>
+      </c>
+      <c r="F656" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G656" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7866888/jadwal-kick-off-super-league-championship-dan-liga-putri-20262027-catat-tanggalnya</t>
+        </is>
+      </c>
+      <c r="H656" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/VBz6VCmSehzqT9rfwL9t4QXveDU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Persib-Bandung-berhasil-meraih-gelar-juara-Super-League-20252026.jpg</t>
+        </is>
+      </c>
+      <c r="I656" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>Kubu Yaqut Bantah KPK Sita Rp100 Miliar saat Geledah Rumah Eks Menag: Tak Ada Uang Selembar Pun</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:48:54 +0700</t>
+        </is>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>Mellisa menyatakan narasi yang menyebut KPK menyita uang Rp 100 miliar dari rumah Yaqut, tidak benar.</t>
+        </is>
+      </c>
+      <c r="F657" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G657" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866887/kubu-yaqut-bantah-kpk-sita-rp100-miliar-saat-geledah-rumah-eks-menag-tak-ada-uang-selembar-pun</t>
+        </is>
+      </c>
+      <c r="H657" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/1c6TMgqEDReVN4O5qe9cNoMcmmc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/melissa-bantaaaahhhh.jpg</t>
+        </is>
+      </c>
+      <c r="I657" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>Spesifikasi Kapal Mewah Grand Maloekoe yang Bawa Rombongan Jessica Mila ke Pulau Padar saat Ditutup</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:48:27 +0700</t>
+        </is>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>Rombongan Jessica Mila yang mendatangi Pulau Padar menggunakan kapal mewah Grand Maloekoe jadi sorotan.</t>
+        </is>
+      </c>
+      <c r="F658" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G658" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7866886/spesifikasi-kapal-mewah-grand-maloekoe-yang-bawa-rombongan-jessica-mila-ke-pulau-padar-saat-ditutup</t>
+        </is>
+      </c>
+      <c r="H658" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/S1aHyqxvCXmNSxS9G5nu-RgKrz4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/keindahan-pulau-padar-labuan-bajo_20210329_114748.jpg</t>
+        </is>
+      </c>
+      <c r="I658" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>Bansos PKH dan BPNT Triwulan III 2026 Resmi Disalurkan, Ini Cara Cek Penerimanya</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:48:07 +0700</t>
+        </is>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>Bansos PKH dan BPNT Triwulan III 2026 untuk periode Juli-September terus disalurkan kepada jutaan KPM secara bertahap.</t>
+        </is>
+      </c>
+      <c r="F659" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G659" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866885/bansos-pkh-dan-bpnt-triwulan-iii-2026-resmi-disalurkan-ini-cara-cek-penerimanya</t>
+        </is>
+      </c>
+      <c r="H659" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Hp59702bRqdb4QGtrmgujM6Ebls=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-uang-bansos-1.jpg</t>
+        </is>
+      </c>
+      <c r="I659" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>Uji UU Pelindungan Data Pribadi di MK, Saksi Ungkap Kekhawatiran Bocornya 204 Juta Data Pemilih KPU</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:45:27 +0700</t>
+        </is>
+      </c>
+      <c r="D660" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E660" t="inlineStr">
+        <is>
+          <t>Sidang uji materi Undang-Undang Pelindungan Data Pribadi (UU PDP) di Mahkamah Konstitusi (MK) turut menyinggung isu keamanan data pemilih.</t>
+        </is>
+      </c>
+      <c r="F660" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G660" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866884/uji-uu-pelindungan-data-pribadi-di-mk-saksi-ungkap-kekhawatiran-bocornya-204-juta-data-pemilih-kpu</t>
+        </is>
+      </c>
+      <c r="H660" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/PAbAgyV5hyPTSxXruCP4txKklzA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/gugat-uu-pdp-di-MK.jpg</t>
+        </is>
+      </c>
+      <c r="I660" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>“Kata Siapa?” Istana Buka Suara soal Kabar Pratikno Sakit dan Mundur</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:44:56 +0700</t>
+        </is>
+      </c>
+      <c r="D661" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E661" t="inlineStr">
+        <is>
+          <t>Kabar Pratikno sakit dan mundur dari kabinet mencuat. Prasetyo Hadi merespons dengan pertanyaan singkat yang bikin penasaran.</t>
+        </is>
+      </c>
+      <c r="F661" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G661" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866883/kata-siapa-istana-buka-suara-soal-kabar-pratikno-sakit-dan-mundur</t>
+        </is>
+      </c>
+      <c r="H661" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/40n_NtqmQqryvyMyNWCtt6PdB-c=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Menteri-Sekretaris-Negara-Mensesneg-Prasetyo-Hadi-di-Istana-Kepresidenan-b.jpg</t>
+        </is>
+      </c>
+      <c r="I661" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>Jelang PKKMB UNS 2026: Cerita Maba Garap Tugas 'Dance Challenge' hingga Mental Rantau</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:43:45 +0700</t>
+        </is>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>Maba UNS siap sambut PKKMB 2026. Ada cerita unik tugas 'dance challenge' hingga orang tua asal Medan rela sewa kos di Solo</t>
+        </is>
+      </c>
+      <c r="F662" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G662" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/pendidikan/7866882/jelang-pkkmb-uns-2026-cerita-maba-garap-tugas-dance-challenge-hingga-mental-rantau</t>
+        </is>
+      </c>
+      <c r="H662" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/4G0NWMjUzqUXIUVsEEURnGIRP3A=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Mahasiswa-baru-berfoto-mengenakan-almamater-Universitas-Sebelas-Maret.jpg</t>
+        </is>
+      </c>
+      <c r="I662" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>Mendikti Saintek Dorong Pekerja dan Buruh Tempuh Pendidikan Tinggi, Bawa Dampak Positif Masyarakat</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:42:45 +0700</t>
+        </is>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>KSPSI dan Universitas Terbuka (UT) buka akses kuliah bagi pekerja, termasuk pengakuan pengalaman belajar yang bisa mempercepat kelulusan.</t>
+        </is>
+      </c>
+      <c r="F663" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G663" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7866881/mendikti-saintek-dorong-pekerja-dan-buruh-tempuh-pendidikan-tinggi-bawa-dampak-positif-masyarakat</t>
+        </is>
+      </c>
+      <c r="H663" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/tzBDOVxrLDBVSDlbXh27qvBe29A=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/mou-kspsi-dengan.jpg</t>
+        </is>
+      </c>
+      <c r="I663" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>Prakiraan Cuaca BMKG Kepulauan Bangka Belitung Rabu, 12 Agustus 2026: Seluruh Wilayah Berawan</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:42:31 +0700</t>
+        </is>
+      </c>
+      <c r="D664" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>Simak prakiraan cuaca BMKG untuk 7 kabupaten/kota di wilayah Provinsi Kepulauan Bangka Belitung pada Rabu, 12 Agustus 2026 besok.</t>
+        </is>
+      </c>
+      <c r="F664" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G664" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7866880/prakiraan-cuaca-bmkg-kepulauan-bangka-belitung-rabu-12-agustus-2026-seluruh-wilayah-berawan</t>
+        </is>
+      </c>
+      <c r="H664" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/d6Z05zmYE-ZlbOieHWf6t6Q66ws=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/cuaca-cerah-berawan-247.jpg</t>
+        </is>
+      </c>
+      <c r="I664" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>Meski Tampil Memukau di Pramusim, Karier Bek Muda Liverpool Terhalang Izin Kerja di Inggris</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:41:42 +0700</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr">
+        <is>
+          <t>Ifeanyi Ndukwe tampil memukau di laga pramusim, tapi bek 18 tahun itu tak bisa bela Liverpool di laga resmi karena terkendala izin kerja Inggris.</t>
+        </is>
+      </c>
+      <c r="F665" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G665" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7866879/meski-tampil-memukau-di-pramusim-karier-bek-muda-liverpool-terhalang-izin-kerja-di-inggris</t>
+        </is>
+      </c>
+      <c r="H665" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/2Ptks1b2u5Or_qpErExe_Sl1zFE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Wonderkid-Liverpool-Ifeanyi-Ndukwe.jpg</t>
+        </is>
+      </c>
+      <c r="I665" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>Sebelum Tewas Tertabrak KRL di Jurangmangu, Siswi Sempat Tulis Surat Terima Kasih untuk Guru</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:38:42 +0700</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>Siswi tewas tertabrak KRL di Jurangmangu dikenang hangat, beretika, dan penuh perhatian; sekolah siapkan pendampingan emosional.</t>
+        </is>
+      </c>
+      <c r="F666" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G666" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7866878/sebelum-tewas-tertabrak-krl-di-jurangmangu-siswi-sempat-tulis-surat-terima-kasih-untuk-guru</t>
+        </is>
+      </c>
+      <c r="H666" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/uU3KeK61xobdJ3IbGB3Mfc2n0Ww=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Suasana-di-Stasiun-Jurangmangu-32019.jpg</t>
+        </is>
+      </c>
+      <c r="I666" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>Trump Sesumbar AS Kuasai Selat Hormuz, Klaim Ranjau Iran Sudah Disapu Bersih Angkatan Laut</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:36:59 +0700</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr">
+        <is>
+          <t>Trump klaim AS kini menguasai Selat Hormuz dan telah membersihkan ranjau Iran. Namun, lalu lintas kapal masih lesu dan ketegangan kawasan belum mereda</t>
+        </is>
+      </c>
+      <c r="F667" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G667" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7866877/trump-sesumbar-as-kuasai-selat-hormuz-klaim-ranjau-iran-sudah-disapu-bersih-angkatan-laut</t>
+        </is>
+      </c>
+      <c r="H667" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/oDBKmF-o4X7LaPeSgKFA268fB_4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/irak-iran-hormuz-minyak.jpg</t>
+        </is>
+      </c>
+      <c r="I667" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>Perpres Ojol Hampir Rampung, Tinggal Finalisasi Rumusan Layanan Bisnisnya</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:36:56 +0700</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr">
+        <is>
+          <t>Pemerintah sedang memfinalisasi Peraturan Presiden tentang Transportasi Online dan dan memasukkan driver ojol sebagai pelaku UMKM.</t>
+        </is>
+      </c>
+      <c r="F668" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G668" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/bisnis/7866876/perpres-ojol-hampir-rampung-tinggal-finalisasi-rumusan-layanan-bisnisnya</t>
+        </is>
+      </c>
+      <c r="H668" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ToY5RNXIMgCawdSlzIrqK_cvB4s=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Prasetyo-Hadi-usai-acara-pembukaan-Konvensi-Sains.jpg</t>
+        </is>
+      </c>
+      <c r="I668" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>UEFA Rombak Penggunaan VAR, Panduan Penggunaan Disiapkan Khusus</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:35:13 +0700</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>UEFA mengeluarkan panduan resmi dari mereka untuk penggunaan VAR di kompetisi yang berada di bawah naungan mereka.</t>
+        </is>
+      </c>
+      <c r="F669" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G669" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7866875/uefa-rombak-penggunaan-var-panduan-penggunaan-disiapkan-khusus</t>
+        </is>
+      </c>
+      <c r="H669" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/TMVb2tGYVxi4Uz1fYumSRXNSLos=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/VIDEO-ASSISTANT-REFEREE-Wasit-Indonesia-Thoriq-Alkatiri.jpg</t>
+        </is>
+      </c>
+      <c r="I669" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>Bangkit Pascabencana, MIN 4 Aceh Tamiang Kembali Miliki Ruang Belajar Layak</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:33:34 +0700</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>Pemulihan MIN 4 Aceh Tamiang menjadi bagian dari upaya mengembalikan layanan pendidikan di wilayah terdampak bencana.</t>
+        </is>
+      </c>
+      <c r="F670" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G670" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7866874/bangkit-pascabencana-min-4-aceh-tamiang-kembali-miliki-ruang-belajar-layak</t>
+        </is>
+      </c>
+      <c r="H670" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Xy_VAKrCeb-sGCPMuGLokFR9_OQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/renovasi-min-4-aceh-tam.jpg</t>
+        </is>
+      </c>
+      <c r="I670" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>Otomotif</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>iCAR Resmikan Dealer ke-2 di SCBD, Perluas Akses Kendaraan Listrik di Pusat Bisnis Jakarta</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 15:02:03 +0700</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>Ferry kisihandi</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- iCAR Indonesia terus memperluas jaringan dealer di Indonesia melalui peresmian iCAR Andalan SCBD, dealer terbaru hasil kolaborasi dengan Andalan Group. 
+Berlokasi di kawasan pusat bisnis Jakarta,...</t>
+        </is>
+      </c>
+      <c r="F671" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G671" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjlibf472/icar-resmikan-dealer-ke2-di-scbd-perluas-akses-kendaraan-listrik-di-pusat-bisnis-jakarta</t>
+        </is>
+      </c>
+      <c r="H671" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/icar-indonesia-meresmikan-icar-andalan-scbd-dealer-terbaru-hasil_260811145931-618.jpeg</t>
+        </is>
+      </c>
+      <c r="I671" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>Finansial</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>OJK Siapkan Aturan Batas Kepemilikan Saham BEI Pasca-Demutualisasi</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:54:39 +0700</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>Friska Yolandha</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- Otoritas Jasa Keuangan (OJK) tengah mengkaji suatu konsep terkait pembatasan kepemilikan maksimum atas PT Bursa Efek Indonesia (BEI), yang akan dimasukkan sebagai ketentuan dalam Peraturan OJK (POJK)...</t>
+        </is>
+      </c>
+      <c r="F672" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G672" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjlhz3370/ojk-siapkan-aturan-batas-kepemilikan-saham-bei-pascademutualisasi</t>
+        </is>
+      </c>
+      <c r="H672" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/033504600-1785491442-830-556.jpg</t>
+        </is>
+      </c>
+      <c r="I672" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>Energi</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>Pertamina Patra Niaga Jalin Kerja Sama dengan Dukcapil, Perkuat Ketepatan Penyaluran Subsidi Energi</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:12:12 +0700</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>Intan Pratiwi</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA – PT Pertamina Patra Niaga dan Direktorat Jenderal Kependudukan dan Pencatatan Sipil (Ditjen Dukcapil) Kementerian Dalam Negeri menandatangani Perjanjian Kerja Sama (PKS) tentang Pemberian Hak Akses dan Pemanfaatan...</t>
+        </is>
+      </c>
+      <c r="F673" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G673" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjlg0c522/pertamina-patra-niaga-jalin-kerja-sama-dengan-dukcapil-perkuat-ketepatan-penyaluran-subsidi-energi</t>
+        </is>
+      </c>
+      <c r="H673" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/pt-pertamina-patra-niaga-dan-direktorat-jenderal-kependudukan-dan_260811141200-810.jpeg</t>
+        </is>
+      </c>
+      <c r="I673" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>Bisnis</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>Pelindo Multi Terminal Catat Kinerja Positif pada Semester I 2026</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 13:59:37 +0700</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>Friska Yolandha</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- Anak usaha PT Pelabuhan Indonesia (Persero), PT Pelindo Multi Terminal mencatatkan kinerja positif sepanjang Semester I 2026. SVP Sekretariat Perusahaan Pelindo Multi Terminal, Finan Syaifullah menyampaikan performa...</t>
+        </is>
+      </c>
+      <c r="F674" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G674" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjlffd370/pelindo-multi-terminal-catat-kinerja-positif-pada-semester-i-2026</t>
+        </is>
+      </c>
+      <c r="H674" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/_260625140731-748.png</t>
+        </is>
+      </c>
+      <c r="I674" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>Pertanian</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>Gejolak Harga Ayam di Tingkat Peternak, Ini Langkah yang Disiapkan Menteri Amran</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 13:55:56 +0700</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>Ahmad Fikri Noor</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, MAKASSAR -- Menteri Pertanian (Mentan) Andi Amran Sulaiman mengatakan pemerintah telah mengambil sejumlah langkah untuk mengatasi kendala yang dialami pengusaha, khususnya peternak ayam skala kecil. Amran Sulaiman di Makassar,...</t>
+        </is>
+      </c>
+      <c r="F675" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G675" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjlf98490/gejolak-harga-ayam-di-tingkat-peternak-ini-langkah-yang-disiapkan-menteri-amran</t>
+        </is>
+      </c>
+      <c r="H675" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/menteri-pertanian-mentan-andi-amran_260730145848-982.jpg</t>
+        </is>
+      </c>
+      <c r="I675" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>Jaksa Beberkan 27 Nama Penerima Uang dari Kasus Korupsi Kuota Haji Khusus</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:54:05 +0700</t>
+        </is>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>Angka yang mengalir ribuan hingga hingga jutaan dolar Amerika Serikat.</t>
+        </is>
+      </c>
+      <c r="F676" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G676" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267091/jaksa-beberkan-27-nama-penerima-uang-dari-kasus-korupsi-kuota-haji-khusus</t>
+        </is>
+      </c>
+      <c r="H676" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/Kcc9tinbWO-BlcvrzhwjP66t9xo=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9321231/original/009653200_1786434165-IMG_20260811_135837_642.jpg</t>
+        </is>
+      </c>
+      <c r="I676" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>Jaksa Agung Lantik 15 Kajati Baru, Berikut Daftarnya</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:52:44 +0700</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>Jaksa Agung melantik 15 Kajati baru, Sutikno ditunjuk memimpin Kejati Daerah Khusus Jakarta.</t>
+        </is>
+      </c>
+      <c r="F677" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G677" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267066/jaksa-agung-lantik-15-kajati-baru-berikut-daftarnya</t>
+        </is>
+      </c>
+      <c r="H677" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/Yo5lT28An9SWE-jU_7jwadGWHig=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9321214/original/065490500_1786433230-72289.jpg</t>
+        </is>
+      </c>
+      <c r="I677" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>Istana Tanggapi Isu Pratikno Sakit dan Mundur dari Menko PMK</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:06:22 +0700</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>Pratikno dipastikan dalam keadaan sehat.</t>
+        </is>
+      </c>
+      <c r="F678" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G678" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267027/istana-tanggapi-isu-pratikno-sakit-dan-mundur-dari-menko-pmk</t>
+        </is>
+      </c>
+      <c r="H678" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/cZ7D2E3mgROFKh5jB2cRxitzHZs=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/5429260/original/030041500_1764578706-Menteri_Koordinator_Bidang_Pembangunan_Manusia_dan_Kebudayaan__Menko_PMK___Pratikno__Membahas_Perihal_Screen_Time_dan_Kesehatan_Mental_Anak.jpg</t>
+        </is>
+      </c>
+      <c r="I678" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>Terungkap Awal Mula Ratusan Senjata Tersembunyi di Sekolah Jaksel</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:09:29 +0700</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>Pemeriksaan dilakukan di tiga ruangan, yakni ruang kerja eks ketua pengurus, ruang kerja eks sekretaris, serta ruang sarana dan prasarana.</t>
+        </is>
+      </c>
+      <c r="F679" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G679" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267049/terungkap-awal-mula-ratusan-senjata-tersembunyi-di-sekolah-jaksel</t>
+        </is>
+      </c>
+      <c r="H679" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/ETTDU2qEXOzAfRQOJ_Mo1H87TaE=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9317518/original/012310700_1786017988-Bungker.webp</t>
+        </is>
+      </c>
+      <c r="I679" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>DKI Tawarkan 41 Aset Milik SKPD, Bidik Investasi Rp 13,1 T</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:00:39 +0700</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>Jakarta membuka peluang investasi dari 41 aset dengan nilai fantastis.</t>
+        </is>
+      </c>
+      <c r="F680" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G680" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267033/dki-tawarkan-41-aset-milik-skpd-bidik-investasi-rp-131-t</t>
+        </is>
+      </c>
+      <c r="H680" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/DMN55_i-MOmhSUpVkYalQRTbCqk=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9321182/original/059652700_1786431601-fa13744b-1936-4aaa-9bac-1142fe76d418.jpg</t>
+        </is>
+      </c>
+      <c r="I680" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>Momen Kiai Anwar Zahid Terduduk di Pinggir Jalan Usai Kecelakaan</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:07:29 +0700</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr">
+        <is>
+          <t>Anwar Zahid terlihat duduk di pinggir jalan setelah kecelakaan. Dia mengenakan kemeja biru dan sarung tanpa alas kaki.</t>
+        </is>
+      </c>
+      <c r="F681" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G681" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267024/momen-kiai-anwar-zahid-terduduk-di-pinggir-jalan-usai-kecelakaan</t>
+        </is>
+      </c>
+      <c r="H681" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/nxBkJ0PQhGFf1fSMuinrfWXvbhw=/0x0:498x281/673x379/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9321169/original/028536600_1786431222-WhatsApp_Image_2026-08-11_at_13.23.08.jpeg</t>
+        </is>
+      </c>
+      <c r="I681" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>Sidang Perdana Yaqut Didakwa Rugikan Negara Rp 622 Miliar</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 13:54:06 +0700</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>Mantan Menteri Agama Yaqut Cholil Qoumas didakwa menerima USD271.500 dalam perkara dugaan korupsi pembagian kuota haji dan penyelenggaraan ibadah haji periode 2023-2024. Dakwaan dibacakan di Pengadilan Tipikor Jakarta, Selasa (11/8/2026). Jaksa juga mendakwa Yaqut terlibat dalam pengisian kuota haji khusus tambahan dengan jemaah tanpa masa tunggu. Perkara tersebut disebut menimbulkan kerugian negara lebih dari Rp 622 miliar berdasarkan laporan pemeriksaan investigatif BPK.</t>
+        </is>
+      </c>
+      <c r="F682" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G682" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/photo/read/8267016/sidang-perdana-yaqut-didakwa-rugikan-negara-rp-622-miliar</t>
+        </is>
+      </c>
+      <c r="H682" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/26W93yGTfQ9cKfAXNkCELGOQoJQ=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9321155/original/021946300_1786430943-ya1.jpg</t>
+        </is>
+      </c>
+      <c r="I682" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>SDN Kebayoran Lama Selatan 09 dan 11 Akan Digabung, Gedung Baru Ditargetkan Rampung Setahun</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 15:06:14 +0700</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr">
+        <is>
+          <t>SDN Kebayoran Lama Selatan 09 akan digabung dengan SDN Kebayoran Lama Selatan 11. Kedua gedung akan dibongkar dan dibangun ulang dalam setahun.</t>
+        </is>
+      </c>
+      <c r="F683" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G683" t="inlineStr">
+        <is>
+          <t>https://megapolitan.kompas.com/read/2026/08/11/15060751/sdn-kebayoran-lama-selatan-09-dan-11-akan-digabung-gedung-baru</t>
+        </is>
+      </c>
+      <c r="H683" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/pWlBYooKUUhEeV1FbfnCux5Ac0s=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/07/21/6a5ef7461e48a.jpeg</t>
+        </is>
+      </c>
+      <c r="I683" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>Ketika Bendera Merah Putih Tak Lagi Ramai Diburu, Pedagang Rasakan Lesunya Daya Beli</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 15:06:14 +0700</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>Meski omzet anjlok lebih dari 50%, Budiman pedagang bendera musiman di Tangerang tak gentar. Baginya, merah putih adalah tradisi dan hormat pada para pahlawan.</t>
+        </is>
+      </c>
+      <c r="F684" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G684" t="inlineStr">
+        <is>
+          <t>https://megapolitan.kompas.com/read/2026/08/11/14572991/ketika-bendera-merah-putih-tak-lagi-ramai-diburu-pedagang-rasakan-lesunya</t>
+        </is>
+      </c>
+      <c r="H684" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/hcwlM_-Nl37vQth-mRauUBsutvI=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/11/6a7abaf0ba928.jpg</t>
+        </is>
+      </c>
+      <c r="I684" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>Diduga Gejala Keracunan MBG Kambuh, 7 Siswa SMPN 3 Candimulyo Magelang Kembali Dirawat</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 15:06:14 +0700</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>Sebelumnya, sebanyak 26 siswa SMP 3 Candimulyo dilaporkan keracunan MBG pada 7 Agustus lalu.</t>
+        </is>
+      </c>
+      <c r="F685" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G685" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/08/11/143820678/diduga-gejala-keracunan-mbg-kambuh-7-siswa-smpn-3-candimulyo-magelang</t>
+        </is>
+      </c>
+      <c r="H685" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/DdCunleASRWX8Wicn6QGvk-WFww=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/11/6a7ac5abc4f14.jpg</t>
+        </is>
+      </c>
+      <c r="I685" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I581"/>
+  <autoFilter ref="A1:I685"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-11 11:41 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-11.xlsx
+++ b/data/berita_2026-08-11.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$992</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1088</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I992"/>
+  <dimension ref="A1:I1088"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -47062,8 +47062,4521 @@
         </is>
       </c>
     </row>
+    <row r="993">
+      <c r="A993" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B993" t="inlineStr">
+        <is>
+          <t>Askrindo pertahankan peringkat kredit proyeksi stabil idAA+</t>
+        </is>
+      </c>
+      <c r="C993" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:35:05 +0700</t>
+        </is>
+      </c>
+      <c r="D993" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E993" t="inlineStr">
+        <is>
+          <t>PT Asuransi Kredit Indonesia (Persero) atau Askrindo mempertahankan peringkat kredit proyeksi stabil idAA+ (Stable ...</t>
+        </is>
+      </c>
+      <c r="F993" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G993" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689615/askrindo-pertahankan-peringkat-kredit-proyeksi-stabil-idaa-</t>
+        </is>
+      </c>
+      <c r="H993" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/WhatsApp-Image-2026-08-11-at-15.11.54.jpeg</t>
+        </is>
+      </c>
+      <c r="I993" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B994" t="inlineStr">
+        <is>
+          <t>Kortastipidkor Polri: Dedi Congor tersangka kasus gratifikasi</t>
+        </is>
+      </c>
+      <c r="C994" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:33:26 +0700</t>
+        </is>
+      </c>
+      <c r="D994" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E994" t="inlineStr">
+        <is>
+          <t>Korps Pemberantasan Tindak Pidana Korupsi (Kortastipidkor) Polri menyatakan bahwa Pejabat Fungsional Bea Cukai Madya, ...</t>
+        </is>
+      </c>
+      <c r="F994" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G994" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689612/kortastipidkor-polri-dedi-congor-tersangka-kasus-gratifikasi</t>
+        </is>
+      </c>
+      <c r="H994" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/08/kpk-periksa-ahmad-dedi-sebagai-saksi-2786367.jpg</t>
+        </is>
+      </c>
+      <c r="I994" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B995" t="inlineStr">
+        <is>
+          <t>Dieng Culture Festival 28-30 Agustus 2026 usung "Spirit of Harmony"</t>
+        </is>
+      </c>
+      <c r="C995" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:31:34 +0700</t>
+        </is>
+      </c>
+      <c r="D995" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E995" t="inlineStr">
+        <is>
+          <t>Pergelaran Dieng Culture Festival (DCF) 2026 di kawasan Candi Dieng, Dieng Kulon, Kabupaten Banjarnegara, Jawa ...</t>
+        </is>
+      </c>
+      <c r="F995" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G995" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689611/dieng-culture-festival-28-30-agustus-2026-usung-spirit-of-harmony</t>
+        </is>
+      </c>
+      <c r="H995" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1002097496.jpg</t>
+        </is>
+      </c>
+      <c r="I995" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B996" t="inlineStr">
+        <is>
+          <t>Program MBG pulau terluar di Simeuleu mulai Oktober 2026</t>
+        </is>
+      </c>
+      <c r="C996" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:31:29 +0700</t>
+        </is>
+      </c>
+      <c r="D996" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E996" t="inlineStr">
+        <is>
+          <t>Penanggung Jawab Badan Gizi Nasional (BGN) Kabupaten Simeulue Zainuddin menyatakan program Makanan Bergizi Gratis (MBG) ...</t>
+        </is>
+      </c>
+      <c r="F996" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G996" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689608/program-mbg-pulau-terluar-di-simeuleu-mulai-oktober-2026</t>
+        </is>
+      </c>
+      <c r="H996" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/sekolah-pulau-terluar.jpeg</t>
+        </is>
+      </c>
+      <c r="I996" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B997" t="inlineStr">
+        <is>
+          <t>BI catat kinerja penjualan eceran Juni 2026 stabil</t>
+        </is>
+      </c>
+      <c r="C997" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:30:54 +0700</t>
+        </is>
+      </c>
+      <c r="D997" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E997" t="inlineStr">
+        <is>
+          <t>Bank Indonesia (BI) mencatat kinerja penjualan eceran pada Juni 2026 masih relatif stabil.
+Dalam Survei Penjualan ...</t>
+        </is>
+      </c>
+      <c r="F997" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G997" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689607/bi-catat-kinerja-penjualan-eceran-juni-2026-stabil</t>
+        </is>
+      </c>
+      <c r="H997" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/WhatsApp-Image-2026-05-13-at-11.55.22.jpeg</t>
+        </is>
+      </c>
+      <c r="I997" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B998" t="inlineStr">
+        <is>
+          <t>Ketum PBNU tegaskan Muktamar ke-35 fokus program dan arah kepemimpinan</t>
+        </is>
+      </c>
+      <c r="C998" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:30:44 +0700</t>
+        </is>
+      </c>
+      <c r="D998" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E998" t="inlineStr">
+        <is>
+          <t>Ketua Umum Pengurus Besar Nahdlatul Ulama (PBNU) KH Yahya Cholil Staquf yang akrab disapa “Gus Yahya” ...</t>
+        </is>
+      </c>
+      <c r="F998" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G998" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689604/ketum-pbnu-tegaskan-muktamar-ke-35-fokus-program-dan-arah-kepemimpinan</t>
+        </is>
+      </c>
+      <c r="H998" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG_1870.jpeg</t>
+        </is>
+      </c>
+      <c r="I998" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B999" t="inlineStr">
+        <is>
+          <t>Balai TNGR: Kebakaran lahan di kawasan Rinjani telah padam</t>
+        </is>
+      </c>
+      <c r="C999" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:29:50 +0700</t>
+        </is>
+      </c>
+      <c r="D999" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E999" t="inlineStr">
+        <is>
+          <t>Balai Taman Nasional Gunung Rinjani (TNGR) Nusa Tenggara Barat (NTB) menyatakan kebakaran permukaan lahan di sekitar ...</t>
+        </is>
+      </c>
+      <c r="F999" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G999" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689600/balai-tngr-kebakaran-lahan-di-kawasan-rinjani-telah-padam</t>
+        </is>
+      </c>
+      <c r="H999" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1005763318.jpg</t>
+        </is>
+      </c>
+      <c r="I999" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1000" t="inlineStr">
+        <is>
+          <t>Mendagri: Bayi lahir di luar faskes bisa dapat akta kelahiran digital</t>
+        </is>
+      </c>
+      <c r="C1000" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:27:05 +0700</t>
+        </is>
+      </c>
+      <c r="D1000" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1000" t="inlineStr">
+        <is>
+          <t>Menteri Dalam Negeri Muhammad Tito Karnavian memastikan layanan penerbitan akta kelahiran digital tetap bisa dinikmati ...</t>
+        </is>
+      </c>
+      <c r="F1000" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1000" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689596/mendagri-bayi-lahir-di-luar-faskes-bisa-dapat-akta-kelahiran-digital</t>
+        </is>
+      </c>
+      <c r="H1000" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1000583719.jpg</t>
+        </is>
+      </c>
+      <c r="I1000" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1001" t="inlineStr">
+        <is>
+          <t>Bapas Jakpus minta masyarakat hapus stigma terhadap mantan napi</t>
+        </is>
+      </c>
+      <c r="C1001" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:25:38 +0700</t>
+        </is>
+      </c>
+      <c r="D1001" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1001" t="inlineStr">
+        <is>
+          <t>Balai Pemasyarakatan (Bapas) Jakarta Pusat meminta masyarakat menghapus stigma terhadap mantan narapidana yang sedang ...</t>
+        </is>
+      </c>
+      <c r="F1001" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1001" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689595/bapas-jakpus-minta-masyarakat-hapus-stigma-terhadap-mantan-napi</t>
+        </is>
+      </c>
+      <c r="H1001" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1000836307.jpg</t>
+        </is>
+      </c>
+      <c r="I1001" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1002" t="inlineStr">
+        <is>
+          <t>CATL dan BYD berlomba kembangkan baterai "solid-state" pada 2027</t>
+        </is>
+      </c>
+      <c r="C1002" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:25:35 +0700</t>
+        </is>
+      </c>
+      <c r="D1002" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E1002" t="inlineStr">
+        <is>
+          <t>Dua produsen baterai kendaraan listrik (EV) terbesar China, CATL dan BYD, tengah berlomba mengembangkan teknologi ...</t>
+        </is>
+      </c>
+      <c r="F1002" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1002" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5689588/catl-dan-byd-berlomba-kembangkan-baterai-solid-state-pada-2027</t>
+        </is>
+      </c>
+      <c r="H1002" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/02/02/catl-factory.jpeg.jpg</t>
+        </is>
+      </c>
+      <c r="I1002" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1003" t="inlineStr">
+        <is>
+          <t>Hujan lebat mengancam, Beijing aktifkan respons kendali banjir</t>
+        </is>
+      </c>
+      <c r="C1003" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:25:34 +0700</t>
+        </is>
+      </c>
+      <c r="D1003" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1003" t="inlineStr">
+        <is>
+          <t>Pemerintah Beijing, China, pada Selasa mengaktifkan respons darurat pengendalian banjir Level II, level kedua ...</t>
+        </is>
+      </c>
+      <c r="F1003" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1003" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689592/hujan-lebat-mengancam-beijing-aktifkan-respons-kendali-banjir</t>
+        </is>
+      </c>
+      <c r="H1003" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/CjkinzN000020_20260811_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I1003" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1004" t="inlineStr">
+        <is>
+          <t>Eks presiden Suriah Bashar Al-Assad divonis mati secara "in absentia"</t>
+        </is>
+      </c>
+      <c r="C1004" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:25:14 +0700</t>
+        </is>
+      </c>
+      <c r="D1004" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1004" t="inlineStr">
+        <is>
+          <t>Mantan presiden Suriah Bashar Al-Assad beserta adiknya, Maher Al-Assad, dijatuhi hukuman mati dalam ketidakhadiran atau ...</t>
+        </is>
+      </c>
+      <c r="F1004" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1004" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689585/eks-presiden-suriah-bashar-al-assad-divonis-mati-secara-in-absentia</t>
+        </is>
+      </c>
+      <c r="H1004" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/02/23/thumbs_b_c_81edbce52422bafd7fba35e612901db4.jpg</t>
+        </is>
+      </c>
+      <c r="I1004" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1005" t="inlineStr">
+        <is>
+          <t>Wakil Ketua MPR soroti penebangan pohon ilegal di lapang padel Bandung</t>
+        </is>
+      </c>
+      <c r="C1005" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:25:02 +0700</t>
+        </is>
+      </c>
+      <c r="D1005" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1005" t="inlineStr">
+        <is>
+          <t>Wakil Ketua MPR RI Eddy Soeparno menyoroti kasus penebangan 10 pohon secara ilegal di Jalan LLRE Martadinata (Riau), ...</t>
+        </is>
+      </c>
+      <c r="F1005" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1005" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689584/wakil-ketua-mpr-soroti-penebangan-pohon-ilegal-di-lapang-padel-bandung</t>
+        </is>
+      </c>
+      <c r="H1005" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG_9446.jpeg</t>
+        </is>
+      </c>
+      <c r="I1005" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1006" t="inlineStr">
+        <is>
+          <t>KuCoin Raih Sertifikasi ISO 22301:2019, Perkuat Ketahanan Operasional</t>
+        </is>
+      </c>
+      <c r="C1006" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:23:52 +0700</t>
+        </is>
+      </c>
+      <c r="D1006" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1006" t="inlineStr">
+        <is>
+          <t>Di tengah pesatnya perkembangan aset digital dalam sistem keuangan global, kemampuan menjaga kesinambungan layanan ...</t>
+        </is>
+      </c>
+      <c r="F1006" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1006" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689580/kucoin-raih-sertifikasi-iso-223012019-perkuat-ketahanan-operasional</t>
+        </is>
+      </c>
+      <c r="H1006" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/KuCoin-Raih-ISO-223012019.jpg</t>
+        </is>
+      </c>
+      <c r="I1006" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1007" t="inlineStr">
+        <is>
+          <t>Kementerian Pariwisata dukung pengembangan Parapuar dan Golo Mori</t>
+        </is>
+      </c>
+      <c r="C1007" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:22:10 +0700</t>
+        </is>
+      </c>
+      <c r="D1007" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1007" t="inlineStr">
+        <is>
+          <t>Kementerian Pariwisata mendukung percepatan pengembangan daerah wisata Parapuar dan Golo Mori sebagai bagian dari ...</t>
+        </is>
+      </c>
+      <c r="F1007" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1007" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689576/kementerian-pariwisata-dukung-pengembangan-parapuar-dan-golo-mori</t>
+        </is>
+      </c>
+      <c r="H1007" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/Menteri-Pariwisata-di-Parapuar.jpeg</t>
+        </is>
+      </c>
+      <c r="I1007" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1008" t="inlineStr">
+        <is>
+          <t>Menteri UMKM: Perpres transportasi digital beri manfaat ekonomi ojol</t>
+        </is>
+      </c>
+      <c r="C1008" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:21:28 +0700</t>
+        </is>
+      </c>
+      <c r="D1008" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1008" t="inlineStr">
+        <is>
+          <t>Menteri Usaha Mikro, Kecil, dan Menengah (UMKM) Maman Abdurrahman mengungkapkan Peraturan Presiden (Perpres) tentang ...</t>
+        </is>
+      </c>
+      <c r="F1008" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1008" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689573/menteri-umkm-perpres-transportasi-digital-beri-manfaat-ekonomi-ojol</t>
+        </is>
+      </c>
+      <c r="H1008" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1040.jpg</t>
+        </is>
+      </c>
+      <c r="I1008" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1009" t="inlineStr">
+        <is>
+          <t>"Pertemuan teh susu" gantikan rapat formal warga lintas etnis Xinjiang</t>
+        </is>
+      </c>
+      <c r="C1009" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:19:01 +0700</t>
+        </is>
+      </c>
+      <c r="D1009" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1009" t="inlineStr">
+        <is>
+          <t>Di sebuah komunitas di Daerah Otonom Uighur Xinjiang, China barat laut, teh susu bukanlah sekadar minuman.    Saat ...</t>
+        </is>
+      </c>
+      <c r="F1009" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1009" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689569/pertemuan-teh-susu-gantikan-rapat-formal-warga-lintas-etnis-xinjiang</t>
+        </is>
+      </c>
+      <c r="H1009" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/CjkinzN000022_20260811_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I1009" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1010" t="inlineStr">
+        <is>
+          <t>Beasiswa YPMAK siapkan SDM Mimika untuk bangun daerah</t>
+        </is>
+      </c>
+      <c r="C1010" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:18:25 +0700</t>
+        </is>
+      </c>
+      <c r="D1010" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1010" t="inlineStr">
+        <is>
+          <t>Program beasiswa Yayasan Pengembangan Masyarakat Amungme dan Kamoro (YPMAK) menyiapkan sumber daya manusia asal Mimika, ...</t>
+        </is>
+      </c>
+      <c r="F1010" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1010" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689565/beasiswa-ypmak-siapkan-sdm-mimika-untuk-bangun-daerah</t>
+        </is>
+      </c>
+      <c r="H1010" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/WhatsApp-Image-2026-08-11-at-15.55.57_1.jpeg</t>
+        </is>
+      </c>
+      <c r="I1010" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1011" t="inlineStr">
+        <is>
+          <t>Legislator: Soekarno Cup panggung talenta muda pesepak bola Indonesia</t>
+        </is>
+      </c>
+      <c r="C1011" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:16:45 +0700</t>
+        </is>
+      </c>
+      <c r="D1011" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1011" t="inlineStr">
+        <is>
+          <t>Anggota DPRD DKI Jakarta Hardiyanto Kenneth menilai turnamen sepakbola Soekarno Cup 2026 yang digelar di Jawa Timur ...</t>
+        </is>
+      </c>
+      <c r="F1011" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1011" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689563/legislator-soekarno-cup-panggung-talenta-muda-pesepak-bola-indonesia</t>
+        </is>
+      </c>
+      <c r="H1011" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/WhatsApp-Image-2026-08-11-at-17.24.00.jpeg</t>
+        </is>
+      </c>
+      <c r="I1011" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1012" t="inlineStr">
+        <is>
+          <t>Indonesia bidik investasi AI via ASOCIO Digital Summit 2026 di Jakarta</t>
+        </is>
+      </c>
+      <c r="C1012" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:15:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1012" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1012" t="inlineStr">
+        <is>
+          <t>Indonesia membidik investasi, transfer teknologi dan akses pasar industri digital melalui ASOCIO Digital &amp; AI ...</t>
+        </is>
+      </c>
+      <c r="F1012" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1012" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689557/indonesia-bidik-investasi-ai-via-asocio-digital-summit-2026-di-jakarta</t>
+        </is>
+      </c>
+      <c r="H1012" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/F5DE283F-B921-4A52-A45C-5CC6650B327D.jpeg</t>
+        </is>
+      </c>
+      <c r="I1012" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1013" t="inlineStr">
+        <is>
+          <t>Target inklusi keuangan tercapai lebih cepat</t>
+        </is>
+      </c>
+      <c r="C1013" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:15:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1013" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1013" t="inlineStr">
+        <is>
+          <t>Akses masyarakat terhadap layanan keuangan terus meningkat, bahkan melampaui target yang ditetapkan dalam Rencana ...</t>
+        </is>
+      </c>
+      <c r="F1013" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1013" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/infografik/5689549/target-inklusi-keuangan-tercapai-lebih-cepat</t>
+        </is>
+      </c>
+      <c r="H1013" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/20260811-Target-inklusi-keuangan-tercapai-lebih-cepat.jpg</t>
+        </is>
+      </c>
+      <c r="I1013" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1014" t="inlineStr">
+        <is>
+          <t>Papua kirim 30 ton kopra senilai Rp516 juta ke Surabaya</t>
+        </is>
+      </c>
+      <c r="C1014" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:12:32 +0700</t>
+        </is>
+      </c>
+      <c r="D1014" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1014" t="inlineStr">
+        <is>
+          <t>ANTARA - Pemerintah Provinsi Papua melepas pengiriman 30 ton kopra hasil produksi petani Kabupaten Sarmi dengan nilai ...</t>
+        </is>
+      </c>
+      <c r="F1014" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1014" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5689513/papua-kirim-30-ton-kopra-senilai-rp516-juta-ke-surabaya</t>
+        </is>
+      </c>
+      <c r="H1014" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/PAPUA-KIRIM-30-TON-KOPRA-SENILAI-RP516-JUTA-KE-SURABAYA.jpg</t>
+        </is>
+      </c>
+      <c r="I1014" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1015" t="inlineStr">
+        <is>
+          <t>KRP rawat tradisi dan perjuangan Reyog jadi warisan budaya dunia</t>
+        </is>
+      </c>
+      <c r="C1015" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:07:59 +0700</t>
+        </is>
+      </c>
+      <c r="D1015" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1015" t="inlineStr">
+        <is>
+          <t>Komunitas Reyog Ponorogo (KRP) terus menunjukkan komitmennya dalam menjaga, merawat, dan memperkenalkan kesenian Reyog ...</t>
+        </is>
+      </c>
+      <c r="F1015" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1015" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689553/krp-rawat-tradisi-dan-perjuangan-reyog-jadi-warisan-budaya-dunia</t>
+        </is>
+      </c>
+      <c r="H1015" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/WhatsApp-Image-2026-08-11-at-16.56.57.jpeg</t>
+        </is>
+      </c>
+      <c r="I1015" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1016" t="inlineStr">
+        <is>
+          <t>Indocement wujudkan rumah layak untuk tukang yang mengabdi 51 tahun</t>
+        </is>
+      </c>
+      <c r="C1016" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:07:33 +0700</t>
+        </is>
+      </c>
+      <c r="D1016" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1016" t="inlineStr">
+        <is>
+          <t>PT Indocement Tunggal Prakarsa Tbk mewujudkan rumah layak bagi Sonijan (68), tukang bangunan di Lampung yang telah ...</t>
+        </is>
+      </c>
+      <c r="F1016" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1016" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689552/indocement-wujudkan-rumah-layak-untuk-tukang-yang-mengabdi-51-tahun</t>
+        </is>
+      </c>
+      <c r="H1016" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1003330149.jpg</t>
+        </is>
+      </c>
+      <c r="I1016" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1017" t="inlineStr">
+        <is>
+          <t>Menko PMK Pratikno bantah rumor dirinya minta mundur karena sakit</t>
+        </is>
+      </c>
+      <c r="C1017" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:01:34 +0700</t>
+        </is>
+      </c>
+      <c r="D1017" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1017" t="inlineStr">
+        <is>
+          <t>Menteri Koordinator Bidang Pembangunan Manusia dan Kebudayaan Pratikno membantah rumor yang menyebut dirinya ...</t>
+        </is>
+      </c>
+      <c r="F1017" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1017" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689547/menko-pmk-pratikno-bantah-rumor-dirinya-minta-mundur-karena-sakit</t>
+        </is>
+      </c>
+      <c r="H1017" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG_5576.jpg</t>
+        </is>
+      </c>
+      <c r="I1017" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1018" t="inlineStr">
+        <is>
+          <t>Mentan ajak maba Unhas berinovasi untuk kedaulatan pangan</t>
+        </is>
+      </c>
+      <c r="C1018" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:58:34 +0700</t>
+        </is>
+      </c>
+      <c r="D1018" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1018" t="inlineStr">
+        <is>
+          <t>Menteri Pertanian sekaligus Ketua Umum Ikatan Alumni Universitas Hasanuddin Andi Amran Sulaiman, mengajak 10.401 ...</t>
+        </is>
+      </c>
+      <c r="F1018" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1018" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689545/mentan-ajak-maba-unhas-berinovasi-untuk-kedaulatan-pangan</t>
+        </is>
+      </c>
+      <c r="H1018" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG-20260811-WA0088.jpg</t>
+        </is>
+      </c>
+      <c r="I1018" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1019" t="inlineStr">
+        <is>
+          <t>Pemkot Palangka Raya perpanjang status tanggap darurat karhutla dan kekeringan hingga 8 September 2026</t>
+        </is>
+      </c>
+      <c r="C1019" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:58:19 +0700</t>
+        </is>
+      </c>
+      <c r="D1019" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1019" t="inlineStr">
+        <is>
+          <t>Petugas berupaya memadamkan kebakaran lahan di Petuk Katimpun, Palangka Raya, Kalimantan Tengah.</t>
+        </is>
+      </c>
+      <c r="F1019" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1019" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5689543/pemkot-palangka-raya-perpanjang-status-tanggap-darurat-karhutla-dan-kekeringan-hingga-8-september-2026</t>
+        </is>
+      </c>
+      <c r="H1019" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/Status-Tanggap-Darurat-Karhutla-Dan-Kekeringan-Di-Palangka-Raya-110826-Aul-3.jpg</t>
+        </is>
+      </c>
+      <c r="I1019" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1020" t="inlineStr">
+        <is>
+          <t>Nusron sebut transformasi pelayanan pertanahan untuk tutup gerak mafia</t>
+        </is>
+      </c>
+      <c r="C1020" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:58:07 +0700</t>
+        </is>
+      </c>
+      <c r="D1020" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1020" t="inlineStr">
+        <is>
+          <t>Menteri Agraria dan Tata Ruang/Kepala Badan Pertanahan Nasional (ATR/BPN) Nusron Wahid mengatakan bahwa transformasi ...</t>
+        </is>
+      </c>
+      <c r="F1020" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1020" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689539/nusron-sebut-transformasi-pelayanan-pertanahan-untuk-tutup-gerak-mafia</t>
+        </is>
+      </c>
+      <c r="H1020" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG_20260803_175241.jpg</t>
+        </is>
+      </c>
+      <c r="I1020" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1021" t="inlineStr">
+        <is>
+          <t>Bapas Jakpus catat kasus narkoba dominasi klien pembebasan bersyarat</t>
+        </is>
+      </c>
+      <c r="C1021" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:55:21 +0700</t>
+        </is>
+      </c>
+      <c r="D1021" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1021" t="inlineStr">
+        <is>
+          <t>Balai Pemasyarakatan (Bapas) Jakarta Pusat mencatat kasus narkotika menjadi jenis perkara yang paling banyak ...</t>
+        </is>
+      </c>
+      <c r="F1021" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1021" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689535/bapas-jakpus-catat-kasus-narkoba-dominasi-klien-pembebasan-bersyarat</t>
+        </is>
+      </c>
+      <c r="H1021" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1000836313.jpg</t>
+        </is>
+      </c>
+      <c r="I1021" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1022" t="inlineStr">
+        <is>
+          <t>Unhas wakili Indonesia dalam Konferensi Perdamaian di Hiroshima</t>
+        </is>
+      </c>
+      <c r="C1022" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:54:28 +0700</t>
+        </is>
+      </c>
+      <c r="D1022" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1022" t="inlineStr">
+        <is>
+          <t>Universitas Hasanuddin menjadi satu-satunya perguruan tinggi dari Indonesia yang terlibat dalam 6th University ...</t>
+        </is>
+      </c>
+      <c r="F1022" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1022" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689532/unhas-wakili-indonesia-dalam-konferensi-perdamaian-di-hiroshima</t>
+        </is>
+      </c>
+      <c r="H1022" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG-20260811-WA0055.jpg</t>
+        </is>
+      </c>
+      <c r="I1022" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1023" t="inlineStr">
+        <is>
+          <t>BCA Syariah sebut emas masih jadi pilihan investasi jangka panjang</t>
+        </is>
+      </c>
+      <c r="C1023" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:53:45 +0700</t>
+        </is>
+      </c>
+      <c r="D1023" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1023" t="inlineStr">
+        <is>
+          <t>PT Bank BCA Syariah mengatakan emas masih menjadi instrumen investasi pilihan masyarakat untuk jangka ...</t>
+        </is>
+      </c>
+      <c r="F1023" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1023" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689531/bca-syariah-sebut-emas-masih-jadi-pilihan-investasi-jangka-panjang</t>
+        </is>
+      </c>
+      <c r="H1023" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG_0507.jpeg</t>
+        </is>
+      </c>
+      <c r="I1023" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1024" t="inlineStr">
+        <is>
+          <t>Gubernur Jateng: Penanganan sampah butuh aksi bersama</t>
+        </is>
+      </c>
+      <c r="C1024" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:53:06 +0700</t>
+        </is>
+      </c>
+      <c r="D1024" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1024" t="inlineStr">
+        <is>
+          <t>Gubernur Jawa Tengah (Jateng) Ahmad Luthfi menyatakan penanganan sampah di wilayah tersebut membutuhkan aksi ...</t>
+        </is>
+      </c>
+      <c r="F1024" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1024" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689528/gubernur-jateng-penanganan-sampah-butuh-aksi-bersama</t>
+        </is>
+      </c>
+      <c r="H1024" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1002097440.jpg</t>
+        </is>
+      </c>
+      <c r="I1024" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1025" t="inlineStr">
+        <is>
+          <t>Maluku hadirkan replika rumah Laksamana Maeda sambut HUT ke-81 RI</t>
+        </is>
+      </c>
+      <c r="C1025" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:51:34 +0700</t>
+        </is>
+      </c>
+      <c r="D1025" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1025" t="inlineStr">
+        <is>
+          <t>Pemerintah Provinsi Maluku menghadirkan replika rumah Laksamana Tadashi Maeda di Kota Ambon sebagai bagian dari ...</t>
+        </is>
+      </c>
+      <c r="F1025" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1025" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689527/maluku-hadirkan-replika-rumah-laksamana-maeda-sambut-hut-ke-81-ri</t>
+        </is>
+      </c>
+      <c r="H1025" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/Tanpa-Judul_2.jpg</t>
+        </is>
+      </c>
+      <c r="I1025" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1026" t="inlineStr">
+        <is>
+          <t>Pemkot Jaksel bagikan bendera Merah Putih jelang peringatan HUT RI</t>
+        </is>
+      </c>
+      <c r="C1026" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:47:31 +0700</t>
+        </is>
+      </c>
+      <c r="D1026" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1026" t="inlineStr">
+        <is>
+          <t>Pemerintah Kota Jakarta Selatan melakukan Gerakan Pembagian Bendera Merah Putih menjelang peringatan Hari Ulang Tahun ...</t>
+        </is>
+      </c>
+      <c r="F1026" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1026" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689523/pemkot-jaksel-bagikan-bendera-merah-putih-jelang-peringatan-hut-ri</t>
+        </is>
+      </c>
+      <c r="H1026" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1001022944.jpg</t>
+        </is>
+      </c>
+      <c r="I1026" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1027" t="inlineStr">
+        <is>
+          <t>Airlangga: Satgas Debottlenecking selesaikan 124 aduan perusahaan</t>
+        </is>
+      </c>
+      <c r="C1027" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:46:17 +0700</t>
+        </is>
+      </c>
+      <c r="D1027" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1027" t="inlineStr">
+        <is>
+          <t>Menteri Koordinator Bidang Perekonomian Airlangga Hartarto menyebut Satgas Debottlenecking telah menyelesaikan 124 dari ...</t>
+        </is>
+      </c>
+      <c r="F1027" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1027" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689519/airlangga-satgas-debottlenecking-selesaikan-124-aduan-perusahaan</t>
+        </is>
+      </c>
+      <c r="H1027" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/779C2F71-F737-4EB6-AB41-D3E05C413485.jpeg</t>
+        </is>
+      </c>
+      <c r="I1027" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1028" t="inlineStr">
+        <is>
+          <t>Dirjen Bea Cukai sebut pembenahan kinerja instansinya mulai terlihat</t>
+        </is>
+      </c>
+      <c r="C1028" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:45:16 +0700</t>
+        </is>
+      </c>
+      <c r="D1028" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1028" t="inlineStr">
+        <is>
+          <t>Direktur Jenderal Bea dan Cukai Djaka Budi Utama menanggapi soal tenggat waktu yang diberikan Menteri Keuangan Purbaya ...</t>
+        </is>
+      </c>
+      <c r="F1028" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1028" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689516/dirjen-bea-cukai-sebut-pembenahan-kinerja-instansinya-mulai-terlihat</t>
+        </is>
+      </c>
+      <c r="H1028" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/e8bb8266-c29a-48d2-be88-451361dbd840.jpeg</t>
+        </is>
+      </c>
+      <c r="I1028" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1029" t="inlineStr">
+        <is>
+          <t>Mentan ancam cabut izin pelaku manipulasi harga pakan dan telur</t>
+        </is>
+      </c>
+      <c r="C1029" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:43:22 +0700</t>
+        </is>
+      </c>
+      <c r="D1029" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1029" t="inlineStr">
+        <is>
+          <t>Menteri Pertanian (Mentan) Andi Amran Sulaiman mengancam mencabut izin usaha pelaku manipulasi harga pakan dan telur ...</t>
+        </is>
+      </c>
+      <c r="F1029" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1029" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689511/mentan-ancam-cabut-izin-pelaku-manipulasi-harga-pakan-dan-telur</t>
+        </is>
+      </c>
+      <c r="H1029" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1347084.jpg</t>
+        </is>
+      </c>
+      <c r="I1029" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1030" t="inlineStr">
+        <is>
+          <t>Warga Pulau Seribu sambut transportasi laut dikelola Transjakarta</t>
+        </is>
+      </c>
+      <c r="C1030" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:42:22 +0700</t>
+        </is>
+      </c>
+      <c r="D1030" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1030" t="inlineStr">
+        <is>
+          <t>Warga Pulau Sabira, Kabupaten Kepulauan Seribu, Agung, menyambut positif rencana pengalihan pengelolaan transportasi ...</t>
+        </is>
+      </c>
+      <c r="F1030" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1030" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689509/warga-pulauseribu-sambut-transportasi-laut-dikelola-transjakarta</t>
+        </is>
+      </c>
+      <c r="H1030" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/20260811105212.jpeg</t>
+        </is>
+      </c>
+      <c r="I1030" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1031" t="inlineStr">
+        <is>
+          <t>KJRI Kuching gelar rangkaian HUT ke-81 di Sarawak</t>
+        </is>
+      </c>
+      <c r="C1031" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:41:42 +0700</t>
+        </is>
+      </c>
+      <c r="D1031" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1031" t="inlineStr">
+        <is>
+          <t>Konsulat Jenderal Republik Indonesia (KJRI) Kuching bersama masyarakat Indonesia menggelar rangkaian kegiatan ...</t>
+        </is>
+      </c>
+      <c r="F1031" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1031" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689508/kjri-kuching-gelar-rangkaian-hut-ke-81-di-sarawak</t>
+        </is>
+      </c>
+      <c r="H1031" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/DSC08638_1.jpg</t>
+        </is>
+      </c>
+      <c r="I1031" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1032" t="inlineStr">
+        <is>
+          <t>HIMKI bidik pengembangan kekuatan ekspor industri kerajinan di Jabar</t>
+        </is>
+      </c>
+      <c r="C1032" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:41:31 +0700</t>
+        </is>
+      </c>
+      <c r="D1032" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1032" t="inlineStr">
+        <is>
+          <t>Himpunan Industri Mebel dan Kerajinan Indonesia (HIMKI) membidik Kawasan Priangan, Jawa Barat (Jabar), sebagai sentra ...</t>
+        </is>
+      </c>
+      <c r="F1032" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1032" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689504/himki-bidik-pengembangan-kekuatan-ekspor-industri-kerajinan-di-jabar</t>
+        </is>
+      </c>
+      <c r="H1032" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/Roadshow-Himki.jpg</t>
+        </is>
+      </c>
+      <c r="I1032" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1033" t="inlineStr">
+        <is>
+          <t>Rakor Konflik Agraria, Mendes Rekomendasikan Solusi Desa dalam Kawasan Hutan</t>
+        </is>
+      </c>
+      <c r="C1033" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:31:10 +0700</t>
+        </is>
+      </c>
+      <c r="D1033" t="inlineStr">
+        <is>
+          <t>Chayyara Zulghifary</t>
+        </is>
+      </c>
+      <c r="E1033" t="inlineStr">
+        <is>
+          <t>Menteri Yandri Susanto merekomendasikan solusi untuk konflik agraria di desa, melibatkan kementerian terkait dan memastikan pemulihan masyarakat.</t>
+        </is>
+      </c>
+      <c r="F1033" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1033" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614179/rakor-konflik-agraria-mendes-rekomendasikan-solusi-desa-dalam-kawasan-hutan</t>
+        </is>
+      </c>
+      <c r="H1033" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/kemendes-1786447831798.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1033" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1034" t="inlineStr">
+        <is>
+          <t>Bejat! Guru Ngaji di Serang Diduga Cabuli Bocah 9 Tahun</t>
+        </is>
+      </c>
+      <c r="C1034" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:30:22 +0700</t>
+        </is>
+      </c>
+      <c r="D1034" t="inlineStr">
+        <is>
+          <t>Arief Ikhsanudin</t>
+        </is>
+      </c>
+      <c r="E1034" t="inlineStr">
+        <is>
+          <t>Seorang guru ngaji berinisial MS ditangkap karena mencabuli muridnya yang berusia 9 tahun. Pencabulan terjadi dua kali di rumah korban saat orang tua tidak ada.</t>
+        </is>
+      </c>
+      <c r="F1034" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1034" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614178/bejat-guru-ngaji-di-serang-diduga-cabuli-bocah-9-tahun</t>
+        </is>
+      </c>
+      <c r="H1034" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2023/12/21/ilustrasi-kekerasan-pada-anak_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1034" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1035" t="inlineStr">
+        <is>
+          <t>Pramono Terima Banyak Masukan Jalur Sepeda Dihapus: Akan Dibahas Khusus</t>
+        </is>
+      </c>
+      <c r="C1035" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:21:38 +0700</t>
+        </is>
+      </c>
+      <c r="D1035" t="inlineStr">
+        <is>
+          <t>Brigitta Belia Permata Sari</t>
+        </is>
+      </c>
+      <c r="E1035" t="inlineStr">
+        <is>
+          <t>Warga Jakarta usulkan penghapusan jalur sepeda di jalan protokol. Gubernur Pramono Anung akan evaluasi penggunaan fasilitas sepeda untuk mengurangi kemacetan.</t>
+        </is>
+      </c>
+      <c r="F1035" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1035" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614156/pramono-terima-banyak-masukan-jalur-sepeda-dihapus-akan-dibahas-khusus</t>
+        </is>
+      </c>
+      <c r="H1035" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/04/pramono-anung-beliadetikcom-1785834009810_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1035" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1036" t="inlineStr">
+        <is>
+          <t>Wamensos Minta Bupati Mandailing Natal Kebut Pengajuan Sekolah Rakyat</t>
+        </is>
+      </c>
+      <c r="C1036" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:20:24 +0700</t>
+        </is>
+      </c>
+      <c r="D1036" t="inlineStr">
+        <is>
+          <t>Moch. Prima Fauzi</t>
+        </is>
+      </c>
+      <c r="E1036" t="inlineStr">
+        <is>
+          <t>Wamensos Agus Jabo mendorong Pemkab Mandailing Natal percepat pembangunan Sekolah Rakyat dan pemutakhiran Data Tunggal Sosial untuk program pemerintah.</t>
+        </is>
+      </c>
+      <c r="F1036" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1036" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614081/wamensos-minta-bupati-mandailing-natal-kebut-pengajuan-sekolah-rakyat</t>
+        </is>
+      </c>
+      <c r="H1036" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/wamensos-agus-jabo-1786445183993_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1036" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1037">
+      <c r="A1037" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1037" t="inlineStr">
+        <is>
+          <t>Perusak Palang Kereta di Sleman Ternyata Juga Rusak Bendera di Bantul</t>
+        </is>
+      </c>
+      <c r="C1037" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:18:58 +0700</t>
+        </is>
+      </c>
+      <c r="D1037" t="inlineStr">
+        <is>
+          <t>Pradito Rida</t>
+        </is>
+      </c>
+      <c r="E1037" t="inlineStr">
+        <is>
+          <t>Polisi selidiki perusakan tiang dan bendera merah putih di Bantul. Pelaku, mahasiswa luar Jogja, diduga dalam kondisi mabuk saat beraksi.</t>
+        </is>
+      </c>
+      <c r="F1037" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1037" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614153/perusak-palang-kereta-di-sleman-ternyata-juga-rusak-bendera-di-bantul</t>
+        </is>
+      </c>
+      <c r="H1037" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2022/03/21/teks-undang-undang-dasar-1945-pembukaan-hingga-maknanya_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1037" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1038" t="inlineStr">
+        <is>
+          <t>Kejagung Gandeng PPATK Telusuri Uang TTPU di Kasus Febrie</t>
+        </is>
+      </c>
+      <c r="C1038" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:17:40 +0700</t>
+        </is>
+      </c>
+      <c r="D1038" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E1038" t="inlineStr">
+        <is>
+          <t>Kejagung RI menggandeng PPATK untuk mengusut kasus TPPU mantan Jampidsus Febrie Adriansyah. Penelusuran aliran uang dilakukan dengan hati-hati dan profesional.</t>
+        </is>
+      </c>
+      <c r="F1038" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1038" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614152/kejagung-gandeng-ppatk-telusuri-uang-ttpu-di-kasus-febrie</t>
+        </is>
+      </c>
+      <c r="H1038" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/febrie-adriansyah-dibawa-ke-kejagung-untuk-diperiksa-tim-9-1786087110132_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1038" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1039" t="inlineStr">
+        <is>
+          <t>USU Buka Suara Terkait Dugaan Pengosongan Paksa Gereja Chapel</t>
+        </is>
+      </c>
+      <c r="C1039" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:13:42 +0700</t>
+        </is>
+      </c>
+      <c r="D1039" t="inlineStr">
+        <is>
+          <t>Rechtin Hani Ritonga</t>
+        </is>
+      </c>
+      <c r="E1039" t="inlineStr">
+        <is>
+          <t>Puluhan jemaat Gereja POUK Chapel USU histeris setelah pengosongan paksa. USU menjelaskan relokasi untuk renovasi demi peningkatan fasilitas ibadah.</t>
+        </is>
+      </c>
+      <c r="F1039" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1039" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614145/usu-buka-suara-terkait-dugaan-pengosongan-paksa-gereja-chapel</t>
+        </is>
+      </c>
+      <c r="H1039" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/10/gereja-di-usu-1786348148267_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1039" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1040" t="inlineStr">
+        <is>
+          <t>Kepala BGN Minta Kejati dan Kejari Ikut Awasi Pelaksanaan Program MBG</t>
+        </is>
+      </c>
+      <c r="C1040" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:11:40 +0700</t>
+        </is>
+      </c>
+      <c r="D1040" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E1040" t="inlineStr">
+        <is>
+          <t>Sudaryono meminta langsung kepada Jaksa Agung ST Burhanuddin agar kejati dan kejari ikut mendampingi dan mengawasi pelaksanaan program Makan Bergizi Gratis.</t>
+        </is>
+      </c>
+      <c r="F1040" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1040" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614139/kepala-bgn-minta-kejati-dan-kejari-ikut-awasi-pelaksanaan-program-mbg</t>
+        </is>
+      </c>
+      <c r="H1040" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/jajaran-bgn-menyambangi-kejagung-untuk-bersilaturahmi-sekaligus-meminta-pendampingan-dan-pengawasan-pelaksanaan-program-makan--1786440210989_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1040" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1041" t="inlineStr">
+        <is>
+          <t>Pratikno Bantah Isu Mundur dari Menko PMK: Saya Lagi Bertugas di Bromo</t>
+        </is>
+      </c>
+      <c r="C1041" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:05:13 +0700</t>
+        </is>
+      </c>
+      <c r="D1041" t="inlineStr">
+        <is>
+          <t>Firda Cynthia Anggrainy</t>
+        </is>
+      </c>
+      <c r="E1041" t="inlineStr">
+        <is>
+          <t>Menko PMK Pratikno membantah rumor sakit dan mundur. Ia aktif mengikuti rapat penanganan kebakaran hutan di Bromo, memastikan tetap bertugas.</t>
+        </is>
+      </c>
+      <c r="F1041" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1041" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614134/pratikno-bantah-isu-mundur-dari-menko-pmk-saya-lagi-bertugas-di-bromo</t>
+        </is>
+      </c>
+      <c r="H1041" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/menko-pmk-pratikno-cek-karhutla-di-bromo-1786446259408_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1041" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1042" t="inlineStr">
+        <is>
+          <t>Akta Kelahiran Kini Semakin Mudah, Langsung Terbit Setelah Bayi Lahir</t>
+        </is>
+      </c>
+      <c r="C1042" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:59:51 +0700</t>
+        </is>
+      </c>
+      <c r="D1042" t="inlineStr">
+        <is>
+          <t>Inkana Putri</t>
+        </is>
+      </c>
+      <c r="E1042" t="inlineStr">
+        <is>
+          <t>Pemerintah Digitalisasi Penerbitan Akta Kelahiran, integrasi SIAK di Puskesmas Pasar Minggu. Proses penerbitan dokumen kependudukan lebih cepat &amp; efisien.</t>
+        </is>
+      </c>
+      <c r="F1042" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1042" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614117/akta-kelahiran-kini-semakin-mudah-langsung-terbit-setelah-bayi-lahir</t>
+        </is>
+      </c>
+      <c r="H1042" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/kemenpan-rb-1786445973378_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1042" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1043" t="inlineStr">
+        <is>
+          <t>Jaksa Agung Minta Kajati Beri Perhatian Kasus Terkait Hajat Hidup Masyarakat</t>
+        </is>
+      </c>
+      <c r="C1043" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:56:08 +0700</t>
+        </is>
+      </c>
+      <c r="D1043" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E1043" t="inlineStr">
+        <is>
+          <t>Jaksa Agung ST Burhanuddin meminta para kajati memberikan perhatian khusus terhadap kasus-kasus yang menyangkut hajat hidup masyarakat.</t>
+        </is>
+      </c>
+      <c r="F1043" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1043" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614111/jaksa-agung-minta-kajati-beri-perhatian-kasus-terkait-hajat-hidup-masyarakat</t>
+        </is>
+      </c>
+      <c r="H1043" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/jaksa-agung-st-burhanuddin-meminta-para-kajati-memberikan-perhatian-khusus-terhadap-kasus-kasus-yang-menyangkut-hajat-hidup-ma-1786445750598_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1043" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1044" t="inlineStr">
+        <is>
+          <t>Soekarno Cup 2026, Kenneth PDIP Dorong Talenta Muda Berani Bermimpi Besar</t>
+        </is>
+      </c>
+      <c r="C1044" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:55:26 +0700</t>
+        </is>
+      </c>
+      <c r="D1044" t="inlineStr">
+        <is>
+          <t>Dea Duta Aulia</t>
+        </is>
+      </c>
+      <c r="E1044" t="inlineStr">
+        <is>
+          <t>Politisi PDI Perjuangan Hardiyanto Kenneth apresiasi Soekarno Cup 2026, menekankan pentingnya pembinaan sepakbola untuk talenta muda Indonesia.</t>
+        </is>
+      </c>
+      <c r="F1044" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1044" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614108/soekarno-cup-2026-kenneth-pdip-dorong-talenta-muda-berani-bermimpi-besar</t>
+        </is>
+      </c>
+      <c r="H1044" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/politisi-pdi-perjuangan-hardiyanto-kenneth-mengapresiasi-diadakannya-soekarno-cup-2026-1786445694184_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1044" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1045" t="inlineStr">
+        <is>
+          <t>Nusron soal Isu Reshuffle Usai 17 Agustus: Tak Elok Menteri Ngomong Itu</t>
+        </is>
+      </c>
+      <c r="C1045" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:54:38 +0700</t>
+        </is>
+      </c>
+      <c r="D1045" t="inlineStr">
+        <is>
+          <t>Dwi Rahmawati</t>
+        </is>
+      </c>
+      <c r="E1045" t="inlineStr">
+        <is>
+          <t>Menteri ATR/BPN Nusron Wahid menanggapi isu reshuffle kabinet. Dia menegaskan semua prerogatif presiden dan tak elok menteri membahas hal itu.</t>
+        </is>
+      </c>
+      <c r="F1045" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1045" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614107/nusron-soal-isu-reshuffle-usai-17-agustus-tak-elok-menteri-ngomong-itu</t>
+        </is>
+      </c>
+      <c r="H1045" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/menteri-atr-bpn-nusron-wahid-di-dpr-dwi-rahmawatidetik-1786445662574.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1045" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1046" t="inlineStr">
+        <is>
+          <t>Rangkul Generasi Muda, PDIP Lantik Dewan Taruna Merah Putih</t>
+        </is>
+      </c>
+      <c r="C1046" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:52:56 +0700</t>
+        </is>
+      </c>
+      <c r="D1046" t="inlineStr">
+        <is>
+          <t>Dea Duta Aulia</t>
+        </is>
+      </c>
+      <c r="E1046" t="inlineStr">
+        <is>
+          <t>PDI Perjuangan melantik DPP Taruna Merah Putih untuk merangkul generasi muda. Fokus pada pendidikan politik dan mengubah persepsi politik menjadi lebih positif.</t>
+        </is>
+      </c>
+      <c r="F1046" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1046" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614099/rangkul-generasi-muda-pdip-lantik-dewan-taruna-merah-putih</t>
+        </is>
+      </c>
+      <c r="H1046" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/pdip-1786445540734_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1046" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1047">
+      <c r="A1047" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1047" t="inlineStr">
+        <is>
+          <t>Pigai Perintahkan Jajaran KemenHAM Bantu Kendalikan Dampak El Nino</t>
+        </is>
+      </c>
+      <c r="C1047" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:47:03 +0700</t>
+        </is>
+      </c>
+      <c r="D1047" t="inlineStr">
+        <is>
+          <t>Chayyara Zulghifary</t>
+        </is>
+      </c>
+      <c r="E1047" t="inlineStr">
+        <is>
+          <t>Menteri HAM Natalius Pigai perintahkan KemenHAM RI untuk berkoordinasi dengan pemerintah daerah dalam mengatasi dampak fenomena El Nino.</t>
+        </is>
+      </c>
+      <c r="F1047" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1047" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614082/pigai-perintahkan-jajaran-kemenham-bantu-kendalikan-dampak-el-nino</t>
+        </is>
+      </c>
+      <c r="H1047" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/menteri-hak-asasi-manusia-ham-natalius-pigai-1786445195449.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1047" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1048">
+      <c r="A1048" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1048" t="inlineStr">
+        <is>
+          <t>Mahasiswa Mabuk Jadi Tersangka Tabrak Lari Aiptu Asep, 2 Anggota TNI Jadi Saksi</t>
+        </is>
+      </c>
+      <c r="C1048" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:46:16 +0700</t>
+        </is>
+      </c>
+      <c r="D1048" t="inlineStr">
+        <is>
+          <t>Wisma Putra</t>
+        </is>
+      </c>
+      <c r="E1048" t="inlineStr">
+        <is>
+          <t>Polisi menetapkan mahasiswa berinisial A sebagai tersangka tabrak lari yang menewaskan Aiptu Asep Suhara. Pelaku mengemudi dalam kondisi mabuk.</t>
+        </is>
+      </c>
+      <c r="F1048" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1048" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614084/mahasiswa-mabuk-jadi-tersangka-tabrak-lari-aiptu-asep-2-anggota-tni-jadi-saksi</t>
+        </is>
+      </c>
+      <c r="H1048" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/konferensi-pers-kasus-tabrak-lari-di-bandung-1786438422534_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1048" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1049">
+      <c r="A1049" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1049" t="inlineStr">
+        <is>
+          <t>Viral TPS Liar Cilincing, Pram Minta Pengelola Diberhentikan dan Disanksi</t>
+        </is>
+      </c>
+      <c r="C1049" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:44:17 +0700</t>
+        </is>
+      </c>
+      <c r="D1049" t="inlineStr">
+        <is>
+          <t>Brigitta Belia Permata Sari</t>
+        </is>
+      </c>
+      <c r="E1049" t="inlineStr">
+        <is>
+          <t>Hamparan sampah di Cilincing, Jakut ramai disorot publik. Gubernur DKI Pramono Anung meminta pihak swasta pengelola TPS itu diberhentikan dan diberi sanksi.</t>
+        </is>
+      </c>
+      <c r="F1049" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1049" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614073/viral-tps-liar-cilincing-pram-minta-pengelola-diberhentikan-dan-disanksi</t>
+        </is>
+      </c>
+      <c r="H1049" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/05/08/gunungan-sampah-liar-cemari-kawasan-cilincing-1778231251896_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1049" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1050">
+      <c r="A1050" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1050" t="inlineStr">
+        <is>
+          <t>Andre Rosiade Terima Aspirasi Serikat Pekerja PT Pos, Dorong Solusi Bersama Danantara</t>
+        </is>
+      </c>
+      <c r="C1050" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:43:28 +0700</t>
+        </is>
+      </c>
+      <c r="D1050" t="inlineStr">
+        <is>
+          <t>Anggi Muliawati</t>
+        </is>
+      </c>
+      <c r="E1050" t="inlineStr">
+        <is>
+          <t>Andre Rosiade mengatakan Komisi VI DPR akan fasilitasi pertemuan antara serikat pekerja dan PT Pos Indonesia untuk membahas isu kesejahteraan dan hak pekerja.</t>
+        </is>
+      </c>
+      <c r="F1050" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1050" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614071/andre-rosiade-terima-aspirasi-serikat-pekerja-pt-pos-dorong-solusi-bersama-danantara</t>
+        </is>
+      </c>
+      <c r="H1050" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/komisi-iv-dpr-menerima-audiensi-serikat-pekerja-pt-pos-indonesia-1786443565666_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1050" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1051">
+      <c r="A1051" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1051" t="inlineStr">
+        <is>
+          <t>Pramono Kecam Challenge Hafalan Qur'an demi Miras: Nodai Kehidupan Keagamaan</t>
+        </is>
+      </c>
+      <c r="C1051" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:42:14 +0700</t>
+        </is>
+      </c>
+      <c r="D1051" t="inlineStr">
+        <is>
+          <t>Brigitta Belia Permata Sari</t>
+        </is>
+      </c>
+      <c r="E1051" t="inlineStr">
+        <is>
+          <t>Gubernur DKI Jakarta Pramono Anung mengecam promosi miras yang mengaitkan dengan hafalan Al-Qur'an. Ia minta tindakan tegas agar hal ini tidak terjadi lagi.</t>
+        </is>
+      </c>
+      <c r="F1051" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1051" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614068/pramono-kecam-challenge-hafalan-quran-demi-miras-nodai-kehidupan-keagamaan</t>
+        </is>
+      </c>
+      <c r="H1051" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/gubernur-dki-jakarta-pramono-anung-1786444893623_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1051" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1052">
+      <c r="A1052" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1052" t="inlineStr">
+        <is>
+          <t>Menkes Ungkap Ada 300 Ribu Pecandu Narkoba di Indonesia</t>
+        </is>
+      </c>
+      <c r="C1052" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:41:30 +0700</t>
+        </is>
+      </c>
+      <c r="D1052" t="inlineStr">
+        <is>
+          <t>Rizky Adha Mahendra</t>
+        </is>
+      </c>
+      <c r="E1052" t="inlineStr">
+        <is>
+          <t>Menkes Budi Gunadi Sadikin mengungkapkan 300 ribu pecandu narkoba di Indonesia, banyak di penjara. Ia mendorong rehabilitasi untuk pemulihan dan produktivitas.</t>
+        </is>
+      </c>
+      <c r="F1052" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1052" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614064/menkes-ungkap-ada-300-ribu-pecandu-narkoba-di-indonesia</t>
+        </is>
+      </c>
+      <c r="H1052" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/10/07/rsppn-gandeng-china-kembangkan-pengobatan-tradisional-1759829199185_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1052" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1053">
+      <c r="A1053" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1053" t="inlineStr">
+        <is>
+          <t>Sinergi Kemensos dan INABA Entaskan Kemiskinan Melalui Sekolah Rakyat</t>
+        </is>
+      </c>
+      <c r="C1053" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:40:35 +0700</t>
+        </is>
+      </c>
+      <c r="D1053" t="inlineStr">
+        <is>
+          <t>Moch. Prima Fauzi</t>
+        </is>
+      </c>
+      <c r="E1053" t="inlineStr">
+        <is>
+          <t>Kementerian Sosial dan Universitas Indonesia Membangun (INABA) menandatangani MoU untuk memperkuat kolaborasi dalam pengentasan kemiskinan.</t>
+        </is>
+      </c>
+      <c r="F1053" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1053" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614063/sinergi-kemensos-dan-inaba-entaskan-kemiskinan-melalui-sekolah-rakyat</t>
+        </is>
+      </c>
+      <c r="H1053" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/kemensos-kerja-sama-dengan-inaba-entaskan-kemiskinan-1786444816995_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1053" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1054">
+      <c r="A1054" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1054" t="inlineStr">
+        <is>
+          <t>Kejagung Hati-hati Usut Kasus Febrie: Yang Kita Hadapi Mantan Pendekar Hukum</t>
+        </is>
+      </c>
+      <c r="C1054" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:39:29 +0700</t>
+        </is>
+      </c>
+      <c r="D1054" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E1054" t="inlineStr">
+        <is>
+          <t>Kapuspenkum Kejagung Anang Supriatna mengatakan pihaknya siap buka-bukaan di persidangan dalam membeberkan peran dari Febrie Adriansyah.</t>
+        </is>
+      </c>
+      <c r="F1054" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1054" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614061/kejagung-hati-hati-usut-kasus-febrie-yang-kita-hadapi-mantan-pendekar-hukum</t>
+        </is>
+      </c>
+      <c r="H1054" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/02/03/kapuspenkum-kejagung-anang-supriatna-1770098880799_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1054" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1055">
+      <c r="A1055" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1055" t="inlineStr">
+        <is>
+          <t>Polisi Pastikan Saepul Pemutilasi Pria di Depok Pelaku Tunggal</t>
+        </is>
+      </c>
+      <c r="C1055" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 15:01:11 +0700</t>
+        </is>
+      </c>
+      <c r="D1055" t="inlineStr">
+        <is>
+          <t>Devi Puspitasari</t>
+        </is>
+      </c>
+      <c r="E1055" t="inlineStr">
+        <is>
+          <t>Polisi mengatakan Saepul pemutilasi pria adalah pelaku tunggal. Dipastikan tidak ada keterlibatan pihak lain dalam perkara ini</t>
+        </is>
+      </c>
+      <c r="F1055" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1055" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8613723/polisi-pastikan-saepul-pemutilasi-pria-di-depok-pelaku-tunggal</t>
+        </is>
+      </c>
+      <c r="H1055" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/polisi-menggelar-reka-ulang-kasus-mutilasi-pria-di-depok-tersangka-saepul-ikut-dihadirkan-1786424451846_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1055" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1056">
+      <c r="A1056" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1056" t="inlineStr">
+        <is>
+          <t>Prabowo Mau Alihkan Sebagian Keuntungan Danantara untuk Cadangan APBN</t>
+        </is>
+      </c>
+      <c r="C1056" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:57:45 +0700</t>
+        </is>
+      </c>
+      <c r="D1056" t="inlineStr">
+        <is>
+          <t>Heri Purnomo</t>
+        </is>
+      </c>
+      <c r="E1056" t="inlineStr">
+        <is>
+          <t>Menteri Keuangan Purbaya mengungkapkan rencana Prabowo untuk mengalihkan sebagian keuntungan Danantara sebagai cadangan APBN. Besaran kontribusi masih dibahas.</t>
+        </is>
+      </c>
+      <c r="F1056" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1056" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8614116/prabowo-mau-alihkan-sebagian-keuntungan-danantara-untuk-cadangan-apbn</t>
+        </is>
+      </c>
+      <c r="H1056" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/10/presiden-prabowo-subianto-saat-acara-peresmian-bendungan-di-lombok-1783667921544_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1056" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1057">
+      <c r="A1057" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B1057" t="inlineStr">
+        <is>
+          <t>Eks Suami Aura Kasih Ungkap Alasan Balik ke Indonesia</t>
+        </is>
+      </c>
+      <c r="C1057" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:07:38 +0700</t>
+        </is>
+      </c>
+      <c r="D1057" t="inlineStr">
+        <is>
+          <t>Febryantino Nur Pratama</t>
+        </is>
+      </c>
+      <c r="E1057" t="inlineStr">
+        <is>
+          <t>Eryck Amaral kembali ke Indonesia untuk menghabiskan waktu bersama putrinya, Arabella.</t>
+        </is>
+      </c>
+      <c r="F1057" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1057" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8612488/eks-suami-aura-kasih-ungkap-alasan-balik-ke-indonesia</t>
+        </is>
+      </c>
+      <c r="H1057" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/06/08/eryck-amaral-1_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1057" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1058">
+      <c r="A1058" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1058" t="inlineStr">
+        <is>
+          <t>Istana Siapkan Tambahan 3.400 Kursi untuk HUT ke-81 RI, Pendaftar Membeludak</t>
+        </is>
+      </c>
+      <c r="C1058" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:32:49 +0700</t>
+        </is>
+      </c>
+      <c r="D1058" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1058" t="inlineStr">
+        <is>
+          <t>Prasetyo Hadi mengumumkan penambahan 3.400 kursi undangan menyusul membeludaknya jumlah pendaftar yang mencapai lebih dari 336 ribu orang.</t>
+        </is>
+      </c>
+      <c r="F1058" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1058" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867038/istana-siapkan-tambahan-3400-kursi-untuk-hut-ke-81-ri-pendaftar-membeludak</t>
+        </is>
+      </c>
+      <c r="H1058" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/oHgOnMumZx2eDe3eQfY_LcDLSRA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Prasetyo-Hadi-di-Kompleks-Parlemen-23072026.jpg</t>
+        </is>
+      </c>
+      <c r="I1058" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1059">
+      <c r="A1059" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1059" t="inlineStr">
+        <is>
+          <t>HFX International Berjangka Dukung E-Sports Kapolri Cup 2026, Siapkan Talenta Digital Indonesia</t>
+        </is>
+      </c>
+      <c r="C1059" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:31:46 +0700</t>
+        </is>
+      </c>
+      <c r="D1059" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1059" t="inlineStr">
+        <is>
+          <t>Dukungan HFX ini  menjadi bagian dari upaya perusahaan untuk ikut mendorong terciptanya ruang pengembangan bagi generasi muda</t>
+        </is>
+      </c>
+      <c r="F1059" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1059" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/adv/7867037/hfx-international-berjangka-dukung-e-sports-kapolri-cup-2026-siapkan-talenta-digital-indonesia</t>
+        </is>
+      </c>
+      <c r="H1059" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/r8IUS0wdW8s1PsNNxOkWUWcl_sA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/HFX-International-Berjangka-mendukung-E-Sports-Kapolri-Cup-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I1059" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1060">
+      <c r="A1060" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1060" t="inlineStr">
+        <is>
+          <t>Mensesneg Ungkap Ada 25 Calon Dubes yang Diajukan Prabowo ke DPR</t>
+        </is>
+      </c>
+      <c r="C1060" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:30:57 +0700</t>
+        </is>
+      </c>
+      <c r="D1060" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1060" t="inlineStr">
+        <is>
+          <t>Presiden mengajukan 25 calon duta besar (dubes) Republik Indonesia, dalam surat presiden (surpres) yang telah dikirim ke DPR, pada Senin (10/8/2026).</t>
+        </is>
+      </c>
+      <c r="F1060" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1060" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867036/mensesneg-ungkap-ada-25-calon-dubes-yang-diajukan-prabowo-ke-dpr</t>
+        </is>
+      </c>
+      <c r="H1060" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/40n_NtqmQqryvyMyNWCtt6PdB-c=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Menteri-Sekretaris-Negara-Mensesneg-Prasetyo-Hadi-di-Istana-Kepresidenan-b.jpg</t>
+        </is>
+      </c>
+      <c r="I1060" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1061">
+      <c r="A1061" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1061" t="inlineStr">
+        <is>
+          <t>Megawati Minta Taruna Merah Putih Jadi Ruang Terbuka Pendidikan Politik Generasi Muda</t>
+        </is>
+      </c>
+      <c r="C1061" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:30:31 +0700</t>
+        </is>
+      </c>
+      <c r="D1061" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1061" t="inlineStr">
+        <is>
+          <t>Megawati saat memimpin langsung pelantikan pengurus DPP TMP di Kantor DPP PDIP, Jalan Diponegoro, Menteng, Jakarta Pusat, Selasa (11/8/2026).</t>
+        </is>
+      </c>
+      <c r="F1061" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1061" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867035/megawati-minta-taruna-merah-putih-jadi-ruang-terbuka-pendidikan-politik-generasi-muda</t>
+        </is>
+      </c>
+      <c r="H1061" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/iPK6MfxQSoCui5NXOx8keM179iQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/tmp-megawati-4.jpg</t>
+        </is>
+      </c>
+      <c r="I1061" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1062">
+      <c r="A1062" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1062" t="inlineStr">
+        <is>
+          <t>Fraksi PAN Kecam Promosi Minuman Keras Menggunakan Ayat Suci Alquran</t>
+        </is>
+      </c>
+      <c r="C1062" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:29:58 +0700</t>
+        </is>
+      </c>
+      <c r="D1062" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1062" t="inlineStr">
+        <is>
+          <t>PAN mengecam keras aksi promosi minuman keras yang diduga menggunakan ayat suci Al-Quran sebagai bagian dari tantangan berhadiah.</t>
+        </is>
+      </c>
+      <c r="F1062" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1062" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867034/fraksi-pan-kecam-promosi-minuman-keras-menggunakan-ayat-suci-alquran</t>
+        </is>
+      </c>
+      <c r="H1062" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/obyAq-9wBAJdeS3JzwLeLMisNxs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Anggota-DPR-RI-Verrell-Bramasta-saat-mengikuti-rapat-di-Komisi-X-Gedung-DPR-RI.jpg</t>
+        </is>
+      </c>
+      <c r="I1062" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1063" t="inlineStr">
+        <is>
+          <t>AS Roma Menggeliat Lagi di Bursa Transfer, Giallorossi Datangkan Bek Baru</t>
+        </is>
+      </c>
+      <c r="C1063" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:28:37 +0700</t>
+        </is>
+      </c>
+      <c r="D1063" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1063" t="inlineStr">
+        <is>
+          <t>AS Roma mendatangkan bek asal Argentina, Nahuel Molina, dari Atletico Madrid senilai 18 juta Euro untuk memperkuat lini belakang mereka.</t>
+        </is>
+      </c>
+      <c r="F1063" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1063" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7867033/as-roma-menggeliat-lagi-di-bursa-transfer-giallorossi-datangkan-bek-baru</t>
+        </is>
+      </c>
+      <c r="H1063" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/SRQdWanRop5LtrNKgXA80jLLrFg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/AS-Roma-Eldor-Shomurodov-74.jpg</t>
+        </is>
+      </c>
+      <c r="I1063" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1064">
+      <c r="A1064" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1064" t="inlineStr">
+        <is>
+          <t>Kunci Gitar Lagu Kau Yang Utama - Syahrini: Kau Selalu Akan Menjadi yang Utama yang Bertakhta</t>
+        </is>
+      </c>
+      <c r="C1064" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:28:21 +0700</t>
+        </is>
+      </c>
+      <c r="D1064" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1064" t="inlineStr">
+        <is>
+          <t>Kunci gitar lagu Kau Yang Utama - Syahrini chord dasar mudah dimainkan: kau selalu akan menjadi yang utama  yang bertakhta di hatiku untuk selama.</t>
+        </is>
+      </c>
+      <c r="F1064" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1064" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/musik/7867032/kunci-gitar-lagu-kau-yang-utama-syahrini-kau-selalu-akan-menjadi-yang-utama-yang-bertakhta</t>
+        </is>
+      </c>
+      <c r="H1064" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/MJbiAjzVSUq6jvpH4Ihys6ac5WI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Syahrini-tanggapi-isu-kontroversi-Cannes.jpg</t>
+        </is>
+      </c>
+      <c r="I1064" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1065">
+      <c r="A1065" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1065" t="inlineStr">
+        <is>
+          <t>Kunci Gitar Lagu Karma - Cokelat: Selamat Tinggal Sayang</t>
+        </is>
+      </c>
+      <c r="C1065" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:28:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1065" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1065" t="inlineStr">
+        <is>
+          <t>Berikut ini merupakan chord kunci gitar lagu Karma yang dipopulerkan oleh grup band Cokelat, dimainkan dari kunci C.</t>
+        </is>
+      </c>
+      <c r="F1065" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1065" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/musik/7867031/kunci-gitar-lagu-karma-cokelat-selamat-tinggal-sayang</t>
+        </is>
+      </c>
+      <c r="H1065" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/GphyHvOUni2z8m3vRko7OvuuWYQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Potret-seseorang-sedang-bermain-gitar-dengan-kunci-chord-dasar-mudah-dimainkan.jpg</t>
+        </is>
+      </c>
+      <c r="I1065" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1066">
+      <c r="A1066" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1066" t="inlineStr">
+        <is>
+          <t>Kunci Gitar Lagu Back To Me - Kodaline: You've Got a Whole Lot of Life Left So Don't Give Up</t>
+        </is>
+      </c>
+      <c r="C1066" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:27:28 +0700</t>
+        </is>
+      </c>
+      <c r="D1066" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1066" t="inlineStr">
+        <is>
+          <t>Kunci gitar lagu Back To Me - Kodaline chord dasar mudah dimainkan: You've got a whole lot of life left So don't give up quite yet, come back to me.</t>
+        </is>
+      </c>
+      <c r="F1066" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1066" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/musik/7867030/kunci-gitar-lagu-back-to-me-kodaline-youve-got-a-whole-lot-of-life-left-so-dont-give-up</t>
+        </is>
+      </c>
+      <c r="H1066" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/eR3zla2C-eLuRKdct7nJlHf_pG0=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Potret-gitar-akustik-untuk-kunci-chord-dasar-mudah-dimainkan-ifan-main-gitar.jpg</t>
+        </is>
+      </c>
+      <c r="I1066" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1067">
+      <c r="A1067" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1067" t="inlineStr">
+        <is>
+          <t>Dalami Karakter Sophia di Film Seni Merayu Tuhan, Lutesha Sampai Tanya Teman soal Cinta Beda Agama</t>
+        </is>
+      </c>
+      <c r="C1067" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:26:50 +0700</t>
+        </is>
+      </c>
+      <c r="D1067" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1067" t="inlineStr">
+        <is>
+          <t>Aktris Lutesha Sadhewa sampai belajar ke teman-temannya yang pernah pacaran beda agama demi dalami karakter Sophia di Film Seni Merayu Tuhan.</t>
+        </is>
+      </c>
+      <c r="F1067" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1067" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7867029/dalami-karakter-sophia-di-film-seni-merayu-tuhan-lutesha-sampai-tanya-teman-soal-cinta-beda-agama</t>
+        </is>
+      </c>
+      <c r="H1067" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/6QDU-A5OOgZKMGf3STeqKDQEYbs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Lutesha-1-12062026.jpg</t>
+        </is>
+      </c>
+      <c r="I1067" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1068">
+      <c r="A1068" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1068" t="inlineStr">
+        <is>
+          <t>“Enggak, Saya di Bromo”, Jawaban Pratikno Saat Isu Mundur Beredar</t>
+        </is>
+      </c>
+      <c r="C1068" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:25:18 +0700</t>
+        </is>
+      </c>
+      <c r="D1068" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1068" t="inlineStr">
+        <is>
+          <t>Isu Pratikno sakit dan mundur kembali beredar. Ia berada di Bromo, sementara Istana memastikan kabar tersebut tidak benar.</t>
+        </is>
+      </c>
+      <c r="F1068" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1068" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867028/enggak-saya-di-bromo-jawaban-pratikno-saat-isu-mundur-beredar</t>
+        </is>
+      </c>
+      <c r="H1068" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/u0NInv8a37nGL6w162QjOkUPogw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Menko-PMK-Pratiknotengah-di-Kawasan-Bromo.jpg</t>
+        </is>
+      </c>
+      <c r="I1068" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1069">
+      <c r="A1069" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1069" t="inlineStr">
+        <is>
+          <t>Tiket Malaysia vs Vietnam Naik 66 Persen, FAM Jadi Sasaran Kritik Suporter</t>
+        </is>
+      </c>
+      <c r="C1069" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:13:57 +0700</t>
+        </is>
+      </c>
+      <c r="D1069" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1069" t="inlineStr">
+        <is>
+          <t>Kenaikan harga tiket semifinal Piala AFF 2026 Malaysia vs Vietnam menuai kritik suporter, di tengah misi memutus rekor buruk.</t>
+        </is>
+      </c>
+      <c r="F1069" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1069" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7867027/tiket-malaysia-vs-vietnam-naik-66-persen-fam-jadi-sasaran-kritik-suporter</t>
+        </is>
+      </c>
+      <c r="H1069" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/1WNe2Qaqla-dt4wi-y3ufRMaWz8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Duel-pemain-Malaysia-melawan-Laos-pada-pertandingan-lanjutan-Grup-F.jpg</t>
+        </is>
+      </c>
+      <c r="I1069" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1070">
+      <c r="A1070" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1070" t="inlineStr">
+        <is>
+          <t>50 Ide Nama Regu Pramuka Putra-Putri yang Unik dan Berkesan, Cocok untuk Kegiatan di Sekolah</t>
+        </is>
+      </c>
+      <c r="C1070" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:09:52 +0700</t>
+        </is>
+      </c>
+      <c r="D1070" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1070" t="inlineStr">
+        <is>
+          <t>Pemilihan nama regu dapat memperkuat identitas dan kekompakan anggota, sehingga nama yang unik dan bermakna cocok digunakan.</t>
+        </is>
+      </c>
+      <c r="F1070" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1070" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867026/50-ide-nama-regu-pramuka-putra-putri-yang-unik-dan-berkesan-cocok-untuk-kegiatan-di-sekolah</t>
+        </is>
+      </c>
+      <c r="H1070" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/jo-cczR-g1VXqTpl5fVdiPXq8q0=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/pemkot-malang-gelar-peringatan-hari-pramuka_20230819_130208.jpg</t>
+        </is>
+      </c>
+      <c r="I1070" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1071">
+      <c r="A1071" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1071" t="inlineStr">
+        <is>
+          <t>Prakiraan Cuaca Kota Sorong Rabu, 12 Agustus 2026: Mayoritas Wilayah Berawan</t>
+        </is>
+      </c>
+      <c r="C1071" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:08:32 +0700</t>
+        </is>
+      </c>
+      <c r="D1071" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1071" t="inlineStr">
+        <is>
+          <t>BMKG memprakirakan, cuaca berawan akan mendominasi langit Kota Sorong, Provinsi Papua Barat Daya, pada Rabu (12/8/2026).</t>
+        </is>
+      </c>
+      <c r="F1071" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1071" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7867025/prakiraan-cuaca-kota-sorong-rabu-12-agustus-2026-mayoritas-wilayah-berawan</t>
+        </is>
+      </c>
+      <c r="H1071" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/T3-SSNlj5aoy3q2FcSs_HLhT1Ok=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/cuaca-berawan-343r.jpg</t>
+        </is>
+      </c>
+      <c r="I1071" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1072">
+      <c r="A1072" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1072" t="inlineStr">
+        <is>
+          <t>Sawah di Gresik Terancam Kekeringan, Ratusan Hektare Terdampak, Mentan: Tak Boleh Dianggap Remeh</t>
+        </is>
+      </c>
+      <c r="C1072" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:07:37 +0700</t>
+        </is>
+      </c>
+      <c r="D1072" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1072" t="inlineStr">
+        <is>
+          <t>Ratusan hektare sawah di Gresik terancam kekeringan. Mentan Amran turun langsung ke lokasi dan siapkan dua solusi jitu untuk para petani.</t>
+        </is>
+      </c>
+      <c r="F1072" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1072" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7867024/sawah-di-gresik-terancam-kekeringan-ratusan-hektare-terdampak-mentan-tak-boleh-dianggap-remeh</t>
+        </is>
+      </c>
+      <c r="H1072" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/eLF2WvXGH06viVoEEOjZss2qkdU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/menteri-pertanian-Andi-Amran-Sulaiman-saat-kunjungan-ke-gresik-kemarau-kekeringan.jpg</t>
+        </is>
+      </c>
+      <c r="I1072" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1073">
+      <c r="A1073" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1073" t="inlineStr">
+        <is>
+          <t>Aset BCA Syariah Tumbuh 17,2 Persen Jadi Rp20,7 Triliun hingga Juni 2026</t>
+        </is>
+      </c>
+      <c r="C1073" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:04:09 +0700</t>
+        </is>
+      </c>
+      <c r="D1073" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1073" t="inlineStr">
+        <is>
+          <t>Pertumbuhan juga terlihat dari laba setelah pajak atau profit after tax (PAT) yang naik 9,2 persen YoY menjadi Rp109 miliar.</t>
+        </is>
+      </c>
+      <c r="F1073" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1073" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/bisnis/7867023/aset-bca-syariah-tumbuh-172-persen-jadi-rp207-triliun-hingga-juni-2026</t>
+        </is>
+      </c>
+      <c r="H1073" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/M9XheOB5uguig5j8A2qbspXrE8E=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/bca-syariah-002.jpg</t>
+        </is>
+      </c>
+      <c r="I1073" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1074">
+      <c r="A1074" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1074" t="inlineStr">
+        <is>
+          <t>Tingkatkan Kesejahteraan Petani, Produktivitas Pertanian di Dua Wilayah Digenjot</t>
+        </is>
+      </c>
+      <c r="C1074" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:00:50 +0700</t>
+        </is>
+      </c>
+      <c r="D1074" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1074" t="inlineStr">
+        <is>
+          <t>PPI menyalurkan sarana pendukung kegiatan pertanian berupa 13 unit sprayer pestisida kepada tiga Gapoktan di kedua wilayah pertanian</t>
+        </is>
+      </c>
+      <c r="F1074" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1074" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/bisnis/7867022/tingkatkan-kesejahteraan-petani-produktivitas-pertanian-di-dua-wilayah-digenjot</t>
+        </is>
+      </c>
+      <c r="H1074" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/SXUeN1MHSU5FIX52c-5ssOmmTQA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/gapoktan-PPI-di-indramayu.jpg</t>
+        </is>
+      </c>
+      <c r="I1074" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1075">
+      <c r="A1075" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1075" t="inlineStr">
+        <is>
+          <t>Sepanjang 2026, Bea Cukai Klaim Gagalkan Peredaran 1,2 Miliar Batang Rokok Ilegal</t>
+        </is>
+      </c>
+      <c r="C1075" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:56:02 +0700</t>
+        </is>
+      </c>
+      <c r="D1075" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1075" t="inlineStr">
+        <is>
+          <t>hingga 31 Juli 2026, Bea Cukai telah menggagalkan lebih dari 1 miliar batang rokok ilegal beredar untuk konsumen dalam negeri.</t>
+        </is>
+      </c>
+      <c r="F1075" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1075" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/bisnis/7867021/sepanjang-2026-bea-cukai-klaim-gagalkan-peredaran-12-miliar-batang-rokok-ilegal</t>
+        </is>
+      </c>
+      <c r="H1075" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ZtjSZdLN0na1W9fF4cZ3CaaG_X8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Dirjen-Bea-Cukai-Kemenkeu-Djaka-Budhi-Utama-saat-konpers-rokok-ilegal-di-priok.jpg</t>
+        </is>
+      </c>
+      <c r="I1075" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1076">
+      <c r="A1076" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1076" t="inlineStr">
+        <is>
+          <t>Menpora Erick Thohir Apresiasi Dukungan Pramono Anung untuk FIFA ASEAN Cup 2026</t>
+        </is>
+      </c>
+      <c r="C1076" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:55:29 +0700</t>
+        </is>
+      </c>
+      <c r="D1076" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1076" t="inlineStr">
+        <is>
+          <t>Pengalaman Pramono dalam membantu penyelenggaraan FIFA U-17 World Cup 2023 di Indonesia menjadi salah satu modal penting</t>
+        </is>
+      </c>
+      <c r="F1076" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1076" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7867020/menpora-erick-thohir-apresiasi-dukungan-pramono-anung-untuk-fifa-asean-cup-2026</t>
+        </is>
+      </c>
+      <c r="H1076" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/BLNOUsr0p6SbsFdC7cZ-6zvK9HU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Menteri-Pemuda-dan-Olahraga-Menpora-Erick-Thohir-1221.jpg</t>
+        </is>
+      </c>
+      <c r="I1076" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1077">
+      <c r="A1077" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1077" t="inlineStr">
+        <is>
+          <t>Putrinya Dituding Selingkuhan Rizky Billar, Avi Basalamah: Ini Proses Hidup</t>
+        </is>
+      </c>
+      <c r="C1077" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:52:58 +0700</t>
+        </is>
+      </c>
+      <c r="D1077" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1077" t="inlineStr">
+        <is>
+          <t>Bersama sang suami, Ramzi, Avi berkomitmen untuk menjaga keharmonisan keluarga agar tetap berjalan normal di tengah proses hukum yang berjalan.</t>
+        </is>
+      </c>
+      <c r="F1077" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1077" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7867019/putrinya-dituding-selingkuhan-rizky-billar-avi-basalamah-ini-proses-hidup</t>
+        </is>
+      </c>
+      <c r="H1077" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/sj4sFJY9tnZ0ZxQBKNLggAS_vJ8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Avi-Basalamah-1-11082026.jpg</t>
+        </is>
+      </c>
+      <c r="I1077" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1078">
+      <c r="A1078" t="inlineStr">
+        <is>
+          <t>Otomotif</t>
+        </is>
+      </c>
+      <c r="B1078" t="inlineStr">
+        <is>
+          <t>Jaringan Purnajual Xpeng Merambah Jawa Tengah Lewat Semarang</t>
+        </is>
+      </c>
+      <c r="C1078" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:25:58 +0700</t>
+        </is>
+      </c>
+      <c r="D1078" t="inlineStr">
+        <is>
+          <t>Israr Itah</t>
+        </is>
+      </c>
+      <c r="E1078" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- Jaringan layanan menjadi salah satu kebutuhan penting bagi merek otomotif yang tengah memperluas pasar. Semakin banyak dealer akan membuat konsumen lebih mudah memperoleh akses penjualan, perawatan, dan...</t>
+        </is>
+      </c>
+      <c r="F1078" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1078" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjlrra348/jaringan-purnajual-xpeng-merambah-jawa-tengah-lewat-semarang</t>
+        </is>
+      </c>
+      <c r="H1078" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/xpeng-experience-service-center_260811182314-782.jpg</t>
+        </is>
+      </c>
+      <c r="I1078" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="1079">
+      <c r="A1079" t="inlineStr">
+        <is>
+          <t>Bisnis</t>
+        </is>
+      </c>
+      <c r="B1079" t="inlineStr">
+        <is>
+          <t>Desa Tambakmekar Kembangkan Wisata Alam dan Budaya Lewat Pinus Kujang</t>
+        </is>
+      </c>
+      <c r="C1079" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1079" t="inlineStr">
+        <is>
+          <t>Satria K Yudha</t>
+        </is>
+      </c>
+      <c r="E1079" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, SUBANG -- Desa Tambakmekar, Kecamatan Jalancagak, Kabupaten Subang, Jawa Barat, mengembangkan potensi wisata berbasis alam dan kearifan lokal melalui Festival Pinus Kujang 2026. Kegiatan yang digelar di kawasan Timman...</t>
+        </is>
+      </c>
+      <c r="F1079" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1079" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjlmzf416/desa-tambakmekar-kembangkan-wisata-alam-dan-budaya-lewat-pinus-kujang</t>
+        </is>
+      </c>
+      <c r="H1079" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/kegiatan-festival-pinus-kujang-di-desa-tambakmekar-kecamatan-jalancagak_260811164118-858.jpeg</t>
+        </is>
+      </c>
+      <c r="I1079" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="1080">
+      <c r="A1080" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1080" t="inlineStr">
+        <is>
+          <t>Kejagung Ungkap Alasan Periksa Pegawai BI di Kasus TPPU Febrie</t>
+        </is>
+      </c>
+      <c r="C1080" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:06:01 +0700</t>
+        </is>
+      </c>
+      <c r="D1080" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1080" t="inlineStr">
+        <is>
+          <t>Kejagung terus mendalami kasus TPPU yang menjerat mantan Jampidsus Febrie Adriansyah.</t>
+        </is>
+      </c>
+      <c r="F1080" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1080" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267373/kejagung-ungkap-alasan-periksa-pegawai-bi-di-kasus-tppu-febrie</t>
+        </is>
+      </c>
+      <c r="H1080" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/2WEvQ2hmLFTijz9iyBipOx1Njqg=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9318624/original/089072000_1786113401-IMG_3067.jpg</t>
+        </is>
+      </c>
+      <c r="I1080" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1081">
+      <c r="A1081" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1081" t="inlineStr">
+        <is>
+          <t>Viral TPS Liar di Cilincing, Pramono Buka Suara</t>
+        </is>
+      </c>
+      <c r="C1081" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:02:30 +0700</t>
+        </is>
+      </c>
+      <c r="D1081" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1081" t="inlineStr">
+        <is>
+          <t>Gunungan sampah hampir setinggi rumah warga di Cilincing, Jakarta Utara, viral di media sossial.</t>
+        </is>
+      </c>
+      <c r="F1081" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1081" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267371/viral-tps-liar-di-cilincing-pramono-buka-suara</t>
+        </is>
+      </c>
+      <c r="H1081" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/7a5oAtHzUp_PhFOGhcN9vSJrY40=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9321518/original/073330700_1786446145-eff6749f-e90e-491d-85af-deb70b9fe17a.jpg</t>
+        </is>
+      </c>
+      <c r="I1081" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1082">
+      <c r="A1082" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1082" t="inlineStr">
+        <is>
+          <t>Seskab Teddy: 40 Persen Peserta Magang Nasional Langsung Direkrut Kerja</t>
+        </is>
+      </c>
+      <c r="C1082" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:03:11 +0700</t>
+        </is>
+      </c>
+      <c r="D1082" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1082" t="inlineStr">
+        <is>
+          <t>Salah satu peserta magang di Jakarta memperoleh penghasilan sekitar Rp 5,5 juta hingga Rp 5,7 juta per bulan.</t>
+        </is>
+      </c>
+      <c r="F1082" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1082" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267372/seskab-teddy-40-persen-peserta-magang-nasional-langsung-direkrut-kerja</t>
+        </is>
+      </c>
+      <c r="H1082" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/JkD3uD5S4C7mq_CyLE-cj09TyT0=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9321110/original/098803900_1786429030-email-attachment_2026_08_11_ariefhakim-at-klyid_ada-kuota-150-ribu-orang-magang-nasional-angkatan-2-dibuka-bertahap-hingga-oktober-2026_1000404420.jpg</t>
+        </is>
+      </c>
+      <c r="I1082" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1083">
+      <c r="A1083" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1083" t="inlineStr">
+        <is>
+          <t>Pramono Yakin Transjakarta Bisa Kelola Transportasi Kepulauan Seribu</t>
+        </is>
+      </c>
+      <c r="C1083" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:50:22 +0700</t>
+        </is>
+      </c>
+      <c r="D1083" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1083" t="inlineStr">
+        <is>
+          <t>Tahun 2027, transportasi Kepulauan Seribu ditargetkan sepenuhnya dikelola Transjakarta.</t>
+        </is>
+      </c>
+      <c r="F1083" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1083" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267355/pramono-yakin-transjakarta-bisa-kelola-transportasi-kepulauan-seribu</t>
+        </is>
+      </c>
+      <c r="H1083" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/XfeHQTc02O4ALPSqS-HfpuOkmNo=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/5341440/original/005282500_1757313161-IMG_9023.jpeg</t>
+        </is>
+      </c>
+      <c r="I1083" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1084">
+      <c r="A1084" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1084" t="inlineStr">
+        <is>
+          <t>AHY Sebut Jakarta di Bawah Pramono Bisa Jadi Contoh, Ini Alasannya</t>
+        </is>
+      </c>
+      <c r="C1084" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:58:39 +0700</t>
+        </is>
+      </c>
+      <c r="D1084" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1084" t="inlineStr">
+        <is>
+          <t>Tantangannya bukan menghentikan urbanisasi, melainkan memastikan kota-kota memiliki standar, sumber daya, dan sistem logistik yang mampu menopang pertumbuhan.</t>
+        </is>
+      </c>
+      <c r="F1084" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1084" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267363/ahy-sebut-jakarta-di-bawah-pramono-bisa-jadi-contoh-ini-alasannya</t>
+        </is>
+      </c>
+      <c r="H1084" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/3BVkMgQGOEqyQmwPCKocWE51fuM=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9321513/original/078925900_1786445913-8dbdc105-046a-48f0-88eb-4a1babc96d88.jpg</t>
+        </is>
+      </c>
+      <c r="I1084" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1085">
+      <c r="A1085" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1085" t="inlineStr">
+        <is>
+          <t>DPR Minta Polisi Tindak Challenge Alquran Hadiah Miras: Umat Bisa Marah</t>
+        </is>
+      </c>
+      <c r="C1085" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:43:16 +0700</t>
+        </is>
+      </c>
+      <c r="D1085" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1085" t="inlineStr">
+        <is>
+          <t>Pasha menilai aparat perlu segera bertindak agar persoalan tersebut tidak memicu kemarahan masyarakat.</t>
+        </is>
+      </c>
+      <c r="F1085" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1085" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267341/dpr-minta-polisi-tindak-challenge-alquran-hadiah-miras-umat-bisa-marah</t>
+        </is>
+      </c>
+      <c r="H1085" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/Fp5iC-vppn7dJSzwqGEBlrLz0gY=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9321055/original/059736500_1786425649-Jepretan_Layar_2025-08-11_pukul_12.15.34.jpg</t>
+        </is>
+      </c>
+      <c r="I1085" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1086">
+      <c r="A1086" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="B1086" t="inlineStr">
+        <is>
+          <t>Vietnam dan Australia Makin Mesra, Sepakat Perkuat Kerja Sama Pertahanan</t>
+        </is>
+      </c>
+      <c r="C1086" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:41:14 +0700</t>
+        </is>
+      </c>
+      <c r="D1086" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E1086" t="inlineStr">
+        <is>
+          <t>Pemerintah Australia dan Vietnam semakin mesra dan sepakat untuk memperdalam kemitraan strategis komprehensif.</t>
+        </is>
+      </c>
+      <c r="F1086" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1086" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/global/read/2026/08/11/184100970/vietnam-dan-australia-makin-mesra-sepakat-perkuat-kerja-sama-pertahanan</t>
+        </is>
+      </c>
+      <c r="H1086" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/sbCV6TSUbqSqLPp6cu7bf52vi3U=/0x0:1023x682/1200x675/filters:watermark(data/photo/2026/01/30/697c81ac46b81.png,0,-0,1)/data/photo/2025/08/20/68a53ceb248e6.jpg</t>
+        </is>
+      </c>
+      <c r="I1086" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1087">
+      <c r="A1087" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1087" t="inlineStr">
+        <is>
+          <t>Pemerintah Luncurkan Digitalisasi Penerbitan Akta Lahir, Bayi Lahir Bisa Langsung Dapatkan Akta</t>
+        </is>
+      </c>
+      <c r="C1087" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:41:14 +0700</t>
+        </is>
+      </c>
+      <c r="D1087" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E1087" t="inlineStr">
+        <is>
+          <t>Melalui layanan ini, akta kelahiran dapat diterbitkan secara otomatis dan dikirim secara daring sesaat setelah bayi lahir di fasilitas</t>
+        </is>
+      </c>
+      <c r="F1087" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1087" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/08/11/18234501/pemerintah-luncurkan-digitalisasi-penerbitan-akta-lahir-bayi-lahir-bisa</t>
+        </is>
+      </c>
+      <c r="H1087" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/OQinD-MsYkhl0oMkgVRNveSgMSM=/160x107:1440x959/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/11/6a7b02396ad05.jpg</t>
+        </is>
+      </c>
+      <c r="I1087" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1088">
+      <c r="A1088" t="inlineStr">
+        <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
+      <c r="B1088" t="inlineStr">
+        <is>
+          <t>Pernah Tuntaskan Full Marathon di Usia 60 Tahun, Ini Kisah Restu Didik Menekuni Lari</t>
+        </is>
+      </c>
+      <c r="C1088" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:41:14 +0700</t>
+        </is>
+      </c>
+      <c r="D1088" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E1088" t="inlineStr">
+        <is>
+          <t>Mulai lari di usia 54 tahun, Restu Didik berhasil menuntaskan full marathon di usia 60 tahun dan kini tetap konsisten berlari.</t>
+        </is>
+      </c>
+      <c r="F1088" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1088" t="inlineStr">
+        <is>
+          <t>https://lifestyle.kompas.com/read/2026/08/11/180500820/pernah-tuntaskan-full-marathon-di-usia-60-tahun-ini-kisah-restu-didik</t>
+        </is>
+      </c>
+      <c r="H1088" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/FFQHUNEHPHTglA2_BAP8CGJfeVQ=/0x0:1280x853/1200x675/filters:watermark(data/photo/2026/01/30/697c817ed68bb.png,0,-0,1)/data/photo/2026/08/10/6a79c8cc14073.jpg</t>
+        </is>
+      </c>
+      <c r="I1088" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I992"/>
+  <autoFilter ref="A1:I1088"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-11 12:42 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-11.xlsx
+++ b/data/berita_2026-08-11.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1088</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1177</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1088"/>
+  <dimension ref="A1:I1177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -51575,8 +51575,4191 @@
         </is>
       </c>
     </row>
+    <row r="1089">
+      <c r="A1089" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1089" t="inlineStr">
+        <is>
+          <t>Wagub Jatim dorong inovasi Umsura menjadi produk siap pakai</t>
+        </is>
+      </c>
+      <c r="C1089" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:35:31 +0700</t>
+        </is>
+      </c>
+      <c r="D1089" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1089" t="inlineStr">
+        <is>
+          <t>Wakil Gubernur Jawa Timur Emil Elestianto Dardak mendorong 38 inovasi teknologi tepat guna hasil Kuliah Kerja Nyata ...</t>
+        </is>
+      </c>
+      <c r="F1089" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1089" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689724/wagub-jatim-dorong-inovasi-umsura-menjadi-produk-siap-pakai</t>
+        </is>
+      </c>
+      <c r="H1089" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1347464.jpg</t>
+        </is>
+      </c>
+      <c r="I1089" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1090">
+      <c r="A1090" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1090" t="inlineStr">
+        <is>
+          <t>Kementerian UMKM sebut ojol harus naik kelas dalam segala aspek</t>
+        </is>
+      </c>
+      <c r="C1090" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:31:49 +0700</t>
+        </is>
+      </c>
+      <c r="D1090" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1090" t="inlineStr">
+        <is>
+          <t>Kementerian Usaha Mikro Kecil dan Menengah (UMKM) menyebutkan driver atau pengemudi ojek online (ojol) harus ...</t>
+        </is>
+      </c>
+      <c r="F1090" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1090" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689723/kementerian-umkm-sebut-ojol-harus-naik-kelas-dalam-segala-aspek</t>
+        </is>
+      </c>
+      <c r="H1090" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1041.jpg</t>
+        </is>
+      </c>
+      <c r="I1090" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1091">
+      <c r="A1091" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1091" t="inlineStr">
+        <is>
+          <t>Sumedang anggarkan minimal Rp100 miliar untuk perbaiki jalan pada 2027</t>
+        </is>
+      </c>
+      <c r="C1091" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:27:23 +0700</t>
+        </is>
+      </c>
+      <c r="D1091" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1091" t="inlineStr">
+        <is>
+          <t>Pemerintah Kabupaten (Pemkab) Sumedang, Jawa Barat, menyiapkan anggaran minimal Rp100 miliar untuk perbaikan ...</t>
+        </is>
+      </c>
+      <c r="F1091" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1091" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689721/sumedang-anggarkan-minimal-rp100-miliar-untuk-perbaiki-jalan-pada-2027</t>
+        </is>
+      </c>
+      <c r="H1091" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/492210.jpg</t>
+        </is>
+      </c>
+      <c r="I1091" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1092" t="inlineStr">
+        <is>
+          <t>Pramono segera bahas soal jalur sepeda di DKI</t>
+        </is>
+      </c>
+      <c r="C1092" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:27:06 +0700</t>
+        </is>
+      </c>
+      <c r="D1092" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1092" t="inlineStr">
+        <is>
+          <t>Gubernur DKI Jakarta Pramono Anung Wibowo bersama jajaran segera membahas jalur sepeda di sejumlah ruas jalan ...</t>
+        </is>
+      </c>
+      <c r="F1092" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1092" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689720/pramono-segera-bahas-soal-jalur-sepeda-di-dki</t>
+        </is>
+      </c>
+      <c r="H1092" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG_6814.jpeg</t>
+        </is>
+      </c>
+      <c r="I1092" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1093">
+      <c r="A1093" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1093" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro jadi tuan rumah peluncuran MotoGP 2027</t>
+        </is>
+      </c>
+      <c r="C1093" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:25:22 +0700</t>
+        </is>
+      </c>
+      <c r="D1093" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1093" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro, Brasil, terpilih menjadi tuan rumah peluncuran musim MotoGP 2027 yang akan digelar di Pantai Botafogo ...</t>
+        </is>
+      </c>
+      <c r="F1093" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1093" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689717/rio-de-janeiro-jadi-tuan-rumah-peluncuran-motogp-2027</t>
+        </is>
+      </c>
+      <c r="H1093" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/01/14/antarafoto-francesco-bagnaia-juara-motogp-mandalika-2023-151023-as-7-1.jpg</t>
+        </is>
+      </c>
+      <c r="I1093" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1094">
+      <c r="A1094" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1094" t="inlineStr">
+        <is>
+          <t>Pelatihan upacara HUT Ke-81 RI bagi pasien ODGJ</t>
+        </is>
+      </c>
+      <c r="C1094" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:23:39 +0700</t>
+        </is>
+      </c>
+      <c r="D1094" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1094" t="inlineStr">
+        <is>
+          <t>Pasien dengan gangguan jiwa (ODGJ) memberikan hormat kepada bendera Merah Putih saat pelatihan upacara di Yayasan ...</t>
+        </is>
+      </c>
+      <c r="F1094" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1094" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5689716/pelatihan-upacara-hut-ke-81-ri-bagi-pasien-odgj</t>
+        </is>
+      </c>
+      <c r="H1094" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/Pelatihan-upacara-HUT-ke-81-RI-bagi-pasien-ODGJ-110826-ryl-5.jpg</t>
+        </is>
+      </c>
+      <c r="I1094" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1095">
+      <c r="A1095" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1095" t="inlineStr">
+        <is>
+          <t>Kementerian UMKM dan OJK sepakat akselerasi akses pembiayaan UMKM</t>
+        </is>
+      </c>
+      <c r="C1095" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:23:36 +0700</t>
+        </is>
+      </c>
+      <c r="D1095" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1095" t="inlineStr">
+        <is>
+          <t>Kementerian Usaha Mikro Kecil Menengah (UMKM) dan Otoritas Jasa Keuangan (OJK) bersepakat melakukan akselerasi akses ...</t>
+        </is>
+      </c>
+      <c r="F1095" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1095" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689715/kementerian-umkm-dan-ojk-sepakat-akselerasi-akses-pembiayaan-umkm</t>
+        </is>
+      </c>
+      <c r="H1095" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/WhatsApp-Image-2026-08-11-at-18.20.09.jpeg</t>
+        </is>
+      </c>
+      <c r="I1095" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1096" t="inlineStr">
+        <is>
+          <t>Aceh Besar percepat penanganan sawah terdampak kekeringan</t>
+        </is>
+      </c>
+      <c r="C1096" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:23:33 +0700</t>
+        </is>
+      </c>
+      <c r="D1096" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1096" t="inlineStr">
+        <is>
+          <t>Pemerintah Kabupaten Aceh Besar terus berupaya mengatasi kekeringan sawah milik petani akibat kemarau panjang yang ...</t>
+        </is>
+      </c>
+      <c r="F1096" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1096" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689711/aceh-besar-percepat-penanganan-sawah-terdampak-kekeringan</t>
+        </is>
+      </c>
+      <c r="H1096" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/WhatsApp-Image-2026-08-11-at-18.55.54.jpeg</t>
+        </is>
+      </c>
+      <c r="I1096" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1097">
+      <c r="A1097" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1097" t="inlineStr">
+        <is>
+          <t>Pramono minta Presiden Prabowo resmikan LRT Kelapa Gading-Manggarai</t>
+        </is>
+      </c>
+      <c r="C1097" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:23:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1097" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1097" t="inlineStr">
+        <is>
+          <t>Gubernur DKI Jakarta Pramono Anung Wibowo mengaku dirinya sudah meminta kepada Presiden Prabowo Subianto untuk ...</t>
+        </is>
+      </c>
+      <c r="F1097" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1097" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689709/pramono-minta-presiden-prabowo-resmikan-lrt-kelapa-gading-manggarai</t>
+        </is>
+      </c>
+      <c r="H1097" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG_6814.jpeg</t>
+        </is>
+      </c>
+      <c r="I1097" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1098">
+      <c r="A1098" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1098" t="inlineStr">
+        <is>
+          <t>Kemenhub pacu modernisasi transportasi darat lewat kolaborasi global</t>
+        </is>
+      </c>
+      <c r="C1098" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:22:11 +0700</t>
+        </is>
+      </c>
+      <c r="D1098" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1098" t="inlineStr">
+        <is>
+          <t>Kementerian Perhubungan (Kemenhub) memperkuat modernisasi transportasi darat melalui penguatan kolaborasi internasional ...</t>
+        </is>
+      </c>
+      <c r="F1098" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1098" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689708/kemenhub-pacu-modernisasi-transportasi-darat-lewat-kolaborasi-global</t>
+        </is>
+      </c>
+      <c r="H1098" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/E6442E4B-CB1E-4A96-99D8-94A8FF3089E5.jpeg</t>
+        </is>
+      </c>
+      <c r="I1098" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1099" t="inlineStr">
+        <is>
+          <t>Kemarau, 8,7 juta liter air telah disalurkan ke 23 daerah di Jabar</t>
+        </is>
+      </c>
+      <c r="C1099" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:20:06 +0700</t>
+        </is>
+      </c>
+      <c r="D1099" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1099" t="inlineStr">
+        <is>
+          <t>Pemerintah Provinsi (Pemprov) Jawa Barat (Jabar) menyebut mereka bersama tim gabungan telah menyalurkan sebanyak 8,7 ...</t>
+        </is>
+      </c>
+      <c r="F1099" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1099" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689704/kemarau-87-juta-liter-air-telah-disalurkan-ke-23-daerah-di-jabar</t>
+        </is>
+      </c>
+      <c r="H1099" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1002091225.jpg</t>
+        </is>
+      </c>
+      <c r="I1099" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1100">
+      <c r="A1100" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1100" t="inlineStr">
+        <is>
+          <t>Pemprov NTB targetkan legalitas lahan segera tuntas di Gili Trawangan</t>
+        </is>
+      </c>
+      <c r="C1100" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:18:35 +0700</t>
+        </is>
+      </c>
+      <c r="D1100" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1100" t="inlineStr">
+        <is>
+          <t>Pemerintah Provinsi Nusa Tenggara Barat (NTB) menargetkan seluruh persoalan legalitas terkait status kepemilikan lahan ...</t>
+        </is>
+      </c>
+      <c r="F1100" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1100" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689703/pemprov-ntb-targetkan-legalitas-lahan-segera-tuntas-di-gili-trawangan</t>
+        </is>
+      </c>
+      <c r="H1100" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1001449206.jpg</t>
+        </is>
+      </c>
+      <c r="I1100" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1101">
+      <c r="A1101" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1101" t="inlineStr">
+        <is>
+          <t>Kejagung ungkap alasan Rinaldi Umar batal jadi Dirdik Jampidsus baru</t>
+        </is>
+      </c>
+      <c r="C1101" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:18:31 +0700</t>
+        </is>
+      </c>
+      <c r="D1101" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1101" t="inlineStr">
+        <is>
+          <t>Kepala Pusat Penerangan Hukum Kejaksaan Agung Anang Supriatna mengungkapkan alasan Rinaldi Umar batal diangkat ...</t>
+        </is>
+      </c>
+      <c r="F1101" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1101" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689701/kejagung-ungkap-alasan-rinaldi-umar-batal-jadi-dirdik-jampidsus-baru</t>
+        </is>
+      </c>
+      <c r="H1101" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1000087747.jpg</t>
+        </is>
+      </c>
+      <c r="I1101" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1102">
+      <c r="A1102" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1102" t="inlineStr">
+        <is>
+          <t>Rayakan Kemerdekaan, Pelajar di Manokwari ikuti lomba gerak jalan HUT RI</t>
+        </is>
+      </c>
+      <c r="C1102" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:17:08 +0700</t>
+        </is>
+      </c>
+      <c r="D1102" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1102" t="inlineStr">
+        <is>
+          <t>Pelajar mengikuti lomba gerak jalan dalam rangka HUT Ke-81 Republik Indonesia di Manokwari, Papua Barat.</t>
+        </is>
+      </c>
+      <c r="F1102" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1102" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5689700/rayakan-kemerdekaan-pelajar-di-manokwari-ikuti-lomba-gerak-jalan-hut-ri</t>
+        </is>
+      </c>
+      <c r="H1102" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/Lomba-Gerak-Jalan-HUT-RI-Di-Manokwari-110826-ci-2.jpg</t>
+        </is>
+      </c>
+      <c r="I1102" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1103">
+      <c r="A1103" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1103" t="inlineStr">
+        <is>
+          <t>Kemenekraf jadikan Tomohon kota florikultura berdaya saing global</t>
+        </is>
+      </c>
+      <c r="C1103" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:15:48 +0700</t>
+        </is>
+      </c>
+      <c r="D1103" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1103" t="inlineStr">
+        <is>
+          <t>Kementerian Ekonomi Kreatif menilai Kota Tomohon, Sulawesi Utara, sebagai destinasi wisata yang membawa identitas lokal ...</t>
+        </is>
+      </c>
+      <c r="F1103" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1103" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689697/kemenekraf-jadikan-tomohon-kota-florikultura-berdaya-saing-global</t>
+        </is>
+      </c>
+      <c r="H1103" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1000595716.jpg</t>
+        </is>
+      </c>
+      <c r="I1103" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1104">
+      <c r="A1104" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1104" t="inlineStr">
+        <is>
+          <t>Pemprov Sumbar siapkan penyitaan aset penunggak pajak air permukaan</t>
+        </is>
+      </c>
+      <c r="C1104" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:14:17 +0700</t>
+        </is>
+      </c>
+      <c r="D1104" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1104" t="inlineStr">
+        <is>
+          <t>ANTARA - Pemerintah Provinsi Sumatera Barat menyiapkan langkah penyitaan aset terhadap perusahaan sawit yang menunggak ...</t>
+        </is>
+      </c>
+      <c r="F1104" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1104" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5689631/pemprov-sumbar-siapkan-penyitaan-aset-penunggak-pajak-air-permukaan</t>
+        </is>
+      </c>
+      <c r="H1104" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/PEMPROV-SUMBAR-SIAPKAN-PENYITAAN-ASET-PENUNGGAK-PAJAK-AIR-PERMUKAAN.jpg</t>
+        </is>
+      </c>
+      <c r="I1104" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1105">
+      <c r="A1105" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1105" t="inlineStr">
+        <is>
+          <t>Gandeng Nintendo, RI dorong pengembang gim lokal mendunia</t>
+        </is>
+      </c>
+      <c r="C1105" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:11:18 +0700</t>
+        </is>
+      </c>
+      <c r="D1105" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1105" t="inlineStr">
+        <is>
+          <t>ANTARA - Pemerintah Indonesia resmi menjajaki kerja sama dengan raksasa industri gim dunia, Nintendo, agar dapat ...</t>
+        </is>
+      </c>
+      <c r="F1105" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1105" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5689561/gandeng-nintendo-ri-dorong-pengembang-gim-lokal-mendunia</t>
+        </is>
+      </c>
+      <c r="H1105" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Sequence-13.13_41_35_18.Still486.jpg</t>
+        </is>
+      </c>
+      <c r="I1105" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1106">
+      <c r="A1106" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1106" t="inlineStr">
+        <is>
+          <t>Tanah Laut jadikan pengelolaan sampah penopang pariwisata</t>
+        </is>
+      </c>
+      <c r="C1106" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:10:31 +0700</t>
+        </is>
+      </c>
+      <c r="D1106" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1106" t="inlineStr">
+        <is>
+          <t>Pemerintah Kabupaten Tanah Laut (Pemkab Tala), Kalimantan Selatan, menjadikan pengelolaan sampah sebagai bagian dari ...</t>
+        </is>
+      </c>
+      <c r="F1106" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1106" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689692/tanah-laut-jadikan-pengelolaan-sampah-penopang-pariwisata</t>
+        </is>
+      </c>
+      <c r="H1106" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG_20260810_171835.jpg</t>
+        </is>
+      </c>
+      <c r="I1106" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1107">
+      <c r="A1107" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1107" t="inlineStr">
+        <is>
+          <t>BKPRMI minta promosi miras dikaitkan hafalan Al Quran diusut</t>
+        </is>
+      </c>
+      <c r="C1107" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:10:31 +0700</t>
+        </is>
+      </c>
+      <c r="D1107" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1107" t="inlineStr">
+        <is>
+          <t>DPP Badan Komunikasi Pemuda Remaja Masjid Indonesia (BKPRMI) meminta pihak terkait untuk mengevaluasi konten promosi ...</t>
+        </is>
+      </c>
+      <c r="F1107" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1107" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689689/bkprmi-minta-promosi-miras-dikaitkan-hafalan-al-quran-diusut</t>
+        </is>
+      </c>
+      <c r="H1107" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/dok-ketum-bkprmi.jpg</t>
+        </is>
+      </c>
+      <c r="I1107" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1108">
+      <c r="A1108" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1108" t="inlineStr">
+        <is>
+          <t>Tokyo menaikkan subsidi pembelian kendaraan listrik dan hibrida</t>
+        </is>
+      </c>
+      <c r="C1108" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:07:27 +0700</t>
+        </is>
+      </c>
+      <c r="D1108" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E1108" t="inlineStr">
+        <is>
+          <t>Pemerintah Metropolitan Tokyo di Jepang menaikkan subsidi dalam pembelian kendaraan listrik dan hibrida guna ...</t>
+        </is>
+      </c>
+      <c r="F1108" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1108" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5689688/tokyo-menaikkan-subsidi-pembelian-kendaraan-listrik-dan-hibrida</t>
+        </is>
+      </c>
+      <c r="H1108" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2023/03/20/shutterstock_735265675.jpg</t>
+        </is>
+      </c>
+      <c r="I1108" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1109">
+      <c r="A1109" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1109" t="inlineStr">
+        <is>
+          <t>Konsultan usulkan debitur skor SLIK 2 dipermudah peroleh kredit</t>
+        </is>
+      </c>
+      <c r="C1109" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:06:16 +0700</t>
+        </is>
+      </c>
+      <c r="D1109" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1109" t="inlineStr">
+        <is>
+          <t>Konsultan dan Perencana Keuangan Elvi Diana mengusulkan agar Otoritas Jasa Keuangan (OJK) maupun penyelenggara industri ...</t>
+        </is>
+      </c>
+      <c r="F1109" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1109" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689684/konsultan-usulkan-debitur-skor-slik-2-dipermudah-peroleh-kredit</t>
+        </is>
+      </c>
+      <c r="H1109" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2018/02/Sosialisasi-SLIK-OJK-230218-pf-3.jpg</t>
+        </is>
+      </c>
+      <c r="I1109" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1110" t="inlineStr">
+        <is>
+          <t>BMW siapkan pembaruan untuk BMW seri 5 touring, akan diproduksi 2027</t>
+        </is>
+      </c>
+      <c r="C1110" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:05:50 +0700</t>
+        </is>
+      </c>
+      <c r="D1110" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E1110" t="inlineStr">
+        <is>
+          <t>BMW saat ini tengah mempersiapkan pembaruan untuk BMW seri 5 touring yang diperkirakan bahwa produksi akan dimulai di ...</t>
+        </is>
+      </c>
+      <c r="F1110" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1110" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5689680/bmw-siapkan-pembaruan-untuk-bmw-seri-5-touring-akan-diproduksi-2027</t>
+        </is>
+      </c>
+      <c r="H1110" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/08/20/IMG_20240820_143100.jpg</t>
+        </is>
+      </c>
+      <c r="I1110" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1111" t="inlineStr">
+        <is>
+          <t>BPK: Mahkamah Agung tindak lanjuti 96,65 persen rekomendasi BPK</t>
+        </is>
+      </c>
+      <c r="C1111" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:03:47 +0700</t>
+        </is>
+      </c>
+      <c r="D1111" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1111" t="inlineStr">
+        <is>
+          <t>Anggota I Badan Pemeriksa Keuangan (BPK) Nyoman Adhi Suryadnyana menyampaikan bahwa Mahkamah Agung telah ...</t>
+        </is>
+      </c>
+      <c r="F1111" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1111" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689676/bpk-mahkamah-agung-tindak-lanjuti-9665-persen-rekomendasi-bpk</t>
+        </is>
+      </c>
+      <c r="H1111" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/WhatsApp-Image-2026-08-06-at-15.26.03.jpeg</t>
+        </is>
+      </c>
+      <c r="I1111" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1112" t="inlineStr">
+        <is>
+          <t>Diskop catat 174 KDKMP beroperasi di Bali didominasi gerai sembako</t>
+        </is>
+      </c>
+      <c r="C1112" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:03:27 +0700</t>
+        </is>
+      </c>
+      <c r="D1112" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1112" t="inlineStr">
+        <is>
+          <t>Dinas Koperasi dan UKM (Diskop UKM) Bali mencatat dari 716 Koperasi Desa Kelurahan Merah Putih (KDKMP) di Bali telah ...</t>
+        </is>
+      </c>
+      <c r="F1112" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1112" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689675/diskop-catat-174-kdkmp-beroperasi-di-bali-didominasi-gerai-sembako</t>
+        </is>
+      </c>
+      <c r="H1112" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/31/nilai-transaksi-kopdes-merah-putih-bali-310726-nhw-6.jpg</t>
+        </is>
+      </c>
+      <c r="I1112" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1113" t="inlineStr">
+        <is>
+          <t>I.League pastikan larangan suporter tandang resmi dicabut musim depan</t>
+        </is>
+      </c>
+      <c r="C1113" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:01:50 +0700</t>
+        </is>
+      </c>
+      <c r="D1113" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1113" t="inlineStr">
+        <is>
+          <t>Operator kompetisi sepak bola Indonesia I.League memastikan kebijakan larangan suporter tandang sudah dicabut untuk ...</t>
+        </is>
+      </c>
+      <c r="F1113" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1113" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689671/ileague-pastikan-larangan-suporter-tandang-resmi-dicabut-musim-depan</t>
+        </is>
+      </c>
+      <c r="H1113" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/01/12/Persib-Bandung-Menang-Melawan-Persija-Jakarta-110126-DAN-01.jpg</t>
+        </is>
+      </c>
+      <c r="I1113" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1114" t="inlineStr">
+        <is>
+          <t>Dharma Jaya dorong kemandirian pangan di Jakarta, kurangi sapi impor</t>
+        </is>
+      </c>
+      <c r="C1114" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:01:45 +0700</t>
+        </is>
+      </c>
+      <c r="D1114" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1114" t="inlineStr">
+        <is>
+          <t>Perumda Dharma Jaya mendorong kemandirian pangan di Jakarta melalui penguatan produksi protein hewani dan pengembangan ...</t>
+        </is>
+      </c>
+      <c r="F1114" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1114" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689669/dharma-jaya-dorong-kemandirian-pangan-di-jakarta-kurangi-sapi-impor</t>
+        </is>
+      </c>
+      <c r="H1114" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1000306724.jpg</t>
+        </is>
+      </c>
+      <c r="I1114" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1115" t="inlineStr">
+        <is>
+          <t>Trump dikawal sistem rudal Avenger saat main golf di New Jersey</t>
+        </is>
+      </c>
+      <c r="C1115" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:01:43 +0700</t>
+        </is>
+      </c>
+      <c r="D1115" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1115" t="inlineStr">
+        <is>
+          <t>Presiden Amerika Serikat Donald Trump mendapat pengawalan ketat dari sistem rudal darat-ke-udara (SAM) bertipe Avenger ...</t>
+        </is>
+      </c>
+      <c r="F1115" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1115" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689667/trump-dikawal-sistem-rudal-avenger-saat-main-golf-di-new-jersey</t>
+        </is>
+      </c>
+      <c r="H1115" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/07/19/2024-07-19T023529Z_224256324_HP1EK7J07712I_RTRMADP_3_USA-ELECTION-REPUBLICANS-CONVENTION.jpg</t>
+        </is>
+      </c>
+      <c r="I1115" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1116" t="inlineStr">
+        <is>
+          <t>Airlangga: Pertalite dan biodiesel RI masih aman meski gejolak global</t>
+        </is>
+      </c>
+      <c r="C1116" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:01:39 +0700</t>
+        </is>
+      </c>
+      <c r="D1116" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1116" t="inlineStr">
+        <is>
+          <t>Menteri Koordinator Bidang Perekonomian Airlangga Hartarto memastikan pasokan Pertalite dan biodiesel Indonesia tetap ...</t>
+        </is>
+      </c>
+      <c r="F1116" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1116" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689663/airlangga-pertalite-dan-biodiesel-ri-masih-aman-meski-gejolak-global</t>
+        </is>
+      </c>
+      <c r="H1116" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/779C2F71-F737-4EB6-AB41-D3E05C413485.jpg</t>
+        </is>
+      </c>
+      <c r="I1116" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1117" t="inlineStr">
+        <is>
+          <t>Perkuat diplomasi di Samudera Hindia, Kemlu luncurkan Satgas IORA 2026</t>
+        </is>
+      </c>
+      <c r="C1117" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:01:26 +0700</t>
+        </is>
+      </c>
+      <c r="D1117" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1117" t="inlineStr">
+        <is>
+          <t>Kementerian Luar Negeri meluncurkan “Satuan Tugas Indian Ocean Rim Association (IORA) Indonesia 2026”, ...</t>
+        </is>
+      </c>
+      <c r="F1117" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1117" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689659/perkuat-diplomasi-di-samudera-hindia-kemlu-luncurkan-satgas-iora-2026</t>
+        </is>
+      </c>
+      <c r="H1117" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/17864220736a7aa339335ea_IMG_9150_JPG.jpeg</t>
+        </is>
+      </c>
+      <c r="I1117" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1118" t="inlineStr">
+        <is>
+          <t>USK siap perkuat kolaborasi pendidikan di Aceh</t>
+        </is>
+      </c>
+      <c r="C1118" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:00:16 +0700</t>
+        </is>
+      </c>
+      <c r="D1118" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1118" t="inlineStr">
+        <is>
+          <t>Universitas Syiah Kuala (USK) Banda Aceh menyatakan siap memperkuat kolaborasi dan sinergi dengan UIN Ar-Raniry dalam ...</t>
+        </is>
+      </c>
+      <c r="F1118" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1118" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689655/usk-siap-perkuat-kolaborasi-pendidikan-di-aceh</t>
+        </is>
+      </c>
+      <c r="H1118" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/DSC03268.JPG.jpeg</t>
+        </is>
+      </c>
+      <c r="I1118" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1119" t="inlineStr">
+        <is>
+          <t>KSP kawal percepatan realisasi investasi dan hilirisasi nasional</t>
+        </is>
+      </c>
+      <c r="C1119" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:59:20 +0700</t>
+        </is>
+      </c>
+      <c r="D1119" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1119" t="inlineStr">
+        <is>
+          <t>ANTARA - Kepala Staf Kepresidenan Jenderal TNI (Purn.) Prof. Dr. Dudung Abdurachman, menggelar pertemuan dengan Wakil ...</t>
+        </is>
+      </c>
+      <c r="F1119" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1119" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5689581/ksp-kawal-percepatan-realisasi-investasi-dan-hilirisasi-nasional</t>
+        </is>
+      </c>
+      <c r="H1119" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Sequence-13.13_44_48_04.Still487.jpg</t>
+        </is>
+      </c>
+      <c r="I1119" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1120" t="inlineStr">
+        <is>
+          <t>Pramono kecam tantangan hafal Al Quran berhadiah miras di acara musik</t>
+        </is>
+      </c>
+      <c r="C1120" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:58:34 +0700</t>
+        </is>
+      </c>
+      <c r="D1120" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1120" t="inlineStr">
+        <is>
+          <t>Gubernur DKI Jakarta Pramono Anung Wibowo mengecam aksi tantangan hafalan Al Quran berhadiah minuman keras (miras) di ...</t>
+        </is>
+      </c>
+      <c r="F1120" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1120" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689651/pramono-kecam-tantangan-hafal-al-quran-berhadiah-miras-di-acara-musik</t>
+        </is>
+      </c>
+      <c r="H1120" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG_6813.jpeg</t>
+        </is>
+      </c>
+      <c r="I1120" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1121">
+      <c r="A1121" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1121" t="inlineStr">
+        <is>
+          <t>Menag: UIN Ar-Raniry Aceh harus jadi pusat peradaban Islam modern</t>
+        </is>
+      </c>
+      <c r="C1121" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:57:09 +0700</t>
+        </is>
+      </c>
+      <c r="D1121" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1121" t="inlineStr">
+        <is>
+          <t>Menteri Agama (Menag) Nasaruddin Umar menyatakan Universitas Islam Negeri (UIN) Ar-Raniry Banda Aceh harus ...</t>
+        </is>
+      </c>
+      <c r="F1121" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1121" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689648/menag-uin-ar-raniry-aceh-harus-jadi-pusat-peradaban-islam-modern</t>
+        </is>
+      </c>
+      <c r="H1121" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/menag.jpg</t>
+        </is>
+      </c>
+      <c r="I1121" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1122" t="inlineStr">
+        <is>
+          <t>Bupati Pati: Telur peternak lokal diprioritaskan penuhi kebutuhan SPPG</t>
+        </is>
+      </c>
+      <c r="C1122" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:56:20 +0700</t>
+        </is>
+      </c>
+      <c r="D1122" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1122" t="inlineStr">
+        <is>
+          <t>Pelaksana tugas (Plt) Bupati Pati Risma Ardhi Chandra menegaskan kebutuhan telur bagi Satuan Pelayanan Pemenuhan ...</t>
+        </is>
+      </c>
+      <c r="F1122" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1122" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689645/bupati-pati-telur-peternak-lokal-diprioritaskan-penuhi-kebutuhan-sppg</t>
+        </is>
+      </c>
+      <c r="H1122" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/TELUR-PATI-LOKAL-SPPG.jpg</t>
+        </is>
+      </c>
+      <c r="I1122" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1123" t="inlineStr">
+        <is>
+          <t>Laga Persija vs Persib digelar di Jakarta dengan kehadiran penonton</t>
+        </is>
+      </c>
+      <c r="C1123" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:56:18 +0700</t>
+        </is>
+      </c>
+      <c r="D1123" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1123" t="inlineStr">
+        <is>
+          <t>Direktur Utama I.League Ferry Paulus memastikan duel klasik antara Persija Jakarta versus Persib Bandung pada kompetisi ...</t>
+        </is>
+      </c>
+      <c r="F1123" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1123" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689644/laga-persija-vs-persib-digelar-di-jakarta-dengan-kehadiran-penonton</t>
+        </is>
+      </c>
+      <c r="H1123" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/11/persija-jakarta-kalahkan-persebaya-surabaya-2770671.jpg</t>
+        </is>
+      </c>
+      <c r="I1123" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1124" t="inlineStr">
+        <is>
+          <t>KAI Sampaikan Permohonan Maaf atas Gangguan Access by KAI, Pemulihan Sistem Terus Dilakukan</t>
+        </is>
+      </c>
+      <c r="C1124" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:55:16 +0700</t>
+        </is>
+      </c>
+      <c r="D1124" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1124" t="inlineStr">
+        <is>
+          <t>PT Kereta Api Indonesia (Persero) menyampaikan permohonan maaf kepada seluruh pelanggan atas gangguan pada layanan ...</t>
+        </is>
+      </c>
+      <c r="F1124" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1124" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689640/kai-sampaikan-permohonan-maaf-atas-gangguan-access-by-kai-pemulihan-sistem-terus-dilakukan</t>
+        </is>
+      </c>
+      <c r="H1124" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/Gangguan-Access-by-KAI.jpg</t>
+        </is>
+      </c>
+      <c r="I1124" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1125" t="inlineStr">
+        <is>
+          <t>Megawati lantik Taruna Merah Putih yang dipimpin Diah Pikatan Haprani</t>
+        </is>
+      </c>
+      <c r="C1125" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:54:29 +0700</t>
+        </is>
+      </c>
+      <c r="D1125" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1125" t="inlineStr">
+        <is>
+          <t>Ketua Umum DPP PDI Perjuangan Megawati Soekarnoputri melantik kepengurusan organisasi pemuda Dewan Pimpinan Pusat ...</t>
+        </is>
+      </c>
+      <c r="F1125" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1125" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689639/megawati-lantik-taruna-merah-putih-yang-dipimpin-diah-pikatan-haprani</t>
+        </is>
+      </c>
+      <c r="H1125" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1001303745.jpg</t>
+        </is>
+      </c>
+      <c r="I1125" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1126" t="inlineStr">
+        <is>
+          <t>Dugaan penistaan agama di festival musik, sejumlah pihak dilaporkan</t>
+        </is>
+      </c>
+      <c r="C1126" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:51:59 +0700</t>
+        </is>
+      </c>
+      <c r="D1126" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1126" t="inlineStr">
+        <is>
+          <t>Tim Hukum Muslim melaporkan lima orang ke Polda Metro Jaya atas dugaan tindak pidana penistaan agama yang terjadi dalam ...</t>
+        </is>
+      </c>
+      <c r="F1126" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1126" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689637/dugaan-penistaan-agama-di-festival-musik-sejumlah-pihak-dilaporkan</t>
+        </is>
+      </c>
+      <c r="H1126" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1000913553.jpg</t>
+        </is>
+      </c>
+      <c r="I1126" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1127" t="inlineStr">
+        <is>
+          <t>JPU: 27 pihak dan 313 PIHK terima aliran dana dari kasus korupsi haji</t>
+        </is>
+      </c>
+      <c r="C1127" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:50:41 +0700</t>
+        </is>
+      </c>
+      <c r="D1127" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1127" t="inlineStr">
+        <is>
+          <t>Jaksa Penuntut Umum dari Komisi Pemberantasan Korupsi (KPK) Fahmi Idris menduga terdapat sebanyak 27 pihak dan 313 ...</t>
+        </is>
+      </c>
+      <c r="F1127" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1127" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689636/jpu-27-pihak-dan-313-pihk-terima-aliran-dana-dari-kasus-korupsi-haji</t>
+        </is>
+      </c>
+      <c r="H1127" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/Yaqut-Cholil-Didakwa-Rugikan-Negara-Ratusan-Miliar-110826-Bay-3.jpg</t>
+        </is>
+      </c>
+      <c r="I1127" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1128" t="inlineStr">
+        <is>
+          <t>Dosen PTS gugat aturan pendanaan pendidikan tinggi ke MK</t>
+        </is>
+      </c>
+      <c r="C1128" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:49:18 +0700</t>
+        </is>
+      </c>
+      <c r="D1128" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1128" t="inlineStr">
+        <is>
+          <t>Seorang dosen perguruan tinggi swasta (PTS) mengajukan uji materi Undang-Undang Nomor 12 Tahun 2012 tentang Pendidikan ...</t>
+        </is>
+      </c>
+      <c r="F1128" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1128" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689635/dosen-pts-gugat-aturan-pendanaan-pendidikan-tinggi-ke-mk</t>
+        </is>
+      </c>
+      <c r="H1128" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1000001970.jpg</t>
+        </is>
+      </c>
+      <c r="I1128" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1129" t="inlineStr">
+        <is>
+          <t>Kemendikdasmen perkuat kompetensi guru vokasi jawab dunia kerja</t>
+        </is>
+      </c>
+      <c r="C1129" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:48:40 +0700</t>
+        </is>
+      </c>
+      <c r="D1129" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1129" t="inlineStr">
+        <is>
+          <t>Kementerian Pendidikan Dasar dan Menengah (Kemendikdasmen) kembali membuka program Peningkatan Kompetensi bagi Pendidik ...</t>
+        </is>
+      </c>
+      <c r="F1129" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1129" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689632/kemendikdasmen-perkuat-kompetensi-guru-vokasi-jawab-dunia-kerja</t>
+        </is>
+      </c>
+      <c r="H1129" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1000232710.jpg</t>
+        </is>
+      </c>
+      <c r="I1129" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1130" t="inlineStr">
+        <is>
+          <t>Kemenbud: Budaya pemersatu bangsa dan antar umat beragama</t>
+        </is>
+      </c>
+      <c r="C1130" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:46:22 +0700</t>
+        </is>
+      </c>
+      <c r="D1130" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1130" t="inlineStr">
+        <is>
+          <t>Staf Khusus Kementerian Kebudayaan (Kemenbud) Sri Eko Sriyanto Galgendu menegaskan bahwa kebudayaan memiliki peran ...</t>
+        </is>
+      </c>
+      <c r="F1130" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1130" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689629/kemenbud-budaya-pemersatu-bangsa-dan-antar-umat-beragama</t>
+        </is>
+      </c>
+      <c r="H1130" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/budaya.jpg.jpeg</t>
+        </is>
+      </c>
+      <c r="I1130" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1131" t="inlineStr">
+        <is>
+          <t>Pemerintah pastikan tidak ada PPPK dirumahkan</t>
+        </is>
+      </c>
+      <c r="C1131" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:43:58 +0700</t>
+        </is>
+      </c>
+      <c r="D1131" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1131" t="inlineStr">
+        <is>
+          <t>Menteri Dalam Negeri Muhammad Tito Karnavian menyatakan pemerintah menyiapkan tiga skema untuk mendukung ...</t>
+        </is>
+      </c>
+      <c r="F1131" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1131" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689628/pemerintah-pastikan-tidak-ada-pppk-dirumahkan</t>
+        </is>
+      </c>
+      <c r="H1131" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/Rapat-persiapan-pembangunan-rumah-layak-huni-di-Papua-150426-fzn-7.jpg</t>
+        </is>
+      </c>
+      <c r="I1131" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1132" t="inlineStr">
+        <is>
+          <t>PBNU minta Kemenag lebih perketat izin pesantren guna cegah kekerasan</t>
+        </is>
+      </c>
+      <c r="C1132" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:42:09 +0700</t>
+        </is>
+      </c>
+      <c r="D1132" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1132" t="inlineStr">
+        <is>
+          <t>Pengurus Besar Nahdlatul Ulama (PBNU) meminta Kementerian Agama (Kemenag) agar lebih memperketat lagi perizinan ...</t>
+        </is>
+      </c>
+      <c r="F1132" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1132" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689625/pbnu-minta-kemenag-lebih-perketat-izin-pesantren-guna-cegah-kekerasan</t>
+        </is>
+      </c>
+      <c r="H1132" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG_1871.jpeg</t>
+        </is>
+      </c>
+      <c r="I1132" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1133" t="inlineStr">
+        <is>
+          <t>Bareskrim Terbitkan 2 DPO Kasus Narkoba Five Stars Bali, Salah Satunya Owner</t>
+        </is>
+      </c>
+      <c r="C1133" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:23:55 +0700</t>
+        </is>
+      </c>
+      <c r="D1133" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E1133" t="inlineStr">
+        <is>
+          <t>Dittipid Narkoba Bareskrim Polri menerbitkan dua DPO terkait peredaran narkoba di THM Five Stars, Denpasar. Ciri-ciri dan domisili pelaku diungkap.</t>
+        </is>
+      </c>
+      <c r="F1133" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1133" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614268/bareskrim-terbitkan-2-dpo-kasus-narkoba-five-stars-bali-salah-satunya-owner</t>
+        </is>
+      </c>
+      <c r="H1133" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/07/bareskrim-polri-mengungkap-peredaran-di-five-stars-denpasar-bali-dan-mengamankan-53-orang-1786079431797_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1133" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1134" t="inlineStr">
+        <is>
+          <t>Gus Alex Didakwa Perkaya Diri Sendiri Rp 93,6 Miliar di Kasus Kuota Haji</t>
+        </is>
+      </c>
+      <c r="C1134" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:17:12 +0700</t>
+        </is>
+      </c>
+      <c r="D1134" t="inlineStr">
+        <is>
+          <t>Mulia Budi</t>
+        </is>
+      </c>
+      <c r="E1134" t="inlineStr">
+        <is>
+          <t>Gus Alex didakwa korupsi kuota haji, merugikan negara Rp 622 miliar. Tiga terdakwa terlibat, termasuk mantan Menag Yaqut Cholil Qoumas.</t>
+        </is>
+      </c>
+      <c r="F1134" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1134" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614250/gus-alex-didakwa-perkaya-diri-sendiri-rp-93-6-miliar-di-kasus-kuota-haji</t>
+        </is>
+      </c>
+      <c r="H1134" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/03/17/gus-alex-langsung-diborgol-eks-stafsus-yaqut-cholil-qoumas-resmi-ditahan-kpk-1773736846668_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1134" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1135">
+      <c r="A1135" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1135" t="inlineStr">
+        <is>
+          <t>Polisi Selidiki Kasus 36 Kambing Disembelih, Pelaku Diduga Lebih dari 1 Orang</t>
+        </is>
+      </c>
+      <c r="C1135" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:13:38 +0700</t>
+        </is>
+      </c>
+      <c r="D1135" t="inlineStr">
+        <is>
+          <t>Arief Ikhsanudin</t>
+        </is>
+      </c>
+      <c r="E1135" t="inlineStr">
+        <is>
+          <t>Polres Serang selidiki pencurian 46 kambing yang disembelih di sawah. Korban alami kerugian Rp50 juta. Pelaku diduga lebih dari satu orang.</t>
+        </is>
+      </c>
+      <c r="F1135" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1135" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614247/polisi-selidiki-kasus-36-kambing-disembelih-pelaku-diduga-lebih-dari-1-orang</t>
+        </is>
+      </c>
+      <c r="H1135" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/tkp-pencurian-dan-penyembelihan-kambing-1786450353007_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1135" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1136">
+      <c r="A1136" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1136" t="inlineStr">
+        <is>
+          <t>Perusahaan Angkut Sampah Ke TPS Ilegal di Cilincing Didenda Rp 10 Juta</t>
+        </is>
+      </c>
+      <c r="C1136" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:11:21 +0700</t>
+        </is>
+      </c>
+      <c r="D1136" t="inlineStr">
+        <is>
+          <t>Brigitta Belia Permata Sari</t>
+        </is>
+      </c>
+      <c r="E1136" t="inlineStr">
+        <is>
+          <t>Pemprov DKI Jakarta denda PT SBCI Rp10 juta karena buang sampah ilegal di Cilincing. DLH tegaskan pengawasan akan diperkuat untuk mencegah pelanggaran serupa.</t>
+        </is>
+      </c>
+      <c r="F1136" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1136" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614235/perusahaan-angkut-sampah-ke-tps-ilegal-di-cilincing-didenda-rp-10-juta</t>
+        </is>
+      </c>
+      <c r="H1136" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/05/08/gunungan-sampah-liar-cemari-kawasan-cilincing-1778231251974_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1136" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1137">
+      <c r="A1137" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1137" t="inlineStr">
+        <is>
+          <t>Kakorlantas Ajak Driver Ojol Jadi Pelopor Keselamatan Lalu Lintas, Perkuat Sinergi</t>
+        </is>
+      </c>
+      <c r="C1137" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:01:59 +0700</t>
+        </is>
+      </c>
+      <c r="D1137" t="inlineStr">
+        <is>
+          <t>Herianto Batubara</t>
+        </is>
+      </c>
+      <c r="E1137" t="inlineStr">
+        <is>
+          <t>Kakorlantas Polri Irjen Wibowo bertemu komunitas ojol untuk memperkuat sinergi dalam keselamatan lalu lintas. Ojol diharapkan jadi mitra keselamatan di jalan.</t>
+        </is>
+      </c>
+      <c r="F1137" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1137" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614227/kakorlantas-ajak-driver-ojol-jadi-pelopor-keselamatan-lalu-lintas-perkuat-sinergi</t>
+        </is>
+      </c>
+      <c r="H1137" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/kakorlantas-ajak-driver-ojol-jadi-pelopor-keselamatan-lalu-lintas-1786449624135_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1137" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1138" t="inlineStr">
+        <is>
+          <t>KP2MI Buka Pendaftaran Pelatihan Asta Mandala SMK Go Global Tahap Pertama</t>
+        </is>
+      </c>
+      <c r="C1138" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:55:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1138" t="inlineStr">
+        <is>
+          <t>Dea Duta Aulia</t>
+        </is>
+      </c>
+      <c r="E1138" t="inlineStr">
+        <is>
+          <t>Kementerian P2MI buka pendaftaran Pelatihan SMK Go Global untuk 500.000 calon pekerja migran. Program ini siapkan generasi muda hadapi pasar kerja internasional</t>
+        </is>
+      </c>
+      <c r="F1138" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1138" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614210/kp2mi-buka-pendaftaran-pelatihan-asta-mandala-smk-go-global-tahap-pertama</t>
+        </is>
+      </c>
+      <c r="H1138" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/kp2mi-1786449281276.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1138" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1139" t="inlineStr">
+        <is>
+          <t>Jaksa Agung Minta Jajaran Jaga Integritas dan Hidup Sederhana</t>
+        </is>
+      </c>
+      <c r="C1139" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:43:46 +0700</t>
+        </is>
+      </c>
+      <c r="D1139" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E1139" t="inlineStr">
+        <is>
+          <t>Jaksa Agung ST Burhanuddin melantik 15 Kajati, menekankan pentingnya integritas dan pola hidup sederhana. Dia juga mendorong transparansi dan pengawasan ketat.</t>
+        </is>
+      </c>
+      <c r="F1139" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1139" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614198/jaksa-agung-minta-jajaran-jaga-integritas-dan-hidup-sederhana</t>
+        </is>
+      </c>
+      <c r="H1139" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/03/13/jaksa-agung-st-burhanuddin-1773341038180_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1139" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1140" t="inlineStr">
+        <is>
+          <t>Challenge Hafalan Qur'an Demi Miras Saat Konser Dilaporkan ke Polda Metro</t>
+        </is>
+      </c>
+      <c r="C1140" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:38:18 +0700</t>
+        </is>
+      </c>
+      <c r="D1140" t="inlineStr">
+        <is>
+          <t>Wildan Noviansah</t>
+        </is>
+      </c>
+      <c r="E1140" t="inlineStr">
+        <is>
+          <t>Kasus promosi miras berkedok tantangan hafalan Al-Qur'an di konser The Sounds Project dilaporkan ke polisi. Penyelidikan sedang berlangsung.</t>
+        </is>
+      </c>
+      <c r="F1140" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1140" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614190/challenge-hafalan-quran-demi-miras-saat-konser-dilaporkan-ke-polda-metro</t>
+        </is>
+      </c>
+      <c r="H1140" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/tim-hukum-muslim-melaporkan-kasus-challenge-hafalan-quran-demi-miras-ke-polda-metro-jaya-1786448216677_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1140" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1141" t="inlineStr">
+        <is>
+          <t>Purbaya &amp;amp; Bahlil Sepakat Harga BBM Subsidi Tak Bakal Naik</t>
+        </is>
+      </c>
+      <c r="C1141" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:00:57 +0700</t>
+        </is>
+      </c>
+      <c r="D1141" t="inlineStr">
+        <is>
+          <t>Heri Purnomo</t>
+        </is>
+      </c>
+      <c r="E1141" t="inlineStr">
+        <is>
+          <t>Menteri ESDM Bahlil dan Menteri Keuangan Purbaya sepakat harga BBM subsidi tidak akan naik, meski harga minyak dunia fluktuatif.</t>
+        </is>
+      </c>
+      <c r="F1141" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1141" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8614186/purbaya-bahlil-sepakat-harga-bbm-subsidi-tak-bakal-naik</t>
+        </is>
+      </c>
+      <c r="H1141" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/10/04/purbaya-dan-bahlil-1759581063819_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1141" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B1142" t="inlineStr">
+        <is>
+          <t>Hoax Selingkuh dengan Asila Berujung Laporan, Rizky Billar Ingin Pelaku Jera</t>
+        </is>
+      </c>
+      <c r="C1142" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:07:11 +0700</t>
+        </is>
+      </c>
+      <c r="D1142" t="inlineStr">
+        <is>
+          <t>Febryantino Nur Pratama</t>
+        </is>
+      </c>
+      <c r="E1142" t="inlineStr">
+        <is>
+          <t>Rizky Billar mendampingi Lesti Kejora dan Asila Maisa dalam pemeriksaan di Polda Metro Jaya terkait laporan penyebaran berita bohong. Billar mau pelaku jera.</t>
+        </is>
+      </c>
+      <c r="F1142" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1142" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8613786/hoax-selingkuh-dengan-asila-berujung-laporan-rizky-billar-ingin-pelaku-jera</t>
+        </is>
+      </c>
+      <c r="H1142" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/rizky-billar-lesti-kejora-dan-asilla-1786424585636_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1142" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B1143" t="inlineStr">
+        <is>
+          <t>Potret Nikah Pebulutangkis Leo Rolly Carnando dengan Indah</t>
+        </is>
+      </c>
+      <c r="C1143" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:33:13 +0700</t>
+        </is>
+      </c>
+      <c r="D1143" t="inlineStr">
+        <is>
+          <t>Mauludi Rismoyo</t>
+        </is>
+      </c>
+      <c r="E1143" t="inlineStr">
+        <is>
+          <t>Kabar soal pebulutangkis Leo Rolly Carnando dengan Indah Cahya Sari benar adanya. Indah membagikan foto nikah.</t>
+        </is>
+      </c>
+      <c r="F1143" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1143" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8614126/potret-nikah-pebulutangkis-leo-rolly-carnando-dengan-indah</t>
+        </is>
+      </c>
+      <c r="H1143" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/leo-rolly-carnando-1786446060203_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1143" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1144" t="inlineStr">
+        <is>
+          <t>Dokter Ungkap Kanker Payudara dan Serviks Sering Berkembang Tanpa Gejala, Penting Skrining Rutin</t>
+        </is>
+      </c>
+      <c r="C1144" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:31:50 +0700</t>
+        </is>
+      </c>
+      <c r="D1144" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1144" t="inlineStr">
+        <is>
+          <t>Banyak pasien kanker payudara memeriksakan diri setelah menemukan benjolan dan merasa nyeri. Padahal belum tentu itu muncul saat kanker di tahap awal.</t>
+        </is>
+      </c>
+      <c r="F1144" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1144" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7867061/dokter-ungkap-kanker-payudara-dan-serviks-sering-berkembang-tanpa-gejala-penting-skrining-rutin</t>
+        </is>
+      </c>
+      <c r="H1144" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/hFidTCUrtHAR90zYoVe4NCXEPUc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ILUSTRASI-KANKER-SERVIKS-1.jpg</t>
+        </is>
+      </c>
+      <c r="I1144" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1145" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya Bongkar Peredaran Narkoba Lewat Ekspedisi di Jakarta Pusat, 7 Paket Sabu Disita</t>
+        </is>
+      </c>
+      <c r="C1145" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:30:46 +0700</t>
+        </is>
+      </c>
+      <c r="D1145" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1145" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya menggagalkan peredaran narkotika jenis sabu yang diduga dikirim menggunakan modus paket ekspedisi di wilayah Jakarta Pusat.</t>
+        </is>
+      </c>
+      <c r="F1145" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1145" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7867060/polda-metro-jaya-bongkar-peredaran-narkoba-lewat-ekspedisi-di-jakarta-pusat-7-paket-sabu-disita</t>
+        </is>
+      </c>
+      <c r="H1145" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/PzAsSaUTeWBvvqRQGt7e-1rxfyA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/rilis-kasus-narkoba-polda-metro-jaya-e.jpg</t>
+        </is>
+      </c>
+      <c r="I1145" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1146" t="inlineStr">
+        <is>
+          <t>Hanya 20,14 Persen Penyandang Disabilitas Masuk Dunia Kerja, Karyanya Masih Terbatas</t>
+        </is>
+      </c>
+      <c r="C1146" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:26:07 +0700</t>
+        </is>
+      </c>
+      <c r="D1146" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1146" t="inlineStr">
+        <is>
+          <t>Data Kemenaker mencatat, dari sekitar 17 juta penyandang disabilitas usia produktif, hanya 20,14 persen yang masuk dalam angkatan kerja.</t>
+        </is>
+      </c>
+      <c r="F1146" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1146" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867059/hanya-2014-persen-penyandang-disabilitas-masuk-dunia-kerja-karyanya-masih-terbatas</t>
+        </is>
+      </c>
+      <c r="H1146" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/oZltZiwirt3OEOiFCb00Np07XmY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Nurdini-Prihastiti-1.jpg</t>
+        </is>
+      </c>
+      <c r="I1146" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1147" t="inlineStr">
+        <is>
+          <t>Sidang Yaqut: KPK Ungkap Pengaturan Kuota Haji, USD1 Juta untuk Pansus dan Kerugian Rp622 Miliar</t>
+        </is>
+      </c>
+      <c r="C1147" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:24:58 +0700</t>
+        </is>
+      </c>
+      <c r="D1147" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1147" t="inlineStr">
+        <is>
+          <t>Yaqut Cholil Qoumas menyiapkan USD 1 juta untuk mempengaruhi hasil Pansus Angket Haji di DPR Tahun 2024.</t>
+        </is>
+      </c>
+      <c r="F1147" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1147" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867058/sidang-yaqut-kpk-ungkap-pengaturan-kuota-haji-usd1-juta-untuk-pansus-dan-kerugian-rp622-miliar</t>
+        </is>
+      </c>
+      <c r="H1147" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/hQOLdcKo2PFpCgJrAjSiIBiOS6M=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Yaqut-Jalani-Sidang-Perdana-Kasus-Korupsi-Kuota-Haji_20260811_145757.jpg</t>
+        </is>
+      </c>
+      <c r="I1147" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1148" t="inlineStr">
+        <is>
+          <t>Beat Takeshi Kritik Pendaki Gunung Fuji, 2 WNI Jadi Sorotan karena Pakai Payung</t>
+        </is>
+      </c>
+      <c r="C1148" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:24:47 +0700</t>
+        </is>
+      </c>
+      <c r="D1148" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1148" t="inlineStr">
+        <is>
+          <t>Beat Takeshi kritik pendaki Gunung Fuji yang tak siap dan dukung aturan lebih tegas, termasuk biaya pendakian dan asuransi untuk operasi penyelamatan</t>
+        </is>
+      </c>
+      <c r="F1148" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1148" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7867057/beat-takeshi-kritik-pendaki-gunung-fuji-2-wni-jadi-sorotan-karena-pakai-payung</t>
+        </is>
+      </c>
+      <c r="H1148" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/W80YeOER7fokSbD-Vo1YrMfQISc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/orangpayung11111.jpg</t>
+        </is>
+      </c>
+      <c r="I1148" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1149" t="inlineStr">
+        <is>
+          <t>3 Alasan Rodri Ragu ke Real Madrid hingga Pilih Barcelona</t>
+        </is>
+      </c>
+      <c r="C1149" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:24:17 +0700</t>
+        </is>
+      </c>
+      <c r="D1149" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1149" t="inlineStr">
+        <is>
+          <t>Rodri dikabarkan batal ke Real Madrid setelah memiliki sejumlah keraguan. Barcelona kemudian datang dan selangkah lagi mendapatkan sang gelandang.</t>
+        </is>
+      </c>
+      <c r="F1149" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1149" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7867056/3-alasan-rodri-ragu-ke-real-madrid-hingga-pilih-barcelona</t>
+        </is>
+      </c>
+      <c r="H1149" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/_VpOqU99lj-Oz2bEhTHowlCuKvY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Rodri-Raih-Ballon-dOr_20241029_113921.jpg</t>
+        </is>
+      </c>
+      <c r="I1149" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1150" t="inlineStr">
+        <is>
+          <t>Dana PTN dan PTS Dinilai Belum Adil, Riset Dosen Terkendala Anggaran</t>
+        </is>
+      </c>
+      <c r="C1150" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:22:28 +0700</t>
+        </is>
+      </c>
+      <c r="D1150" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1150" t="inlineStr">
+        <is>
+          <t>Dosen PTS menggugat aturan pendanaan pendidikan tinggi ke MK setelah anggaran riset disebut semakin terbatas.</t>
+        </is>
+      </c>
+      <c r="F1150" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1150" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867055/dana-ptn-dan-pts-dinilai-belum-adil-riset-dosen-terkendala-anggaran</t>
+        </is>
+      </c>
+      <c r="H1150" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/oAcRRDSjQ7nHVcXmoaAOIcOmd4Q=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/sidang-uji-materi-Undang-Undang-Nomor-12-Tahun-2012-UU-Pendidikan-Tinggi-Mahkamah-Konstitusi-MK.jpg</t>
+        </is>
+      </c>
+      <c r="I1150" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1151" t="inlineStr">
+        <is>
+          <t>KPK Buka Suara Soal Winda Lorenza, Sempat Dipanggil Untuk Telusuri Aliran Uang Korupsi Bea Cukai</t>
+        </is>
+      </c>
+      <c r="C1151" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:19:59 +0700</t>
+        </is>
+      </c>
+      <c r="D1151" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1151" t="inlineStr">
+        <is>
+          <t>KPK akhirnya buka suara mengenai sosok Winda Lorenza Gowasa yang tewas penuh kejanggalan di Medan, Sumatera Utara.</t>
+        </is>
+      </c>
+      <c r="F1151" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1151" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867054/kpk-buka-suara-soal-winda-lorenza-sempat-dipanggil-untuk-telusuri-aliran-uang-korupsi-bea-cukai</t>
+        </is>
+      </c>
+      <c r="H1151" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/E0yUvTRc5-LVa7G_JqpQdDfSl7M=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Juru-Bicara-KPK-Budi-Prasetyo-2742026.jpg</t>
+        </is>
+      </c>
+      <c r="I1151" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1152" t="inlineStr">
+        <is>
+          <t>Kunci Jawaban Matematika Kelas 5 SD Halaman 197 Kurikulum Merdeka Bab 7, Membuat Segitiga</t>
+        </is>
+      </c>
+      <c r="C1152" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:19:29 +0700</t>
+        </is>
+      </c>
+      <c r="D1152" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1152" t="inlineStr">
+        <is>
+          <t>Kunci jawaban Matematika Kelas 5 SD halaman 197 membahas kelompok sedotan yang bisa dan tidak bisa membentuk segitiga.</t>
+        </is>
+      </c>
+      <c r="F1152" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1152" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/pendidikan/7867053/kunci-jawaban-matematika-kelas-5-sd-halaman-197-kurikulum-merdeka-bab-7-membuat-segitiga</t>
+        </is>
+      </c>
+      <c r="H1152" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/1JPKJGa96_InI21Y0aEE8NCU4z4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/SISWA-SD-BELAJAR-20.jpg</t>
+        </is>
+      </c>
+      <c r="I1152" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1153" t="inlineStr">
+        <is>
+          <t>Viral Challenge Hafalan Surat Alquran Berhadiah Miras, YKMI Desak Cabut Izin Edar</t>
+        </is>
+      </c>
+      <c r="C1153" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:17:33 +0700</t>
+        </is>
+      </c>
+      <c r="D1153" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1153" t="inlineStr">
+        <is>
+          <t>YKMI menilai promosi tersebut melecehkan agama dan mendesak pemerintah serta aparat mengambil tindakan.</t>
+        </is>
+      </c>
+      <c r="F1153" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1153" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867052/viral-challenge-hafalan-surat-alquran-berhadiah-miras-ykmi-desak-cabut-izin-edar</t>
+        </is>
+      </c>
+      <c r="H1153" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/WO5gUct79rm2w14vW8VLt3rKtHQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Ferry-Irawan-YMKI.jpg</t>
+        </is>
+      </c>
+      <c r="I1153" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1154" t="inlineStr">
+        <is>
+          <t>Stres hingga Depresi Gegara Skripsi? Psikolog Beri Saran untuk Mahasiswa Tingkat Akhir</t>
+        </is>
+      </c>
+      <c r="C1154" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:16:30 +0700</t>
+        </is>
+      </c>
+      <c r="D1154" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1154" t="inlineStr">
+        <is>
+          <t>Psikolog menyarankan mahasiswa menghadapi stres skripsi dengan fokus pada hal yang bisa dikontrol dan tidak ragu mencari bantuan.</t>
+        </is>
+      </c>
+      <c r="F1154" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1154" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/lifestyle/7867051/stres-hingga-depresi-gegara-skripsi-psikolog-beri-saran-untuk-mahasiswa-tingkat-akhir</t>
+        </is>
+      </c>
+      <c r="H1154" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/om_yS8jzPPdVEHqZCFP9CIRqb1E=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/PSiswa-MAN-3-Padang-Ledakkan-Bom-di-Sekolah-Gegara-Di-bully-Psikolog-Tegaskan-Dia-Bukan-Anak-Jahat.jpg</t>
+        </is>
+      </c>
+      <c r="I1154" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1155" t="inlineStr">
+        <is>
+          <t>Kunci Jawaban Matematika Kelas 5 SD Halaman 196 Kurikulum Merdeka, Eksplorasi Membuat Segitiga</t>
+        </is>
+      </c>
+      <c r="C1155" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:15:51 +0700</t>
+        </is>
+      </c>
+      <c r="D1155" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1155" t="inlineStr">
+        <is>
+          <t>Kunci jawaban Matematika Kelas 5 SD halaman 196 membahas cara menentukan tiga panjang sisi yang dapat membentuk segitiga.</t>
+        </is>
+      </c>
+      <c r="F1155" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1155" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/pendidikan/7867050/kunci-jawaban-matematika-kelas-5-sd-halaman-196-kurikulum-merdeka-eksplorasi-membuat-segitiga</t>
+        </is>
+      </c>
+      <c r="H1155" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/1JPKJGa96_InI21Y0aEE8NCU4z4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/SISWA-SD-BELAJAR-20.jpg</t>
+        </is>
+      </c>
+      <c r="I1155" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1156" t="inlineStr">
+        <is>
+          <t>Prakiraan Cuaca Flores Besok Rabu 12 Agustus 2026: Labuan Bajo dan Ende Cerah hingga Cerah Berawan</t>
+        </is>
+      </c>
+      <c r="C1156" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:15:06 +0700</t>
+        </is>
+      </c>
+      <c r="D1156" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1156" t="inlineStr">
+        <is>
+          <t>Berikut detail prakiraan cuaca di beberapa kota terkenal di Flores untuk Rabu (12/8/2026) berdasarkan prakiraan BMKG:</t>
+        </is>
+      </c>
+      <c r="F1156" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1156" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7867049/prakiraan-cuaca-flores-besok-rabu-12-agustus-2026-labuan-bajo-dan-ende-cerah-hingga-cerah-berawan</t>
+        </is>
+      </c>
+      <c r="H1156" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/L57Bkzw0Fujr2ABxB4iWPb-V7SE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/danau-tiwusora-di-kabupaten-ende-flores-ntt.jpg</t>
+        </is>
+      </c>
+      <c r="I1156" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1157" t="inlineStr">
+        <is>
+          <t>Destry Damayanti Calon Gubernur BI, Anggota DPR Eric Hermawan: Kemampuannya Tak Perlu Diragukan</t>
+        </is>
+      </c>
+      <c r="C1157" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:59:06 +0700</t>
+        </is>
+      </c>
+      <c r="D1157" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1157" t="inlineStr">
+        <is>
+          <t>Eric Hermawan, menilai sosok Destry Damayanti sebagai figur yang pas untuk menjabat sebagai Gubernur Bank Indonesia (BI) definitif.</t>
+        </is>
+      </c>
+      <c r="F1157" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1157" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867048/destry-damayanti-calon-gubernur-bi-anggota-dpr-eric-hermawan-kemampuannya-tak-perlu-diragukan</t>
+        </is>
+      </c>
+      <c r="H1157" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/gMctDY3Den6hm7aAheqS9w41TQE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Destry-Damayanti-di-Istana-32102.jpg</t>
+        </is>
+      </c>
+      <c r="I1157" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1158" t="inlineStr">
+        <is>
+          <t>Penerapan K3 ke Pekerja Sawit Berdampak Positif ke Produktivitas Industri</t>
+        </is>
+      </c>
+      <c r="C1158" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:56:39 +0700</t>
+        </is>
+      </c>
+      <c r="D1158" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1158" t="inlineStr">
+        <is>
+          <t>implementasi K3 harus diterapkan secara menyeluruh di seluruh rantai industri sawit mulai dari perkebunan hingga pabrik pengolahan</t>
+        </is>
+      </c>
+      <c r="F1158" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1158" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/bisnis/7867047/penerapan-k3-ke-pekerja-sawit-berdampak-positif-ke-produktivitas-industri</t>
+        </is>
+      </c>
+      <c r="H1158" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/T1sIpuSqdVF6MvUOF5E5MjDnhQE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Penerapan-standar-keselamatan-dan-kesehatan-kerja-K3-di-perkebunan.jpg</t>
+        </is>
+      </c>
+      <c r="I1158" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1159" t="inlineStr">
+        <is>
+          <t>Gimik Bermuatan SARA Dinilai Bisa Picu Perpecahan, Anggota DPR Minta Polisi Bertindak Tegas</t>
+        </is>
+      </c>
+      <c r="C1159" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:56:36 +0700</t>
+        </is>
+      </c>
+      <c r="D1159" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1159" t="inlineStr">
+        <is>
+          <t>Abdullah menyoroti maraknya gimik di ruang publik dan media sosial yang dinilai merendahkan suku, agama, ras, dan antargolongan (SARA).</t>
+        </is>
+      </c>
+      <c r="F1159" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1159" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867046/gimik-bermuatan-sara-dinilai-bisa-picu-perpecahan-anggota-dpr-minta-polisi-bertindak-tegas</t>
+        </is>
+      </c>
+      <c r="H1159" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/S7niCuPoL-On6Ah57kIk9Zp3z9c=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Anggota-DPR-RI-Abdullah-Soroti-Kasus-Brimob-Lindas-Ojol.jpg</t>
+        </is>
+      </c>
+      <c r="I1159" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1160" t="inlineStr">
+        <is>
+          <t>Habis Indonesia Gantian Malaysia, Kans Vietnam Ulangi Pembantaian di Piala AFF 2026</t>
+        </is>
+      </c>
+      <c r="C1160" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:55:36 +0700</t>
+        </is>
+      </c>
+      <c r="D1160" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1160" t="inlineStr">
+        <is>
+          <t>Vietnam diprediksi bakal menyingkirkan Malaysia dengan cara memalukan di semifinal Piala AFF 2026.</t>
+        </is>
+      </c>
+      <c r="F1160" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1160" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7867045/habis-indonesia-gantian-malaysia-kans-vietnam-ulangi-pembantaian-di-piala-aff-2026</t>
+        </is>
+      </c>
+      <c r="H1160" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/u8AMguqjsVPB9v5yd1u6daLPdnU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Timnas-Indonesia-Dicukur-Timnas-Vietnam-3-0_20260804_070349.jpg</t>
+        </is>
+      </c>
+      <c r="I1160" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1161" t="inlineStr">
+        <is>
+          <t>Kronologi Penyelamatan Ibu dan Bayi 6 Bulan Ditemukan Hidup di Balik Reruntuhan Gempa Cali Kolombia</t>
+        </is>
+      </c>
+      <c r="C1161" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:51:36 +0700</t>
+        </is>
+      </c>
+      <c r="D1161" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1161" t="inlineStr">
+        <is>
+          <t>Tim SAR menemukan ibu dan bayinya yang berusia enam bulan masih hidup di balik reruntuhan bangunan akibat gempa di Cali, Kolombia</t>
+        </is>
+      </c>
+      <c r="F1161" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1161" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7867044/kronologi-penyelamatan-ibu-dan-bayi-6-bulan-ditemukan-hidup-di-balik-reruntuhan-gempa-cali-kolombia</t>
+        </is>
+      </c>
+      <c r="H1161" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/hzWx5otJiYfuvi7E1WBaYnCcYqs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/KONDISI-KOTA-PEREIRA-SETELAH-GEMPA-GUNCANG-KOLOMBIA.jpg</t>
+        </is>
+      </c>
+      <c r="I1161" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1162" t="inlineStr">
+        <is>
+          <t>Purbaya Targetkan Pembenahan Bea Cukai hingga September 2026, Djaka Budhi Minta Bantuan Masyarakat</t>
+        </is>
+      </c>
+      <c r="C1162" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:50:19 +0700</t>
+        </is>
+      </c>
+      <c r="D1162" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1162" t="inlineStr">
+        <is>
+          <t>Djaka mengkaui, pembenahan terhadap internal Bea Cukai akan maksimal apabila ada peran dari stakeholder lainnya.</t>
+        </is>
+      </c>
+      <c r="F1162" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1162" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/bisnis/7867043/purbaya-targetkan-pembenahan-bea-cukai-hingga-september-2026-djaka-budhi-minta-bantuan-masyarakat</t>
+        </is>
+      </c>
+      <c r="H1162" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ZtjSZdLN0na1W9fF4cZ3CaaG_X8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Dirjen-Bea-Cukai-Kemenkeu-Djaka-Budhi-Utama-saat-konpers-rokok-ilegal-di-priok.jpg</t>
+        </is>
+      </c>
+      <c r="I1162" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1163" t="inlineStr">
+        <is>
+          <t>Peringatan Dini 6 Ibu Kota Pulau Jawa Besok Rabu 12 Agustus: Jakarta Cerah, Jogja Udara Kabur</t>
+        </is>
+      </c>
+      <c r="C1163" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:49:21 +0700</t>
+        </is>
+      </c>
+      <c r="D1163" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1163" t="inlineStr">
+        <is>
+          <t>Peringatan dini BMKG di 6 Ibu Kota di Pulau Jawa. Mulai dari Jakarta, Bandung, hingga Semarang pada (12/8/2026).</t>
+        </is>
+      </c>
+      <c r="F1163" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1163" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867042/peringatan-dini-6-ibu-kota-pulau-jawa-besok-rabu-12-agustus-jakarta-cerah-jogja-udara-kabur</t>
+        </is>
+      </c>
+      <c r="H1163" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Ew22ZWpIXWs0i0Fg5jOcsd0PKDk=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/cuaca-cerah-sekali.jpg</t>
+        </is>
+      </c>
+      <c r="I1163" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B1164" t="inlineStr">
+        <is>
+          <t>Menteri UMKM Maman Janjikan Perpres Ojol Segera Terbit</t>
+        </is>
+      </c>
+      <c r="C1164" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:35:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1164" t="inlineStr">
+        <is>
+          <t>Novina Putri Bestari</t>
+        </is>
+      </c>
+      <c r="E1164" t="inlineStr">
+        <is>
+          <t>Menteri UMKM Maman Abdurrahman menjanjikan Perpres Ojol akan segera terbit</t>
+        </is>
+      </c>
+      <c r="F1164" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1164" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260811191928-37-758413/menteri-umkm-maman-janjikan-perpres-ojol-segera-terbit</t>
+        </is>
+      </c>
+      <c r="H1164" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/menteri-umkm-maman-abdurrahman-saat-doorstop-usai-acara-umkm-finance-summit-2026-dengan-tema-penguatan-akses-pembiayaan-dan-ek-1786422817800_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1164" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1165">
+      <c r="A1165" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B1165" t="inlineStr">
+        <is>
+          <t>Petaka Baru Datang dari China, Satu Dunia Terancam Jadi Korban</t>
+        </is>
+      </c>
+      <c r="C1165" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1165" t="inlineStr">
+        <is>
+          <t>Redaksi</t>
+        </is>
+      </c>
+      <c r="E1165" t="inlineStr">
+        <is>
+          <t>Microsoft mengungkap kelompok peretas China, Storm-1175, yang menyebarkan ransomware baru, StormEncryptor. Simak!</t>
+        </is>
+      </c>
+      <c r="F1165" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1165" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260811120046-37-758220/petaka-baru-datang-dari-china-satu-dunia-terancam-jadi-korban</t>
+        </is>
+      </c>
+      <c r="H1165" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2022/09/11/siapakah-bjorka-hacker-yang-bikin-pemerintah-ri-ketar-ketir_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1165" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B1166" t="inlineStr">
+        <is>
+          <t>Batu Dipakai Ganjal Pintu, Ternyata Harta Karun Rp 20 Miliar</t>
+        </is>
+      </c>
+      <c r="C1166" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:20:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1166" t="inlineStr">
+        <is>
+          <t>Redaksi</t>
+        </is>
+      </c>
+      <c r="E1166" t="inlineStr">
+        <is>
+          <t>Seorang nenek di Romania menemukan batu 3,5 kg yang ternyata adalah amber raksasa bernilai Rp 20 miliar.</t>
+        </is>
+      </c>
+      <c r="F1166" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1166" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260811145624-37-758308/batu-dipakai-ganjal-pintu-ternyata-harta-karun-rp-20-miliar</t>
+        </is>
+      </c>
+      <c r="H1166" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2024/09/12/bongkahan-amber-seberat-35-kilogram-itu-merupakan-potongan-rumanit-terbesar-yang-pernah-ditemukan_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1166" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1167">
+      <c r="A1167" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B1167" t="inlineStr">
+        <is>
+          <t>Jadi Bangunan Cerdas, RS dan Pabrik Ini Mampu Tekan Cost dan Downtime</t>
+        </is>
+      </c>
+      <c r="C1167" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:57:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1167" t="inlineStr">
+        <is>
+          <t>Khoirul Anam</t>
+        </is>
+      </c>
+      <c r="E1167" t="inlineStr">
+        <is>
+          <t>Indonesia menargetkan penurunan emisi gas rumah kaca hingga 43% pada 2030, salah satunya lewat penerapan Bangunan Gedung Cerdas.</t>
+        </is>
+      </c>
+      <c r="F1167" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1167" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260811171626-37-758386/jadi-bangunan-cerdas-rs-dan-pabrik-ini-mampu-tekan-cost-downtime</t>
+        </is>
+      </c>
+      <c r="H1167" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/smc-rumah-sakit-telogorejo-semarang-1786445781245_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1167" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1168">
+      <c r="A1168" t="inlineStr">
+        <is>
+          <t>Energi</t>
+        </is>
+      </c>
+      <c r="B1168" t="inlineStr">
+        <is>
+          <t>Rapat dengan Bahlil, Purbaya Janji Pembatasan Pembelian Pertalite Dilakukan Bertahap</t>
+        </is>
+      </c>
+      <c r="C1168" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:09:28 +0700</t>
+        </is>
+      </c>
+      <c r="D1168" t="inlineStr">
+        <is>
+          <t>Ahmad Fikri Noor</t>
+        </is>
+      </c>
+      <c r="E1168" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- Menteri Energi dan Sumber Daya Mineral (ESDM) dan Menteri Keuangan (Menkeu) Purbaya Yudhi Sadewa melaksanakan pertemuan untuk membahas mekanisme penyaluran BBM bersubsidi. Purbaya mengatakan, pengendalian subsidi bahan...</t>
+        </is>
+      </c>
+      <c r="F1168" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1168" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjltrs490/rapat-dengan-bahlil-purbaya-janji-pembatasan-pembelian-pertalite-dilakukan-bertahap</t>
+        </is>
+      </c>
+      <c r="H1168" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/096319300-1780650844-830-556.jpg</t>
+        </is>
+      </c>
+      <c r="I1168" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="1169">
+      <c r="A1169" t="inlineStr">
+        <is>
+          <t>Energi</t>
+        </is>
+      </c>
+      <c r="B1169" t="inlineStr">
+        <is>
+          <t>Bahlil Temui Purbaya Bahas Pembatasan Pembelian Pertalite</t>
+        </is>
+      </c>
+      <c r="C1169" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:03:37 +0700</t>
+        </is>
+      </c>
+      <c r="D1169" t="inlineStr">
+        <is>
+          <t>Ahmad Fikri Noor</t>
+        </is>
+      </c>
+      <c r="E1169" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- Menteri Energi dan Sumber Daya Mineral (ESDM) Bahlil Lahadalia menemui Menteri Keuangan (Menkeu) Purbaya Yudhi Sadewa. Pertemuan itu membahas penyaluran subsidi bahan bakar minyak (BBM) agar tepat...</t>
+        </is>
+      </c>
+      <c r="F1169" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1169" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjlti1490/bahlil-temui-purbaya-bahas-pembatasan-pembelian-pertalite</t>
+        </is>
+      </c>
+      <c r="H1169" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/006092900-1760884175-830-556.jpg</t>
+        </is>
+      </c>
+      <c r="I1169" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="1170">
+      <c r="A1170" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1170" t="inlineStr">
+        <is>
+          <t>Polisi Tangkap 2 Pelaku Penyekapan Lansia Ngaku Anggota KPK</t>
+        </is>
+      </c>
+      <c r="C1170" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:38:27 +0700</t>
+        </is>
+      </c>
+      <c r="D1170" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1170" t="inlineStr">
+        <is>
+          <t>Polisi mengamankan dua pria yang diduga terlibat dalam tindak pidana pencurian dengan pemberatan disertai penyekapan terhadap lansia di Tangsel.</t>
+        </is>
+      </c>
+      <c r="F1170" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1170" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267437/polisi-tangkap-2-pelaku-penyekapan-lansia-ngaku-anggota-kpk</t>
+        </is>
+      </c>
+      <c r="H1170" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/EvCoV8tn_M-VP-PCM52zvLmQyM4=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9321574/original/082974800_1786451876-IMG-20260811-WA0026.jpg</t>
+        </is>
+      </c>
+      <c r="I1170" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1171">
+      <c r="A1171" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1171" t="inlineStr">
+        <is>
+          <t>Sempat Dikira Gantung Diri, Wanita di Tangerang Ternyata Dibunuh Kekasih</t>
+        </is>
+      </c>
+      <c r="C1171" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:32:52 +0700</t>
+        </is>
+      </c>
+      <c r="D1171" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1171" t="inlineStr">
+        <is>
+          <t>Korban ditemukan dalam kondisi tergantung yang awalnya diduga sebagai bunuh diri.</t>
+        </is>
+      </c>
+      <c r="F1171" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1171" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267431/sempat-dikira-gantung-diri-wanita-di-tangerang-ternyata-dibunuh-kekasih</t>
+        </is>
+      </c>
+      <c r="H1171" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/elDNxj19Ao1xJh5eehIKyL9IihU=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/849467/original/025285500_1428837125-Ilustrasi-pembunuhan-wanita-2.jpg</t>
+        </is>
+      </c>
+      <c r="I1171" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1172">
+      <c r="A1172" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1172" t="inlineStr">
+        <is>
+          <t>Fokus Rangkul Generasi Muda, PDIP Lantik Taruna Merah Putih</t>
+        </is>
+      </c>
+      <c r="C1172" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:03:39 +0700</t>
+        </is>
+      </c>
+      <c r="D1172" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1172" t="inlineStr">
+        <is>
+          <t>PDI Perjuangan menegaskan fokus partai dalam merangkul generasi muda.</t>
+        </is>
+      </c>
+      <c r="F1172" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1172" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267415/fokus-rangkul-generasi-muda-pdip-lantik-taruna-merah-putih</t>
+        </is>
+      </c>
+      <c r="H1172" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/m48HfJYPaJEZKeA4JZOFEYcJ3b0=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9321561/original/095047900_1786449805-DSC02530.jpg.jpeg</t>
+        </is>
+      </c>
+      <c r="I1172" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1173">
+      <c r="A1173" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1173" t="inlineStr">
+        <is>
+          <t>Pakar Usul RUU Perampasan Aset Diubah Jadi RUU Melindungi Aset</t>
+        </is>
+      </c>
+      <c r="C1173" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:51:51 +0700</t>
+        </is>
+      </c>
+      <c r="D1173" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1173" t="inlineStr">
+        <is>
+          <t>RUU Perampasan Aset berpotensi memberikan kewenangan besar kepada negara untuk mengambil alih hak milik pribadi.</t>
+        </is>
+      </c>
+      <c r="F1173" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1173" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267408/pakar-usul-ruu-perampasan-aset-diubah-jadi-ruu-melindungi-aset</t>
+        </is>
+      </c>
+      <c r="H1173" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/P0blfdNw0Xxs6u842ruS_IXQRUQ=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/8137362/original/092189600_1780989441-RUU_Polri.jpeg</t>
+        </is>
+      </c>
+      <c r="I1173" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1174">
+      <c r="A1174" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1174" t="inlineStr">
+        <is>
+          <t>Tantangan Hafalan Alquran Berhadiah Miras Dilaporkan ke Bareskrim</t>
+        </is>
+      </c>
+      <c r="C1174" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:36:19 +0700</t>
+        </is>
+      </c>
+      <c r="D1174" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1174" t="inlineStr">
+        <is>
+          <t>Kegiatan berupa challenge atau tantangan yang melibatkan Alquran dinilai bermasalah dari sisi etika dan moral.</t>
+        </is>
+      </c>
+      <c r="F1174" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1174" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267399/tantangan-hafalan-alquran-berhadiah-miras-dilaporkan-ke-bareskrim</t>
+        </is>
+      </c>
+      <c r="H1174" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/iHD_QgF-uP8FSa50xdyMeQkNYRU=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9321537/original/088033500_1786448173-IMG_2876.jpeg</t>
+        </is>
+      </c>
+      <c r="I1174" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1175">
+      <c r="A1175" t="inlineStr">
+        <is>
+          <t>Money</t>
+        </is>
+      </c>
+      <c r="B1175" t="inlineStr">
+        <is>
+          <t>Harga Minyak Mentah Melonjak 2 Persen Usai Kesepakatan Damai AS-Iran Kian Buntu</t>
+        </is>
+      </c>
+      <c r="C1175" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:42:23 +0700</t>
+        </is>
+      </c>
+      <c r="D1175" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E1175" t="inlineStr">
+        <is>
+          <t>Pada Senin kemarin, pemerintahan Trump memperpanjang penangguhan undang-undang pengiriman.</t>
+        </is>
+      </c>
+      <c r="F1175" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1175" t="inlineStr">
+        <is>
+          <t>https://money.kompas.com/read/2026/08/11/194216126/harga-minyak-mentah-melonjak-2-persen-usai-kesepakatan-damai-as-iran-kian</t>
+        </is>
+      </c>
+      <c r="H1175" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/eX6M2TeyVC73j-CvAId9vaXzdrA=/0x0:1496x997/1200x675/filters:watermark(data/photo/2026/01/30/697c815e7ef28.png,0,-0,1)/data/photo/2026/02/28/69a26f1c57fb7.jpg</t>
+        </is>
+      </c>
+      <c r="I1175" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1176">
+      <c r="A1176" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B1176" t="inlineStr">
+        <is>
+          <t>Gelombang Tinggi Terjang Pesisir Kebumen, Puluhan Warung dan Kios Rusak</t>
+        </is>
+      </c>
+      <c r="C1176" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:42:23 +0700</t>
+        </is>
+      </c>
+      <c r="D1176" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E1176" t="inlineStr">
+        <is>
+          <t>Berikut dampak gelombang tinggi di kawasan pesisir selatan Kabupaten Kebumen, Jawa Tengah, pada Selasa (11/8/2026).</t>
+        </is>
+      </c>
+      <c r="F1176" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1176" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/08/11/192102678/gelombang-tinggi-terjang-pesisir-kebumen-puluhan-warung-dan-kios-rusak</t>
+        </is>
+      </c>
+      <c r="H1176" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/jEQBgdw-vBS65LR6lKzvHD_J0oA=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/11/6a7b095514f9b.jpg</t>
+        </is>
+      </c>
+      <c r="I1176" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1177">
+      <c r="A1177" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B1177" t="inlineStr">
+        <is>
+          <t>Relawan Sound Horeg Temui Jokowi di Solo, Siap Kawal Gibran di Pilpres 2029</t>
+        </is>
+      </c>
+      <c r="C1177" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:42:23 +0700</t>
+        </is>
+      </c>
+      <c r="D1177" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E1177" t="inlineStr">
+        <is>
+          <t>'Arahan dari beliau suruh menunggu dulu. Arahannya begitu,' ungkapnya.</t>
+        </is>
+      </c>
+      <c r="F1177" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1177" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/08/11/190029878/relawan-sound-horeg-temui-jokowi-di-solo-siap-kawal-gibran-di-pilpres-2029</t>
+        </is>
+      </c>
+      <c r="H1177" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/nnUbOMKlD9faKR9GqE97AVjun5A=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/11/6a7b0a34d3f3f.jpg</t>
+        </is>
+      </c>
+      <c r="I1177" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I1088"/>
+  <autoFilter ref="A1:I1177"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-11 14:14 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-11.xlsx
+++ b/data/berita_2026-08-11.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1177</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1279</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1177"/>
+  <dimension ref="A1:I1279"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -55758,8 +55758,4802 @@
         </is>
       </c>
     </row>
+    <row r="1178">
+      <c r="A1178" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1178" t="inlineStr">
+        <is>
+          <t>Gamba Osaka dan CAHN lolos ke fase liga ACL Elite</t>
+        </is>
+      </c>
+      <c r="C1178" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:09:41 +0700</t>
+        </is>
+      </c>
+      <c r="D1178" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1178" t="inlineStr">
+        <is>
+          <t>Gamba Osaka dan Cong An Hanoi FC (CAHN) lolos ke fase liga AFC Champions League (ACL) Elite wilayah Timur setelah ...</t>
+        </is>
+      </c>
+      <c r="F1178" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1178" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689932/gamba-osaka-dan-cahn-lolos-ke-fase-liga-acl-elite</t>
+        </is>
+      </c>
+      <c r="H1178" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/image-39.jpg</t>
+        </is>
+      </c>
+      <c r="I1178" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1179">
+      <c r="A1179" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1179" t="inlineStr">
+        <is>
+          <t>Mentan percepat bantuan pompa dan sumur dangkal untuk petani di Gresik</t>
+        </is>
+      </c>
+      <c r="C1179" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:09:09 +0700</t>
+        </is>
+      </c>
+      <c r="D1179" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1179" t="inlineStr">
+        <is>
+          <t>Menteri Pertanian Andi Amran Sulaiman mempercepat penanganan kekeringan di Kabupaten Gresik, Jawa ...</t>
+        </is>
+      </c>
+      <c r="F1179" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1179" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689929/mentan-percepat-bantuan-pompa-dan-sumur-dangkal-untuk-petani-di-gresik</t>
+        </is>
+      </c>
+      <c r="H1179" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/WhatsApp-Image-2026-08-11-at-21.01.17.jpeg</t>
+        </is>
+      </c>
+      <c r="I1179" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1180">
+      <c r="A1180" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1180" t="inlineStr">
+        <is>
+          <t>Deltras FC datangkan dua pemain perkuat skuad di musim 2026/2027</t>
+        </is>
+      </c>
+      <c r="C1180" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:05:31 +0700</t>
+        </is>
+      </c>
+      <c r="D1180" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1180" t="inlineStr">
+        <is>
+          <t>Deltras FC Sidoarjo mendatangkan penjaga gawang Samuel Reimas dan gelandang senior Rizky Pellu untuk memperkuat ...</t>
+        </is>
+      </c>
+      <c r="F1180" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1180" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689925/deltras-fc-datangkan-dua-pemain-perkuat-skuad-di-musim-2026-2027</t>
+        </is>
+      </c>
+      <c r="H1180" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/ANTARA-2026-08-11T163721.534.jpg.jpeg</t>
+        </is>
+      </c>
+      <c r="I1180" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1181">
+      <c r="A1181" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1181" t="inlineStr">
+        <is>
+          <t>Petugas berjibaku padamkan kebakaran lahan di Kertapati Palembang</t>
+        </is>
+      </c>
+      <c r="C1181" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:05:09 +0700</t>
+        </is>
+      </c>
+      <c r="D1181" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1181" t="inlineStr">
+        <is>
+          <t>Api membakar lahan di Karya Jaya, Kecamatan Kertapati, Palembang, Sumatera Selatan.</t>
+        </is>
+      </c>
+      <c r="F1181" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1181" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5689924/petugas-berjibaku-padamkan-kebakaran-lahan-di-kertapati-palembang</t>
+        </is>
+      </c>
+      <c r="H1181" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/Upaya-pemadaman-kebakaran-lahan-di-Kertapati-Palembang-110826-Lmo-5.jpg</t>
+        </is>
+      </c>
+      <c r="I1181" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1182">
+      <c r="A1182" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1182" t="inlineStr">
+        <is>
+          <t>Manggala Agni masih berjibaku padamkan karhutla di Rohil dan Bengkalis</t>
+        </is>
+      </c>
+      <c r="C1182" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:04:45 +0700</t>
+        </is>
+      </c>
+      <c r="D1182" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1182" t="inlineStr">
+        <is>
+          <t>Manggala Agni Daerah Operasi Dumai, Provinsi Riau, masih berjibaku memadamkan kebakaran hutan dan lahan (karhutla) ...</t>
+        </is>
+      </c>
+      <c r="F1182" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1182" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689923/manggala-agni-masih-berjibaku-padamkan-karhutla-di-rohil-dan-bengkalis</t>
+        </is>
+      </c>
+      <c r="H1182" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1000705378.jpg</t>
+        </is>
+      </c>
+      <c r="I1182" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1183">
+      <c r="A1183" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1183" t="inlineStr">
+        <is>
+          <t>Menkop mendorong Agrinas bangun ekosistem sawit seperti Felda Malaysia</t>
+        </is>
+      </c>
+      <c r="C1183" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:03:30 +0700</t>
+        </is>
+      </c>
+      <c r="D1183" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1183" t="inlineStr">
+        <is>
+          <t>Menteri Koperasi (Menkop) Ferry Juliantono mendorong PT Agrinas Palma Nusantara (Persero) mengembangkan ekosistem ...</t>
+        </is>
+      </c>
+      <c r="F1183" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1183" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689920/menkop-mendorong-agrinas-bangun-ekosistem-sawit-seperti-felda-malaysia</t>
+        </is>
+      </c>
+      <c r="H1183" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/tempImageRyzPec.jpg</t>
+        </is>
+      </c>
+      <c r="I1183" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1184">
+      <c r="A1184" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1184" t="inlineStr">
+        <is>
+          <t>KPK ungkap konstruksi korupsi kuota Haji, negara rugi Rp622 mililar</t>
+        </is>
+      </c>
+      <c r="C1184" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:01:27 +0700</t>
+        </is>
+      </c>
+      <c r="D1184" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1184" t="inlineStr">
+        <is>
+          <t>ANTARA - Komisi Pemberantasan Korupsi (KPK) membeberkan konstruksi dugaan tindak pidana korupsi pengalokasian kuota ...</t>
+        </is>
+      </c>
+      <c r="F1184" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1184" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5689895/kpk-ungkap-konstruksi-korupsi-kuota-haji-negara-rugi-rp622-mililar</t>
+        </is>
+      </c>
+      <c r="H1184" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KPK-UNGKAP-KONSTRUKSI-KORUPSI-KUOTA-HAJI-KERUGIAN-NEGARA-RP622-M.jpg</t>
+        </is>
+      </c>
+      <c r="I1184" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1185">
+      <c r="A1185" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1185" t="inlineStr">
+        <is>
+          <t>Kementan optimalkan rumah pompa untuk 600 hektare sawah di Lamongan</t>
+        </is>
+      </c>
+      <c r="C1185" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:58:38 +0700</t>
+        </is>
+      </c>
+      <c r="D1185" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1185" t="inlineStr">
+        <is>
+          <t>Kementerian Pertanian mengoptimalkan penggunaan rumah pompa di salah satu lokasi di Kabupaten Lamongan yang ...</t>
+        </is>
+      </c>
+      <c r="F1185" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1185" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689915/kementan-optimalkan-rumah-pompa-untuk-600-hektare-sawah-di-lamongan</t>
+        </is>
+      </c>
+      <c r="H1185" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/WhatsApp-Image-2026-08-11-at-20.27.36.jpeg</t>
+        </is>
+      </c>
+      <c r="I1185" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1186">
+      <c r="A1186" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1186" t="inlineStr">
+        <is>
+          <t>Jaksa sebut Yaqut siapkan 1 juta dolar AS pengaruhi Pansus Haji</t>
+        </is>
+      </c>
+      <c r="C1186" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:58:25 +0700</t>
+        </is>
+      </c>
+      <c r="D1186" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1186" t="inlineStr">
+        <is>
+          <t>Jaksa Penuntut Umum Komisi Pemberantasan Korupsi (KPK) menyebut mantan Menteri Agama Yaqut Cholil Qoumas diduga ...</t>
+        </is>
+      </c>
+      <c r="F1186" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1186" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689912/jaksa-sebut-yaqut-siapkan-1-juta-dolar-as-pengaruhi-pansus-haji</t>
+        </is>
+      </c>
+      <c r="H1186" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/yaqut-cholil-didakwa-rugikan-negara-ratusan-miliar-2838961.jpg</t>
+        </is>
+      </c>
+      <c r="I1186" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1187">
+      <c r="A1187" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1187" t="inlineStr">
+        <is>
+          <t>Zero ODOL mulai 2027, Kakorlantas ingatkan distribusi harus lancar</t>
+        </is>
+      </c>
+      <c r="C1187" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:58:15 +0700</t>
+        </is>
+      </c>
+      <c r="D1187" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1187" t="inlineStr">
+        <is>
+          <t>Kakorlantas Polri Irjen Pol. Wibowo mengingatkan jajaran bahwa distribusi barang maupun bahan pokok harus tetap lancar ...</t>
+        </is>
+      </c>
+      <c r="F1187" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1187" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689911/zero-odol-mulai-2027-kakorlantas-ingatkan-distribusi-harus-lancar</t>
+        </is>
+      </c>
+      <c r="H1187" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1000087748.jpg</t>
+        </is>
+      </c>
+      <c r="I1187" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1188">
+      <c r="A1188" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1188" t="inlineStr">
+        <is>
+          <t>OJK sebut pengembangan UMKM dilakukan dengan pendekatan lebih sistemik</t>
+        </is>
+      </c>
+      <c r="C1188" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:58:12 +0700</t>
+        </is>
+      </c>
+      <c r="D1188" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1188" t="inlineStr">
+        <is>
+          <t>Kepala Eksekutif Pengawas Perbankan Otoritas Jasa Keuangan (OJK) Dian Ediana Rae mengatakan pengembangan usaha mikro ...</t>
+        </is>
+      </c>
+      <c r="F1188" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1188" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689908/ojk-sebut-pengembangan-umkm-dilakukan-dengan-pendekatan-lebih-sistemik</t>
+        </is>
+      </c>
+      <c r="H1188" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/posalia-sulteng-digifest-2026-2839153.jpeg</t>
+        </is>
+      </c>
+      <c r="I1188" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1189">
+      <c r="A1189" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1189" t="inlineStr">
+        <is>
+          <t>Topan Chan-hom terjang Jepang, Tokyo siaga banjir</t>
+        </is>
+      </c>
+      <c r="C1189" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:57:47 +0700</t>
+        </is>
+      </c>
+      <c r="D1189" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1189" t="inlineStr">
+        <is>
+          <t>Topan Chan-hom menerjang wilayah daratan Kanto di Jepang timur, yang juga mencakup kawasan Tokyo, pada ...</t>
+        </is>
+      </c>
+      <c r="F1189" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1189" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689905/topan-chan-hom-terjang-jepang-tokyo-siaga-banjir</t>
+        </is>
+      </c>
+      <c r="H1189" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2023/08/10/2023-08-10T000000Z_2137806987_MT1YOMIUR000TGJLC3_RTRMADP_3_TYPHOON-NO-6-KHANUN-STRAYS-IN-JAPAN.jpg</t>
+        </is>
+      </c>
+      <c r="I1189" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1190">
+      <c r="A1190" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1190" t="inlineStr">
+        <is>
+          <t>BNPB targetkan dua titik karhutla Bromo bisa padam pekan ini</t>
+        </is>
+      </c>
+      <c r="C1190" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:53:09 +0700</t>
+        </is>
+      </c>
+      <c r="D1190" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1190" t="inlineStr">
+        <is>
+          <t>Badan Nasional Penanggulangan Bencana (BNPB) menargetkan dua titik api yang masih belum padam di kebakaran hutan dan ...</t>
+        </is>
+      </c>
+      <c r="F1190" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1190" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689904/bnpb-targetkan-dua-titik-karhutla-bromo-bisa-padam-pekan-ini</t>
+        </is>
+      </c>
+      <c r="H1190" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/WhatsApp-Image-2026-08-11-at-20.32.22.jpeg</t>
+        </is>
+      </c>
+      <c r="I1190" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1191">
+      <c r="A1191" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1191" t="inlineStr">
+        <is>
+          <t>Juventus tutup pramusim di Australia dengan kemenangan</t>
+        </is>
+      </c>
+      <c r="C1191" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:50:46 +0700</t>
+        </is>
+      </c>
+      <c r="D1191" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1191" t="inlineStr">
+        <is>
+          <t>Juventus menutup laga pramusim di Australia dengan kemenangan 2-0 atas sesama klub asal Italia Palermo di ...</t>
+        </is>
+      </c>
+      <c r="F1191" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1191" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689903/juventus-tutup-pramusim-di-australia-dengan-kemenangan</t>
+        </is>
+      </c>
+      <c r="H1191" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/image-38.jpg</t>
+        </is>
+      </c>
+      <c r="I1191" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1192">
+      <c r="A1192" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1192" t="inlineStr">
+        <is>
+          <t>Suriah kecam Kolombia akui "kedaulatan Israel" di Dataran Tinggi Golan</t>
+        </is>
+      </c>
+      <c r="C1192" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:50:22 +0700</t>
+        </is>
+      </c>
+      <c r="D1192" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1192" t="inlineStr">
+        <is>
+          <t>Suriah dengan tegas mengecam pengakuan Kolombia yang mengakui "kedaulatan Israel" di Dataran Tinggi ...</t>
+        </is>
+      </c>
+      <c r="F1192" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1192" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689899/suriah-kecam-kolombia-akui-kedaulatan-israel-di-dataran-tinggi-golan</t>
+        </is>
+      </c>
+      <c r="H1192" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/12/03/Golan.jpg</t>
+        </is>
+      </c>
+      <c r="I1192" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1193">
+      <c r="A1193" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1193" t="inlineStr">
+        <is>
+          <t>BPBD catat 1.077 kejadian karhutla di Sumsel hingga Agustus 2026</t>
+        </is>
+      </c>
+      <c r="C1193" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:50:18 +0700</t>
+        </is>
+      </c>
+      <c r="D1193" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1193" t="inlineStr">
+        <is>
+          <t>ANTARA - Eskalasi kebakaran hutan dan lahan atau karhutla di Sumatera Selatan terus meningkat seiring memasuki puncak ...</t>
+        </is>
+      </c>
+      <c r="F1193" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1193" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5689693/bpbd-catat-1077-kejadian-karhutla-di-sumsel-hingga-agustus-2026</t>
+        </is>
+      </c>
+      <c r="H1193" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/SANS_BPBD-CATAT-1.077-KEJADIAN-KARHUTLA-DI-SUMSEL-HINGGA-AGUSTUS-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I1193" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1194">
+      <c r="A1194" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1194" t="inlineStr">
+        <is>
+          <t>Hanura usul kursi pertama diberikan caleg nomor urut 1</t>
+        </is>
+      </c>
+      <c r="C1194" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:48:48 +0700</t>
+        </is>
+      </c>
+      <c r="D1194" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1194" t="inlineStr">
+        <is>
+          <t>Partai Hanura mengusulkan sistem pemilu legislatif dengan mekanisme kombinasi proporsional tertutup dan terbuka, yakni ...</t>
+        </is>
+      </c>
+      <c r="F1194" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1194" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689891/hanura-usul-kursi-pertama-diberikan-caleg-nomor-urut-1</t>
+        </is>
+      </c>
+      <c r="H1194" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1000583793.jpg</t>
+        </is>
+      </c>
+      <c r="I1194" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1195">
+      <c r="A1195" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1195" t="inlineStr">
+        <is>
+          <t>AUM BNI Private tercatat tumbuh 21 persen hingga kuartal II 2026</t>
+        </is>
+      </c>
+      <c r="C1195" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:48:39 +0700</t>
+        </is>
+      </c>
+      <c r="D1195" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1195" t="inlineStr">
+        <is>
+          <t>PT Bank Negara Indonesia (Persero) Tbk atau BNI mencatat aset kelolaan (asset under management/AUM) BNI Private tumbuh ...</t>
+        </is>
+      </c>
+      <c r="F1195" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1195" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689888/aum-bni-private-tercatat-tumbuh-21-persen-hingga-kuartal-ii-2026</t>
+        </is>
+      </c>
+      <c r="H1195" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1000675745.jpg</t>
+        </is>
+      </c>
+      <c r="I1195" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1196">
+      <c r="A1196" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1196" t="inlineStr">
+        <is>
+          <t>Pemkab Pasuruan kerahkan 3 tangki air bantu padamkan kebakaran Bromo</t>
+        </is>
+      </c>
+      <c r="C1196" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:48:28 +0700</t>
+        </is>
+      </c>
+      <c r="D1196" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1196" t="inlineStr">
+        <is>
+          <t>Pemerintah Kabupaten (Pemkab) Pasuruan, Jawa Timur, mengerahkan tiga kendaraan tangki air dan satu kendaraan ...</t>
+        </is>
+      </c>
+      <c r="F1196" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1196" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689884/pemkab-pasuruan-kerahkan-3-tangki-air-bantu-padamkan-kebakaran-bromo</t>
+        </is>
+      </c>
+      <c r="H1196" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/ANTARA-2026-08-11T194712.702.jpg.jpeg</t>
+        </is>
+      </c>
+      <c r="I1196" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1197">
+      <c r="A1197" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1197" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya tangkap pelaku pembunuhan-pemerkosaan di Tangerang</t>
+        </is>
+      </c>
+      <c r="C1197" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:48:11 +0700</t>
+        </is>
+      </c>
+      <c r="D1197" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1197" t="inlineStr">
+        <is>
+          <t>Ditreskrimum Polda Metro Jaya membekuk seorang pelaku pembunuhan dan pemerkosaan yang beraksi di sebuah rumah kontrakan ...</t>
+        </is>
+      </c>
+      <c r="F1197" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1197" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689883/polda-metro-jaya-tangkap-pelaku-pembunuhan-pemerkosaan-di-tangerang</t>
+        </is>
+      </c>
+      <c r="H1197" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1000913631.jpg</t>
+        </is>
+      </c>
+      <c r="I1197" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1198">
+      <c r="A1198" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1198" t="inlineStr">
+        <is>
+          <t>Menhan RI dan Wamenhan AS bahas penguatan kerja sama pertahanan</t>
+        </is>
+      </c>
+      <c r="C1198" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:43:55 +0700</t>
+        </is>
+      </c>
+      <c r="D1198" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1198" t="inlineStr">
+        <is>
+          <t>Menteri Pertahanan (Menhan) RI Sjafrie Sjamsoeddin membahas rencana penguatan kerja sama bidang pertahanan dengan Wakil ...</t>
+        </is>
+      </c>
+      <c r="F1198" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1198" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689879/menhan-ri-dan-wamenhan-as-bahas-penguatan-kerja-sama-pertahanan</t>
+        </is>
+      </c>
+      <c r="H1198" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1001569954.jpg</t>
+        </is>
+      </c>
+      <c r="I1198" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1199">
+      <c r="A1199" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1199" t="inlineStr">
+        <is>
+          <t>Karhutla Palangka Raya meluas, pemkot perpanjang status darurat</t>
+        </is>
+      </c>
+      <c r="C1199" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:42:49 +0700</t>
+        </is>
+      </c>
+      <c r="D1199" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1199" t="inlineStr">
+        <is>
+          <t>ANTARA - Luas lahan terdampak kebakaran hutan dan lahan (karhutla) di Kota Palangka Raya, Kalimantan Tengah, terus ...</t>
+        </is>
+      </c>
+      <c r="F1199" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1199" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5689537/karhutla-palangka-raya-meluas-pemkot-perpanjang-status-darurat</t>
+        </is>
+      </c>
+      <c r="H1199" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KARHUTLA-PALANGKA-RAYA-MELUAS-PEMKOT-PERPANJANG-STATUS-DARURAT.jpg</t>
+        </is>
+      </c>
+      <c r="I1199" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1200">
+      <c r="A1200" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1200" t="inlineStr">
+        <is>
+          <t>PBB: Hampir 5.000 rumah, 24 faskes rusak akibat gempa Kolombia</t>
+        </is>
+      </c>
+      <c r="C1200" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:40:55 +0700</t>
+        </is>
+      </c>
+      <c r="D1200" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1200" t="inlineStr">
+        <is>
+          <t>Gempa bumi dahsyat bermagnitudo 7,4 yang mengguncang Kolombia pada Senin (10/8) merusak hampir 5.000 rumah dan 24 ...</t>
+        </is>
+      </c>
+      <c r="F1200" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1200" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689877/pbb-hampir-5000-rumah-24-faskes-rusak-akibat-gempa-kolombia</t>
+        </is>
+      </c>
+      <c r="H1200" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/Reruntuhan-gedung-akibat-gempa-Kolombia.jpg</t>
+        </is>
+      </c>
+      <c r="I1200" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1201">
+      <c r="A1201" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1201" t="inlineStr">
+        <is>
+          <t>Menko Airlangga sebut calon Gubernur PFII sudah ada dari pemerintah</t>
+        </is>
+      </c>
+      <c r="C1201" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:40:43 +0700</t>
+        </is>
+      </c>
+      <c r="D1201" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1201" t="inlineStr">
+        <is>
+          <t>Menteri Koordinator Bidang Perekonomian Airlangga Hartarto menyatakan calon Gubernur Pusat Finansial Internasional ...</t>
+        </is>
+      </c>
+      <c r="F1201" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1201" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689873/menko-airlangga-sebut-calon-gubernur-pfii-sudah-ada-dari-pemerintah</t>
+        </is>
+      </c>
+      <c r="H1201" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/4A66028E-AC15-4B2B-BF63-6F00D047171E.jpeg</t>
+        </is>
+      </c>
+      <c r="I1201" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1202">
+      <c r="A1202" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1202" t="inlineStr">
+        <is>
+          <t>Pemprov Kalsel dorong pesantren adaptif tanpa kehilangan jati diri</t>
+        </is>
+      </c>
+      <c r="C1202" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:40:14 +0700</t>
+        </is>
+      </c>
+      <c r="D1202" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1202" t="inlineStr">
+        <is>
+          <t>Pemerintah Provinsi (Pemprov) Kalimantan Selatan (Kalsel) mendorong pesantren mengembangkan pendekatan pendidikan yang ...</t>
+        </is>
+      </c>
+      <c r="F1202" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1202" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689869/pemprov-kalsel-dorong-pesantren-adaptif-tanpa-kehilangan-jati-diri</t>
+        </is>
+      </c>
+      <c r="H1202" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG_1873.jpeg</t>
+        </is>
+      </c>
+      <c r="I1202" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1203">
+      <c r="A1203" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1203" t="inlineStr">
+        <is>
+          <t>Pemkot Semarang prioritaskan skrining kesehatan bagi perempuan</t>
+        </is>
+      </c>
+      <c r="C1203" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:39:07 +0700</t>
+        </is>
+      </c>
+      <c r="D1203" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1203" t="inlineStr">
+        <is>
+          <t>ANTARA - Pemerintah Kota Semarang menggelar layanan Cek Kesehatan Gratis (CKG) di Balai Kota Semarang pada 10-12 ...</t>
+        </is>
+      </c>
+      <c r="F1203" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1203" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5689747/pemkot-semarang-prioritaskan-skrining-kesehatan-bagi-perempuan</t>
+        </is>
+      </c>
+      <c r="H1203" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/SANS_PEMKOT-SEMARANG-PRIORITASKAN-SKRINING-KESEHATAN-BAGI-PEREMPUAN_1.jpg</t>
+        </is>
+      </c>
+      <c r="I1203" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1204">
+      <c r="A1204" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1204" t="inlineStr">
+        <is>
+          <t>Pemerintah berupaya tingkatkan keselamatan wisata bahari</t>
+        </is>
+      </c>
+      <c r="C1204" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:39:06 +0700</t>
+        </is>
+      </c>
+      <c r="D1204" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1204" t="inlineStr">
+        <is>
+          <t>Kementerian Pariwisata menjalankan program pelatihan bagi sumber daya manusia pariwisata dalam ...</t>
+        </is>
+      </c>
+      <c r="F1204" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1204" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689868/pemerintah-berupaya-tingkatkan-keselamatan-wisata-bahari</t>
+        </is>
+      </c>
+      <c r="H1204" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/WhatsApp-Image-2026-08-11-at-14.10.27.jpeg</t>
+        </is>
+      </c>
+      <c r="I1204" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1205">
+      <c r="A1205" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1205" t="inlineStr">
+        <is>
+          <t>Peneliti ingatkan ancaman gelombang panas laut bagi kesehatan manusia</t>
+        </is>
+      </c>
+      <c r="C1205" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:38:56 +0700</t>
+        </is>
+      </c>
+      <c r="D1205" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1205" t="inlineStr">
+        <is>
+          <t>Gelombang panas laut (marine heatwaves) menimbulkan ancaman yang semakin besar terhadap kesehatan manusia, dengan ...</t>
+        </is>
+      </c>
+      <c r="F1205" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1205" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689864/peneliti-ingatkan-ancaman-gelombang-panas-laut-bagi-kesehatan-manusia</t>
+        </is>
+      </c>
+      <c r="H1205" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/CjkinzN000023_20260811_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I1205" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1206">
+      <c r="A1206" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1206" t="inlineStr">
+        <is>
+          <t>Liga Putri Indonesia mulai kick off Oktober 2026, Erick: Kita bangkit</t>
+        </is>
+      </c>
+      <c r="C1206" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:36:53 +0700</t>
+        </is>
+      </c>
+      <c r="D1206" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1206" t="inlineStr">
+        <is>
+          <t>ANTARA - Liga Putri Indonesia (Indonesia Women's League) 2026/2027 resmi melaksanakan kick off pada 17 ...</t>
+        </is>
+      </c>
+      <c r="F1206" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1206" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5689621/liga-putri-indonesia-mulai-kick-off-oktober-2026-erick-kita-bangkit</t>
+        </is>
+      </c>
+      <c r="H1206" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Sequence-13.13_46_42_02.Still488.jpg</t>
+        </is>
+      </c>
+      <c r="I1206" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1207">
+      <c r="A1207" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1207" t="inlineStr">
+        <is>
+          <t>ATR/BPN kuatkan integritas ASN melalui pendidikan antikorupsi</t>
+        </is>
+      </c>
+      <c r="C1207" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:36:43 +0700</t>
+        </is>
+      </c>
+      <c r="D1207" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1207" t="inlineStr">
+        <is>
+          <t>Kementerian Agraria dan Tata Ruang/Badan Pertanahan Nasional (ATR/BPN) bekerja sama dengan Komisi Pemberantasan Korupsi ...</t>
+        </is>
+      </c>
+      <c r="F1207" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1207" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689861/atr-bpn-kuatkan-integritas-asn-melalui-pendidikan-antikorupsi</t>
+        </is>
+      </c>
+      <c r="H1207" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG_20260811_200228.jpg</t>
+        </is>
+      </c>
+      <c r="I1207" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1208">
+      <c r="A1208" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1208" t="inlineStr">
+        <is>
+          <t>Menag tandai pembangunan baru MIN 5 Pidie Jaya di atas tanah hibah</t>
+        </is>
+      </c>
+      <c r="C1208" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:36:24 +0700</t>
+        </is>
+      </c>
+      <c r="D1208" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1208" t="inlineStr">
+        <is>
+          <t>Menteri Agama (Menag) Nasaruddin Umar menandai pembangunan baru Madrasah Ibtidaiyah Negeri (MIN) 5 Pidie Jaya, Aceh ...</t>
+        </is>
+      </c>
+      <c r="F1208" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1208" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689857/menag-tandai-pembangunan-baru-min-5-pidie-jaya-di-atas-tanah-hibah</t>
+        </is>
+      </c>
+      <c r="H1208" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG-20260811-WA0012.jpg</t>
+        </is>
+      </c>
+      <c r="I1208" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1209">
+      <c r="A1209" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1209" t="inlineStr">
+        <is>
+          <t>BNN gandeng tiga kementerian siapkan penyintas masuk dunia kerja</t>
+        </is>
+      </c>
+      <c r="C1209" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:36:14 +0700</t>
+        </is>
+      </c>
+      <c r="D1209" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1209" t="inlineStr">
+        <is>
+          <t>Badan Narkotika Nasional (BNN) bersama tiga kementerian mengintegrasikan penanganan penyintas penyalahgunaan narkotika ...</t>
+        </is>
+      </c>
+      <c r="F1209" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1209" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689856/bnn-gandeng-tiga-kementerian-siapkan-penyintas-masuk-dunia-kerja</t>
+        </is>
+      </c>
+      <c r="H1209" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1003330639.jpg</t>
+        </is>
+      </c>
+      <c r="I1209" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1210">
+      <c r="A1210" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1210" t="inlineStr">
+        <is>
+          <t>BNPB: Pemadaman api di Bromo andalkan pasokan air Danau Ranu Pani</t>
+        </is>
+      </c>
+      <c r="C1210" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:35:20 +0700</t>
+        </is>
+      </c>
+      <c r="D1210" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1210" t="inlineStr">
+        <is>
+          <t>Badan Nasional Penanggulangan Bencana (BNPB) menyatakan tidak ada sumber air lain yang bisa dimanfaatkan selain ...</t>
+        </is>
+      </c>
+      <c r="F1210" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1210" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689852/bnpb-pemadaman-api-di-bromo-andalkan-pasokan-air-danau-ranu-pani</t>
+        </is>
+      </c>
+      <c r="H1210" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG-20260811-WA0029_1.jpg</t>
+        </is>
+      </c>
+      <c r="I1210" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1211" t="inlineStr">
+        <is>
+          <t>Korban tewas gempa Kolombia bertambah jadi 224 orang</t>
+        </is>
+      </c>
+      <c r="C1211" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:34:09 +0700</t>
+        </is>
+      </c>
+      <c r="D1211" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1211" t="inlineStr">
+        <is>
+          <t>Jumlah korban tewas akibat gempa bumi yang mengguncang Kolombia pada Senin (10/8) bertambah menjadi 224 orang, seperti ...</t>
+        </is>
+      </c>
+      <c r="F1211" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1211" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689851/korban-tewas-gempa-kolombia-bertambah-jadi-224-orang</t>
+        </is>
+      </c>
+      <c r="H1211" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/AT_LEAST_18_KILLED_AS_MAGNITUDE_74_EARTHQUAKE_HITS_COLOMBIA.jpg</t>
+        </is>
+      </c>
+      <c r="I1211" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1212" t="inlineStr">
+        <is>
+          <t>WEGE-RDM KSO Resmi Mulai Pembangunan Gedung Poliklinik RSUD Temanggung Senilai Rp 155,4 Miliar</t>
+        </is>
+      </c>
+      <c r="C1212" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:33:36 +0700</t>
+        </is>
+      </c>
+      <c r="D1212" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1212" t="inlineStr">
+        <is>
+          <t>Jakarta (ANTARA) – PT Wijaya Karya Bangunan Gedung Tbk (WEGE) yang tergabung dalam WEGE-RDM KSO secara resmi ...</t>
+        </is>
+      </c>
+      <c r="F1212" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1212" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689849/wege-rdm-kso-resmi-mulai-pembangunan-gedung-poliklinik-rsud-temanggung-senilai-rp-1554-miliar</t>
+        </is>
+      </c>
+      <c r="H1212" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/WIKA-Ground-Breaking.jpg</t>
+        </is>
+      </c>
+      <c r="I1212" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1213">
+      <c r="A1213" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1213" t="inlineStr">
+        <is>
+          <t>Trump berganti pesawat setelah kunjungan ke Turkiye</t>
+        </is>
+      </c>
+      <c r="C1213" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:32:57 +0700</t>
+        </is>
+      </c>
+      <c r="D1213" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1213" t="inlineStr">
+        <is>
+          <t>Presiden Amerika Serikat (AS) Donald Trump secara diam-diam berganti pesawat saat bertolak dari Turkiye setelah ...</t>
+        </is>
+      </c>
+      <c r="F1213" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1213" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689845/trump-berganti-pesawat-setelah-kunjungan-ke-turkiye</t>
+        </is>
+      </c>
+      <c r="H1213" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/CjkinzN000025_20260811_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I1213" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1214" t="inlineStr">
+        <is>
+          <t>Bakamla RI gelar latihan gabungan dengan Malaysia dan Singapura</t>
+        </is>
+      </c>
+      <c r="C1214" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:31:08 +0700</t>
+        </is>
+      </c>
+      <c r="D1214" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1214" t="inlineStr">
+        <is>
+          <t>ANTARA - Badan Keamanan Laut Republik Indonesia  (Bakamla RI) menggelar latihan gabungan bersama ...</t>
+        </is>
+      </c>
+      <c r="F1214" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1214" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5689577/bakamla-ri-gelar-latihan-gabungan-dengan-malaysia-dan-singapura</t>
+        </is>
+      </c>
+      <c r="H1214" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/BAKAMLA-RI-GELAR-LATIHAN-GABUNGAN-DENGAN-MALAYSIA-DAN-SINGAPURA.jpg</t>
+        </is>
+      </c>
+      <c r="I1214" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1215" t="inlineStr">
+        <is>
+          <t>Pegadaian perkuat literasi keuangan pekerja informal di Tangerang</t>
+        </is>
+      </c>
+      <c r="C1215" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:30:33 +0700</t>
+        </is>
+      </c>
+      <c r="D1215" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1215" t="inlineStr">
+        <is>
+          <t>PT Pegadaian memperkuat literasi dan inklusi keuangan pekerja sektor informal melalui edukasi pengelolaan keuangan bagi ...</t>
+        </is>
+      </c>
+      <c r="F1215" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1215" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689844/pegadaian-perkuat-literasi-keuangan-pekerja-informal-di-tangerang</t>
+        </is>
+      </c>
+      <c r="H1215" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1000179867.jpg</t>
+        </is>
+      </c>
+      <c r="I1215" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1216" t="inlineStr">
+        <is>
+          <t>Pemkot Jakbar perketat pengawasan "pak ogah" di exit tol Rawa Buaya</t>
+        </is>
+      </c>
+      <c r="C1216" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:28:57 +0700</t>
+        </is>
+      </c>
+      <c r="D1216" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1216" t="inlineStr">
+        <is>
+          <t>Petugas gabungan Satpol PP dan Suku Dinas Perhubungan Jakarta Barat meningkatkan pengawasan terhadap pengatur lalu ...</t>
+        </is>
+      </c>
+      <c r="F1216" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1216" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689841/pemkot-jakbar-perketat-pengawasan-pak-ogah-di-exit-tol-rawa-buaya</t>
+        </is>
+      </c>
+      <c r="H1216" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG_20260811_200925.v1.jpg</t>
+        </is>
+      </c>
+      <c r="I1216" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1217">
+      <c r="A1217" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1217" t="inlineStr">
+        <is>
+          <t>Pengacara Yaqut pertanyakan negara rugi Rp622 miliar kasus kuota haji</t>
+        </is>
+      </c>
+      <c r="C1217" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:26:30 +0700</t>
+        </is>
+      </c>
+      <c r="D1217" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1217" t="inlineStr">
+        <is>
+          <t>ANTARA - Penasihat hukum mantan Menteri Agama Yaqut Cholil Qoumas, Mellisa Anggraini, di Pengadilan Negara Jakarta ...</t>
+        </is>
+      </c>
+      <c r="F1217" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1217" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5689617/pengacara-yaqut-pertanyakan-negara-rugi-rp622-miliar-kasus-kuota-haji</t>
+        </is>
+      </c>
+      <c r="H1217" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/PENGACARA-YAQUT-PERTANYAKAN-NEGARA-RUGI-RP622-MILIAR-KASUS-KUOTA-HAJI.jpg</t>
+        </is>
+      </c>
+      <c r="I1217" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1218">
+      <c r="A1218" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1218" t="inlineStr">
+        <is>
+          <t>Kemenpora ajak warga mendaftar Merdeka Run 2026 dibuka 12 Agustus</t>
+        </is>
+      </c>
+      <c r="C1218" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:25:36 +0700</t>
+        </is>
+      </c>
+      <c r="D1218" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1218" t="inlineStr">
+        <is>
+          <t>Kementerian Pemuda dan Olahraga (Kemenpora) mengajak semua elemen warga mengikuti Merdeka Run 2026 yang ...</t>
+        </is>
+      </c>
+      <c r="F1218" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1218" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689840/kemenpora-ajak-warga-mendaftar-merdeka-run-2026-dibuka-12-agustus</t>
+        </is>
+      </c>
+      <c r="H1218" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2023/10/26/Resize_20231026_225833_3699.jpg</t>
+        </is>
+      </c>
+      <c r="I1218" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1219">
+      <c r="A1219" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1219" t="inlineStr">
+        <is>
+          <t>Wamendagri soroti kesiapan APBD tangani kekerasan perempuan-anak</t>
+        </is>
+      </c>
+      <c r="C1219" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:24:52 +0700</t>
+        </is>
+      </c>
+      <c r="D1219" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1219" t="inlineStr">
+        <is>
+          <t>Wakil Menteri Dalam Negeri Bima Arya Sugiarto meminta pemerintah daerah untuk memperkuat sistem pelayanan terpadu dalam ...</t>
+        </is>
+      </c>
+      <c r="F1219" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1219" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689839/wamendagri-soroti-kesiapan-apbd-tangani-kekerasan-perempuan-anak</t>
+        </is>
+      </c>
+      <c r="H1219" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/28/IMG_4925.jpeg</t>
+        </is>
+      </c>
+      <c r="I1219" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1220">
+      <c r="A1220" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1220" t="inlineStr">
+        <is>
+          <t>Pemko Banjarmasin bagikan 10.000 bendera, tumbuhkan nasionalisme warga</t>
+        </is>
+      </c>
+      <c r="C1220" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:20:32 +0700</t>
+        </is>
+      </c>
+      <c r="D1220" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1220" t="inlineStr">
+        <is>
+          <t>ANTARA - Guna Menyemarakkan Hari Ulang Tahun Ke-81 Kemerdekaan Republik Indonesia, Pemerintah Kota Banjarmasin ...</t>
+        </is>
+      </c>
+      <c r="F1220" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1220" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5689751/pemko-banjarmasin-bagikan-10000-bendera-tumbuhkan-nasionalisme-warga</t>
+        </is>
+      </c>
+      <c r="H1220" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Sequence-13.13_52_35_01.Still490.jpg</t>
+        </is>
+      </c>
+      <c r="I1220" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1221" t="inlineStr">
+        <is>
+          <t>Perpres Ojol masuk finalisasi, pemerintah lengkapi formula pola bisnis</t>
+        </is>
+      </c>
+      <c r="C1221" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:20:25 +0700</t>
+        </is>
+      </c>
+      <c r="D1221" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1221" t="inlineStr">
+        <is>
+          <t>ANTARA - Menteri Sekretaris Negara (Mensesneg) Prasetyo Hadi, Selasa (11/8), menyebut bahwa Perpres terkait Ojek Online ...</t>
+        </is>
+      </c>
+      <c r="F1221" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1221" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5689252/perpres-ojol-masuk-finalisasi-pemerintah-lengkapi-formula-pola-bisnis</t>
+        </is>
+      </c>
+      <c r="H1221" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/PERPRES-OJOL-MASUK-FINALISASI-PEMERINTAH-LENGKAPI-FORMULA-POLA-BISNIS.jpg</t>
+        </is>
+      </c>
+      <c r="I1221" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1222" t="inlineStr">
+        <is>
+          <t>BPK: SPKN 2026 jadi transformasi standar pemeriksaan sektor publik RI</t>
+        </is>
+      </c>
+      <c r="C1222" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:20:03 +0700</t>
+        </is>
+      </c>
+      <c r="D1222" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1222" t="inlineStr">
+        <is>
+          <t>Wakil Ketua Badan Pemeriksa Keuangan (BPK) Budi Prijono menyatakan Standar Pemeriksaan Keuangan Negara (SPKN) 2026 ...</t>
+        </is>
+      </c>
+      <c r="F1222" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1222" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689832/bpk-spkn-2026-jadi-transformasi-standar-pemeriksaan-sektor-publik-ri</t>
+        </is>
+      </c>
+      <c r="H1222" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/WhatsApp-Image-2026-08-06-at-15.29.02.jpeg</t>
+        </is>
+      </c>
+      <c r="I1222" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1223">
+      <c r="A1223" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1223" t="inlineStr">
+        <is>
+          <t>Megawati: Partai politik perlu riset dan sains</t>
+        </is>
+      </c>
+      <c r="C1223" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:19:23 +0700</t>
+        </is>
+      </c>
+      <c r="D1223" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1223" t="inlineStr">
+        <is>
+          <t>Ketua Umum DPP PDI Perjuangan Megawati Soekarnoputri menekankan pentingnya riset berbasis sains dalam tubuh partai ...</t>
+        </is>
+      </c>
+      <c r="F1223" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1223" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689829/megawati-partai-politik-perlu-riset-dan-sains</t>
+        </is>
+      </c>
+      <c r="H1223" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1000583723.jpg</t>
+        </is>
+      </c>
+      <c r="I1223" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1224">
+      <c r="A1224" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1224" t="inlineStr">
+        <is>
+          <t>Waspadai karhutla, Banjarmasin gelar apel penanggulangan bencana</t>
+        </is>
+      </c>
+      <c r="C1224" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:17:01 +0700</t>
+        </is>
+      </c>
+      <c r="D1224" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1224" t="inlineStr">
+        <is>
+          <t>ANTARA - Kepolisian Resor Kota Banjarmasin menggelar apel pasukan penanggulangan bencana kebakaran hutan dan lahan yang ...</t>
+        </is>
+      </c>
+      <c r="F1224" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1224" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5689729/waspadai-karhutla-banjarmasin-gelar-apel-penanggulangan-bencana</t>
+        </is>
+      </c>
+      <c r="H1224" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Sequence-13.13_48_48_24.Still489.jpg</t>
+        </is>
+      </c>
+      <c r="I1224" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1225">
+      <c r="A1225" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1225" t="inlineStr">
+        <is>
+          <t>BMKG: El Nino kuat picu Sumsel makin kering hingga September</t>
+        </is>
+      </c>
+      <c r="C1225" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:15:34 +0700</t>
+        </is>
+      </c>
+      <c r="D1225" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1225" t="inlineStr">
+        <is>
+          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) menyebut fenomena El Nino berstatus kuat menyebabkan kondisi ...</t>
+        </is>
+      </c>
+      <c r="F1225" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1225" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689827/bmkg-el-nino-kuat-picu-sumsel-makin-kering-hingga-september</t>
+        </is>
+      </c>
+      <c r="H1225" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/prediksi-puncak-musim-kemarau-di-sumatera-selatan-2835887.jpg</t>
+        </is>
+      </c>
+      <c r="I1225" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1226">
+      <c r="A1226" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1226" t="inlineStr">
+        <is>
+          <t>Pemkot Jakbar perkuat kerja sama lintas sektor turunkan stunting</t>
+        </is>
+      </c>
+      <c r="C1226" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:14:43 +0700</t>
+        </is>
+      </c>
+      <c r="D1226" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1226" t="inlineStr">
+        <is>
+          <t>Pemerintah Kota Jakarta Barat memperkuat kerja sama lintas sektor untuk intervensi percepatan penurunan kasus anak ...</t>
+        </is>
+      </c>
+      <c r="F1226" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1226" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689824/pemkot-jakbar-perkuat-kerja-sama-lintas-sektor-turunkan-stunting</t>
+        </is>
+      </c>
+      <c r="H1226" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/24/IMG_20260723_212803.v1.jpg</t>
+        </is>
+      </c>
+      <c r="I1226" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1227">
+      <c r="A1227" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1227" t="inlineStr">
+        <is>
+          <t>Polisi: situasi pascaricuh di Tabang Kukar telah kondusif</t>
+        </is>
+      </c>
+      <c r="C1227" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:13:26 +0700</t>
+        </is>
+      </c>
+      <c r="D1227" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1227" t="inlineStr">
+        <is>
+          <t>ANTARA - Kepolisian mengamankan situasi dan memastikan kondusivitas di wilayah Kecamatan Tabang, Kabupaten Kutai ...</t>
+        </is>
+      </c>
+      <c r="F1227" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1227" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5689172/polisi-situasi-pascaricuh-di-tabang-kukar-telah-kondusif</t>
+        </is>
+      </c>
+      <c r="H1227" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/POLISI-SITUASI-PASCARICUH-DI-TABANG-KUKAR-TELAH-KONDUSIF.jpg</t>
+        </is>
+      </c>
+      <c r="I1227" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1228">
+      <c r="A1228" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1228" t="inlineStr">
+        <is>
+          <t>Bamsoet Dorong Kampus Selaraskan Pendidikan dengan Kebutuhan Dunia Kerja</t>
+        </is>
+      </c>
+      <c r="C1228" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:02:15 +0700</t>
+        </is>
+      </c>
+      <c r="D1228" t="inlineStr">
+        <is>
+          <t>Moch. Prima Fauzi</t>
+        </is>
+      </c>
+      <c r="E1228" t="inlineStr">
+        <is>
+          <t>Bambang Soesatyo mengusulkan tiga program studi baru di UNPERBA untuk 2026, mendukung pendidikan tinggi yang relevan dengan kebutuhan industri.</t>
+        </is>
+      </c>
+      <c r="F1228" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1228" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614374/bamsoet-dorong-kampus-selaraskan-pendidikan-dengan-kebutuhan-dunia-kerja</t>
+        </is>
+      </c>
+      <c r="H1228" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/20/anggota-dpr-ri-bambang-soesatyo-1784547923074.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1228" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1229">
+      <c r="A1229" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1229" t="inlineStr">
+        <is>
+          <t>KPK Libatkan BPKP dalam Pemeriksaan Rudy Tanoe untuk Hitung Kerugian Negara</t>
+        </is>
+      </c>
+      <c r="C1229" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:57:43 +0700</t>
+        </is>
+      </c>
+      <c r="D1229" t="inlineStr">
+        <is>
+          <t>Adrial akbar</t>
+        </is>
+      </c>
+      <c r="E1229" t="inlineStr">
+        <is>
+          <t>KPK memeriksa Rudy Tanoe terkait dugaan korupsi bansos 2020. Pemeriksaan melibatkan BPKP untuk menghitung kerugian negara dalam pengadaan bantuan.</t>
+        </is>
+      </c>
+      <c r="F1229" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1229" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614371/kpk-libatkan-bpkp-dalam-pemeriksaan-rudy-tanoe-untuk-hitung-kerugian-negara</t>
+        </is>
+      </c>
+      <c r="H1229" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2021/03/02/gedung-baru-kpk-7_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1229" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1230">
+      <c r="A1230" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1230" t="inlineStr">
+        <is>
+          <t>Pria di Bogor Diikat di Tiang Usai Kepergok Curi Uang Kotak Amal Masjid</t>
+        </is>
+      </c>
+      <c r="C1230" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:48:41 +0700</t>
+        </is>
+      </c>
+      <c r="D1230" t="inlineStr">
+        <is>
+          <t>M Solihin</t>
+        </is>
+      </c>
+      <c r="E1230" t="inlineStr">
+        <is>
+          <t>Pria bernama Asmanto ditangkap setelah mencuri uang kotak amal masjid di Bogor. Ia pura-pura solat sebelum aksinya dan mengaku sudah dua kali melakukannya.</t>
+        </is>
+      </c>
+      <c r="F1230" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1230" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614351/pria-di-bogor-diikat-di-tiang-usai-kepergok-curi-uang-kotak-amal-masjid</t>
+        </is>
+      </c>
+      <c r="H1230" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/maling-kotak-amal-di-bogor-diikat-di-tiang-listrik-dok-istimewa-1786456096957_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1230" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1231">
+      <c r="A1231" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1231" t="inlineStr">
+        <is>
+          <t>Jatanras PMJ Tangkap Pelaku Pembunuhan dan Pemerkosaan di Tangerang</t>
+        </is>
+      </c>
+      <c r="C1231" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:43:59 +0700</t>
+        </is>
+      </c>
+      <c r="D1231" t="inlineStr">
+        <is>
+          <t>Zunita Putri</t>
+        </is>
+      </c>
+      <c r="E1231" t="inlineStr">
+        <is>
+          <t>Seorang wanita berinisial SNA (20) ditemukan tewas di kontrakan di Tangerang, diduga korban pembunuhan dan pemerkosaan. Pelaku ditangkap dalam 24 jam.</t>
+        </is>
+      </c>
+      <c r="F1231" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1231" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614346/jatanras-pmj-tangkap-pelaku-pembunuhan-dan-pemerkosaan-di-tangerang</t>
+        </is>
+      </c>
+      <c r="H1231" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/tkp-pembunuhan-dan-pemerkosaan-di-tangerang-1786455813903_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1231" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1232">
+      <c r="A1232" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1232" t="inlineStr">
+        <is>
+          <t>Uji Coba E-voting, Kemenkum Libatkan Pegawai Pilih Kakanwil Jatim</t>
+        </is>
+      </c>
+      <c r="C1232" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:36:19 +0700</t>
+        </is>
+      </c>
+      <c r="D1232" t="inlineStr">
+        <is>
+          <t>Angelina Vioni</t>
+        </is>
+      </c>
+      <c r="E1232" t="inlineStr">
+        <is>
+          <t>Kemenkum uji coba e-voting untuk pengisian jabatan, meningkatkan transparansi dan manajemen talenta. Langkah ini diharapkan memperkuat tata kelola birokrasi.</t>
+        </is>
+      </c>
+      <c r="F1232" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1232" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614341/uji-coba-e-voting-kemenkum-libatkan-pegawai-pilih-kakanwil-jatim</t>
+        </is>
+      </c>
+      <c r="H1232" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/kemenkum-1786455205202_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1232" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1233">
+      <c r="A1233" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1233" t="inlineStr">
+        <is>
+          <t>Menkop Dorong Hilirisasi Sawit Berbasis Koperasi untuk Sejahterakan Petani</t>
+        </is>
+      </c>
+      <c r="C1233" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:32:35 +0700</t>
+        </is>
+      </c>
+      <c r="D1233" t="inlineStr">
+        <is>
+          <t>Chayyara Zulghifary</t>
+        </is>
+      </c>
+      <c r="E1233" t="inlineStr">
+        <is>
+          <t>Program hilirisasi kelapa sawit berbasis koperasi diharapkan meningkatkan kesejahteraan petani. Dukungan dari berbagai pihak penting untuk keberhasilan ini.</t>
+        </is>
+      </c>
+      <c r="F1233" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1233" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614339/menkop-dorong-hilirisasi-sawit-berbasis-koperasi-untuk-sejahterakan-petani</t>
+        </is>
+      </c>
+      <c r="H1233" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/kemenkop-1786455130445_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1233" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1234">
+      <c r="A1234" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1234" t="inlineStr">
+        <is>
+          <t>Wamendagri Ribka Haluk Sambut Anak Papua Lanjutkan Sekolah di Tangerang</t>
+        </is>
+      </c>
+      <c r="C1234" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:21:37 +0700</t>
+        </is>
+      </c>
+      <c r="D1234" t="inlineStr">
+        <is>
+          <t>Nada Herwando Kartika</t>
+        </is>
+      </c>
+      <c r="E1234" t="inlineStr">
+        <is>
+          <t>Wamendagri Ribka Haluk menyambut 65 pelajar Papua di Jakarta. Mereka akan melanjutkan pendidikan di Tangerang setelah perjalanan laut tujuh hari.</t>
+        </is>
+      </c>
+      <c r="F1234" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1234" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614319/wamendagri-ribka-haluk-sambut-anak-papua-lanjutkan-sekolah-di-tangerang</t>
+        </is>
+      </c>
+      <c r="H1234" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/kemendagri-1786454396856_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1234" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1235">
+      <c r="A1235" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1235" t="inlineStr">
+        <is>
+          <t>Waka MPR Dorong Penataan Ulang Sistem Pendidikan di Indonesia</t>
+        </is>
+      </c>
+      <c r="C1235" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:21:17 +0700</t>
+        </is>
+      </c>
+      <c r="D1235" t="inlineStr">
+        <is>
+          <t>Dea Duta Aulia</t>
+        </is>
+      </c>
+      <c r="E1235" t="inlineStr">
+        <is>
+          <t>Waka MPR Lestari Moerdijat tekankan pentingnya transformasi pendidikan untuk lahirkan lulusan yang kritis dan berkarakter, selaras dengan kebutuhan pasar kerja.</t>
+        </is>
+      </c>
+      <c r="F1235" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1235" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614318/waka-mpr-dorong-penataan-ulang-sistem-pendidikan-di-indonesia</t>
+        </is>
+      </c>
+      <c r="H1235" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/05/02/wakil-ketua-mpr-lestari-moerdijat-1777717773159_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1235" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1236">
+      <c r="A1236" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1236" t="inlineStr">
+        <is>
+          <t>Empat Lembaga Teken MoU Rehabilitasi hingga Pemberdayaan Napza</t>
+        </is>
+      </c>
+      <c r="C1236" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:16:48 +0700</t>
+        </is>
+      </c>
+      <c r="D1236" t="inlineStr">
+        <is>
+          <t>Chayyara Zulghifary</t>
+        </is>
+      </c>
+      <c r="E1236" t="inlineStr">
+        <is>
+          <t>Kemensos, Kemenkes, Kemenaker, dan BNN tandatangani MoU untuk penanganan terpadu korban penyalahgunaan Napza, dari rehabilitasi hingga penempatan kerja.</t>
+        </is>
+      </c>
+      <c r="F1236" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1236" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614315/empat-lembaga-teken-mou-rehabilitasi-hingga-pemberdayaan-napza</t>
+        </is>
+      </c>
+      <c r="H1236" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/kemensos-1786453983320_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1236" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1237">
+      <c r="A1237" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1237" t="inlineStr">
+        <is>
+          <t>Megawati Lantik Pinka Haprani-Andi Widjajanto Pimpin Organisasi Sayap PDIP</t>
+        </is>
+      </c>
+      <c r="C1237" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:10:05 +0700</t>
+        </is>
+      </c>
+      <c r="D1237" t="inlineStr">
+        <is>
+          <t>Dwi Rahmawati</t>
+        </is>
+      </c>
+      <c r="E1237" t="inlineStr">
+        <is>
+          <t>Megawati Soekarnoputri melantik pimpinan organisasi sayap PDIP, termasuk Pinka Haprani dan Andi Widjajanto, untuk memperkuat konsolidasi dan riset partai.</t>
+        </is>
+      </c>
+      <c r="F1237" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1237" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614312/megawati-lantik-pinka-haprani-andi-widjajanto-pimpin-organisasi-sayap-pdip</t>
+        </is>
+      </c>
+      <c r="H1237" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/ketua-umum-dpp-pdi-perjuangan-pdip-megawati-soekarnoputri-melantik-pimpinan-organisasi-sayap-dan-badan-partai-dok-ist-1786453772423_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1237" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1238">
+      <c r="A1238" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1238" t="inlineStr">
+        <is>
+          <t>Ulah Maling di Serang Sembelih Puluhan Kambing di Pematang Sawah</t>
+        </is>
+      </c>
+      <c r="C1238" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:00:45 +0700</t>
+        </is>
+      </c>
+      <c r="D1238" t="inlineStr">
+        <is>
+          <t>Tim detikcom</t>
+        </is>
+      </c>
+      <c r="E1238" t="inlineStr">
+        <is>
+          <t>Aksi pencurian puluhan kambing terjadi di Kabupaten Serang, Banten. Kambing-kambing itu diduga disembelih sebelum diangkut dan dibawa kabur.</t>
+        </is>
+      </c>
+      <c r="F1238" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1238" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614304/ulah-maling-di-serang-sembelih-puluhan-kambing-di-pematang-sawah</t>
+        </is>
+      </c>
+      <c r="H1238" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/lokasi-kandang-kambing-yang-dicuri-ariefdetikcom-1786427491486_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1238" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1239">
+      <c r="A1239" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1239" t="inlineStr">
+        <is>
+          <t>Ramai di Medsos, Komentar Warganet Soal Videotron 'Hujan Anggur' di Jakarta</t>
+        </is>
+      </c>
+      <c r="C1239" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:00:25 +0700</t>
+        </is>
+      </c>
+      <c r="D1239" t="inlineStr">
+        <is>
+          <t>Rahmat Khairurizqi</t>
+        </is>
+      </c>
+      <c r="E1239" t="inlineStr">
+        <is>
+          <t>Visual 'hujan anggur' di videotron Jakarta menarik perhatian warganet. Beragam respons muncul, dari ketertarikan hingga komentar tentang HiFruit.</t>
+        </is>
+      </c>
+      <c r="F1239" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1239" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614286/ramai-di-medsos-komentar-warganet-soal-videotron-hujan-anggur-di-jakarta</t>
+        </is>
+      </c>
+      <c r="H1239" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/viral-hujan-anggur-di-jakarta-iklan-ini-bikin-warga-berhenti-menoleh-1786451271811_43.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1239" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1240">
+      <c r="A1240" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1240" t="inlineStr">
+        <is>
+          <t>Banjir Bertahun-tahun di Bulak Barat Depok Kini Telah Surut</t>
+        </is>
+      </c>
+      <c r="C1240" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:47:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1240" t="inlineStr">
+        <is>
+          <t>Devi Puspitasari</t>
+        </is>
+      </c>
+      <c r="E1240" t="inlineStr">
+        <is>
+          <t>Banjir di Bulak Barat, Depok, yang berkepanjangan kini telah surut. Pemerintah setempat melakukan normalisasi sungai dan merencanakan pembangunan jembatan baru.</t>
+        </is>
+      </c>
+      <c r="F1240" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1240" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614290/banjir-bertahun-tahun-di-bulak-barat-depok-kini-telah-surut</t>
+        </is>
+      </c>
+      <c r="H1240" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/banjir-di-bulak-barat-depok-yang-berkepanjangan-kini-telah-surut-pemerintah-setempat-melakukan-normalisasi-sungai-devi-pdetikc-1786452277211_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1240" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1241">
+      <c r="A1241" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1241" t="inlineStr">
+        <is>
+          <t>Perwira TNI Didakwa Selundupkan Sabu di Kepri, Paket Ditulis 'Selamat Umrah'</t>
+        </is>
+      </c>
+      <c r="C1241" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:44:35 +0700</t>
+        </is>
+      </c>
+      <c r="D1241" t="inlineStr">
+        <is>
+          <t>Nizar Aldi</t>
+        </is>
+      </c>
+      <c r="E1241" t="inlineStr">
+        <is>
+          <t>Mayor Laut Faisal Mulia didakwa menyelundupkan 12 paket sabu ke pesawat militer. Ia ditangkap setelah interogasi terkait pengiriman narkoba.</t>
+        </is>
+      </c>
+      <c r="F1241" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1241" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614288/perwira-tni-didakwa-selundupkan-sabu-di-kepri-paket-ditulis-selamat-umrah</t>
+        </is>
+      </c>
+      <c r="H1241" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2023/03/03/ilustrasi-hukum-2_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1241" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1242">
+      <c r="A1242" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1242" t="inlineStr">
+        <is>
+          <t>Muncul 'Hujan Anggur' di Jakarta, Videotron Ini Curi Perhatian Warga</t>
+        </is>
+      </c>
+      <c r="C1242" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:40:56 +0700</t>
+        </is>
+      </c>
+      <c r="D1242" t="inlineStr">
+        <is>
+          <t>Rahmat Khairurizqi</t>
+        </is>
+      </c>
+      <c r="E1242" t="inlineStr">
+        <is>
+          <t>Visual unik 'hujan anggur' menghiasi videotron Jakarta, menarik perhatian di tengah iklan. Iklan HiFruit ini menciptakan pengalaman visual yang menonjol.</t>
+        </is>
+      </c>
+      <c r="F1242" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1242" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614284/muncul-hujan-anggur-di-jakarta-videotron-ini-curi-perhatian-warga</t>
+        </is>
+      </c>
+      <c r="H1242" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/viral-hujan-anggur-di-jakarta-iklan-ini-bikin-warga-berhenti-menoleh-1786451271811_43.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1242" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1243">
+      <c r="A1243" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1243" t="inlineStr">
+        <is>
+          <t>Koalisi Sipil Kritik Pernyataan Panglima TNI Tanggung Jawab Keamanan Indonesia</t>
+        </is>
+      </c>
+      <c r="C1243" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:37:44 +0700</t>
+        </is>
+      </c>
+      <c r="D1243" t="inlineStr">
+        <is>
+          <t>Tim detikcom</t>
+        </is>
+      </c>
+      <c r="E1243" t="inlineStr">
+        <is>
+          <t>Koalisi Masyarakat Sipil mengecam pernyataan Panglima TNI tentang tanggung jawab keamanan. Mereka khawatir akan pengaburan fungsi TNI dalam urusan sipil.</t>
+        </is>
+      </c>
+      <c r="F1243" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1243" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614282/koalisi-sipil-kritik-pernyataan-panglima-tni-tanggung-jawab-keamanan-indonesia</t>
+        </is>
+      </c>
+      <c r="H1243" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/08/09/ilustrasi-tni-1754727401560.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1243" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1244">
+      <c r="A1244" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1244" t="inlineStr">
+        <is>
+          <t>4 Kesimpulan Komisi III DPR soal Kasus Tewasnya Eks Istri Polisi di Medan</t>
+        </is>
+      </c>
+      <c r="C1244" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:33:46 +0700</t>
+        </is>
+      </c>
+      <c r="D1244" t="inlineStr">
+        <is>
+          <t>Dwi Rahmawati</t>
+        </is>
+      </c>
+      <c r="E1244" t="inlineStr">
+        <is>
+          <t>Komisi III DPR RI mengeluarkan 4 kesimpulan terkait kematian eks istri polisi di Medan, mendesak penyidikan transparan dan akuntabel.</t>
+        </is>
+      </c>
+      <c r="F1244" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1244" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614277/4-kesimpulan-komisi-iii-dpr-soal-kasus-tewasnya-eks-istri-polisi-di-medan</t>
+        </is>
+      </c>
+      <c r="H1244" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/komisi-iii-dpr-ri-menggelar-rapat-dengar-pendapat-rdp-dan-rapat-dengar-pendapat-umum-rdpu-membahas-kasus-kematian-eks-istri-br-1786451602067_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1244" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1245">
+      <c r="A1245" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1245" t="inlineStr">
+        <is>
+          <t>Mantan Sekjen Kementerian ESDM Rida Mulyana Meninggal Dunia</t>
+        </is>
+      </c>
+      <c r="C1245" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:40:30 +0700</t>
+        </is>
+      </c>
+      <c r="D1245" t="inlineStr">
+        <is>
+          <t>Heri Purnomo</t>
+        </is>
+      </c>
+      <c r="E1245" t="inlineStr">
+        <is>
+          <t>Mantan Sekretaris Jenderal Kementerian Energi dan Sumber Daya Mineral (ESDM) Rida Mulyana meninggal dunia pada Selasa (11/8/2026).</t>
+        </is>
+      </c>
+      <c r="F1245" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1245" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8614344/mantan-sekjen-kementerian-esdm-rida-mulyana-meninggal-dunia</t>
+        </is>
+      </c>
+      <c r="H1245" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2018/10/04/25efc886-7cad-437b-b73e-2130e142219b_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1245" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1246">
+      <c r="A1246" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1246" t="inlineStr">
+        <is>
+          <t>Kata Bahlil soal Kabar Reshuffle Kabinet Usai 17 Agustus</t>
+        </is>
+      </c>
+      <c r="C1246" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:22:57 +0700</t>
+        </is>
+      </c>
+      <c r="D1246" t="inlineStr">
+        <is>
+          <t>Heri Purnomo</t>
+        </is>
+      </c>
+      <c r="E1246" t="inlineStr">
+        <is>
+          <t>Menteri ESDM Bahlil Lahadalia merespons isu reshuffle kabinet yang disebut-sebut akan dilakukan Presiden Prabowo Subianto setelah 17 Agustus 2026.</t>
+        </is>
+      </c>
+      <c r="F1246" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1246" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8614324/kata-bahlil-soal-kabar-reshuffle-kabinet-usai-17-agustus</t>
+        </is>
+      </c>
+      <c r="H1246" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/04/bahlil-lahadalia-1785840108228_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1246" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1247">
+      <c r="A1247" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1247" t="inlineStr">
+        <is>
+          <t>Sederet Capaian Kinerja BUMN di Bawah Danantara</t>
+        </is>
+      </c>
+      <c r="C1247" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:04:22 +0700</t>
+        </is>
+      </c>
+      <c r="D1247" t="inlineStr">
+        <is>
+          <t>Ignacio Geordi Oswaldo</t>
+        </is>
+      </c>
+      <c r="E1247" t="inlineStr">
+        <is>
+          <t>Program konsolidasi dan transformasi BUMN yang dijalankan Danantara sejak awal pembentukannya mulai menunjukkan hasil yang konkret.</t>
+        </is>
+      </c>
+      <c r="F1247" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1247" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8614307/sederet-capaian-kinerja-bumn-di-bawah-danantara</t>
+        </is>
+      </c>
+      <c r="H1247" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/07/01/wisma-danantara-indonesia-1751345496316_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1247" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1248">
+      <c r="A1248" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1248" t="inlineStr">
+        <is>
+          <t>Cegah Longsor, KemenPU Perkuat Ruas Padang Panjang-Sicincin di Lembah Anai</t>
+        </is>
+      </c>
+      <c r="C1248" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:35:26 +0700</t>
+        </is>
+      </c>
+      <c r="D1248" t="inlineStr">
+        <is>
+          <t>Nada Herwando</t>
+        </is>
+      </c>
+      <c r="E1248" t="inlineStr">
+        <is>
+          <t>Kementerian PU memperkuat jalan dan lereng di Padang Panjang-Sicincin untuk ketahanan infrastruktur menghadapi bencana. Proyek ini selesai pada Juli 2026.</t>
+        </is>
+      </c>
+      <c r="F1248" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1248" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/infrastruktur/d-8614281/cegah-longsor-kemenpu-perkuat-ruas-padang-panjang-sicincin-di-lembah-anai</t>
+        </is>
+      </c>
+      <c r="H1248" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/kementerian-pu-1786451641619_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1248" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1249">
+      <c r="A1249" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1249" t="inlineStr">
+        <is>
+          <t>Rp 20,5 T Telah Mengalir ke 490 Pemda, Purbaya: Cukup untuk Bayar Gaji PPPK</t>
+        </is>
+      </c>
+      <c r="C1249" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:30:06 +0700</t>
+        </is>
+      </c>
+      <c r="D1249" t="inlineStr">
+        <is>
+          <t>Heri Purnomo</t>
+        </is>
+      </c>
+      <c r="E1249" t="inlineStr">
+        <is>
+          <t>Menteri Keuangan Purbaya Yudhi Sadewa mengumumkan penyaluran Rp 20,5 triliun untuk 490 Pemda, cukup untuk membayar gaji ASN dan PPPK.</t>
+        </is>
+      </c>
+      <c r="F1249" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1249" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8614194/rp-20-5-t-telah-mengalir-ke-490-pemda-purbaya-cukup-untuk-bayar-gaji-pppk</t>
+        </is>
+      </c>
+      <c r="H1249" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/23/menkeu-purbaya-1784785896260_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1249" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1250">
+      <c r="A1250" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B1250" t="inlineStr">
+        <is>
+          <t>Haru dan Bahagia Ivan Gunawan Exhibition Nusanova Dapat Rekor MURI</t>
+        </is>
+      </c>
+      <c r="C1250" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:02:39 +0700</t>
+        </is>
+      </c>
+      <c r="D1250" t="inlineStr">
+        <is>
+          <t>Desi Puspasari</t>
+        </is>
+      </c>
+      <c r="E1250" t="inlineStr">
+        <is>
+          <t>Ivan Gunawan terharu Nusanova 2.0: Sekar Jagat mendapatkan rekor MURI. Dia memecahkan pameran busana imersif pertama berbasis corak batik Sekar Jagat Madura.</t>
+        </is>
+      </c>
+      <c r="F1250" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1250" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8613990/haru-dan-bahagia-ivan-gunawan-exhibition-nusanova-dapat-rekor-muri</t>
+        </is>
+      </c>
+      <c r="H1250" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/ivan-gunawan-1786441529083_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1250" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1251">
+      <c r="A1251" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1251" t="inlineStr">
+        <is>
+          <t>Satu WNI dan Dua Warga Pakistan Tewas Diserang Houthi, Akankah Islamabad Terjun ke Perang?</t>
+        </is>
+      </c>
+      <c r="C1251" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:50:15 +0700</t>
+        </is>
+      </c>
+      <c r="D1251" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1251" t="inlineStr">
+        <is>
+          <t>Bagi Pakistan, persoalan jadi lebih sensitif karena dua warga negaranya jadi korban. Mereka baru bergabung dalam pakta pertahanan Turki-Saudi</t>
+        </is>
+      </c>
+      <c r="F1251" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1251" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7867107/satu-wni-dan-dua-warga-pakistan-tewas-diserang-houthi-akankah-islamabad-terjun-ke-perang</t>
+        </is>
+      </c>
+      <c r="H1251" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/sKTjW2IWme_tj-rBEFT9DF7gqhA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/PAKTA-PERTAHANAN-Bendera-Arab-Saudi-Pakistan-dan-Turki.jpg</t>
+        </is>
+      </c>
+      <c r="I1251" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1252">
+      <c r="A1252" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1252" t="inlineStr">
+        <is>
+          <t>Soal Isu Demo Agustus 2025 Berulang, Ray Rangkuti: Tak Ada Indikasi, tapi Lampu Kuning bagi Prabowo</t>
+        </is>
+      </c>
+      <c r="C1252" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:47:01 +0700</t>
+        </is>
+      </c>
+      <c r="D1252" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1252" t="inlineStr">
+        <is>
+          <t>Ray Rangkuti menilai, publik sudah semakin resah dengan pemerintahan Prabowo-Gibran, dan hal itu makin terlihat dari survei SMRC terbaru.</t>
+        </is>
+      </c>
+      <c r="F1252" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1252" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867106/soal-isu-demo-agustus-2025-berulang-ray-rangkuti-tak-ada-indikasi-tapi-lampu-kuning-bagi-prabowo</t>
+        </is>
+      </c>
+      <c r="H1252" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/0iL7xMX-_zskwBZCe2XRTCl1Bzs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/prabowo-kadin-dks.jpg</t>
+        </is>
+      </c>
+      <c r="I1252" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1253">
+      <c r="A1253" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1253" t="inlineStr">
+        <is>
+          <t>Orang Kaya Mulai Kurangi Properti, Saham dan Kripto Dinilai Lebih Menarik</t>
+        </is>
+      </c>
+      <c r="C1253" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:44:40 +0700</t>
+        </is>
+      </c>
+      <c r="D1253" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1253" t="inlineStr">
+        <is>
+          <t>Penjualan properti kelas atas melambat karena orang kaya mengurangi aset properti dan beralih ke saham serta kripto yang dinilai lebih…</t>
+        </is>
+      </c>
+      <c r="F1253" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1253" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7867105/orang-kaya-mulai-kurangi-properti-saham-dan-kripto-dinilai-lebih-menarik</t>
+        </is>
+      </c>
+      <c r="H1253" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/UNKBC5WcfRV_cLsFJWHGS_vnnvE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/BDeutsche-Welle77982382_403.jpg.jpg</t>
+        </is>
+      </c>
+      <c r="I1253" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1254">
+      <c r="A1254" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1254" t="inlineStr">
+        <is>
+          <t>Sejarah Baru CAHN FC Tembus Liga Champions Asia 2026/2027, Sepak Bola Vietnam Naik Kelas</t>
+        </is>
+      </c>
+      <c r="C1254" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:44:19 +0700</t>
+        </is>
+      </c>
+      <c r="D1254" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1254" t="inlineStr">
+        <is>
+          <t>Sejarah baru diukir salah satu klub Vietnam yang berhasil menembus putaran final Liga Champions Asia musim 2026/2027.</t>
+        </is>
+      </c>
+      <c r="F1254" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1254" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7867104/sejarah-baru-cahn-fc-tembus-liga-champions-asia-20262027-sepak-bola-vietnam-naik-kelas</t>
+        </is>
+      </c>
+      <c r="H1254" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/IInQZ2cgGLMiezomp6XB8qOu4_k=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/pelatih-kepala-timnas-thailand-alexandre-polking_20211229_202645.jpg</t>
+        </is>
+      </c>
+      <c r="I1254" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1255">
+      <c r="A1255" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1255" t="inlineStr">
+        <is>
+          <t>Raffi Ahmad Dorong Kolaborasi Anak Muda Jadi Penggerak Transformasi Digital</t>
+        </is>
+      </c>
+      <c r="C1255" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:44:06 +0700</t>
+        </is>
+      </c>
+      <c r="D1255" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1255" t="inlineStr">
+        <is>
+          <t>Raffi Ahmad mendorong kolaborasi pemerintah dan pemuda diperkuat untuk memanfaatkan transformasi digital, termasuk AI, bagi pendidikan,</t>
+        </is>
+      </c>
+      <c r="F1255" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1255" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867103/raffi-ahmad-dorong-kolaborasi-anak-muda-jadi-penggerak-transformasi-digital</t>
+        </is>
+      </c>
+      <c r="H1255" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/8G7DhYEeY8_HDZm-rOs30XeMDkU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/raffi-audiensi-dengan-dpp.jpg</t>
+        </is>
+      </c>
+      <c r="I1255" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1256">
+      <c r="A1256" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1256" t="inlineStr">
+        <is>
+          <t>Cegah Kekerasan Terhadap Santri, Kemenag Hingga KPAI Rumuskan Pedoman Safeguarding Pesantren</t>
+        </is>
+      </c>
+      <c r="C1256" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:42:56 +0700</t>
+        </is>
+      </c>
+      <c r="D1256" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1256" t="inlineStr">
+        <is>
+          <t>Pedoman Safeguarding Pesantren Ramah Anak akan menjadi panduan bersama dalam memperkuat sistem pencegahan tindak kekerasan</t>
+        </is>
+      </c>
+      <c r="F1256" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1256" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867102/cegah-kekerasan-terhadap-santri-kemenag-hingga-kpai-rumuskan-pedoman-safeguarding-pesantren</t>
+        </is>
+      </c>
+      <c r="H1256" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/RJLgc4hbDHHbIMpg3m_gQYsPxBM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Tadarus-Santri-Ponpes-Ar-Raudlatul-Hasanah-Medan_20260221_172957.jpg</t>
+        </is>
+      </c>
+      <c r="I1256" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1257">
+      <c r="A1257" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1257" t="inlineStr">
+        <is>
+          <t>Bukan Sekadar Hasil, Xabi Alonso Bangun Fondasi Chelsea di Tur Pramusim</t>
+        </is>
+      </c>
+      <c r="C1257" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:42:47 +0700</t>
+        </is>
+      </c>
+      <c r="D1257" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1257" t="inlineStr">
+        <is>
+          <t>Lebih dari sekadar hasil laga, tur pramusim menjadi momen Xabi Alonso membangun chemistry dan fondasi baru Chelsea.</t>
+        </is>
+      </c>
+      <c r="F1257" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1257" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7867101/bukan-sekadar-hasil-xabi-alonso-bangun-fondasi-chelsea-di-tur-pramusim</t>
+        </is>
+      </c>
+      <c r="H1257" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/SIUs7kjLLjYIblFlkw_JSBUggrM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Chelsea-FC-vs-AC-Milan_20260809_140404.jpg</t>
+        </is>
+      </c>
+      <c r="I1257" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1258">
+      <c r="A1258" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1258" t="inlineStr">
+        <is>
+          <t>Terjemahan Lirik Lagu Purple Rain - Prince: I Never Meant to Cause You any Sorrow</t>
+        </is>
+      </c>
+      <c r="C1258" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:40:02 +0700</t>
+        </is>
+      </c>
+      <c r="D1258" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1258" t="inlineStr">
+        <is>
+          <t>Solo gitarnya di bagian akhir menjadi momen paling emosional dan menjadi penutup yang apik.</t>
+        </is>
+      </c>
+      <c r="F1258" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1258" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/musik/7867100/terjemahan-lirik-lagu-purple-rain-prince-i-never-meant-to-cause-you-any-sorrow</t>
+        </is>
+      </c>
+      <c r="H1258" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/zLN77GXG_MWcQ27NDqNvGgp-QJs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-musik-ilustrasi-lirik-ilustrasi-terjemahan-lirik-lagu.jpg</t>
+        </is>
+      </c>
+      <c r="I1258" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1259">
+      <c r="A1259" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1259" t="inlineStr">
+        <is>
+          <t>Terjemahan Lirik Lagu Slow Dancing in a Burning Room dari John Mayer: We're Going Down</t>
+        </is>
+      </c>
+      <c r="C1259" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:39:32 +0700</t>
+        </is>
+      </c>
+      <c r="D1259" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1259" t="inlineStr">
+        <is>
+          <t>Slow Dancing in a Burning Room sering digunakan oleh banyak musisi muda untuk belajar teknik gitar blues modern.</t>
+        </is>
+      </c>
+      <c r="F1259" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1259" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/musik/7867099/terjemahan-lirik-lagu-slow-dancing-in-a-burning-room-dari-john-mayer-were-going-down</t>
+        </is>
+      </c>
+      <c r="H1259" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/iF9WIvyjtJsIYfbmSdBAvkMvzYI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/john-mayer-hibur-fansnya-di-indonesia-dalam-konser-asia-tour_20190405_213614.jpg</t>
+        </is>
+      </c>
+      <c r="I1259" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1260">
+      <c r="A1260" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1260" t="inlineStr">
+        <is>
+          <t>Terjemahan Lirik Lagu Blackout - Turnstile: Blackout in the Middle of the Light</t>
+        </is>
+      </c>
+      <c r="C1260" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:39:03 +0700</t>
+        </is>
+      </c>
+      <c r="D1260" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1260" t="inlineStr">
+        <is>
+          <t>Berikut ini merupakan terjemahan lirik lagu Blackout yang dipopulerkan oleh grup band asal Baltimore, Turnstile.</t>
+        </is>
+      </c>
+      <c r="F1260" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1260" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/musik/7867098/terjemahan-lirik-lagu-blackout-turnstile-blackout-in-the-middle-of-the-light</t>
+        </is>
+      </c>
+      <c r="H1260" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/zLN77GXG_MWcQ27NDqNvGgp-QJs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-musik-ilustrasi-lirik-ilustrasi-terjemahan-lirik-lagu.jpg</t>
+        </is>
+      </c>
+      <c r="I1260" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1261">
+      <c r="A1261" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1261" t="inlineStr">
+        <is>
+          <t>Kunci Gitar Lagu Sementara - The Paps: Ku Tak Mau Jatuh Cinta untuk Sementara</t>
+        </is>
+      </c>
+      <c r="C1261" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:38:25 +0700</t>
+        </is>
+      </c>
+      <c r="D1261" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1261" t="inlineStr">
+        <is>
+          <t>Berikut ini merupakan chord kunci gitar lagu Sementara yang dipopulerkan oleh grup band The Paps, dimainkan dari kunci Am.</t>
+        </is>
+      </c>
+      <c r="F1261" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1261" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/musik/7867097/kunci-gitar-lagu-sementara-the-paps-ku-tak-mau-jatuh-cinta-untuk-sementara</t>
+        </is>
+      </c>
+      <c r="H1261" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/vZGfIQdrUWUr9aeBMAO6c3gc3O0=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Potret-gitar-akustik-untuk-kunci-chord-dasar-mudah-dimainkan.jpg</t>
+        </is>
+      </c>
+      <c r="I1261" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1262">
+      <c r="A1262" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1262" t="inlineStr">
+        <is>
+          <t>Terjemahan Lirik Lagu New Generation - The SIGIT: We Are the Noodle Generation</t>
+        </is>
+      </c>
+      <c r="C1262" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:37:03 +0700</t>
+        </is>
+      </c>
+      <c r="D1262" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1262" t="inlineStr">
+        <is>
+          <t>Berikut ini merupakan terjemahan lirik lagu New Generation yang dipopulerkan oleh grup band The SIGIT.</t>
+        </is>
+      </c>
+      <c r="F1262" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1262" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/musik/7867096/terjemahan-lirik-lagu-new-generation-the-sigit-we-are-the-noodle-generation</t>
+        </is>
+      </c>
+      <c r="H1262" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/tEq9lHSi3zC8-tIEQ99J9IcoxD8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-terjemahan-lirik-lagu.jpg</t>
+        </is>
+      </c>
+      <c r="I1262" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1263">
+      <c r="A1263" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1263" t="inlineStr">
+        <is>
+          <t>Taiwan Deteksi Pesawat dan Kapal Perang China di Sekitar Wilayahnya</t>
+        </is>
+      </c>
+      <c r="C1263" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:36:56 +0700</t>
+        </is>
+      </c>
+      <c r="D1263" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1263" t="inlineStr">
+        <is>
+          <t>Beijing menganggap Taiwan sebagai bagian dari wilayah China dan menolak gagasan bahwa Taiwan merupakan negara yang terpisah.</t>
+        </is>
+      </c>
+      <c r="F1263" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1263" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7867095/taiwan-deteksi-pesawat-dan-kapal-perang-china-di-sekitar-wilayahnya</t>
+        </is>
+      </c>
+      <c r="H1263" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/04b2exUAkAL41jonI7E-0LjTXnk=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Kapal-Perang-China-Angkatan-Laut-Tiongkok.jpg</t>
+        </is>
+      </c>
+      <c r="I1263" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1264">
+      <c r="A1264" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1264" t="inlineStr">
+        <is>
+          <t>‘Berkarya Lewat Lensa’ Jadi Ruang Jurnalis dan Masyarakat Bercerita Melalui Foto</t>
+        </is>
+      </c>
+      <c r="C1264" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:34:56 +0700</t>
+        </is>
+      </c>
+      <c r="D1264" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1264" t="inlineStr">
+        <is>
+          <t>PFI bersama Nojorono Kudus gelar “Berkarya Lewat Lensa”, ruang ekspresi visual menjaga warisan di tengah perubahan zaman.</t>
+        </is>
+      </c>
+      <c r="F1264" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1264" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7867094/berkarya-lewat-lensa-jadi-ruang-jurnalis-dan-masyarakat-bercerita-melalui-foto</t>
+        </is>
+      </c>
+      <c r="H1264" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ctKK8KNp7E6vPwK-FrLwXXJmN9w=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-fotografi-smartphone.jpg</t>
+        </is>
+      </c>
+      <c r="I1264" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1265">
+      <c r="A1265" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1265" t="inlineStr">
+        <is>
+          <t>Abdul Muhari Dilantik Jadi Deputi Pencegahan BNPB, Ini Sosoknya</t>
+        </is>
+      </c>
+      <c r="C1265" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:34:38 +0700</t>
+        </is>
+      </c>
+      <c r="D1265" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1265" t="inlineStr">
+        <is>
+          <t>Kepala BNPB Letjen TNI Dr Suharyanto mengambil sumpah jabatan Abdul Muhari sebagai Deputi Bidang Pencegahan BNPB</t>
+        </is>
+      </c>
+      <c r="F1265" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1265" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867093/abdul-muhari-dilantik-jadi-deputi-pencegahan-bnpb-ini-sosoknya</t>
+        </is>
+      </c>
+      <c r="H1265" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/c5wKBOF6W6_Peb2ImbRRlDy7GTY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Abdul-Muhari-dilantik-menjadi-Deputi-Bidang-Pencegahan-BNPB.jpg</t>
+        </is>
+      </c>
+      <c r="I1265" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1266">
+      <c r="A1266" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1266" t="inlineStr">
+        <is>
+          <t>Terjemahan Lirik dan Makna Lagu Loser - Tame Impala: So Much for Closure, I Lost Composure</t>
+        </is>
+      </c>
+      <c r="C1266" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:33:32 +0700</t>
+        </is>
+      </c>
+      <c r="D1266" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1266" t="inlineStr">
+        <is>
+          <t>Berikut ini terjemahan lirik dan makna lagu "Loser" karya Tame Impala lengkap dengan profil singkat sang musisi.</t>
+        </is>
+      </c>
+      <c r="F1266" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1266" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/musik/7867092/terjemahan-lirik-dan-makna-lagu-loser-tame-impala-so-much-for-closure-i-lost-composure</t>
+        </is>
+      </c>
+      <c r="H1266" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/8ofGbaRMpqu_gFPWYkenF6qEE2Y=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Potret-ilustrasi-lirik-lagu-terjemahan-musik-mendengarkan-musik.jpg</t>
+        </is>
+      </c>
+      <c r="I1266" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1267">
+      <c r="A1267" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1267" t="inlineStr">
+        <is>
+          <t>Kunci Jawaban Bahasa Indonesia Kawan Seiring Kelas 3 Halaman 22 Kurikulum Merdeka: Aktivitas 6</t>
+        </is>
+      </c>
+      <c r="C1267" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:29:16 +0700</t>
+        </is>
+      </c>
+      <c r="D1267" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1267" t="inlineStr">
+        <is>
+          <t>Soal ini terdapat pada buku Bahasa Indonesia Kawan Seiring Kelas 3 Halaman 22 Kurikulum Merdeka, tepatnya pada Aktivitas 6.</t>
+        </is>
+      </c>
+      <c r="F1267" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1267" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/pendidikan/7867091/kunci-jawaban-bahasa-indonesia-kawan-seiring-kelas-3-halaman-22-kurikulum-merdeka-aktivitas-6</t>
+        </is>
+      </c>
+      <c r="H1267" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/AQ6NUlpft8TPoUd6GxuTuejfIw4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/siswa-SD-belajar-di-sekolah.jpg</t>
+        </is>
+      </c>
+      <c r="I1267" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1268">
+      <c r="A1268" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1268" t="inlineStr">
+        <is>
+          <t>Laut Merah Jadi Front Baru Perang Iran, Houthi Gencarkan Serangan Kapal: Ada WNI Jadi Korban</t>
+        </is>
+      </c>
+      <c r="C1268" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:28:02 +0700</t>
+        </is>
+      </c>
+      <c r="D1268" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1268" t="inlineStr">
+        <is>
+          <t>Sumber dari penjaga pantai Yaman dan pemerintah setempat menyebut tiga awak kapal tewas, terdiri dari dua warga Pakistan dan satu warga Indonesia.</t>
+        </is>
+      </c>
+      <c r="F1268" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1268" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7867090/laut-merah-jadi-front-baru-perang-iran-houthi-gencarkan-serangan-kapal-ada-wni-jadi-korban</t>
+        </is>
+      </c>
+      <c r="H1268" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ic5AbtT--SxS2enYL-jm8r_WyyI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Houthi-serangan-kapal-kargo-di-Laut-Merah.jpg</t>
+        </is>
+      </c>
+      <c r="I1268" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1269">
+      <c r="A1269" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1269" t="inlineStr">
+        <is>
+          <t>Agenda Keliling Dunia Rampung, Chelsea Gantian Sambut Para Bintang</t>
+        </is>
+      </c>
+      <c r="C1269" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:25:15 +0700</t>
+        </is>
+      </c>
+      <c r="D1269" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1269" t="inlineStr">
+        <is>
+          <t>Chelsea mulai akan menyambut para pemain bintang yang bergabung belakangan ke klub, seperti Enzo Fernandez, Morgan Rogers,dan Valentin Barco.</t>
+        </is>
+      </c>
+      <c r="F1269" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1269" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7867089/agenda-keliling-dunia-rampung-chelsea-gantian-sambut-para-bintang</t>
+        </is>
+      </c>
+      <c r="H1269" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/1TZQge9GlQD89HfEuhZSIz5D8rA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Chelsea-FC-vs-AC-Milan_20260809_140223.jpg</t>
+        </is>
+      </c>
+      <c r="I1269" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1270">
+      <c r="A1270" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1270" t="inlineStr">
+        <is>
+          <t>Uji Materi UU Kesehatan, Pemohon Soroti Wewenang MDP KKI: Kasus Dokter Ratna Jadi Acuan</t>
+        </is>
+      </c>
+      <c r="C1270" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:25:01 +0700</t>
+        </is>
+      </c>
+      <c r="D1270" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1270" t="inlineStr">
+        <is>
+          <t>Kasus dokter Ratna di Pangkalpinang menjadi acuan uji UU Kesehatan soal batas kewenangan MDP KKI dan proses hukum dokter</t>
+        </is>
+      </c>
+      <c r="F1270" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1270" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867088/uji-materi-uu-kesehatan-pemohon-soroti-wewenang-mdp-kki-kasus-dokter-ratna-jadi-acuan</t>
+        </is>
+      </c>
+      <c r="H1270" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/zAd483LFybKEViN_GUiehmzCGNY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Mahkamah-Konstitusi-menggelar-sidang-pengucapan-sejumlah-putusan.jpg</t>
+        </is>
+      </c>
+      <c r="I1270" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1271">
+      <c r="A1271" t="inlineStr">
+        <is>
+          <t>Bisnis</t>
+        </is>
+      </c>
+      <c r="B1271" t="inlineStr">
+        <is>
+          <t>KAI Diskon Tiket 17 Persen dan Tarif Rp8 untuk LRT dan KRL</t>
+        </is>
+      </c>
+      <c r="C1271" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:25:38 +0700</t>
+        </is>
+      </c>
+      <c r="D1271" t="inlineStr">
+        <is>
+          <t>Friska Yolandha</t>
+        </is>
+      </c>
+      <c r="E1271" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- PT Kereta Api Indonesia (Persero) atau KAI menghadirkan Promo Spesial 17-8-2026 dalam rangka menyemarakkan Hari Ulang Tahun ke-81 Kemerdekaan Republik Indonesia dengan tema “Bersatu Berdaulat, Rakyat...</t>
+        </is>
+      </c>
+      <c r="F1271" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1271" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjlxaq370/kai-diskon-tiket-17-persen-dan-tarif-rp8-untuk-lrt-dan-krl</t>
+        </is>
+      </c>
+      <c r="H1271" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/jumlah-pengguna-lrt-jabodebek-terus-meningkat-seiring-semakin-banyak_260730175516-557.jpg</t>
+        </is>
+      </c>
+      <c r="I1271" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="1272">
+      <c r="A1272" t="inlineStr">
+        <is>
+          <t>Bisnis</t>
+        </is>
+      </c>
+      <c r="B1272" t="inlineStr">
+        <is>
+          <t>Harga Pakan Naik, Harga Telur Turun, Peternak Unggas Tercekik</t>
+        </is>
+      </c>
+      <c r="C1272" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:57:56 +0700</t>
+        </is>
+      </c>
+      <c r="D1272" t="inlineStr">
+        <is>
+          <t>Gita Amanda</t>
+        </is>
+      </c>
+      <c r="E1272" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, SEMARANG — Para peternak yang tergabung dalam Koperasi Peternak Unggas Sejahtera (KPUS) telah menggelar demonstrasi di sejumlah kabupaten di Provinsi Jawa Tengah (Jateng) pada Senin (10/8/2026). Mereka mengeluhkan terus...</t>
+        </is>
+      </c>
+      <c r="F1272" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1272" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjlw0k423/harga-pakan-naik-harga-telur-turun-peternak-unggas-tercekik</t>
+        </is>
+      </c>
+      <c r="H1272" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/sejumlah-peternak-ayam-di-diy-membentangkan-spanduk-memprotes-mahalnya_260811010152-976.jpeg</t>
+        </is>
+      </c>
+      <c r="I1272" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="1273">
+      <c r="A1273" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1273" t="inlineStr">
+        <is>
+          <t>Lima Pihak Dipolisikan Buntut Tantangan Hafalan Alquran Berhadiah Miras</t>
+        </is>
+      </c>
+      <c r="C1273" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:06:38 +0700</t>
+        </is>
+      </c>
+      <c r="D1273" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1273" t="inlineStr">
+        <is>
+          <t>Tim Hukum Muslim melaporkan perkara ini ke Polda Metro Jaya.</t>
+        </is>
+      </c>
+      <c r="F1273" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1273" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267496/lima-pihak-dipolisikan-buntut-tantangan-hafalan-alquran-berhadiah-miras</t>
+        </is>
+      </c>
+      <c r="H1273" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/zZCEJSPd8hO87JaYrgYkVT8aozU=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9321619/original/023796700_1786457189-03531120-2f6a-4f2a-b03d-ae796cbec761.jpg</t>
+        </is>
+      </c>
+      <c r="I1273" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1274">
+      <c r="A1274" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1274" t="inlineStr">
+        <is>
+          <t>Gus Alex Didakwa Perkaya Diri Rp 93,6 M dari Kasus Kuota Haji</t>
+        </is>
+      </c>
+      <c r="C1274" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:46:01 +0700</t>
+        </is>
+      </c>
+      <c r="D1274" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1274" t="inlineStr">
+        <is>
+          <t>Uang yang diterima Gus Alex tersebut berasal dari sejumlah pihak dalam praktik pengisian kuota haji khusus</t>
+        </is>
+      </c>
+      <c r="F1274" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1274" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267481/gus-alex-didakwa-perkaya-diri-rp-936-m-dari-kasus-kuota-haji</t>
+        </is>
+      </c>
+      <c r="H1274" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/w5ODo7-d0Sp1v14iaP_WyQRa58I=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/5777171/original/051032100_1778679973-1.jpg</t>
+        </is>
+      </c>
+      <c r="I1274" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1275">
+      <c r="A1275" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1275" t="inlineStr">
+        <is>
+          <t>Kejagung: Febrie Adriansyah Mantan Pendekar Hukum, Harus Hati-Hati</t>
+        </is>
+      </c>
+      <c r="C1275" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:26:16 +0700</t>
+        </is>
+      </c>
+      <c r="D1275" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1275" t="inlineStr">
+        <is>
+          <t>Febrie merupakan orang yang memahami hukum sehingga penyidik perlu menyiapkan strategi dalam menangani perkara tersebut.</t>
+        </is>
+      </c>
+      <c r="F1275" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1275" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267464/kejagung-febrie-adriansyah-mantan-pendekar-hukum-harus-hati-hati</t>
+        </is>
+      </c>
+      <c r="H1275" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/A02PfRJ2y22nBz-jXAXGn_wIYFI=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9306887/original/065864800_1784913814-jam8.jpg</t>
+        </is>
+      </c>
+      <c r="I1275" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1276">
+      <c r="A1276" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1276" t="inlineStr">
+        <is>
+          <t>Menko PMK Ungkap Kendala Modifikasi Cuaca untuk Padamkan Kebakaran Bromo</t>
+        </is>
+      </c>
+      <c r="C1276" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:54:47 +0700</t>
+        </is>
+      </c>
+      <c r="D1276" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1276" t="inlineStr">
+        <is>
+          <t>Saat ini masih terdapat dua titik api di kawasan tersebut, turun dari 36 titik pada puncak kebakaran.</t>
+        </is>
+      </c>
+      <c r="F1276" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1276" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267444/menko-pmk-ungkap-kendala-modifikasi-cuaca-untuk-padamkan-kebakaran-bromo</t>
+        </is>
+      </c>
+      <c r="H1276" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/v7T1HIXrr1naqq66YB477MHNM78=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9321359/original/040865600_1786440061-Menko_PMK_Pratikno_rakor_kebakaran_bromo.jpg</t>
+        </is>
+      </c>
+      <c r="I1276" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B1277" t="inlineStr">
+        <is>
+          <t>Polisi Usut Perusakan Lahan, Direktur CV Dzarrin Dijemput Paksa di Gresik</t>
+        </is>
+      </c>
+      <c r="C1277" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:14:51 +0700</t>
+        </is>
+      </c>
+      <c r="D1277" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E1277" t="inlineStr">
+        <is>
+          <t>Direktur CV Dzarrin dijemput paksa terkait dua kasus berbeda di Pamekasan: dugaan perusakan lahan dan korupsi proyek jalan mangkrak senilai miliaran rupiah.</t>
+        </is>
+      </c>
+      <c r="F1277" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1277" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/08/11/211405478/polisi-usut-perusakan-lahan-direktur-cv-dzarrin-dijemput-paksa-di-gresik</t>
+        </is>
+      </c>
+      <c r="H1277" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/2TzBwW3DCPFeMeQ_QhMXMoq2YMU=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/11/6a7b1b17f2cdc.jpg</t>
+        </is>
+      </c>
+      <c r="I1277" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1278">
+      <c r="A1278" t="inlineStr">
+        <is>
+          <t>Cahaya</t>
+        </is>
+      </c>
+      <c r="B1278" t="inlineStr">
+        <is>
+          <t>Surat Ad-Dhuha: Arab, Latin, Arti, Makna, dan Keutamaannya</t>
+        </is>
+      </c>
+      <c r="C1278" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:14:51 +0700</t>
+        </is>
+      </c>
+      <c r="D1278" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E1278" t="inlineStr">
+        <is>
+          <t>Surat Ad-Dhuha merupakan surah ke-93 dalam Al-Qur’an yang terdiri dari 11 ayat. Berikut bacaan lengkap Arab, latin, arti, dan penjelasan lainnya.</t>
+        </is>
+      </c>
+      <c r="F1278" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1278" t="inlineStr">
+        <is>
+          <t>https://cahaya.kompas.com/aktual/26H11204414090/surat-ad-dhuha-arab-latin-arti-makna-dan-keutamaannya</t>
+        </is>
+      </c>
+      <c r="H1278" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/KGfNQwPTuUwSXgO6yDemkYULfrU=/733x0:5093x2906/1200x675/data/photo/2026/07/09/6a4f9394db337.jpg</t>
+        </is>
+      </c>
+      <c r="I1278" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1279">
+      <c r="A1279" t="inlineStr">
+        <is>
+          <t>Money</t>
+        </is>
+      </c>
+      <c r="B1279" t="inlineStr">
+        <is>
+          <t>Garuda Indonesia Sediakan 170.845 Tiket Domestik Gratis Buat Wisatawan Asing</t>
+        </is>
+      </c>
+      <c r="C1279" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:14:51 +0700</t>
+        </is>
+      </c>
+      <c r="D1279" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E1279" t="inlineStr">
+        <is>
+          <t>Garuda Indonesia (Persero) Tbk meluncurkan program free domestic flight atau penerbangan domestik gratis bagi wisatawan asing.</t>
+        </is>
+      </c>
+      <c r="F1279" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1279" t="inlineStr">
+        <is>
+          <t>https://money.kompas.com/read/2026/08/11/201836926/garuda-indonesia-sediakan-170845-tiket-domestik-gratis-buat-wisatawan-asing</t>
+        </is>
+      </c>
+      <c r="H1279" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/LKqMqZcv-AbYqee3C9YXcUvcLK0=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815e7ef28.png,0,-0,1)/data/photo/2026/08/11/6a7b1f598854c.jpg</t>
+        </is>
+      </c>
+      <c r="I1279" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I1177"/>
+  <autoFilter ref="A1:I1279"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-11 15:54 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-11.xlsx
+++ b/data/berita_2026-08-11.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1279</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1356</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1279"/>
+  <dimension ref="A1:I1356"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -60552,8 +60552,3627 @@
         </is>
       </c>
     </row>
+    <row r="1280">
+      <c r="A1280" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1280" t="inlineStr">
+        <is>
+          <t>TNI hadirkan Yuke Dewa 19 pulihkan trauma warga Aceh di momen HUT RI</t>
+        </is>
+      </c>
+      <c r="C1280" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:46:29 +0700</t>
+        </is>
+      </c>
+      <c r="D1280" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1280" t="inlineStr">
+        <is>
+          <t>TNI AD melalui Korem (Danrem) 011/Lilawangsa menghadirkan basis grup musik legendaris Dewa 19 Yuke Sampurna untuk ...</t>
+        </is>
+      </c>
+      <c r="F1280" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1280" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690031/tni-hadirkan-yuke-dewa-19-pulihkan-trauma-warga-aceh-di-momen-hut-ri</t>
+        </is>
+      </c>
+      <c r="H1280" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG-20260811-WA0025.jpg</t>
+        </is>
+      </c>
+      <c r="I1280" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1281">
+      <c r="A1281" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1281" t="inlineStr">
+        <is>
+          <t>Yaqut ajukan perlawanan atas dakwaan korupsi kuota haji</t>
+        </is>
+      </c>
+      <c r="C1281" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:43:54 +0700</t>
+        </is>
+      </c>
+      <c r="D1281" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1281" t="inlineStr">
+        <is>
+          <t>Menteri Agama periode 2020-2024 Yaqut Cholil Qoumas, melalui tim advokatnya, mengajukan perlawanan terkait kasus dugaan ...</t>
+        </is>
+      </c>
+      <c r="F1281" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1281" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690028/yaqut-ajukan-perlawanan-atas-dakwaan-korupsi-kuota-haji</t>
+        </is>
+      </c>
+      <c r="H1281" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/Yaqut-Cholil-Didakwa-Rugikan-Negara-Ratusan-Miliar-110826-Bay-3.jpg</t>
+        </is>
+      </c>
+      <c r="I1281" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1282">
+      <c r="A1282" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1282" t="inlineStr">
+        <is>
+          <t>Kemlu benarkan ABK WNI jadi korban serangan di Bab Al-Mandeb Yaman</t>
+        </is>
+      </c>
+      <c r="C1282" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:42:04 +0700</t>
+        </is>
+      </c>
+      <c r="D1282" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1282" t="inlineStr">
+        <is>
+          <t>Kementerian Luar Negeri (Kemlu) RI membenarkan informasi terkait tiga anak buah kapal (ABK) asal Indonesia yang menjadi ...</t>
+        </is>
+      </c>
+      <c r="F1282" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1282" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690024/kemlu-benarkan-abk-wni-jadi-korban-serangan-di-bab-al-mandeb-yaman</t>
+        </is>
+      </c>
+      <c r="H1282" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/08/06/create-antaranews-logo.jpg</t>
+        </is>
+      </c>
+      <c r="I1282" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1283">
+      <c r="A1283" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1283" t="inlineStr">
+        <is>
+          <t>Nusron beberkan mekanisme penyelesaian konflik agraria</t>
+        </is>
+      </c>
+      <c r="C1283" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:41:34 +0700</t>
+        </is>
+      </c>
+      <c r="D1283" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1283" t="inlineStr">
+        <is>
+          <t>Menteri Agraria dan Tata Ruang (ATR)/Kepala Badan Pertanahan Nasional (BPN) Nusron Wahid menjelaskan bahwa penyelesaian ...</t>
+        </is>
+      </c>
+      <c r="F1283" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1283" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690020/nusron-beberkan-mekanisme-penyelesaian-konflik-agraria</t>
+        </is>
+      </c>
+      <c r="H1283" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG_20260811_223144.jpg</t>
+        </is>
+      </c>
+      <c r="I1283" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1284">
+      <c r="A1284" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1284" t="inlineStr">
+        <is>
+          <t>139 SPPG Surabaya tak serap telur lokal, Mentan copot Korwil</t>
+        </is>
+      </c>
+      <c r="C1284" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:41:22 +0700</t>
+        </is>
+      </c>
+      <c r="D1284" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1284" t="inlineStr">
+        <is>
+          <t>ANTARA - Menteri Pertanian Andi Amran Sulaiman mencopot Koordinator Wilayah Kantor Pelayanan Pemenuhan Gizi Kota ...</t>
+        </is>
+      </c>
+      <c r="F1284" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1284" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5689765/139-sppg-surabaya-tak-serap-telur-lokal-mentan-copot-korwil</t>
+        </is>
+      </c>
+      <c r="H1284" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/SANS_139-SPPG-SURABAYA-TAK-SERAP-TELUR-LOKAL-MENTAN-COPOT-KORWIL.jpg</t>
+        </is>
+      </c>
+      <c r="I1284" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1285">
+      <c r="A1285" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1285" t="inlineStr">
+        <is>
+          <t>Lewat M4CR, Pelestarian Ekosistem Pesisir Jadi Kunci Ketahanan Pangan di Bulungan Kaltara</t>
+        </is>
+      </c>
+      <c r="C1285" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:38:40 +0700</t>
+        </is>
+      </c>
+      <c r="D1285" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1285" t="inlineStr">
+        <is>
+          <t>Hamparan tambak tradisional membentang luas mengikuti garis pantai di Desa Tanjung Buka, Kabupaten Bulungan, ...</t>
+        </is>
+      </c>
+      <c r="F1285" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1285" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690016/lewat-m4cr-pelestarian-ekosistem-pesisir-jadi-kunci-ketahanan-pangan-di-bulungan-kaltara</t>
+        </is>
+      </c>
+      <c r="H1285" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/Program-Mangroves-for-Coastal-Resilience.jpg</t>
+        </is>
+      </c>
+      <c r="I1285" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1286">
+      <c r="A1286" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1286" t="inlineStr">
+        <is>
+          <t>Gita Bahana Nusantara unjuk kesiapan di Pakansari jelang HUT ke-81 RI</t>
+        </is>
+      </c>
+      <c r="C1286" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:37:28 +0700</t>
+        </is>
+      </c>
+      <c r="D1286" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1286" t="inlineStr">
+        <is>
+          <t>Gita Bahana Nusantara (GBN) 2026 menunjukkan kesiapan menjelang peringatan HUT ke-81 Kemerdekaan Republik Indonesia ...</t>
+        </is>
+      </c>
+      <c r="F1286" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1286" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690013/gita-bahana-nusantara-unjuk-kesiapan-di-pakansari-jelang-hut-ke-81-ri</t>
+        </is>
+      </c>
+      <c r="H1286" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1003331040.jpg</t>
+        </is>
+      </c>
+      <c r="I1286" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1287">
+      <c r="A1287" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1287" t="inlineStr">
+        <is>
+          <t>Kabut asap memburuk, sekolah di Pontianak beralih daring</t>
+        </is>
+      </c>
+      <c r="C1287" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:35:47 +0700</t>
+        </is>
+      </c>
+      <c r="D1287" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1287" t="inlineStr">
+        <is>
+          <t>ANTARA - Pemerintah Kota Pontianak, Kalimantan Barat, mengalihkan pembelajaran tatap muka menjadi pembelajaran daring ...</t>
+        </is>
+      </c>
+      <c r="F1287" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1287" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5689769/kabut-asap-memburuk-sekolah-di-pontianak-beralih-daring</t>
+        </is>
+      </c>
+      <c r="H1287" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KABUT-ASAP-MEMBURUK-SEKOLAH-DI-PONTIANAK-BERALIH-DARING.jpg</t>
+        </is>
+      </c>
+      <c r="I1287" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1288" t="inlineStr">
+        <is>
+          <t>Asiana perkenalkan teknologi ubah sampah jadi bahan bakar alternatif</t>
+        </is>
+      </c>
+      <c r="C1288" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:32:51 +0700</t>
+        </is>
+      </c>
+      <c r="D1288" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1288" t="inlineStr">
+        <is>
+          <t>PT Asiana Technologies memperkenalkan pengolahan sampah menjadi bahan bakar alternatif berupa Refuse Derived Fuel (RDF) ...</t>
+        </is>
+      </c>
+      <c r="F1288" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1288" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690012/asiana-perkenalkan-teknologi-ubah-sampah-jadi-bahan-bakar-alternatif</t>
+        </is>
+      </c>
+      <c r="H1288" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG_20260811_220846.jpg</t>
+        </is>
+      </c>
+      <c r="I1288" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1289">
+      <c r="A1289" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1289" t="inlineStr">
+        <is>
+          <t>Komisi VII DPR minta Pemprov NTB benahi destinasi wisata Gili Tramena</t>
+        </is>
+      </c>
+      <c r="C1289" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:28:48 +0700</t>
+        </is>
+      </c>
+      <c r="D1289" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1289" t="inlineStr">
+        <is>
+          <t>Komisi VII DPR RI meminta Pemerintah Provinsi Nusa Tenggara Barat (Pemprov NTB) serius membenahi persoalan di kawasan ...</t>
+        </is>
+      </c>
+      <c r="F1289" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1289" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690011/komisi-vii-dpr-minta-pemprov-ntb-benahi-destinasi-wisata-gili-tramena</t>
+        </is>
+      </c>
+      <c r="H1289" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/b2ba4340-fd3c-4459-ac58-e54cf4341212.jpg</t>
+        </is>
+      </c>
+      <c r="I1289" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1290">
+      <c r="A1290" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1290" t="inlineStr">
+        <is>
+          <t>InJourney menyatakan Mandalika siap sambut MotoGP 2026</t>
+        </is>
+      </c>
+      <c r="C1290" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:24:07 +0700</t>
+        </is>
+      </c>
+      <c r="D1290" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1290" t="inlineStr">
+        <is>
+          <t>PT Aviasi Pariwisata Indonesia (Persero) atau InJourney menyatakan bahwa Sirkuit Internasional Pertamina ...</t>
+        </is>
+      </c>
+      <c r="F1290" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1290" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690007/injourney-menyatakan-mandalika-siap-sambut-motogp-2026</t>
+        </is>
+      </c>
+      <c r="H1290" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/WhatsApp-Image-2026-08-11-at-20.08.05.jpeg</t>
+        </is>
+      </c>
+      <c r="I1290" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1291">
+      <c r="A1291" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1291" t="inlineStr">
+        <is>
+          <t>Wagub Sumut: majukan kualitas pendidikan Nias Barat butuh kolaborasi</t>
+        </is>
+      </c>
+      <c r="C1291" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:19:09 +0700</t>
+        </is>
+      </c>
+      <c r="D1291" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1291" t="inlineStr">
+        <is>
+          <t>Wakil Gubernur (Wagub) Sumatera Utara (Sumut) Surya menegaskan, bahwa memajukan kualitas pendidikan di wilayah ...</t>
+        </is>
+      </c>
+      <c r="F1291" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1291" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690003/wagub-sumut-majukan-kualitas-pendidikan-nias-barat-butuh-kolaborasi</t>
+        </is>
+      </c>
+      <c r="H1291" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1001041644.jpg</t>
+        </is>
+      </c>
+      <c r="I1291" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1292">
+      <c r="A1292" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1292" t="inlineStr">
+        <is>
+          <t>Danantara: PSEL Yogyakarta diproyeksikan aliri listrik 15 ribu rumah</t>
+        </is>
+      </c>
+      <c r="C1292" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:15:41 +0700</t>
+        </is>
+      </c>
+      <c r="D1292" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1292" t="inlineStr">
+        <is>
+          <t>Badan Pengelola Investasi Daya Anagata Nusantara (Danantara) menyebut energi listrik yang dihasilkan dari konstruksi ...</t>
+        </is>
+      </c>
+      <c r="F1292" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1292" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690000/danantara-psel-yogyakarta-diproyeksikan-aliri-listrik-15-ribu-rumah</t>
+        </is>
+      </c>
+      <c r="H1292" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG_20260811_220510.jpg</t>
+        </is>
+      </c>
+      <c r="I1292" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1293">
+      <c r="A1293" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1293" t="inlineStr">
+        <is>
+          <t>Menkop: LPDB siap dukung koperasi bangun pabrik CPO</t>
+        </is>
+      </c>
+      <c r="C1293" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:15:11 +0700</t>
+        </is>
+      </c>
+      <c r="D1293" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1293" t="inlineStr">
+        <is>
+          <t>Menteri Koperasi Ferry Juliantono mengatakan Lembaga Pengelola Dana Bergulir (LPDB) Koperasi siap mendukung pembiayaan ...</t>
+        </is>
+      </c>
+      <c r="F1293" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1293" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689997/menkop-lpdb-siap-dukung-koperasi-bangun-pabrik-cpo</t>
+        </is>
+      </c>
+      <c r="H1293" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/tempImagePrULuy.jpg</t>
+        </is>
+      </c>
+      <c r="I1293" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1294">
+      <c r="A1294" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1294" t="inlineStr">
+        <is>
+          <t>Hanura: Caleg berkualitas jangan sampai kalah karena modal</t>
+        </is>
+      </c>
+      <c r="C1294" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:09:36 +0700</t>
+        </is>
+      </c>
+      <c r="D1294" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1294" t="inlineStr">
+        <is>
+          <t>Partai Hanura menilai sistem pemilu perlu memberikan ruang bagi calon legislatif (caleg) berkualitas agar tidak ...</t>
+        </is>
+      </c>
+      <c r="F1294" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1294" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689996/hanura-caleg-berkualitas-jangan-sampai-kalah-karena-modal</t>
+        </is>
+      </c>
+      <c r="H1294" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1000583792.jpg</t>
+        </is>
+      </c>
+      <c r="I1294" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1295">
+      <c r="A1295" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1295" t="inlineStr">
+        <is>
+          <t>Polisi kumpulkan barang bukti dugaan penistaan agama di festival musik</t>
+        </is>
+      </c>
+      <c r="C1295" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:08:37 +0700</t>
+        </is>
+      </c>
+      <c r="D1295" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1295" t="inlineStr">
+        <is>
+          <t>Polres Metro Jakarta Utara mengumpulkan barang bukti untuk menyelidiki dugaan penistaan agama yang terjadi saat ...</t>
+        </is>
+      </c>
+      <c r="F1295" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1295" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689992/polisi-kumpulkan-barang-bukti-dugaan-penistaan-agama-di-festival-musik</t>
+        </is>
+      </c>
+      <c r="H1295" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1000913154.jpg</t>
+        </is>
+      </c>
+      <c r="I1295" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1296">
+      <c r="A1296" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1296" t="inlineStr">
+        <is>
+          <t>BPBD Sleman tetapkan Siaga Darurat Kekeringan antisipasi El Nino</t>
+        </is>
+      </c>
+      <c r="C1296" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:02:56 +0700</t>
+        </is>
+      </c>
+      <c r="D1296" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1296" t="inlineStr">
+        <is>
+          <t>BPBD Kabupaten Sleman, Daerah Istimewa Yogyakarta, menetapkan Status Siaga Darurat Kekeringan melalui Keputusan Bupati ...</t>
+        </is>
+      </c>
+      <c r="F1296" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1296" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689989/bpbd-sleman-tetapkan-siaga-darurat-kekeringan-antisipasi-el-nino</t>
+        </is>
+      </c>
+      <c r="H1296" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1000050725.jpg</t>
+        </is>
+      </c>
+      <c r="I1296" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1297">
+      <c r="A1297" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1297" t="inlineStr">
+        <is>
+          <t>Agrinas siapkan percontohan plasma sawit berbasis koperasi di Sumut</t>
+        </is>
+      </c>
+      <c r="C1297" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:01:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1297" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1297" t="inlineStr">
+        <is>
+          <t>PT Agrinas Palma Nusantara (Persero) sedang menyiapkan proyek percontohan atau pilot project kemitraan pengembangan ...</t>
+        </is>
+      </c>
+      <c r="F1297" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1297" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689988/agrinas-siapkan-percontohan-plasma-sawit-berbasis-koperasi-di-sumut</t>
+        </is>
+      </c>
+      <c r="H1297" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/WhatsApp-Image-2026-08-11-at-19.13.31-2.jpeg</t>
+        </is>
+      </c>
+      <c r="I1297" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1298">
+      <c r="A1298" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1298" t="inlineStr">
+        <is>
+          <t>Polres Jakbar tahan sopir taksi online terduga pelaku pencabulan</t>
+        </is>
+      </c>
+      <c r="C1298" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:59:56 +0700</t>
+        </is>
+      </c>
+      <c r="D1298" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1298" t="inlineStr">
+        <is>
+          <t>Polres Metro Jakarta Barat menahan pria berinisial ARA (54), sopir taksi daring yang diduga ...</t>
+        </is>
+      </c>
+      <c r="F1298" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1298" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689987/polres-jakbar-tahan-sopir-taksi-online-terduga-pelaku-pencabulan</t>
+        </is>
+      </c>
+      <c r="H1298" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/11/24/1000684130.jpg</t>
+        </is>
+      </c>
+      <c r="I1298" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1299" t="inlineStr">
+        <is>
+          <t>Kaltara lepas 119 anggota pramuka ke Jambore Nasional Cibubur</t>
+        </is>
+      </c>
+      <c r="C1299" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:59:16 +0700</t>
+        </is>
+      </c>
+      <c r="D1299" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1299" t="inlineStr">
+        <is>
+          <t>ANTARA - Pemerintah Provinsi Kalimantan Utara resmi melepas seratus sembilan belas anggota Pramuka Penggalang untuk ...</t>
+        </is>
+      </c>
+      <c r="F1299" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1299" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5689963/kaltara-lepas-119-anggota-pramuka-ke-jambore-nasional-cibubur</t>
+        </is>
+      </c>
+      <c r="H1299" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Sequence-13.14_01_58_01.Still493.jpg</t>
+        </is>
+      </c>
+      <c r="I1299" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1300" t="inlineStr">
+        <is>
+          <t>Pertamina memasok 750 kl avtur untuk Super Garuda Shield 2026</t>
+        </is>
+      </c>
+      <c r="C1300" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:59:13 +0700</t>
+        </is>
+      </c>
+      <c r="D1300" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1300" t="inlineStr">
+        <is>
+          <t>PT Pertamina Patra Niaga Regional Sumatera Bagian Selatan (Sumbagsel) menyiapkan 750 kiloliter (kl) bahan bakar ...</t>
+        </is>
+      </c>
+      <c r="F1300" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1300" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689985/pertamina-memasok-750-kl-avtur-untuk-super-garuda-shield-2026</t>
+        </is>
+      </c>
+      <c r="H1300" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/654313.jpg</t>
+        </is>
+      </c>
+      <c r="I1300" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1301">
+      <c r="A1301" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1301" t="inlineStr">
+        <is>
+          <t>Komisi VII minta NTB segera tuntaskan persoalan pariwisata tiga Gili</t>
+        </is>
+      </c>
+      <c r="C1301" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:57:09 +0700</t>
+        </is>
+      </c>
+      <c r="D1301" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1301" t="inlineStr">
+        <is>
+          <t>ANTARA - Komisi VII DPR RI mendorong Pemerintah Provinsi Nusa Tenggara Barat segera menuntaskan persoalan status ...</t>
+        </is>
+      </c>
+      <c r="F1301" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1301" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5689836/komisi-vii-minta-ntb-segera-tuntaskanpersoalan-pariwisata-tiga-gili</t>
+        </is>
+      </c>
+      <c r="H1301" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/SANS_KOMISI-VII-MINTA-NTB-SEGERA-TUNTASKAN-PERSOALAN-PARIWISATA-TIGA-GILI.jpg</t>
+        </is>
+      </c>
+      <c r="I1301" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1302">
+      <c r="A1302" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1302" t="inlineStr">
+        <is>
+          <t>Usaha telur asin Cilegon produksi 2.000  per hari, tembus pasar Banten</t>
+        </is>
+      </c>
+      <c r="C1302" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:55:55 +0700</t>
+        </is>
+      </c>
+      <c r="D1302" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1302" t="inlineStr">
+        <is>
+          <t>ANTARA - Selama 19 tahun, Murod mengembangkan usaha telur asin dari produksi puluhan butir menjadi 2.000 butir per ...</t>
+        </is>
+      </c>
+      <c r="F1302" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1302" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5689959/usaha-telur-asin-cilegon-produksi-2000-per-hari-tembus-pasar-banten</t>
+        </is>
+      </c>
+      <c r="H1302" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/SANS_USAHA-TELUR-ASIN-CILEGON-PRODUKSI-2.000-PER-HARI-TEMBUS-PASAR-BANTEN.jpg</t>
+        </is>
+      </c>
+      <c r="I1302" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1303">
+      <c r="A1303" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1303" t="inlineStr">
+        <is>
+          <t>GNB sampaikan delapan poin pesan kemerdekaan jelang HUT ke-81 RI</t>
+        </is>
+      </c>
+      <c r="C1303" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:55:11 +0700</t>
+        </is>
+      </c>
+      <c r="D1303" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1303" t="inlineStr">
+        <is>
+          <t>ANTARA - Gerakan Nurani Bangsa (GNB) menggelar sarasehan dan menyampaikan delapan poin pesan kemerdekaan usai sarasehan ...</t>
+        </is>
+      </c>
+      <c r="F1303" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1303" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5689940/gnb-sampaikan-delapan-poin-pesan-kemerdekaan-jelang-hut-ke-81-ri</t>
+        </is>
+      </c>
+      <c r="H1303" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/GNB-SAMPAIKAN-DELAPAN-POIN-PESAN-KEMERDEKAAN-JELANG-HUT-KE-81-RI.jpg</t>
+        </is>
+      </c>
+      <c r="I1303" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1304">
+      <c r="A1304" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1304" t="inlineStr">
+        <is>
+          <t>Garuda dan InJourney berupaya tarik wisman ke lebih banyak destinasi</t>
+        </is>
+      </c>
+      <c r="C1304" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:54:22 +0700</t>
+        </is>
+      </c>
+      <c r="D1304" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1304" t="inlineStr">
+        <is>
+          <t>PT Garuda Indonesia (Persero) Tbk bersama PT Aviasi Pariwisata Indonesia (Persero) atau InJourney berupaya menarik ...</t>
+        </is>
+      </c>
+      <c r="F1304" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1304" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689983/garuda-dan-injourney-berupaya-tarik-wisman-ke-lebih-banyak-destinasi</t>
+        </is>
+      </c>
+      <c r="H1304" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/WhatsApp-Image-2026-08-11-at-20.07.25.jpeg</t>
+        </is>
+      </c>
+      <c r="I1304" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1305">
+      <c r="A1305" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1305" t="inlineStr">
+        <is>
+          <t>Wamenkop sebut penempatan manajer Kopdes masih dipersiapkan</t>
+        </is>
+      </c>
+      <c r="C1305" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:54:12 +0700</t>
+        </is>
+      </c>
+      <c r="D1305" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1305" t="inlineStr">
+        <is>
+          <t>Wakil Menteri Koperasi (Wamenkop) Farida Farichah mengatakan penempatan manajer Koperasi Desa/Kelurahan Merah Putih ...</t>
+        </is>
+      </c>
+      <c r="F1305" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1305" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689979/wamenkop-sebut-penempatan-manajer-kopdes-masih-dipersiapkan</t>
+        </is>
+      </c>
+      <c r="H1305" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/c79qikca.jpg</t>
+        </is>
+      </c>
+      <c r="I1305" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1306">
+      <c r="A1306" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1306" t="inlineStr">
+        <is>
+          <t>Yaqut klaim tak pernah terima uang dari kasus korupsi kuota haji</t>
+        </is>
+      </c>
+      <c r="C1306" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:47:52 +0700</t>
+        </is>
+      </c>
+      <c r="D1306" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1306" t="inlineStr">
+        <is>
+          <t>Menteri Agama periode 2020–2024 Yaqut Cholil Qoumas menyatakan tidak pernah menerima uang satu rupiah pun ...</t>
+        </is>
+      </c>
+      <c r="F1306" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1306" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689975/yaqut-klaim-tak-pernah-terima-uang-dari-kasus-korupsi-kuota-haji</t>
+        </is>
+      </c>
+      <c r="H1306" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/sidang-dakwaan-yaqut-cholil-qoumas-2838672.jpg</t>
+        </is>
+      </c>
+      <c r="I1306" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1307">
+      <c r="A1307" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1307" t="inlineStr">
+        <is>
+          <t>Kemenag penuhi janji bangun ulang MIN 5 Pidie Jaya dengan lebih layak</t>
+        </is>
+      </c>
+      <c r="C1307" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:47:20 +0700</t>
+        </is>
+      </c>
+      <c r="D1307" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1307" t="inlineStr">
+        <is>
+          <t>ANTARA - Bencana banjir bandang yang menerjang desa Mon Senong, Pidie Jaya, Aceh akhir November 2025 lalu. Tidak ...</t>
+        </is>
+      </c>
+      <c r="F1307" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1307" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5689933/kemenag-penuhi-janji-bangun-ulang-min-5-pidie-jaya-dengan-lebih-layak</t>
+        </is>
+      </c>
+      <c r="H1307" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Sequence-13.13_58_33_17.Still492.jpg</t>
+        </is>
+      </c>
+      <c r="I1307" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1308">
+      <c r="A1308" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1308" t="inlineStr">
+        <is>
+          <t>Airlangga: Fundamental ekonomi RI kuat meski hadapi dinamika global</t>
+        </is>
+      </c>
+      <c r="C1308" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:46:55 +0700</t>
+        </is>
+      </c>
+      <c r="D1308" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1308" t="inlineStr">
+        <is>
+          <t>Menteri Koordinator Bidang Perekonomian Airlangga Hartarto menegaskan fundamental ekonomi Indonesia tetap kuat didukung ...</t>
+        </is>
+      </c>
+      <c r="F1308" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1308" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689973/airlangga-fundamental-ekonomi-ri-kuat-meski-hadapi-dinamika-global</t>
+        </is>
+      </c>
+      <c r="H1308" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/47653FDE-6B7E-4613-A53F-FD6C21364C9F.jpeg</t>
+        </is>
+      </c>
+      <c r="I1308" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1309">
+      <c r="A1309" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1309" t="inlineStr">
+        <is>
+          <t>Gempa dahsyat di Kolombia akibatkan 181 orang tewas dan 1.310 terluka</t>
+        </is>
+      </c>
+      <c r="C1309" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:40:21 +0700</t>
+        </is>
+      </c>
+      <c r="D1309" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1309" t="inlineStr">
+        <is>
+          <t>Jumlah korban tewas akibat gempa bumi berkekuatan magnitudo 7,4 yang mengguncang Kolombia, Senin (10/8) meningkat ...</t>
+        </is>
+      </c>
+      <c r="F1309" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1309" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689969/gempa-dahsyat-di-kolombia-akibatkan-181-orang-tewas-dan-1310-terluka</t>
+        </is>
+      </c>
+      <c r="H1309" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/bangunan-runtuh-akibat-gempa-kuat-di-Kolombia.jpg</t>
+        </is>
+      </c>
+      <c r="I1309" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1310">
+      <c r="A1310" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1310" t="inlineStr">
+        <is>
+          <t>Spanyol imbau migran tidak mempertaruhkan nyawa untuk ke Ceuta</t>
+        </is>
+      </c>
+      <c r="C1310" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:39:15 +0700</t>
+        </is>
+      </c>
+      <c r="D1310" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1310" t="inlineStr">
+        <is>
+          <t>Menteri Luar Negeri Spanyol, Selasa, memperingatkan para migran agar tidak mempertaruhkan nyawa dengan mencoba memasuki ...</t>
+        </is>
+      </c>
+      <c r="F1310" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1310" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689968/spanyol-imbau-migran-tidak-mempertaruhkan-nyawa-untuk-ke-ceuta</t>
+        </is>
+      </c>
+      <c r="H1310" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/Ceuta-spanyol.jpg</t>
+        </is>
+      </c>
+      <c r="I1310" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1311">
+      <c r="A1311" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1311" t="inlineStr">
+        <is>
+          <t>Kemendikdasmen wujudkan sekolah sebagai rumah kedua lewat SNT 09 Gowa</t>
+        </is>
+      </c>
+      <c r="C1311" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:38:15 +0700</t>
+        </is>
+      </c>
+      <c r="D1311" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1311" t="inlineStr">
+        <is>
+          <t>Kementerian Pendidikan Dasar dan Menengah (Kemendikdasmen) berhasil mewujudkan sekolah sebagai rumah kedua bagi para ...</t>
+        </is>
+      </c>
+      <c r="F1311" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1311" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689965/kemendikdasmen-wujudkan-sekolah-sebagai-rumah-kedua-lewat-snt-09-gowa</t>
+        </is>
+      </c>
+      <c r="H1311" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1000233119.jpg</t>
+        </is>
+      </c>
+      <c r="I1311" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1312">
+      <c r="A1312" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1312" t="inlineStr">
+        <is>
+          <t>Pemerintah terus kebut penanganan Karhutla di Bromo</t>
+        </is>
+      </c>
+      <c r="C1312" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:29:28 +0700</t>
+        </is>
+      </c>
+      <c r="D1312" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1312" t="inlineStr">
+        <is>
+          <t>Menteri Koordinator Bidang Pembangunan Manusia dan Kebudayaan (Menko PMK) Pratikno menyatakan bahwa pemerintah terus ...</t>
+        </is>
+      </c>
+      <c r="F1312" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1312" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689961/pemerintah-terus-kebut-penanganan-karhutla-di-bromo</t>
+        </is>
+      </c>
+      <c r="H1312" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1000177502.jpg</t>
+        </is>
+      </c>
+      <c r="I1312" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1313">
+      <c r="A1313" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1313" t="inlineStr">
+        <is>
+          <t>Anggota DPR dorong pemberian insentif bagi ibu rumah tangga</t>
+        </is>
+      </c>
+      <c r="C1313" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:24:45 +0700</t>
+        </is>
+      </c>
+      <c r="D1313" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1313" t="inlineStr">
+        <is>
+          <t>Anggota DPR RI Viktor Bungtilu Laiskodat mendorong pemerintah memberikan insentif dan perlindungan bagi ibu rumah ...</t>
+        </is>
+      </c>
+      <c r="F1313" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1313" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689956/anggota-dpr-dorong-pemberian-insentif-bagi-ibu-rumah-tangga</t>
+        </is>
+      </c>
+      <c r="H1313" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1001231248.jpg</t>
+        </is>
+      </c>
+      <c r="I1313" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1314">
+      <c r="A1314" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1314" t="inlineStr">
+        <is>
+          <t>Menteri ESDM menjamin PNBP dari minerba dan migas dapat lampaui target</t>
+        </is>
+      </c>
+      <c r="C1314" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:24:11 +0700</t>
+        </is>
+      </c>
+      <c r="D1314" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1314" t="inlineStr">
+        <is>
+          <t>Menteri Energi dan Sumber Daya Mineral (ESDM) Bahlil Lahadalia menjamin bahwa Penerimaan Negara Bukan Pajak (PNBP) ...</t>
+        </is>
+      </c>
+      <c r="F1314" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1314" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689952/menteri-esdm-menjamin-pnbp-dari-minerba-dan-migas-dapat-lampaui-target</t>
+        </is>
+      </c>
+      <c r="H1314" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG_20260811_211723.jpg</t>
+        </is>
+      </c>
+      <c r="I1314" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1315">
+      <c r="A1315" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1315" t="inlineStr">
+        <is>
+          <t>Aceh Selatan serap dana TKD untuk normalisasi Sungai Krueng Trumon</t>
+        </is>
+      </c>
+      <c r="C1315" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:22:12 +0700</t>
+        </is>
+      </c>
+      <c r="D1315" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1315" t="inlineStr">
+        <is>
+          <t>ANTARA - Melalui dana Transfer Ke Daerah atau TKD yang diberikan oleh pemerintah pusat ke wilayah terdampak bencana, ...</t>
+        </is>
+      </c>
+      <c r="F1315" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1315" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5689919/aceh-selatan-serap-dana-tkd-untuk-normalisasi-sungai-krueng-trumon</t>
+        </is>
+      </c>
+      <c r="H1315" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Sequence-13.13_53_55_03.Still491.jpg</t>
+        </is>
+      </c>
+      <c r="I1315" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1316">
+      <c r="A1316" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1316" t="inlineStr">
+        <is>
+          <t>OJK dan Kementerian UMKM bentuk satgas perluas pembiayaan UMKM</t>
+        </is>
+      </c>
+      <c r="C1316" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:22:04 +0700</t>
+        </is>
+      </c>
+      <c r="D1316" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1316" t="inlineStr">
+        <is>
+          <t>Otoritas Jasa Keuangan (OJK) dan Kementerian Usaha Mikro, Kecil, dan Menengah (UMKM) sepakat untuk membentuk satuan ...</t>
+        </is>
+      </c>
+      <c r="F1316" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1316" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689951/ojk-dan-kementerian-umkm-bentuk-satgas-perluas-pembiayaan-umkm</t>
+        </is>
+      </c>
+      <c r="H1316" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/WhatsApp-Image-2026-08-11-at-15.19.39.jpeg</t>
+        </is>
+      </c>
+      <c r="I1316" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1317">
+      <c r="A1317" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1317" t="inlineStr">
+        <is>
+          <t>Chevrolet akan menghentikan penjualan mobil baru di pasar China</t>
+        </is>
+      </c>
+      <c r="C1317" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:17:11 +0700</t>
+        </is>
+      </c>
+      <c r="D1317" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E1317" t="inlineStr">
+        <is>
+          <t>General Motors telah mengonfirmasi bahwa Chevrolet akan berhenti menjual mobil baru di pasar China, mengakhiri ...</t>
+        </is>
+      </c>
+      <c r="F1317" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1317" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5689947/chevrolet-akan-menghentikan-penjualan-mobil-baru-di-pasar-china</t>
+        </is>
+      </c>
+      <c r="H1317" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2019/10/29/chevrolet.jpg</t>
+        </is>
+      </c>
+      <c r="I1317" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1318">
+      <c r="A1318" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1318" t="inlineStr">
+        <is>
+          <t>Harga hotel di Spanyol melonjak jelang gerhana Matahari total</t>
+        </is>
+      </c>
+      <c r="C1318" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:16:54 +0700</t>
+        </is>
+      </c>
+      <c r="D1318" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1318" t="inlineStr">
+        <is>
+          <t>Harga hotel melonjak tajam dan akomodasi di berbagai wilayah Spanyol sudah habis terjual menjelang gerhana Matahari ...</t>
+        </is>
+      </c>
+      <c r="F1318" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1318" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689943/harga-hotel-di-spanyol-melonjak-jelang-gerhana-matahari-total</t>
+        </is>
+      </c>
+      <c r="H1318" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/09/20/antarafoto-gerhana-matahari-sebagian-di-bekasi-20042023-par-2.jpg</t>
+        </is>
+      </c>
+      <c r="I1318" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1319">
+      <c r="A1319" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1319" t="inlineStr">
+        <is>
+          <t>KKP menangani 1.286 telur penyu di Sambas, hanya 96 layak ditetaskan</t>
+        </is>
+      </c>
+      <c r="C1319" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:15:27 +0700</t>
+        </is>
+      </c>
+      <c r="D1319" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1319" t="inlineStr">
+        <is>
+          <t>Kementerian Kelautan dan Perikanan (KKP) menangani 1.286 butir telur penyu yang ditemukan pada dua lokasi di Kabupaten ...</t>
+        </is>
+      </c>
+      <c r="F1319" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1319" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5689936/kkp-menangani-1286-telur-penyu-di-sambas-hanya-96-layak-ditetaskan</t>
+        </is>
+      </c>
+      <c r="H1319" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/WhatsApp-Image-2026-08-11-at-14.12.40.jpeg</t>
+        </is>
+      </c>
+      <c r="I1319" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1320">
+      <c r="A1320" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1320" t="inlineStr">
+        <is>
+          <t>Progres LRT Jakarta Fase 1B Jelang Diresmikan</t>
+        </is>
+      </c>
+      <c r="C1320" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:32:01 +0700</t>
+        </is>
+      </c>
+      <c r="D1320" t="inlineStr">
+        <is>
+          <t>Muhammad Azzam</t>
+        </is>
+      </c>
+      <c r="E1320" t="inlineStr">
+        <is>
+          <t>Pembangunan LRT Jakarta Fase 1B terus dikebut jelang peresmian. Progres konstruksinya kini telah mencapai 97,99 persen.</t>
+        </is>
+      </c>
+      <c r="F1320" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1320" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/foto-bisnis/d-8614467/progres-lrt-jakarta-fase-1b-jelang-diresmikan</t>
+        </is>
+      </c>
+      <c r="H1320" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/progres-lrt-jakarta-fase-1b-jelang-diresmikan-1786462097440.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1320" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1321">
+      <c r="A1321" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1321" t="inlineStr">
+        <is>
+          <t>Garuda Tebar 170.845 Tiket Gratis buat Wisman</t>
+        </is>
+      </c>
+      <c r="C1321" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:25:16 +0700</t>
+        </is>
+      </c>
+      <c r="D1321" t="inlineStr">
+        <is>
+          <t>Ignacio Geordi Oswaldo</t>
+        </is>
+      </c>
+      <c r="E1321" t="inlineStr">
+        <is>
+          <t>PT Garuda Indonesia (Persero) Tbk bersama PT Aviasi Pariwisata Indonesia (Persero) atau InJourney meluncurkan program peningkatan kunjungan wisatawan.</t>
+        </is>
+      </c>
+      <c r="F1321" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1321" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8614461/garuda-tebar-170-845-tiket-gratis-buat-wisman</t>
+        </is>
+      </c>
+      <c r="H1321" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2015/06/15/769bb45d-da7c-474a-b16a-8134644cb233_169.jpg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1321" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1322">
+      <c r="A1322" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1322" t="inlineStr">
+        <is>
+          <t>MSCI Segera Umumkan Rebalancing Saham, OJK Harap Pembekuan Dicabut</t>
+        </is>
+      </c>
+      <c r="C1322" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:33:02 +0700</t>
+        </is>
+      </c>
+      <c r="D1322" t="inlineStr">
+        <is>
+          <t>Ignacio Geordi Oswaldo</t>
+        </is>
+      </c>
+      <c r="E1322" t="inlineStr">
+        <is>
+          <t>OJK berharap penyedia indeks global, MSCI obyektif menilai peningkatan transparansi pasar modal Indonesia dan segera mencabut pembekuan (freeze).</t>
+        </is>
+      </c>
+      <c r="F1322" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1322" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8614415/msci-segera-umumkan-rebalancing-saham-ojk-harap-pembekuan-dicabut</t>
+        </is>
+      </c>
+      <c r="H1322" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2020/02/13/6d3c742d-cc97-4819-a6ec-77edce240296_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1322" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1323">
+      <c r="A1323" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1323" t="inlineStr">
+        <is>
+          <t>Harga Pertalite Dijamin Tidak Naik sampai Desember</t>
+        </is>
+      </c>
+      <c r="C1323" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:05:06 +0700</t>
+        </is>
+      </c>
+      <c r="D1323" t="inlineStr">
+        <is>
+          <t>Ignacio Geordi Oswaldo</t>
+        </is>
+      </c>
+      <c r="E1323" t="inlineStr">
+        <is>
+          <t>Pemerintah pastikan harga BBM subsidi aman alias tidak naik, sampai Desember.</t>
+        </is>
+      </c>
+      <c r="F1323" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1323" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8614377/harga-pertalite-dijamin-tidak-naik-sampai-desember</t>
+        </is>
+      </c>
+      <c r="H1323" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2022/09/01/antrean-di-spbu-mengular-panic-buying-isu-harga-bbm-naik-1_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1323" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1324">
+      <c r="A1324" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1324" t="inlineStr">
+        <is>
+          <t>Pekerja Informal Persampahan Dapat Keringanan Iuran Jaminan Sosial</t>
+        </is>
+      </c>
+      <c r="C1324" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:00:48 +0700</t>
+        </is>
+      </c>
+      <c r="D1324" t="inlineStr">
+        <is>
+          <t>Rifki Afifan</t>
+        </is>
+      </c>
+      <c r="E1324" t="inlineStr">
+        <is>
+          <t>Pemerintah memberi keringanan iuran jaminan sosial. Kebijakan ini menyasar pekerja informal sektor persampahan.</t>
+        </is>
+      </c>
+      <c r="F1324" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1324" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/foto-bisnis/d-8613599/pekerja-informal-persampahan-dapat-keringanan-iuran-jaminan-sosial</t>
+        </is>
+      </c>
+      <c r="H1324" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/pekerja-informal-persampahan-dapat-keringanan-iuran-jaminan-sosial-ketenagakerjaan-1786431203285_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1324" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1325">
+      <c r="A1325" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1325" t="inlineStr">
+        <is>
+          <t>Produksi Tas Travel Meningkat Jelang Musim Umrah</t>
+        </is>
+      </c>
+      <c r="C1325" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:50:45 +0700</t>
+        </is>
+      </c>
+      <c r="D1325" t="inlineStr">
+        <is>
+          <t>Muhammad Azzam</t>
+        </is>
+      </c>
+      <c r="E1325" t="inlineStr">
+        <is>
+          <t>UMKM pembuat perlengkapan umrah memproduksi ratusan tas travel setiap hari. Pesanan meningkat menjelang musim keberangkatan umrah.</t>
+        </is>
+      </c>
+      <c r="F1325" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1325" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/foto-bisnis/d-8614352/produksi-tas-travel-meningkat-jelang-musim-umrah</t>
+        </is>
+      </c>
+      <c r="H1325" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/produksi-tas-travel-meningkat-jelang-musim-umrah-1786456066313.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1325" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1326">
+      <c r="A1326" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1326" t="inlineStr">
+        <is>
+          <t>Kurang dari 24 Jam, Polisi Tangkap KF Terkait Wanita Muda Tewas di Tangerang</t>
+        </is>
+      </c>
+      <c r="C1326" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:33:32 +0700</t>
+        </is>
+      </c>
+      <c r="D1326" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1326" t="inlineStr">
+        <is>
+          <t>Kurang dari 24 jam setelah kejadian, polisi menangkap KF. Motif dan kronologi kematian wanita muda di Tangerang masih didalami.</t>
+        </is>
+      </c>
+      <c r="F1326" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1326" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7867134/kurang-dari-24-jam-polisi-tangkap-kf-terkait-wanita-muda-tewas-di-tangerang</t>
+        </is>
+      </c>
+      <c r="H1326" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/DlQgAzF77lGyDqvBt6frr4f96q0=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Ilustrasi-penangkapan-terduga-pelaku-tindak-pidana-oleh-polisi.jpg</t>
+        </is>
+      </c>
+      <c r="I1326" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1327">
+      <c r="A1327" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1327" t="inlineStr">
+        <is>
+          <t>Mata Anak Tampak Juling? Coba Cek Pakai Flash HP, Dokter Ungkap Pantulan Cahaya yang Perlu Dicermati</t>
+        </is>
+      </c>
+      <c r="C1327" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:22:27 +0700</t>
+        </is>
+      </c>
+      <c r="D1327" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1327" t="inlineStr">
+        <is>
+          <t>Mata juling atau strabismus pada anak tidak selalu muncul terus-menerus sehingga perlu pengecekan.</t>
+        </is>
+      </c>
+      <c r="F1327" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1327" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7867133/mata-anak-tampak-juling-coba-cek-pakai-flash-hp-dokter-ungkap-pantulan-cahaya-yang-perlu-dicermati</t>
+        </is>
+      </c>
+      <c r="H1327" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/oYC7Eu25ziOyR3hKvcJU_h4-zIA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/bakti-sosial-operasi-mata-juling-jec_20231015_172841.jpg</t>
+        </is>
+      </c>
+      <c r="I1327" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1328">
+      <c r="A1328" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1328" t="inlineStr">
+        <is>
+          <t>Laporan Keuangan BSSN Raih WTP, BPK Rekomendasikan Pembenahan Aset dan Belanja</t>
+        </is>
+      </c>
+      <c r="C1328" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:18:39 +0700</t>
+        </is>
+      </c>
+      <c r="D1328" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1328" t="inlineStr">
+        <is>
+          <t>BSSN meraih opini WTP untuk laporan keuangan 2025, tetapi BPK masih mencatat persoalan aset dan belanja.</t>
+        </is>
+      </c>
+      <c r="F1328" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1328" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867132/laporan-keuangan-bssn-raih-wtp-bpk-rekomendasikan-pembenahan-aset-dan-belanja</t>
+        </is>
+      </c>
+      <c r="H1328" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/arXl4_3ql_Q1vjblzpLd5xy4cXQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-bpk-ri-badan-pemeriksa-keuangan.jpg</t>
+        </is>
+      </c>
+      <c r="I1328" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1329">
+      <c r="A1329" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1329" t="inlineStr">
+        <is>
+          <t>Cadangan Tembus 1,4 Miliar Barel, China Bangun Kekuatan Minyak dari Sisi Pembeli, Bukan Produsen</t>
+        </is>
+      </c>
+      <c r="C1329" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:15:14 +0700</t>
+        </is>
+      </c>
+      <c r="D1329" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1329" t="inlineStr">
+        <is>
+          <t>China bukan merupakan salah satu produsen minyak terbesar dunia. Namun berkat kekuatan uang, mereka mampu membeli dan menstok 1,4 miliar barel minyak.</t>
+        </is>
+      </c>
+      <c r="F1329" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1329" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7867131/cadangan-tembus-14-miliar-barel-china-bangun-kekuatan-minyak-dari-sisi-pembeli-bukan-produsen</t>
+        </is>
+      </c>
+      <c r="H1329" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Q5f1SvaqZD85DlwF31QhRJge_V0=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Kapal-tanker-China-di-Selat-Hormuz.jpg</t>
+        </is>
+      </c>
+      <c r="I1329" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1330">
+      <c r="A1330" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1330" t="inlineStr">
+        <is>
+          <t>Idy Muzayyad: Banyaknya Calon Ketum PBNU Tunjukkan Demokratisasi di Internal NU</t>
+        </is>
+      </c>
+      <c r="C1330" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:14:50 +0700</t>
+        </is>
+      </c>
+      <c r="D1330" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1330" t="inlineStr">
+        <is>
+          <t>Bursa calon Ketum PBNU 2026-2031 makin dinamis. Muncul 7-8 kandidat, NU diingatkan menjaga marwah muktamar dari politik uang.</t>
+        </is>
+      </c>
+      <c r="F1330" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1330" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867130/idy-muzayyad-banyaknya-calon-ketum-pbnu-tunjukkan-demokratisasi-di-internal-nu</t>
+        </is>
+      </c>
+      <c r="H1330" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/atQNf7QsqLrIUVarl0snUrlbjIg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Wawancara-Anggota-Koordinator-Muktamar-Ke-35-PBNU-Idy-Muzayyad_20260811_170744.jpg</t>
+        </is>
+      </c>
+      <c r="I1330" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1331">
+      <c r="A1331" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1331" t="inlineStr">
+        <is>
+          <t>Perang Iran-AS Jadi Ujian AI, IRGC: Rudal Kami Berhasil Hadapi Teknologi Amerika</t>
+        </is>
+      </c>
+      <c r="C1331" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:03:21 +0700</t>
+        </is>
+      </c>
+      <c r="D1331" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1331" t="inlineStr">
+        <is>
+          <t>Teknologi militer Amerika Serikat, termasuk sistem berbasis AI, gagal memberikan keunggulan menentukan dalam menghadapi Iran.</t>
+        </is>
+      </c>
+      <c r="F1331" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1331" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7867129/perang-iran-as-jadi-ujian-ai-irgc-rudal-kami-berhasil-hadapi-teknologi-amerika</t>
+        </is>
+      </c>
+      <c r="H1331" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/nm1ZuVS7uMjwQPa9tQAPPcg-ElY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Rudal-IRGC-ke-Selat-Hormuz-OK.jpg</t>
+        </is>
+      </c>
+      <c r="I1331" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1332">
+      <c r="A1332" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1332" t="inlineStr">
+        <is>
+          <t>Suara untuk yang Tak Bisa Bicara, Pengalaman Pahit Dhisha dan Thomas Kehilangan Hewan Kesayangan</t>
+        </is>
+      </c>
+      <c r="C1332" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:02:04 +0700</t>
+        </is>
+      </c>
+      <c r="D1332" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1332" t="inlineStr">
+        <is>
+          <t>Kehadiran dokter hewan sangat krusial untuk menjadi perpanjangan suara bagi satwa-satwa yang menderita</t>
+        </is>
+      </c>
+      <c r="F1332" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1332" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/lifestyle/7867128/suara-untuk-yang-tak-bisa-bicara-pengalaman-pahit-dhisha-dan-thomas-kehilangan-hewan-kesayangan</t>
+        </is>
+      </c>
+      <c r="H1332" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/GNxXBETlpXzF3A6pTtcjT7exoZw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/suarahwan11111.jpg</t>
+        </is>
+      </c>
+      <c r="I1332" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1333">
+      <c r="A1333" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1333" t="inlineStr">
+        <is>
+          <t>Dikawal Polisi, Oknum Tenaga Kesehatan yang Sempat Bully Pasien BPJS Yurizal Datang ke Bogor</t>
+        </is>
+      </c>
+      <c r="C1333" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:59:09 +0700</t>
+        </is>
+      </c>
+      <c r="D1333" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1333" t="inlineStr">
+        <is>
+          <t>Dua oknum nakes yang sempat membully Yurizal datang ke Bogor meminta maaf kepada keluarga almarhum. Permintaan maaf diterima.</t>
+        </is>
+      </c>
+      <c r="F1333" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1333" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867127/dikawal-polisi-oknum-tenaga-kesehatan-yang-sempat-bully-pasien-bpjs-yurizal-datang-ke-bogor</t>
+        </is>
+      </c>
+      <c r="H1333" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/8RxfNXKwalnCup3VRnRm31keznc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/makam-yurizal-1.jpg</t>
+        </is>
+      </c>
+      <c r="I1333" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1334">
+      <c r="A1334" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1334" t="inlineStr">
+        <is>
+          <t>192 Ribu Bibit Kopi Dihibahkan, Tunas Bumi Fest 2026 Bawa Pesan Menjaga Hutan Wonosobo</t>
+        </is>
+      </c>
+      <c r="C1334" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:55:24 +0700</t>
+        </is>
+      </c>
+      <c r="D1334" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1334" t="inlineStr">
+        <is>
+          <t>Bibit tersebut diberikan kepada Lembaga Masyarakat Desa Hutan (LMDH) dan Kelompok Tani Hutan (KTH)</t>
+        </is>
+      </c>
+      <c r="F1334" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1334" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7867126/192-ribu-bibit-kopi-dihibahkan-tunas-bumi-fest-2026-bawa-pesan-menjaga-hutan-wonosobo</t>
+        </is>
+      </c>
+      <c r="H1334" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/tGVKeIsZzV7MxZZgpfkj-969KM8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Jatubu-Fest111111.jpg</t>
+        </is>
+      </c>
+      <c r="I1334" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1335">
+      <c r="A1335" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1335" t="inlineStr">
+        <is>
+          <t>Koalisi Sipil Kritik Klaim Panglima TNI Bertanggung Jawab atas Kamtibmas</t>
+        </is>
+      </c>
+      <c r="C1335" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:54:27 +0700</t>
+        </is>
+      </c>
+      <c r="D1335" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1335" t="inlineStr">
+        <is>
+          <t>Klaim Panglima TNI soal keamanan masyarakat menuai kritik. Koalisi Sipil mengingatkan batas kewenangan TNI dan Polri.</t>
+        </is>
+      </c>
+      <c r="F1335" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1335" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867125/koalisi-sipil-kritik-klaim-panglima-tni-bertanggung-jawab-atas-kamtibmas</t>
+        </is>
+      </c>
+      <c r="H1335" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/E3QMa9fa3HNSU927YKwVdeDFlnM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Presiden-Prabowo-Hadiri-Upacara-Gelar-Pasukan-dan-Kehormatan-Mil_20250811_110806.jpg</t>
+        </is>
+      </c>
+      <c r="I1335" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1336">
+      <c r="A1336" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1336" t="inlineStr">
+        <is>
+          <t>Jelang Team Launching, Persija TC di Thailand dan Tantang Brisbane Roar</t>
+        </is>
+      </c>
+      <c r="C1336" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:49:54 +0700</t>
+        </is>
+      </c>
+      <c r="D1336" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1336" t="inlineStr">
+        <is>
+          <t>Persija bersiap menyambut Super League 2026/2027 dengan TC di Thailand sebelum meluncurkan tim dan menghadapi Brisbane Roar di JIS.</t>
+        </is>
+      </c>
+      <c r="F1336" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1336" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7867124/jelang-team-launching-persija-tc-di-thailand-dan-tantang-brisbane-roar</t>
+        </is>
+      </c>
+      <c r="H1336" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/crXao2yo-UjEX99RtPnK3s3JExo=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Pemain-Persija-Jakarta-berfoto-bersama-menjelang-laga-perdana-Grup-B-Piala-Presiden-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I1336" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1337">
+      <c r="A1337" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1337" t="inlineStr">
+        <is>
+          <t>Pakar Ingatkan RUU Perampasan Aset Harus Cegah Kekuasaan Dipakai Bungkam Lawan Politik</t>
+        </is>
+      </c>
+      <c r="C1337" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:49:36 +0700</t>
+        </is>
+      </c>
+      <c r="D1337" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1337" t="inlineStr">
+        <is>
+          <t>Ia meminta agar RUU Perampasan Aset secara tegas memberikan jaminan, kewenangan negara tidak dapat disalahgunakan untuk kepentingan politik.</t>
+        </is>
+      </c>
+      <c r="F1337" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1337" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867123/pakar-ingatkan-ruu-perampasan-aset-harus-cegah-kekuasaan-dipakai-bungkam-lawan-politik</t>
+        </is>
+      </c>
+      <c r="H1337" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/qglOIrg4c3lXIy6rB43f30cKECI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/perampasan-aset-skjd.jpg</t>
+        </is>
+      </c>
+      <c r="I1337" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1338">
+      <c r="A1338" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1338" t="inlineStr">
+        <is>
+          <t>Cristiano Ronaldo Sudah Rindu Al Nassr, Rekan Senegara Sudah Gabung Duluan</t>
+        </is>
+      </c>
+      <c r="C1338" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:49:22 +0700</t>
+        </is>
+      </c>
+      <c r="D1338" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1338" t="inlineStr">
+        <is>
+          <t>Cristiano Ronaldo akan kembali ke Al Nassr pada tengah pekan ini untuk berlatih bersama rekan-rekannya menjelang musim 2026/2027.</t>
+        </is>
+      </c>
+      <c r="F1338" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1338" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7867122/cristiano-ronaldo-sudah-rindu-al-nassr-rekan-senegara-sudah-gabung-duluan</t>
+        </is>
+      </c>
+      <c r="H1338" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Cyib7FLfUSF10TPgO8ouC9PoF_0=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Logo-klub-Liga-Arab-Saudi-Al-Nassr.jpg</t>
+        </is>
+      </c>
+      <c r="I1338" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1339">
+      <c r="A1339" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1339" t="inlineStr">
+        <is>
+          <t>Ketahanan Air Masuk Prioritas Nasional, AHY Tekankan Pentingnya Kolaborasi</t>
+        </is>
+      </c>
+      <c r="C1339" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:49:04 +0700</t>
+        </is>
+      </c>
+      <c r="D1339" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1339" t="inlineStr">
+        <is>
+          <t>Pemerintah menempatkan ketahanan air atau water security sebagai salah satu prioritas utama pembangunan nasional, sejajar dengan ketahanan pangan.</t>
+        </is>
+      </c>
+      <c r="F1339" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1339" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867121/ketahanan-air-masuk-prioritas-nasional-ahy-tekankan-pentingnya-kolaborasi</t>
+        </is>
+      </c>
+      <c r="H1339" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/AkC4VRXFN4MZJlBqD48-39W7e_g=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ahy-air-pangan-as.jpg</t>
+        </is>
+      </c>
+      <c r="I1339" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1340">
+      <c r="A1340" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1340" t="inlineStr">
+        <is>
+          <t>Habis Manis Sepah Dibuang: Paul Munster Out, Bhayangkara FC Depak Juru Penyelamat</t>
+        </is>
+      </c>
+      <c r="C1340" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:45:41 +0700</t>
+        </is>
+      </c>
+      <c r="D1340" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1340" t="inlineStr">
+        <is>
+          <t>Kabar mengejutkan datang dari Bhayangkara FC yang resmi memutuskan untuk berpisah dengan Paul Munster sebagai pelatih.</t>
+        </is>
+      </c>
+      <c r="F1340" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1340" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7867120/habis-manis-sepah-dibuang-paul-munster-out-bhayangkara-fc-depak-juru-penyelamat</t>
+        </is>
+      </c>
+      <c r="H1340" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/vSmPHoAl2A9WDAiJstoz1nFTN1w=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Potret-aksi-duel-Bhayangkara-FC-vs-Persita-Tangerang-di-pekan-ke-11-Super-League.jpg</t>
+        </is>
+      </c>
+      <c r="I1340" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1341">
+      <c r="A1341" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1341" t="inlineStr">
+        <is>
+          <t>35.936 Peserta Kapolri Cup 2026, Esports dan Tantangan Literasi Finansial</t>
+        </is>
+      </c>
+      <c r="C1341" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:44:24 +0700</t>
+        </is>
+      </c>
+      <c r="D1341" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1341" t="inlineStr">
+        <is>
+          <t>Kompetisi yang digelar di Indonesia Arena, Gelora Bung Karno itu menghadirkan pertandingan Mobile Legends: Bang Bang (MLBB)</t>
+        </is>
+      </c>
+      <c r="F1341" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1341" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/e-sport/7867119/35936-peserta-kapolri-cup-2026-esports-dan-tantangan-literasi-finansial</t>
+        </is>
+      </c>
+      <c r="H1341" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/GWYK-VELKrbWWVxgCrLj_83cI1g=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/PENGEMBANGAN-TALENTA-Esports-Kapolri-Cup-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I1341" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1342">
+      <c r="A1342" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1342" t="inlineStr">
+        <is>
+          <t>Ukraina Digempur Rudal dan 120 Drone, Zelensky Tuding Rusia Pakai Senjata Korut</t>
+        </is>
+      </c>
+      <c r="C1342" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:36:25 +0700</t>
+        </is>
+      </c>
+      <c r="D1342" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1342" t="inlineStr">
+        <is>
+          <t>Selain rudal, Rusia juga dilaporkan mengerahkan lebih dari 120 drone dalam serangan malam hingga pagi hari.</t>
+        </is>
+      </c>
+      <c r="F1342" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1342" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7867118/ukraina-digempur-rudal-dan-120-drone-zelensky-tuding-rusia-pakai-senjata-korut</t>
+        </is>
+      </c>
+      <c r="H1342" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/t1lTPJsAvsM7FM8Z_QMNTGn3ar0=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/DIHANTAM-RUDAL-BALISTIK-Ibu-kota-Ukraina-Kiev-diserang-oleh-Rusia.jpg</t>
+        </is>
+      </c>
+      <c r="I1342" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1343">
+      <c r="A1343" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1343" t="inlineStr">
+        <is>
+          <t>Mengubah Sampah Menjadi Bahan Bakar, Mengapa Sampah Basah Jadi Kendala?</t>
+        </is>
+      </c>
+      <c r="C1343" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:34:47 +0700</t>
+        </is>
+      </c>
+      <c r="D1343" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1343" t="inlineStr">
+        <is>
+          <t>Salah satu teknologi yang dikembangkan untuk menjawab persoalan tersebut adalah Refuse Derived Fuel (RDF), yakni bahan bakar yang dibuat dari sampah</t>
+        </is>
+      </c>
+      <c r="F1343" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1343" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867117/mengubah-sampah-menjadi-bahan-bakar-mengapa-sampah-basah-jadi-kendala</t>
+        </is>
+      </c>
+      <c r="H1343" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Xsb5OdhuvaqkqAmy-k6mese8NsY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/sampahbasah111111.jpg</t>
+        </is>
+      </c>
+      <c r="I1343" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1344">
+      <c r="A1344" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1344" t="inlineStr">
+        <is>
+          <t>Haaland Puncaki Daftar Gaji Liga Inggris 2026/2027, Rashford Punya Keuntungan dari Klausul Lama</t>
+        </is>
+      </c>
+      <c r="C1344" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:27:17 +0700</t>
+        </is>
+      </c>
+      <c r="D1344" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1344" t="inlineStr">
+        <is>
+          <t>Daftar 10 pemain dengan gaji tertinggi di Liga Inggris 2026/2027, dengan Haaland teratas yang mendapatkan bayaran sekitar Rp12 miliar per pekan.</t>
+        </is>
+      </c>
+      <c r="F1344" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1344" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7867116/haaland-puncaki-daftar-gaji-liga-inggris-20262027-rashford-punya-keuntungan-dari-klausul-lama</t>
+        </is>
+      </c>
+      <c r="H1344" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/5JoIgZ4U65E-o8goXbBIyLYIWEI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Logo-kompetisi-Liga-Inggris-atau-Premier-League.jpg</t>
+        </is>
+      </c>
+      <c r="I1344" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1345">
+      <c r="A1345" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1345" t="inlineStr">
+        <is>
+          <t>Siap Nikah Tahun Depan, Jonathan Frizzy Sebut Ririn Dwi Ariyanti Soulmate Sempurna</t>
+        </is>
+      </c>
+      <c r="C1345" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:24:40 +0700</t>
+        </is>
+      </c>
+      <c r="D1345" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1345" t="inlineStr">
+        <is>
+          <t>Jonathan Frizzy dan Ririn Dwi Ariyanti mantap melangkah ke jenjang pernikahan. Keduanya meminta doa agar rencana baik mereka berjalan lancar.</t>
+        </is>
+      </c>
+      <c r="F1345" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1345" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7867115/siap-nikah-tahun-depan-jonathan-frizzy-sebut-ririn-dwi-ariyanti-soulmate-sempurna</t>
+        </is>
+      </c>
+      <c r="H1345" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/08xUXEebGRYmJGQUXu1SOcDzb4w=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Momen-kebersamaan-Jonathan-Frizzy-dan-Ririn-Dwi-Ariyanti.jpg</t>
+        </is>
+      </c>
+      <c r="I1345" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1346">
+      <c r="A1346" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B1346" t="inlineStr">
+        <is>
+          <t>Diam-Diam Pengendali Emiten Ini Borong 204 Juta Saham di Harga Rp210</t>
+        </is>
+      </c>
+      <c r="C1346" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:35:33 +0700</t>
+        </is>
+      </c>
+      <c r="D1346" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1346" t="inlineStr">
+        <is>
+          <t>Pengendali emiten di bidang pengolahan singkong, PT Budi Starch dan Sweetener (BUDI), Budi Delta Swakarya memborong 204 juta saham (4,54%) perseroan.</t>
+        </is>
+      </c>
+      <c r="F1346" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1346" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260811172750-17-758384/diam-diam-pengendali-emiten-ini-borong-204-juta-saham-di-harga-rp210</t>
+        </is>
+      </c>
+      <c r="H1346" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2019/06/21/ab14131b-0e21-4f01-adff-754949cf6ace_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1346" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1347">
+      <c r="A1347" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B1347" t="inlineStr">
+        <is>
+          <t>RANS Ungkap Penggunaan Dana Hasil IPO, Nagita: Buat Pelunasan Utang</t>
+        </is>
+      </c>
+      <c r="C1347" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:50:08 +0700</t>
+        </is>
+      </c>
+      <c r="D1347" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1347" t="inlineStr">
+        <is>
+          <t>RANS Entertainment, milik Raffi Ahmad, alokasikan dana IPO untuk pelunasan utang dan pengembangan bisnis. Kerja sama strategis dengan Mayora juga diumumkan.</t>
+        </is>
+      </c>
+      <c r="F1347" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1347" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260811180008-17-758395/rans-ungkap-penggunaan-dana-hasil-ipo-nagita-buat-pelunasan-utang</t>
+        </is>
+      </c>
+      <c r="H1347" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/07/27/pt-rans-entertainmen-indonesia-tbk-rans-1785124527605_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1347" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1348">
+      <c r="A1348" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B1348" t="inlineStr">
+        <is>
+          <t>Emiten RI Ini Mau Caplok 1 Pabrik Gula Jumbo dan Bangun 2 Pabrik Baru</t>
+        </is>
+      </c>
+      <c r="C1348" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:35:01 +0700</t>
+        </is>
+      </c>
+      <c r="D1348" t="inlineStr">
+        <is>
+          <t>Romys Binekasri</t>
+        </is>
+      </c>
+      <c r="E1348" t="inlineStr">
+        <is>
+          <t>Emiten produsen gula, PT Aman Agrindo Tbk (GULA) saat ini tengah menjalankan tiga proyek strategis.</t>
+        </is>
+      </c>
+      <c r="F1348" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1348" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260811171357-17-758379/emiten-ri-ini-mau-caplok-1-pabrik-gula-jumbo-dan-bangun-2-pabrik-baru</t>
+        </is>
+      </c>
+      <c r="H1348" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/06/30/layar-menampilkan-pergerakan-indeks-harga-saham-gabungan-ihsg-di-bursa-efek-indonesia-bei-jakarta-selasa-3062026-1782797018492_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1348" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1349">
+      <c r="A1349" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B1349" t="inlineStr">
+        <is>
+          <t>Video: Efek RKAB-Biaya BBM Naik, Penambang Tunda Beli Truk-Alat Berat</t>
+        </is>
+      </c>
+      <c r="C1349" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:00:44 +0700</t>
+        </is>
+      </c>
+      <c r="D1349" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1349" t="inlineStr">
+        <is>
+          <t>RKAB - Biaya BBM Naik Bikin Penambang Tunda Beli Alat Berat, Distributor Kena Imbasnya</t>
+        </is>
+      </c>
+      <c r="F1349" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1349" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260811170703-19-758376/video-efek-rkab-biaya-bbm-naik-penambang-tunda-beli-truk-alat-berat</t>
+        </is>
+      </c>
+      <c r="H1349" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/rkab-biaya-bbm-naik-bikin-penambang-tunda-beli-alat-berat-distributor-kena-imbasnya-1786443365369_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1349" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1350">
+      <c r="A1350" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="B1350" t="inlineStr">
+        <is>
+          <t>Purbaya Ungkap Ada Ide Keuntungan Danantara Masuk APBN</t>
+        </is>
+      </c>
+      <c r="C1350" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:00:18 +0700</t>
+        </is>
+      </c>
+      <c r="D1350" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1350" t="inlineStr">
+        <is>
+          <t>Menkeu Purbaya Yudhi Sadewa menyatakan keuntungan BPI Danantara akan disalurkan ke APBN. Pendapatan Danantara melonjak 400% dalam setahun.</t>
+        </is>
+      </c>
+      <c r="F1350" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1350" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/market/20260811165448-17-758362/purbaya-ungkap-ada-ide-keuntungan-danantara-masuk-apbn</t>
+        </is>
+      </c>
+      <c r="H1350" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/menteri-esdm-bahlil-lahadalia-dan-menteri-keuangan-purbaya-yudhi-sadewa-usai-melakukan-pertemuan-di-kantor-kementerian-keuanga-1786439887710_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1350" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1351">
+      <c r="A1351" t="inlineStr">
+        <is>
+          <t>Otomotif</t>
+        </is>
+      </c>
+      <c r="B1351" t="inlineStr">
+        <is>
+          <t>Daihatsu Catatkan 591 SPK Sepanjang GIIAS 2026, Sigra Jadi Model Terlaris</t>
+        </is>
+      </c>
+      <c r="C1351" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:29:28 +0700</t>
+        </is>
+      </c>
+      <c r="D1351" t="inlineStr">
+        <is>
+          <t>Israr Itah</t>
+        </is>
+      </c>
+      <c r="E1351" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, TANGERANG -- Daihatsu menutup partisipasinya di Gaikindo Indonesia International Auto Show (GIIAS) 2026 dengan hasil positif. Selama 11 hari penyelenggaraan pameran di ICE BSD, Tangerang, merek otomotif asal Jepang...</t>
+        </is>
+      </c>
+      <c r="F1351" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1351" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjm314348/daihatsu-catatkan-591-spk-sepanjang-giias-2026-sigra-jadi-model-terlaris</t>
+        </is>
+      </c>
+      <c r="H1351" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/_260729232327-626.png</t>
+        </is>
+      </c>
+      <c r="I1351" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="1352">
+      <c r="A1352" t="inlineStr">
+        <is>
+          <t>Bisnis</t>
+        </is>
+      </c>
+      <c r="B1352" t="inlineStr">
+        <is>
+          <t>Laba BUMN Melejit, Ada yang Naik 804 Persen dalam Enam Bulan</t>
+        </is>
+      </c>
+      <c r="C1352" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:56:45 +0700</t>
+        </is>
+      </c>
+      <c r="D1352" t="inlineStr">
+        <is>
+          <t>Satria K Yudha</t>
+        </is>
+      </c>
+      <c r="E1352" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA – Sejumlah badan usaha milik negara (BUMN) mencatat pertumbuhan laba signifikan pada semester I 2026, termasuk perusahaan yang sebelumnya mengalami tekanan kinerja. Capaian tersebut menunjukkan adanya perbaikan pada...</t>
+        </is>
+      </c>
+      <c r="F1352" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1352" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjm1dc416/laba-bumn-melejit-ada-yang-naik-804-persen-dalam-enam-bulan</t>
+        </is>
+      </c>
+      <c r="H1352" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/_241119101508-198.png</t>
+        </is>
+      </c>
+      <c r="I1352" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="1353">
+      <c r="A1353" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1353" t="inlineStr">
+        <is>
+          <t>Ditangkap, Ini Tampang Pelaku Pembunuhan dan Pemerkosaan di Tangerang</t>
+        </is>
+      </c>
+      <c r="C1353" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:00:44 +0700</t>
+        </is>
+      </c>
+      <c r="D1353" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1353" t="inlineStr">
+        <is>
+          <t>Polisi menangkap kurang dari 24 jam setelah pelaku melancarkan aksinya.</t>
+        </is>
+      </c>
+      <c r="F1353" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1353" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267522/ditangkap-ini-tampang-pelaku-pembunuhan-dan-pemerkosaan-di-tangerang</t>
+        </is>
+      </c>
+      <c r="H1353" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/PZAYEojI2eFEzzJmj0KuNbn2kMI=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9321632/original/052176900_1786460436-a71e799a-7631-4261-b3b3-a253ab4faad9.jpg</t>
+        </is>
+      </c>
+      <c r="I1353" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1354">
+      <c r="A1354" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1354" t="inlineStr">
+        <is>
+          <t>Mantan Stafsus Yaqut Didakwa Terima 5,2 Juta Dolar AS dan Rp 330 Juta dari Korupsi Kuota Haji</t>
+        </is>
+      </c>
+      <c r="C1354" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:54:04 +0700</t>
+        </is>
+      </c>
+      <c r="D1354" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E1354" t="inlineStr">
+        <is>
+          <t>Eks staf khusus Menteri Agama Yaqut Cholil Qoumas, Ishfah Abidal Azis alias Gus Alex didakwa menerima uang sebesar 5,2 juta dolar AS dan Rp 330 juta.</t>
+        </is>
+      </c>
+      <c r="F1354" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1354" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/08/11/22514641/mantan-stafsus-yaqut-didakwa-terima-52-juta-dolar-as-dan-rp-330-juta-dari</t>
+        </is>
+      </c>
+      <c r="H1354" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/mkdPAvRjMX48rozLcZBVJ_5s3KM=/479x107:2994x1784/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/01/26/6977470578a63.jpeg</t>
+        </is>
+      </c>
+      <c r="I1354" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1355">
+      <c r="A1355" t="inlineStr">
+        <is>
+          <t>Cahaya</t>
+        </is>
+      </c>
+      <c r="B1355" t="inlineStr">
+        <is>
+          <t>Contoh Teks Doa Upacara 17 Agustus 2026 pada Peringatan HUT Ke-81 RI</t>
+        </is>
+      </c>
+      <c r="C1355" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:54:04 +0700</t>
+        </is>
+      </c>
+      <c r="D1355" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E1355" t="inlineStr">
+        <is>
+          <t>Contoh teks doa upacara HUT ke-81 RI pada 17 Agustus 2026 untuk dibacakan saat upacara Hari Kemerdekaan Republik Indonesia.</t>
+        </is>
+      </c>
+      <c r="F1355" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1355" t="inlineStr">
+        <is>
+          <t>https://cahaya.kompas.com/doa-dan-niat/26H11220103190/contoh-teks-doa-upacara-17-agustus-2026-pada-peringatan-hut-ke-81-ri</t>
+        </is>
+      </c>
+      <c r="H1355" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/uPHZcq5iiOIr4YuWHvYAi1_Pq-Y=/0x0:2048x1365/1200x675/data/photo/2025/11/24/69242af6309cc.jpg</t>
+        </is>
+      </c>
+      <c r="I1355" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1356">
+      <c r="A1356" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B1356" t="inlineStr">
+        <is>
+          <t>Dugaan Penyebab Kecelakaan Drag Race Kotamobagu Sulut yang Tewaskan 8 Penonton</t>
+        </is>
+      </c>
+      <c r="C1356" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:54:04 +0700</t>
+        </is>
+      </c>
+      <c r="D1356" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E1356" t="inlineStr">
+        <is>
+          <t>'Semuanya ini masih kita lengkapi, masih kita kembangkan untuk sekali lagi membuat terang perkara ini,' ujarnya.</t>
+        </is>
+      </c>
+      <c r="F1356" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1356" t="inlineStr">
+        <is>
+          <t>https://makassar.kompas.com/read/2026/08/11/210628478/dugaan-penyebab-kecelakaan-drag-race-kotamobagu-sulut-yang-tewaskan-8</t>
+        </is>
+      </c>
+      <c r="H1356" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/qJYtu36N4ZY_lhfCKp-c_wVdyI0=/46x9:1024x662/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/10/6a7952569bb7e.png</t>
+        </is>
+      </c>
+      <c r="I1356" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I1279"/>
+  <autoFilter ref="A1:I1356"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-11 16:48 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-11.xlsx
+++ b/data/berita_2026-08-11.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1356</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1397</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1356"/>
+  <dimension ref="A1:I1397"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -64171,8 +64171,1935 @@
         </is>
       </c>
     </row>
+    <row r="1357">
+      <c r="A1357" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1357" t="inlineStr">
+        <is>
+          <t>KP2MI ungkap opsi, kuota sektor kerja Program SMK Go Global tahun ini</t>
+        </is>
+      </c>
+      <c r="C1357" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 23:42:33 +0700</t>
+        </is>
+      </c>
+      <c r="D1357" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1357" t="inlineStr">
+        <is>
+          <t>Kementerian Pelindungan Pekerja Migran Indonesia (KP2MI) mengungkapkan detail jumlah kebutuhan tenaga kerja, bidang ...</t>
+        </is>
+      </c>
+      <c r="F1357" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1357" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690080/kp2mi-ungkap-opsi-kuota-sektor-kerja-program-smk-go-global-tahun-ini</t>
+        </is>
+      </c>
+      <c r="H1357" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/WhatsApp-Image-2026-08-05-at-13.28.21.jpeg</t>
+        </is>
+      </c>
+      <c r="I1357" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1358">
+      <c r="A1358" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1358" t="inlineStr">
+        <is>
+          <t>KY pastikan proses seleksi calon hakim agung-ad hoc transparan</t>
+        </is>
+      </c>
+      <c r="C1358" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 23:31:52 +0700</t>
+        </is>
+      </c>
+      <c r="D1358" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1358" t="inlineStr">
+        <is>
+          <t>Komisi Yudisial memastikan pelaksanaan seleksi calon hakim agung, calon hakim ad hoc hak asasi manusia, dan calon ...</t>
+        </is>
+      </c>
+      <c r="F1358" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1358" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690069/ky-pastikan-proses-seleksi-calon-hakim-agung-ad-hoc-transparan</t>
+        </is>
+      </c>
+      <c r="H1358" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000012883_1.jpg</t>
+        </is>
+      </c>
+      <c r="I1358" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1359">
+      <c r="A1359" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1359" t="inlineStr">
+        <is>
+          <t>Ketahanan pangan, Kowani dorong hilirisasi singkong berbasis perempuan</t>
+        </is>
+      </c>
+      <c r="C1359" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 23:31:06 +0700</t>
+        </is>
+      </c>
+      <c r="D1359" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1359" t="inlineStr">
+        <is>
+          <t>Kongres Wanita Indonesia (Kowani) mendorong pengembangan hilirisasi singkong berbasis perempuan sebagai bagian dari ...</t>
+        </is>
+      </c>
+      <c r="F1359" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1359" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690065/ketahanan-pangan-kowani-dorong-hilirisasi-singkong-berbasis-perempuan</t>
+        </is>
+      </c>
+      <c r="H1359" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/WhatsApp-Image-2026-08-11-at-14.12.22.jpg</t>
+        </is>
+      </c>
+      <c r="I1359" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1360">
+      <c r="A1360" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1360" t="inlineStr">
+        <is>
+          <t>Kantor Imigrasi Mimika deportasi WNA asal PNG</t>
+        </is>
+      </c>
+      <c r="C1360" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 23:30:24 +0700</t>
+        </is>
+      </c>
+      <c r="D1360" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1360" t="inlineStr">
+        <is>
+          <t>Kantor Imigrasi Kelas II TPI Mimika mendeportasi seorang warga negara asing (WNA) asal Papua New Guinea (PNG) yang ...</t>
+        </is>
+      </c>
+      <c r="F1360" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1360" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690063/kantor-imigrasi-mimika-deportasi-wna-asal-png</t>
+        </is>
+      </c>
+      <c r="H1360" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/Imigrasi-Timika_1.jpg</t>
+        </is>
+      </c>
+      <c r="I1360" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1361">
+      <c r="A1361" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1361" t="inlineStr">
+        <is>
+          <t>InJourney dukung “Free Add-on Domestic Flight” Garuda Indonesia</t>
+        </is>
+      </c>
+      <c r="C1361" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 23:24:57 +0700</t>
+        </is>
+      </c>
+      <c r="D1361" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1361" t="inlineStr">
+        <is>
+          <t>ANTARA - InJourney dan Garuda Indonesia berkolaborasi mendorong kedatangan turis luar negeri lewat layanan “Free ...</t>
+        </is>
+      </c>
+      <c r="F1361" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1361" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5690047/injourney-dukung-free-add-on-domestic-flight-garuda-indonesia</t>
+        </is>
+      </c>
+      <c r="H1361" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/INJOURNEY-DUKUNG-22FREE-ADD-ON-DOMESTIC-FLIGHT-22-GARUDA-INDONESIA.jpg</t>
+        </is>
+      </c>
+      <c r="I1361" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1362">
+      <c r="A1362" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1362" t="inlineStr">
+        <is>
+          <t>Kasus korupsi haji, eks Stafsus Yaqut didakwa perkaya diri Rp93 miliar</t>
+        </is>
+      </c>
+      <c r="C1362" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 23:21:06 +0700</t>
+        </is>
+      </c>
+      <c r="D1362" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1362" t="inlineStr">
+        <is>
+          <t>Mantan Staf Khusus Yaqut Cholil Qoumas, Ishfah Abidal Aziz alias Gus Alex ,didakwa memperkaya diri senilai Rp93,42 ...</t>
+        </is>
+      </c>
+      <c r="F1362" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1362" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690060/kasus-korupsi-haji-eks-stafsus-yaqut-didakwa-perkaya-diri-rp93-miliar</t>
+        </is>
+      </c>
+      <c r="H1362" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/sidang-perdana-gus-alex-2838669.jpg</t>
+        </is>
+      </c>
+      <c r="I1362" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1363">
+      <c r="A1363" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1363" t="inlineStr">
+        <is>
+          <t>Olimpiade Informatika Internasional dibuka di Uzbekistan untuk kali pertama</t>
+        </is>
+      </c>
+      <c r="C1363" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 23:16:54 +0700</t>
+        </is>
+      </c>
+      <c r="D1363" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1363" t="inlineStr">
+        <is>
+          <t>Olimpiade Informatika Internasional ke-38 (IOI 2026) dibuka pada hari Senin di ibu kota Uzbekistan, Tashkent, menurut ...</t>
+        </is>
+      </c>
+      <c r="F1363" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1363" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690056/olimpiade-informatika-internasional-dibuka-di-uzbekistan-untuk-kali-pertama</t>
+        </is>
+      </c>
+      <c r="H1363" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/CjkinzN000016_20260811_CBMFN0A001.jpeg</t>
+        </is>
+      </c>
+      <c r="I1363" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1364">
+      <c r="A1364" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1364" t="inlineStr">
+        <is>
+          <t>Kejaksaan amankan uang Rp1,98 miliar dari kasus korupsi DPRD Ponorogo</t>
+        </is>
+      </c>
+      <c r="C1364" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 23:15:07 +0700</t>
+        </is>
+      </c>
+      <c r="D1364" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1364" t="inlineStr">
+        <is>
+          <t>ANTARA - Kejaksaan Negeri (Kejari) Ponorogo mengamankan uang senilai Rp 1,24 miliar dari penanganan kasus dugaan ...</t>
+        </is>
+      </c>
+      <c r="F1364" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1364" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5690043/kejaksaan-amankan-uang-rp198-miliar-dari-kasus-korupsi-dprd-ponorogo</t>
+        </is>
+      </c>
+      <c r="H1364" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KEJAKSAAN-AMANKAN-UANG-RP1-98-MILIAR-DARI-KASUS-KORUPSI-DPRD-PONOROGO.jpg</t>
+        </is>
+      </c>
+      <c r="I1364" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1365">
+      <c r="A1365" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1365" t="inlineStr">
+        <is>
+          <t>Wuling rangkum ribuan SPK dalam pameran GIIAS 2026</t>
+        </is>
+      </c>
+      <c r="C1365" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 23:14:42 +0700</t>
+        </is>
+      </c>
+      <c r="D1365" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E1365" t="inlineStr">
+        <is>
+          <t>Wuling melaporkan total pemesanan sebesar 3.290 unit kendaraan selama sebelas hari ajang Gaikindo Indonesia ...</t>
+        </is>
+      </c>
+      <c r="F1365" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1365" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5690053/wuling-rangkum-ribuan-spk-dalam-pameran-giias-2026</t>
+        </is>
+      </c>
+      <c r="H1365" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/CjkinzN000026_20260811_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I1365" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1366">
+      <c r="A1366" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1366" t="inlineStr">
+        <is>
+          <t>Kebakaran hutan di Gunung Bromo capai 800 Ha, Jatim prioritaskan OMC</t>
+        </is>
+      </c>
+      <c r="C1366" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 23:04:59 +0700</t>
+        </is>
+      </c>
+      <c r="D1366" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1366" t="inlineStr">
+        <is>
+          <t>ANTARA - Kebakaran hutan di Gunung Bromo telah meluas mencapai 800 hektare lebih. Wilayah Jawa Timur ditetapkan ...</t>
+        </is>
+      </c>
+      <c r="F1366" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1366" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5690035/kebakaran-hutan-di-gunung-bromo-capai-800-ha-jatim-prioritaskan-omc</t>
+        </is>
+      </c>
+      <c r="H1366" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KEBAKARAN-HUTAN-DI-GUNUNG-BROMO-CAPAI-800-HA-JATIM-PRIORITASKAN-OMC.jpg</t>
+        </is>
+      </c>
+      <c r="I1366" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1367">
+      <c r="A1367" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1367" t="inlineStr">
+        <is>
+          <t>Grab Indonesia ajak para mitra bersinergi untuk berkembang</t>
+        </is>
+      </c>
+      <c r="C1367" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 23:04:05 +0700</t>
+        </is>
+      </c>
+      <c r="D1367" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1367" t="inlineStr">
+        <is>
+          <t>Perusahaan layanan transportasi berbasis aplikasi Grab Indonesia mengajak para mitra perusahaan, termasuk pengemudi ...</t>
+        </is>
+      </c>
+      <c r="F1367" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1367" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690045/grab-indonesia-ajak-para-mitra-bersinergi-untuk-berkembang</t>
+        </is>
+      </c>
+      <c r="H1367" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1c86c2d4-d489-4c69-a64c-a632a2ec8d2c.jpeg</t>
+        </is>
+      </c>
+      <c r="I1367" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1368">
+      <c r="A1368" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1368" t="inlineStr">
+        <is>
+          <t>Yogyakarta tuan rumah forum kerja sama antarpemda Indonesia-Tiongkok</t>
+        </is>
+      </c>
+      <c r="C1368" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:53:58 +0700</t>
+        </is>
+      </c>
+      <c r="D1368" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1368" t="inlineStr">
+        <is>
+          <t>Pemerintah Kota Yogyakarta menjadi tuan rumah kegiatan Local Governments Dialogue China- Indonesia on Local Government ...</t>
+        </is>
+      </c>
+      <c r="F1368" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1368" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690040/yogyakarta-tuan-rumah-forum-kerja-sama-antarpemda-indonesia-tiongkok</t>
+        </is>
+      </c>
+      <c r="H1368" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/IMG_20260811_223146.jpg</t>
+        </is>
+      </c>
+      <c r="I1368" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1369">
+      <c r="A1369" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1369" t="inlineStr">
+        <is>
+          <t>KP2MI buka pendaftaran 40 ribu peserta SMK Go Global hingga 16 Agustus</t>
+        </is>
+      </c>
+      <c r="C1369" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:53:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1369" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1369" t="inlineStr">
+        <is>
+          <t>Kementerian Pelindungan Pekerja Migran Indonesia (KP2MI) membuka pendaftaran tahap pertama Pelatihan Peningkatan ...</t>
+        </is>
+      </c>
+      <c r="F1369" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1369" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690036/kp2mi-buka-pendaftaran-40-ribu-peserta-smk-go-global-hingga-16-agustus</t>
+        </is>
+      </c>
+      <c r="H1369" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/WhatsApp-Image-2026-08-11-at-18.32.14.jpeg</t>
+        </is>
+      </c>
+      <c r="I1369" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1370">
+      <c r="A1370" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1370" t="inlineStr">
+        <is>
+          <t>Airlangga minta emiten perkuat kinerja demi jaga kepercayaan pasar</t>
+        </is>
+      </c>
+      <c r="C1370" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:47:38 +0700</t>
+        </is>
+      </c>
+      <c r="D1370" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1370" t="inlineStr">
+        <is>
+          <t>Menteri Koordinator (Menko) Bidang Perekonomian Airlangga Hartarto meminta seluruh emiten memperkuat kinerja, tata ...</t>
+        </is>
+      </c>
+      <c r="F1370" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1370" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690033/airlangga-minta-emiten-perkuat-kinerja-demi-jaga-kepercayaan-pasar</t>
+        </is>
+      </c>
+      <c r="H1370" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/37E20D7A-30BB-48E5-B5C9-D38BC54BF91F.jpeg</t>
+        </is>
+      </c>
+      <c r="I1370" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1371">
+      <c r="A1371" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1371" t="inlineStr">
+        <is>
+          <t>Puntung Rokok Anak Picu Kebakaran Rumah di Grobogan, Sang Ibu Tewas</t>
+        </is>
+      </c>
+      <c r="C1371" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 23:28:14 +0700</t>
+        </is>
+      </c>
+      <c r="D1371" t="inlineStr">
+        <is>
+          <t>Ardian Dwi Kurnia</t>
+        </is>
+      </c>
+      <c r="E1371" t="inlineStr">
+        <is>
+          <t>Kebakaran tragis di Grobogan akibat puntung rokok anak. Seorang ibu tewas setelah api melahap rumah. Kejadian terjadi saat suami melihat asap dari kamar.</t>
+        </is>
+      </c>
+      <c r="F1371" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1371" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614496/puntung-rokok-anak-picu-kebakaran-rumah-di-grobogan-sang-ibu-tewas</t>
+        </is>
+      </c>
+      <c r="H1371" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/rumah-di-geyer-grobogan-terbakar-1786462775941_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1371" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1372">
+      <c r="A1372" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1372" t="inlineStr">
+        <is>
+          <t>Polri Beri Ruang Gen Z dan Alpha, Ada Lomba Mobile Legends hingga Animasi AI</t>
+        </is>
+      </c>
+      <c r="C1372" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 23:21:34 +0700</t>
+        </is>
+      </c>
+      <c r="D1372" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E1372" t="inlineStr">
+        <is>
+          <t>Polri merayakan Hari Bhayangkara ke-80 dengan 'Apresiasi Kreasi Polri Untuk Masyarakat', memberikan penghargaan untuk inovasi dan pengabdian masyarakat.</t>
+        </is>
+      </c>
+      <c r="F1372" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1372" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614494/polri-beri-ruang-gen-z-dan-alpha-ada-lomba-mobile-legends-hingga-animasi-ai</t>
+        </is>
+      </c>
+      <c r="H1372" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/polri-gelar-apresiasi-kreasi-1786465267542_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1372" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1373">
+      <c r="A1373" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1373" t="inlineStr">
+        <is>
+          <t>Momen Hangat Kapolri Beri Ruang Anak untuk Berkarya, dari Dongeng hingga Cita-cita</t>
+        </is>
+      </c>
+      <c r="C1373" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:59:40 +0700</t>
+        </is>
+      </c>
+      <c r="D1373" t="inlineStr">
+        <is>
+          <t>Azhar Bagas Ramadhan</t>
+        </is>
+      </c>
+      <c r="E1373" t="inlineStr">
+        <is>
+          <t>Kapolri Listyo Sigit memberikan ruang bagi anak-anak berbagi cita-cita dan bakat di malam puncak penganugerahan Apresiasi Kreasi Polri untuk Masyarakat.</t>
+        </is>
+      </c>
+      <c r="F1373" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1373" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614486/momen-hangat-kapolri-beri-ruang-anak-untuk-berkarya-dari-dongeng-hingga-cita-cita</t>
+        </is>
+      </c>
+      <c r="H1373" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/kapolri-jenderal-listyo-sigit-prabowo-memberikan-ruang-kepada-tiga-anak-untuk-menunjukkan-kemampuan-sekaligus-menyampaikan-cit-1786463916538_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1373" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1374">
+      <c r="A1374" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1374" t="inlineStr">
+        <is>
+          <t>Simpang Hek Kramat Jati Macet Panjang Malam Ini Imbas Perbaikan Jalan</t>
+        </is>
+      </c>
+      <c r="C1374" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:55:53 +0700</t>
+        </is>
+      </c>
+      <c r="D1374" t="inlineStr">
+        <is>
+          <t>Dwi Rahmawati</t>
+        </is>
+      </c>
+      <c r="E1374" t="inlineStr">
+        <is>
+          <t>Kemacetan parah terjadi di Jalan Raya Bogor, Kramat Jati, akibat perbaikan jalan. Kemacetan terjadi lantaran ada perbaikan jalan.</t>
+        </is>
+      </c>
+      <c r="F1374" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1374" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614485/simpang-hek-kramat-jati-macet-panjang-malam-ini-imbas-perbaikan-jalan</t>
+        </is>
+      </c>
+      <c r="H1374" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/simpang-hek-kramat-jati-macet-panjang-malam-inii-karena-ada-perbaikan-jalan-dwidetikcom-1786463737093_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1374" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1375">
+      <c r="A1375" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1375" t="inlineStr">
+        <is>
+          <t>Truk Tabrak Mobil Lagi Parkir di Kemang Jaksel, Sempat Tutup Jalan</t>
+        </is>
+      </c>
+      <c r="C1375" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:41:54 +0700</t>
+        </is>
+      </c>
+      <c r="D1375" t="inlineStr">
+        <is>
+          <t>Azhar Bagas Ramadhan</t>
+        </is>
+      </c>
+      <c r="E1375" t="inlineStr">
+        <is>
+          <t>Truk menabrak mobil yang terparkir di Jalan Kemang Timur, Jakarta Selatan. Proses evakuasi selesai, lalu lintas kini lancar kembali.</t>
+        </is>
+      </c>
+      <c r="F1375" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1375" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614479/truk-tabrak-mobil-lagi-parkir-di-kemang-jaksel-sempat-tutup-jalan</t>
+        </is>
+      </c>
+      <c r="H1375" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/sebuah-truk-muatan-menabrak-mobil-yang-sedang-terparkir-di-jalan-kemang-timur-jakarta-selatan-screenshot-video-viral-1786462606747_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1375" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1376">
+      <c r="A1376" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1376" t="inlineStr">
+        <is>
+          <t>Respons TNI soal Panglima Dikritik Imbas Pernyataan Tanggung Jawab Keamanan RI</t>
+        </is>
+      </c>
+      <c r="C1376" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:23:31 +0700</t>
+        </is>
+      </c>
+      <c r="D1376" t="inlineStr">
+        <is>
+          <t>Azhar Bagas Ramadhan</t>
+        </is>
+      </c>
+      <c r="E1376" t="inlineStr">
+        <is>
+          <t>TNI merespons kritik terhadap Panglima terkait tanggung jawab keamanan. Koalisi Masyarakat Sipil menilai pernyataan itu berisiko membingungkan fungsi TNI.</t>
+        </is>
+      </c>
+      <c r="F1376" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1376" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614458/respons-tni-soal-panglima-dikritik-imbas-pernyataan-tanggung-jawab-keamanan-ri</t>
+        </is>
+      </c>
+      <c r="H1376" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/09/kapupsen-tni-brigjen-muhammad-nas-dok-istimewa-1783579696895_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1376" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1377">
+      <c r="A1377" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1377" t="inlineStr">
+        <is>
+          <t>Siti Fauziah Sebut Sinergi Bakohumas Perkuat Publikasi Sidang Tahunan MPR</t>
+        </is>
+      </c>
+      <c r="C1377" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:15:16 +0700</t>
+        </is>
+      </c>
+      <c r="D1377" t="inlineStr">
+        <is>
+          <t>Dea Duta Aulia</t>
+        </is>
+      </c>
+      <c r="E1377" t="inlineStr">
+        <is>
+          <t>Plt. Sekjen MPR Siti Fauziah menekankan pentingnya sinergi Bakohumas untuk publikasi Sidang Tahunan MPR 2026 yang informatif dan kredibel. Persiapan sudah 85%.</t>
+        </is>
+      </c>
+      <c r="F1377" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1377" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614455/siti-fauziah-sebut-sinergi-bakohumas-perkuat-publikasi-sidang-tahunan-mpr</t>
+        </is>
+      </c>
+      <c r="H1377" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/mpr-1786461289407_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1377" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1378">
+      <c r="A1378" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1378" t="inlineStr">
+        <is>
+          <t>Neng Eem Tekankan 3 Prinsip Kehumasan Kawal Sidang Tahunan MPR</t>
+        </is>
+      </c>
+      <c r="C1378" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:10:30 +0700</t>
+        </is>
+      </c>
+      <c r="D1378" t="inlineStr">
+        <is>
+          <t>Angelina Vioni</t>
+        </is>
+      </c>
+      <c r="E1378" t="inlineStr">
+        <is>
+          <t>Ketua Fraksi PKB MPR, Neng Eem, menekankan tiga prinsip kehumasan: informatif, kolaboratif, dan kredibel, untuk publikasi Sidang Tahunan MPR 2026.</t>
+        </is>
+      </c>
+      <c r="F1378" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1378" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614454/neng-eem-tekankan-3-prinsip-kehumasan-kawal-sidang-tahunan-mpr</t>
+        </is>
+      </c>
+      <c r="H1378" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/mpr-1786459705861_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1378" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1379">
+      <c r="A1379" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1379" t="inlineStr">
+        <is>
+          <t>Kapolri Anugerahi Pemenang Apresiasi Kreasi Polri untuk Masyarakat</t>
+        </is>
+      </c>
+      <c r="C1379" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:09:59 +0700</t>
+        </is>
+      </c>
+      <c r="D1379" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E1379" t="inlineStr">
+        <is>
+          <t>Kapolri Jenderal Listyo Sigit menghadiri penganugerahan 'Apresiasi Kreasi Polri untuk Masyarakat', merayakan kreativitas dan kolaborasi Polri dan masyarakat.</t>
+        </is>
+      </c>
+      <c r="F1379" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1379" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614453/kapolri-anugerahi-pemenang-apresiasi-kreasi-polri-untuk-masyarakat</t>
+        </is>
+      </c>
+      <c r="H1379" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/kapolri-anugerahi-pemenang-apresiasi-kreasi-polri-untuk-masyarakat-1786460939313_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1379" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1380">
+      <c r="A1380" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1380" t="inlineStr">
+        <is>
+          <t>Senangnya Warga Bulak Barat Depok, Banjir Bertahun-tahun Kini Surut</t>
+        </is>
+      </c>
+      <c r="C1380" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:02:11 +0700</t>
+        </is>
+      </c>
+      <c r="D1380" t="inlineStr">
+        <is>
+          <t>Devi Puspitasari</t>
+        </is>
+      </c>
+      <c r="E1380" t="inlineStr">
+        <is>
+          <t>Banjir di Kampung Bulak Barat, Cipayung, Depok, akhirnya surut setelah normalisasi sungai. Warga bersyukur dan berharap perbaikan jembatan segera selesai.</t>
+        </is>
+      </c>
+      <c r="F1380" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1380" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614444/senangnya-warga-bulak-barat-depok-banjir-bertahun-tahun-kini-surut</t>
+        </is>
+      </c>
+      <c r="H1380" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/banjir-bertahun-tahun-di-depok-surut-1786460487792_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1380" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1381">
+      <c r="A1381" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1381" t="inlineStr">
+        <is>
+          <t>TPS Liar Cilincing Disorot, Pengelolaan Sampah Berbasis RDF Jadi Perhatian</t>
+        </is>
+      </c>
+      <c r="C1381" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:50:57 +0700</t>
+        </is>
+      </c>
+      <c r="D1381" t="inlineStr">
+        <is>
+          <t>Jabbar Ramdhani</t>
+        </is>
+      </c>
+      <c r="E1381" t="inlineStr">
+        <is>
+          <t>Peninjauan TPS liar di Cilincing oleh polsek dan kecamatan berfokus pada pengelolaan sampah berbasis RDF.</t>
+        </is>
+      </c>
+      <c r="F1381" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1381" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614436/tps-liar-cilincing-disorot-pengelolaan-sampah-berbasis-rdf-jadi-perhatian</t>
+        </is>
+      </c>
+      <c r="H1381" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/peninjauan-tps-liar-di-cilincing-oleh-polsek-dan-kecamatan-fokus-pada-pengelolaan-sampah-berbasis-rdf-dok-ist-1786459833382_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1381" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1382">
+      <c r="A1382" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1382" t="inlineStr">
+        <is>
+          <t>Buka Forum Bakohumas MPR, Neng Eem Dorong Sinergi Komunikasi Pemerintah</t>
+        </is>
+      </c>
+      <c r="C1382" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:48:59 +0700</t>
+        </is>
+      </c>
+      <c r="D1382" t="inlineStr">
+        <is>
+          <t>â Nada Herwando Kartika</t>
+        </is>
+      </c>
+      <c r="E1382" t="inlineStr">
+        <is>
+          <t>Ketua Fraksi PKB MPR Neng Eem tekankan pentingnya kehumasan pemerintah untuk menjembatani komunikasi antara pemerintah dan masyarakat dalam Sidang Tahunan MPR.</t>
+        </is>
+      </c>
+      <c r="F1382" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1382" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614434/buka-forum-bakohumas-mpr-neng-eem-dorong-sinergi-komunikasi-pemerintah</t>
+        </is>
+      </c>
+      <c r="H1382" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/mpr-1786461289321_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1382" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1383">
+      <c r="A1383" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1383" t="inlineStr">
+        <is>
+          <t>Tampang Pria Pembunuh dan Pemerkosa Wanita di Tangerang</t>
+        </is>
+      </c>
+      <c r="C1383" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:40:02 +0700</t>
+        </is>
+      </c>
+      <c r="D1383" t="inlineStr">
+        <is>
+          <t>Kadek Melda Luxiana</t>
+        </is>
+      </c>
+      <c r="E1383" t="inlineStr">
+        <is>
+          <t>Polisi tangkap pelaku pembunuhan dan pemerkosaan wanita berinisial SNA (20) di Tangerang. Penangkapan dilakukan kurang dari 24 jam setelah kejadian.</t>
+        </is>
+      </c>
+      <c r="F1383" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1383" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614426/tampang-pria-pembunuh-dan-pemerkosa-wanita-di-tangerang</t>
+        </is>
+      </c>
+      <c r="H1383" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/pelaku-pemerkosa-dan-pembunuhan-wanita-di-tangerang-dok-istimewa-1786459171206.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1383" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1384">
+      <c r="A1384" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1384" t="inlineStr">
+        <is>
+          <t>Lawyer Muslim Adukan Challenge Hafalan Qur'an demi Miras ke Bareskrim</t>
+        </is>
+      </c>
+      <c r="C1384" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:22:35 +0700</t>
+        </is>
+      </c>
+      <c r="D1384" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E1384" t="inlineStr">
+        <is>
+          <t>Asosiasi Lawyer Muslim melaporkan tantangan hafalan Al-Qur'an berhadiah miras ke Bareskrim. Penyelidikan sedang dilakukan terkait dugaan penistaan agama.</t>
+        </is>
+      </c>
+      <c r="F1384" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1384" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614400/lawyer-muslim-adukan-challenge-hafalan-quran-demi-miras-ke-bareskrim</t>
+        </is>
+      </c>
+      <c r="H1384" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/asosiasi-lawyer-muslim-indonesia-almi-mengadukan-tindakan-challenge-hafalan-al-quran-berhadiah-minuman-keras-miras-saat-konser-1786458081129_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1384" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1385">
+      <c r="A1385" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1385" t="inlineStr">
+        <is>
+          <t>Pemerintah Bakal Bentuk Tim Lintas Kementerian Atasi Masalah Agraria</t>
+        </is>
+      </c>
+      <c r="C1385" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:14:28 +0700</t>
+        </is>
+      </c>
+      <c r="D1385" t="inlineStr">
+        <is>
+          <t>Dwi Rahmawati</t>
+        </is>
+      </c>
+      <c r="E1385" t="inlineStr">
+        <is>
+          <t>Mensesneg Prasetyo Hadi umumkan pembentukan tim lintas kementerian untuk menyelesaikan masalah agraria.</t>
+        </is>
+      </c>
+      <c r="F1385" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1385" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614398/pemerintah-bakal-bentuk-tim-lintas-kementerian-atasi-masalah-agraria</t>
+        </is>
+      </c>
+      <c r="H1385" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/20/prasetyo-hadi-1784523183633_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1385" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1386">
+      <c r="A1386" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B1386" t="inlineStr">
+        <is>
+          <t>Dahlia Poland Temukan Tambatan Hati Baru, Pria Sunda-Satu Frekuensi</t>
+        </is>
+      </c>
+      <c r="C1386" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:02:14 +0700</t>
+        </is>
+      </c>
+      <c r="D1386" t="inlineStr">
+        <is>
+          <t>Muhammad Ahsan Nurrijal</t>
+        </is>
+      </c>
+      <c r="E1386" t="inlineStr">
+        <is>
+          <t>Aktris Dahlia Poland bahagia dengan kekasih baru setelah berpisah dari Fandy Christian. Ia menikmati hubungan yang masih dalam tahap pengenalan.</t>
+        </is>
+      </c>
+      <c r="F1386" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1386" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8614328/dahlia-poland-temukan-tambatan-hati-baru-pria-sunda-satu-frekuensi</t>
+        </is>
+      </c>
+      <c r="H1386" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/11/25/dahlia-poland-1764056150319_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1386" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1387">
+      <c r="A1387" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B1387" t="inlineStr">
+        <is>
+          <t>Denny Sumargo Mohon Doa, Istri Jalani Program Bayi Tabung Terakhir</t>
+        </is>
+      </c>
+      <c r="C1387" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:02:06 +0700</t>
+        </is>
+      </c>
+      <c r="D1387" t="inlineStr">
+        <is>
+          <t>Muhammad Ahsan Nurrijal</t>
+        </is>
+      </c>
+      <c r="E1387" t="inlineStr">
+        <is>
+          <t>Denny Sumargo dan Olivia Allan berjuang untuk anak kedua melalui program bayi tabung. Setelah empat kegagalan, mereka berharap percobaan terakhir ini berhasil.</t>
+        </is>
+      </c>
+      <c r="F1387" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1387" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8614317/denny-sumargo-mohon-doa-istri-jalani-program-bayi-tabung-terakhir</t>
+        </is>
+      </c>
+      <c r="H1387" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/denny-sumargo-1786454390420_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1387" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1388">
+      <c r="A1388" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1388" t="inlineStr">
+        <is>
+          <t>Kuasa Hukum Eks Menag Yaqut Jelaskan Duduk Persoalan Pembagian Kuota Haji Tambahan</t>
+        </is>
+      </c>
+      <c r="C1388" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 23:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1388" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1388" t="inlineStr">
+        <is>
+          <t>Kuasa hukum Yaqut Cholil Qoumas menjelaskan duduk persoalan mengenai pembagian kuota haji tambahan tahun 2023-2024 yang dipersoalkan KPK.</t>
+        </is>
+      </c>
+      <c r="F1388" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1388" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867140/kuasa-hukum-eks-menag-yaqut-jelaskan-duduk-persoalan-pembagian-kuota-haji-tambahan</t>
+        </is>
+      </c>
+      <c r="H1388" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/1hVGgaXLegVFCnj-iNku1-8XQW0=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Terdakwa-kasus-dugaan-korupsi-kuota-haji-mantan-Menag-Yaqut-Cholil.jpg</t>
+        </is>
+      </c>
+      <c r="I1388" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1389">
+      <c r="A1389" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1389" t="inlineStr">
+        <is>
+          <t>Kolaborasi DeadSquad Bareng Limbad Sukses Meriahkan Parti Libur 2026</t>
+        </is>
+      </c>
+      <c r="C1389" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 23:29:35 +0700</t>
+        </is>
+      </c>
+      <c r="D1389" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1389" t="inlineStr">
+        <is>
+          <t>Parti Libur 2026 mengusung konsep Caravan yang memadukan festival musik dengan wahana bermain di Batu Night Spectacular (NBS).</t>
+        </is>
+      </c>
+      <c r="F1389" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1389" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7867139/kolaborasi-deadsquad-bareng-limbad-sukses-meriahkan-parti-libur-2026</t>
+        </is>
+      </c>
+      <c r="H1389" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/UqrxxSV_61vei1R96OGYmz_eHJQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Limbad-1-11082026.jpg</t>
+        </is>
+      </c>
+      <c r="I1389" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1390">
+      <c r="A1390" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1390" t="inlineStr">
+        <is>
+          <t>Pria Beristri Bunuh Kekasih di Tangerang, Pelaku Rekayasa Kematian Korban Seolah Gantung Diri</t>
+        </is>
+      </c>
+      <c r="C1390" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 23:04:45 +0700</t>
+        </is>
+      </c>
+      <c r="D1390" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1390" t="inlineStr">
+        <is>
+          <t>Wanita usia 29 tahun berinisial R menjadi korban pembunuhan yang dilakukan kekasihnya berinisial di Pasar Kemis, Kabupaten Tangerang.</t>
+        </is>
+      </c>
+      <c r="F1390" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1390" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7867138/pria-beristri-bunuh-kekasih-di-tangerang-pelaku-rekayasa-kematian-korban-seolah-gantung-diri</t>
+        </is>
+      </c>
+      <c r="H1390" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/a4cQ92m0zPGnlR7WfCm6rl1m9D0=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/kasus-pembunuhan-pasar-kemis.jpg</t>
+        </is>
+      </c>
+      <c r="I1390" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1391">
+      <c r="A1391" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1391" t="inlineStr">
+        <is>
+          <t>Yaqut Bantah Terima Uang Korupsi Kuota Haji, Pertanyakan Pihak yang Raup Keuntungan</t>
+        </is>
+      </c>
+      <c r="C1391" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:52:49 +0700</t>
+        </is>
+      </c>
+      <c r="D1391" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1391" t="inlineStr">
+        <is>
+          <t>Yaqut membantah menerima uang dalam perkara kuota haji dan mempertanyakan pihak yang disebut jaksa memperoleh keuntungan.</t>
+        </is>
+      </c>
+      <c r="F1391" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1391" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867137/yaqut-bantah-terima-uang-korupsi-kuota-haji-pertanyakan-pihak-yang-raup-keuntungan</t>
+        </is>
+      </c>
+      <c r="H1391" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/2hk2ajvAHooPwdG2smD6r2W1zfI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Mantan-Menteri-Agama-Yaqut-Cholil-Qoumas-usai-sidang-perdana-perkara-korupsi-kuota-haji.jpg</t>
+        </is>
+      </c>
+      <c r="I1391" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1392">
+      <c r="A1392" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1392" t="inlineStr">
+        <is>
+          <t>73 Ribu Hektare Sawah Masih Berstatus Kawasan Hutan, Pemerintah Bentuk Tim Agraria</t>
+        </is>
+      </c>
+      <c r="C1392" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:52:02 +0700</t>
+        </is>
+      </c>
+      <c r="D1392" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1392" t="inlineStr">
+        <is>
+          <t>Pemerintah mengatakan 73.000 hektare lahan yang saat ini telah berbentuk sawah masih memiliki status yang dapat masuk dalam kawasan hutan.</t>
+        </is>
+      </c>
+      <c r="F1392" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1392" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867136/73-ribu-hektare-sawah-masih-berstatus-kawasan-hutan-pemerintah-bentuk-tim-agraria</t>
+        </is>
+      </c>
+      <c r="H1392" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/yezKPCYXFWzwWCegljMEEYJiBKY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ILUSTRASI-PERTANIAN-SAWAH.jpg</t>
+        </is>
+      </c>
+      <c r="I1392" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1393">
+      <c r="A1393" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1393" t="inlineStr">
+        <is>
+          <t>Perketat Ekspor Teknologi, China Tangkap Sejumlah Pengusaha Jepang</t>
+        </is>
+      </c>
+      <c r="C1393" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:37:05 +0700</t>
+        </is>
+      </c>
+      <c r="D1393" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1393" t="inlineStr">
+        <is>
+          <t>Informasi itu menyebut sejumlah eksekutif perusahaan Jepang yang memiliki operasi di China menjadi sasaran penyelidikan.</t>
+        </is>
+      </c>
+      <c r="F1393" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1393" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7867135/perketat-ekspor-teknologi-china-tangkap-sejumlah-pengusaha-jepang</t>
+        </is>
+      </c>
+      <c r="H1393" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/rtTV6JXDL-dp4lehWhprdwo1SFQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ILUSTRASI-Bendera-China-dan-Jepang.jpg</t>
+        </is>
+      </c>
+      <c r="I1393" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1394">
+      <c r="A1394" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1394" t="inlineStr">
+        <is>
+          <t>Polisi Kumpulkan Barbuk Kasus Challenge Hafalan Al-Qur'an Berhadiah Miras</t>
+        </is>
+      </c>
+      <c r="C1394" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 23:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1394" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1394" t="inlineStr">
+        <is>
+          <t>Selain rekaman video yang beredar di media sosial, petugas juga memeriksa sejumlah barang bukti lain.</t>
+        </is>
+      </c>
+      <c r="F1394" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1394" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267527/polisi-kumpulkan-barbuk-kasus-challenge-hafalan-al-quran-berhadiah-miras</t>
+        </is>
+      </c>
+      <c r="H1394" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/Fp5iC-vppn7dJSzwqGEBlrLz0gY=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9321055/original/059736500_1786425649-Jepretan_Layar_2025-08-11_pukul_12.15.34.jpg</t>
+        </is>
+      </c>
+      <c r="I1394" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1395">
+      <c r="A1395" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1395" t="inlineStr">
+        <is>
+          <t>Peringatan ke Pegawai, Gus Ipul: Jangan Kebiasaan Habiskan Uang dan Belanja Sembarangan</t>
+        </is>
+      </c>
+      <c r="C1395" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 23:48:32 +0700</t>
+        </is>
+      </c>
+      <c r="D1395" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E1395" t="inlineStr">
+        <is>
+          <t>Mensos Saifullah Yusuf atau Gus Ipul memperingatkan pegawainya agar meninggalkan kebiasaan menghabiskan uang dan belanja anggaran secara sembarangan.</t>
+        </is>
+      </c>
+      <c r="F1395" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1395" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/08/11/23324151/peringatan-ke-pegawai-gus-ipul-jangan-kebiasaan-habiskan-uang-dan-belanja</t>
+        </is>
+      </c>
+      <c r="H1395" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/pKspNR1Miw68Cgbca6xdXgMI_PM=/425x148:3753x2367/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/05/6a73165e5e027.jpeg</t>
+        </is>
+      </c>
+      <c r="I1395" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1396">
+      <c r="A1396" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1396" t="inlineStr">
+        <is>
+          <t>Wakil Menteri Perang AS Temui Menhan Sjafrie, Bahas soal Kelanjutan Kerja Sama Pertahanan</t>
+        </is>
+      </c>
+      <c r="C1396" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 23:48:32 +0700</t>
+        </is>
+      </c>
+      <c r="D1396" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E1396" t="inlineStr">
+        <is>
+          <t>Wakil Menteri Perang Amerika Serikat (AS) bidang Kebijakan Elbridge A. Colby mengunjungi Menteri Pertahanan RI Sjafrie Sjamsoeddin di Kemenhan RI.</t>
+        </is>
+      </c>
+      <c r="F1396" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1396" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/08/11/22202711/wakil-menteri-perang-as-temui-menhan-sjafrie-bahas-soal-kelanjutan-kerja</t>
+        </is>
+      </c>
+      <c r="H1396" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/d6iy2gqD10-O_Sn9zLIxhlhGQOI=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/11/6a7b340b0529f.jpg</t>
+        </is>
+      </c>
+      <c r="I1396" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1397">
+      <c r="A1397" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1397" t="inlineStr">
+        <is>
+          <t>Rinaldi Umar Batal Dilantik Jadi Dirdik Jampidsus, Ini Alasan Kejagung</t>
+        </is>
+      </c>
+      <c r="C1397" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 23:48:32 +0700</t>
+        </is>
+      </c>
+      <c r="D1397" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E1397" t="inlineStr">
+        <is>
+          <t>Alasan Rinaldi Umar batal dilantik sebagai Direktur Penyidikan (Dirdik) pada Jaksa Agung Muda Tindak Pidana Khusus karena alasan pengalaman.</t>
+        </is>
+      </c>
+      <c r="F1397" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1397" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/08/11/21262681/rinaldi-umar-batal-dilantik-jadi-dirdik-jampidsus-ini-alasan-kejagung</t>
+        </is>
+      </c>
+      <c r="H1397" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/RkjlvY0ly1nBMPQx3Rv8uJ7Vyts=/265x66:1297x754/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/03/6a70a42491bfb.jpg</t>
+        </is>
+      </c>
+      <c r="I1397" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I1356"/>
+  <autoFilter ref="A1:I1397"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-11 17:51 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-11.xlsx
+++ b/data/berita_2026-08-11.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1397</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1502</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1397"/>
+  <dimension ref="A1:I1502"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -66098,8 +66098,4943 @@
         </is>
       </c>
     </row>
+    <row r="1398">
+      <c r="A1398" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1398" t="inlineStr">
+        <is>
+          <t>Kaltara dapat bantuan Rp10 miliar lebih dari Presiden Prabowo</t>
+        </is>
+      </c>
+      <c r="C1398" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 23:59:53 +0700</t>
+        </is>
+      </c>
+      <c r="D1398" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1398" t="inlineStr">
+        <is>
+          <t>ANTARA - Gubernur Kalimantan Utara Zainal Arifin Paliwang menyebut Kaltara mendapat bantuan anggaran lebih dari Rp10 ...</t>
+        </is>
+      </c>
+      <c r="F1398" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1398" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5690051/kaltara-dapat-bantuan-rp10-miliar-lebih-dari-presiden-prabowo</t>
+        </is>
+      </c>
+      <c r="H1398" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KALTARA-DAPAT-BANTUAN-RP10-MILIAR-LEBIH-DARI-PRESIDEN-PRABOWO.jpg</t>
+        </is>
+      </c>
+      <c r="I1398" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1399">
+      <c r="A1399" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1399" t="inlineStr">
+        <is>
+          <t>Bapanas: Perpanjangan SPHP jagung pakan demi bantu peternak lokal</t>
+        </is>
+      </c>
+      <c r="C1399" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 23:54:41 +0700</t>
+        </is>
+      </c>
+      <c r="D1399" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1399" t="inlineStr">
+        <is>
+          <t>Kepala Badan Pangan Nasional (Bapanas) Andi Amran Sulaiman menegaskan program Stabilisasi Pasokan dan Harga Pangan ...</t>
+        </is>
+      </c>
+      <c r="F1399" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1399" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690089/bapanas-perpanjangan-sphp-jagung-pakan-demi-bantu-peternak-lokal</t>
+        </is>
+      </c>
+      <c r="H1399" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/3E7505B6-92AA-42E1-8605-933DE8346CB5.jpeg</t>
+        </is>
+      </c>
+      <c r="I1399" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1400">
+      <c r="A1400" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1400" t="inlineStr">
+        <is>
+          <t>OMC malam jadi opsi perkuat penanganan karhutla di Sumsel</t>
+        </is>
+      </c>
+      <c r="C1400" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 23:52:54 +0700</t>
+        </is>
+      </c>
+      <c r="D1400" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1400" t="inlineStr">
+        <is>
+          <t>ANTARA - Operasi Modifikasi Cuaca atau OMC pada malam hari disiapkan sebagai opsi untuk mengoptimalkan penanganan ...</t>
+        </is>
+      </c>
+      <c r="F1400" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1400" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5690072/omc-malam-jadi-opsi-perkuat-penanganan-karhutla-di-sumsel</t>
+        </is>
+      </c>
+      <c r="H1400" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/OMC-MALAM-JADI-OPSI-PERKUAT-PENANGANAN-KARHUTLA-DI-SUMSEL.jpg</t>
+        </is>
+      </c>
+      <c r="I1400" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1401">
+      <c r="A1401" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1401" t="inlineStr">
+        <is>
+          <t>Delapan pemain jadi sorotan dalam World Tour Lausanne 2026</t>
+        </is>
+      </c>
+      <c r="C1401" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 23:52:25 +0700</t>
+        </is>
+      </c>
+      <c r="D1401" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1401" t="inlineStr">
+        <is>
+          <t>Delapan pemain menjadi sorotan utama dalam FIBA 3x3 World Tour Lausanne 2026 di Swiss, pada 14-15 Agustus, mulai dari ...</t>
+        </is>
+      </c>
+      <c r="F1401" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1401" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690088/delapan-pemain-jadi-sorotan-dalam-world-tour-lausanne-2026</t>
+        </is>
+      </c>
+      <c r="H1401" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2018/08/Basket-3-on-3.jpg</t>
+        </is>
+      </c>
+      <c r="I1401" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1402">
+      <c r="A1402" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1402" t="inlineStr">
+        <is>
+          <t>Silver Media Group gaet Chris John untuk kembangkan "Dragon's Dojo"</t>
+        </is>
+      </c>
+      <c r="C1402" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 23:46:10 +0700</t>
+        </is>
+      </c>
+      <c r="D1402" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1402" t="inlineStr">
+        <is>
+          <t>Silver Media Group menggandeng legenda tinju Indonesia, Chris John, untuk mengembangkan seri animasi baru berjudul ...</t>
+        </is>
+      </c>
+      <c r="F1402" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1402" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690084/silver-media-group-gaet-chris-john-untuk-kembangkan-dragons-dojo</t>
+        </is>
+      </c>
+      <c r="H1402" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2023/07/03/IMG_2214.jpeg</t>
+        </is>
+      </c>
+      <c r="I1402" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1403">
+      <c r="A1403" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1403" t="inlineStr">
+        <is>
+          <t>Kemenbud siapkan situs bersejarah Bogor jadi Cagar Budaya Nasional</t>
+        </is>
+      </c>
+      <c r="C1403" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 23:45:10 +0700</t>
+        </is>
+      </c>
+      <c r="D1403" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1403" t="inlineStr">
+        <is>
+          <t>Kementerian Kebudayaan (Kemenbud) menyiapkan sejumlah situs bersejarah di Kabupaten Bogor, Jawa Barat, untuk ditata dan ...</t>
+        </is>
+      </c>
+      <c r="F1403" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1403" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690083/kemenbud-siapkan-situs-bersejarah-bogor-jadi-cagar-budaya-nasional</t>
+        </is>
+      </c>
+      <c r="H1403" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1003331109.jpg</t>
+        </is>
+      </c>
+      <c r="I1403" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1404">
+      <c r="A1404" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1404" t="inlineStr">
+        <is>
+          <t>KPAI Apresiasi Polri Beri Penghargaan ke Anak: Picu Mereka Terus Berkembang</t>
+        </is>
+      </c>
+      <c r="C1404" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 23:43:23 +0700</t>
+        </is>
+      </c>
+      <c r="D1404" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E1404" t="inlineStr">
+        <is>
+          <t>Ketua KPAI Aris Adi Leksono apresiasi penghargaan Polri untuk anak. Ia berharap lebih banyak ruang bagi anak untuk berkreasi dan berprestasi.</t>
+        </is>
+      </c>
+      <c r="F1404" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1404" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614499/kpai-apresiasi-polri-beri-penghargaan-ke-anak-picu-mereka-terus-berkembang</t>
+        </is>
+      </c>
+      <c r="H1404" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/ketua-kpai-aris-adi-leksono-apresiasi-penghargaan-polri-untuk-anak-kurniawan-fdetikcom-1786466595626_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1404" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1405">
+      <c r="A1405" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1405" t="inlineStr">
+        <is>
+          <t>Kak Seto Puji Polri Rangkul Anak Lewat Penghargaan dan Lomba Kreativitas</t>
+        </is>
+      </c>
+      <c r="C1405" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 23:42:19 +0700</t>
+        </is>
+      </c>
+      <c r="D1405" t="inlineStr">
+        <is>
+          <t>Kurniawan Fadilah</t>
+        </is>
+      </c>
+      <c r="E1405" t="inlineStr">
+        <is>
+          <t>Kak Seto apresiasi kegiatan Apresiasi Kreasi Polri untuk Masyarakat. Ia menekankan pentingnya polisi sebagai sahabat anak dan membangun karakter.</t>
+        </is>
+      </c>
+      <c r="F1405" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1405" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614498/kak-seto-puji-polri-rangkul-anak-lewat-penghargaan-dan-lomba-kreativitas</t>
+        </is>
+      </c>
+      <c r="H1405" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/kak-seto-selepas-acara-apresiasi-kreasi-polri-untuk-masyarakat-1786466516186_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1405" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1406">
+      <c r="A1406" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1406" t="inlineStr">
+        <is>
+          <t>Pemerintah Janji Jaga Harga Pakan, Minta Dapur MBG Serap Telur Peternak</t>
+        </is>
+      </c>
+      <c r="C1406" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 22:50:17 +0700</t>
+        </is>
+      </c>
+      <c r="D1406" t="inlineStr">
+        <is>
+          <t>Ignacio Geordi Oswaldo</t>
+        </is>
+      </c>
+      <c r="E1406" t="inlineStr">
+        <is>
+          <t>Menteri Pertanian (Mentan) Andi Amran Sulaiman memastikan harga pakan tetap dijaga hingga akhir tahun</t>
+        </is>
+      </c>
+      <c r="F1406" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1406" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8614483/pemerintah-janji-jaga-harga-pakan-minta-dapur-mbg-serap-telur-peternak</t>
+        </is>
+      </c>
+      <c r="H1406" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/02/harga-telur-di-temanggung-anjlok-jadi-rp17000-rp18000-per-kg-1782966898187_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1406" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1407">
+      <c r="A1407" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1407" t="inlineStr">
+        <is>
+          <t>Solomon Putra Wongso Tampil di Trunk Show Wedding, Hadirkan Sentuhan Tailoring dari London</t>
+        </is>
+      </c>
+      <c r="C1407" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 23:56:26 +0700</t>
+        </is>
+      </c>
+      <c r="D1407" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E1407" t="inlineStr">
+        <is>
+          <t>Solomon Puttra Wongso tampil di trunk show bersama ayahnya, Lianto, membawa perspektif tailoring London ke panggung Jakarta.</t>
+        </is>
+      </c>
+      <c r="F1407" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1407" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/lifestyle/7867141/solomon-putra-wongso-tampil-di-trunk-show-wedding-hadirkan-sentuhan-tailoring-dari-london</t>
+        </is>
+      </c>
+      <c r="H1407" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/fVrRaHo0Tso1W_ZiArEurHdcf6g=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Lianto-Wongso-tengah-bersama-putranya-Solomon-Putra-Wongso-kiri.jpg</t>
+        </is>
+      </c>
+      <c r="I1407" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="1408">
+      <c r="A1408" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1408" t="inlineStr">
+        <is>
+          <t>Perang Saudara Negara Arab, Kuburan Massal Ditemukan</t>
+        </is>
+      </c>
+      <c r="C1408" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:50:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1408" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1408" t="inlineStr">
+        <is>
+          <t>Kuburan massal ditemukan di Kurmuk, Sudan, setelah pasukan militer merebut kota.</t>
+        </is>
+      </c>
+      <c r="F1408" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1408" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811170918-4-758368/perang-saudara-negara-arab-kuburan-massal-ditemukan</t>
+        </is>
+      </c>
+      <c r="H1408" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2023/09/13/jenazah-korban-ditempatkan-di-kuburan-massal-setelah-badai-dahsyat-dan-hujan-lebat-di-libya-di-derna-libya-12-september-2023-4_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1408" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1409">
+      <c r="A1409" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1409" t="inlineStr">
+        <is>
+          <t>Kasus Suap Miliarder Dibatalkan, Pengacaranya sama dengan Presiden</t>
+        </is>
+      </c>
+      <c r="C1409" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:40:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1409" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1409" t="inlineStr">
+        <is>
+          <t>Hakim AS batalkan kasus suap Gautam Adani. Pengacara Adani, Robert Giuffra, merupakan pengacara pribadi Presiden AS Donald Trump.</t>
+        </is>
+      </c>
+      <c r="F1409" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1409" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811164104-4-758357/kasus-suap-miliarder-dibatalkan-pengacaranya-sama-dengan-presiden</t>
+        </is>
+      </c>
+      <c r="H1409" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/05/20/miliarder-india-gautam-adani-reutersstringerfile-photo-1779240974007_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1409" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1410">
+      <c r="A1410" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1410" t="inlineStr">
+        <is>
+          <t>Iran Rombak Struktur Keamanan, Veteran IRGC Naik ke Posisi Kunci</t>
+        </is>
+      </c>
+      <c r="C1410" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1410" t="inlineStr">
+        <is>
+          <t>tfa</t>
+        </is>
+      </c>
+      <c r="E1410" t="inlineStr">
+        <is>
+          <t>Iran melakukan perombakan di jajaran keamanan dengan menunjuk veteran IRGC, termasuk Mohsen Rezaee, di tengah ketegangan dengan AS dan Israel.</t>
+        </is>
+      </c>
+      <c r="F1410" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1410" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811143928-4-758300/iran-rombak-struktur-keamanan-veteran-irgc-naik-ke-posisi-kunci</t>
+        </is>
+      </c>
+      <c r="H1410" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/06/13/seorang-wanita-memegang-bendera-iran-di-jalanan-teheran-iran-10-juni-2026-1781317439422_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1410" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1411">
+      <c r="A1411" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1411" t="inlineStr">
+        <is>
+          <t>CNG 3 Kg Bakal Disubsidi, Tapi Biayanya Lebih Hemat 40% dari LPG</t>
+        </is>
+      </c>
+      <c r="C1411" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:20:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1411" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1411" t="inlineStr">
+        <is>
+          <t>CNG 3 Kg bakal disubsidi pemerintah</t>
+        </is>
+      </c>
+      <c r="F1411" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1411" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811181543-4-758404/cng-3-kg-bakal-disubsidi-tapi-biayanya-lebih-hemat-40-dari-lpg</t>
+        </is>
+      </c>
+      <c r="H1411" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/06/29/ilustrasi-cng-merah-putih-3kg-1782728074855_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1411" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1412">
+      <c r="A1412" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1412" t="inlineStr">
+        <is>
+          <t>Banjir Surut, Potret Pantai Tetangga RI Kini Jadi Lautan Sampah</t>
+        </is>
+      </c>
+      <c r="C1412" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 21:10:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1412" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1412" t="inlineStr">
+        <is>
+          <t>Sampah menumpuk di Pantai Dolomit Manila usai hujan deras akibat Habagat. Limbah terbawa banjir dari saluran air dan permukiman di sekitar kawasan.</t>
+        </is>
+      </c>
+      <c r="F1412" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1412" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811180143-7-758397/banjir-surut-potret-pantai-tetangga-ri-kini-jadi-lautan-sampah</t>
+        </is>
+      </c>
+      <c r="H1412" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/seorang-pekerja-mengumpulkan-sampah-yang-terbawa-arus-ke-sungai-di-tengah-hujan-deras-akibat-angin-muson-barat-daya-di-dekat-g-1786446098324_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1412" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1413">
+      <c r="A1413" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1413" t="inlineStr">
+        <is>
+          <t>Lempeng Samudra Nazca Plate Robek, Gempa Dahsyat Mw7,4 Rusak Kolombia</t>
+        </is>
+      </c>
+      <c r="C1413" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:50:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1413" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1413" t="inlineStr">
+        <is>
+          <t>Gempa Mw7,4 mengguncang Kolombia, menewaskan 138 orang dan melukai ratusan. Daryono menjelaskan penyebab dan dampak gempa dalam-lempeng ini.</t>
+        </is>
+      </c>
+      <c r="F1413" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1413" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811180341-4-758396/lempeng-samudra-nazca-plate-robek-gempa-dahsyat-mw74-rusak-kolombia</t>
+        </is>
+      </c>
+      <c r="H1413" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/suasana-setelah-gempa-bumi-di-dosquebradas-kolombia-senin-1082026-reutersjuan-david-duque-1786405982899_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1413" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1414">
+      <c r="A1414" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1414" t="inlineStr">
+        <is>
+          <t>Gubernur Bank Sentral Libya Mundur di Tengah Tekanan Ekonomi</t>
+        </is>
+      </c>
+      <c r="C1414" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:40:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1414" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1414" t="inlineStr">
+        <is>
+          <t>Pengunduran diri Gubernur Bank Sentral Libya, Naji Issa, memunculkan tantangan ekonomi besar, termasuk belanja pemerintah dan cadangan devisa.</t>
+        </is>
+      </c>
+      <c r="F1414" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1414" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811161659-4-758346/gubernur-bank-sentral-libya-mundur-di-tengah-tekanan-ekonomi</t>
+        </is>
+      </c>
+      <c r="H1414" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/gubernur-bank-sentral-libya-naji-issa-1786440205574_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1414" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1415">
+      <c r="A1415" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1415" t="inlineStr">
+        <is>
+          <t>Freeport Sudah Ajukan Perpanjangan Izin Tambang (IUPK), Ini Kata ESDM</t>
+        </is>
+      </c>
+      <c r="C1415" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:20:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1415" t="inlineStr">
+        <is>
+          <t>Firda Dwi Muliawati</t>
+        </is>
+      </c>
+      <c r="E1415" t="inlineStr">
+        <is>
+          <t>Kementerian ESDM masih mereview permohonan perpanjangan IUPK PT Freeport Indonesia.</t>
+        </is>
+      </c>
+      <c r="F1415" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1415" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811170211-4-758367/freeport-sudah-ajukan-perpanjangan-izin-tambang--iupk--ini-kata-esdm</t>
+        </is>
+      </c>
+      <c r="H1415" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/01/23/dirjen-minerba-kementerian-esdm-tri-winarno-saat-menyampaikan-paparan-dalam-program-cnbc-indonesia-mining-zone-1769160383776_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1415" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1416">
+      <c r="A1416" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1416" t="inlineStr">
+        <is>
+          <t>Siap-Siap China Digulung Petaka, Beijing Darurat</t>
+        </is>
+      </c>
+      <c r="C1416" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 20:10:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1416" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1416" t="inlineStr">
+        <is>
+          <t>Beijing bersiap menghadapi hujan ekstrem mulai 11 Agustus 2026, dengan curah hujan diperkirakan melebihi 200 mm dalam 24 jam, meningkatkan risiko banjir.</t>
+        </is>
+      </c>
+      <c r="F1416" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1416" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811143603-4-758298/siap-siap-china-digulung-petaka-beijing-darurat</t>
+        </is>
+      </c>
+      <c r="H1416" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/10/sebuah-truk-terguling-akibat-angin-kencang-saat-topan-dolphin-menerjang-daratan-di-wenzhou-provinsi-zhejiang-tiongkok-pada-9-a-1786355485482_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1416" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1417">
+      <c r="A1417" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1417" t="inlineStr">
+        <is>
+          <t>Soal Pembatasan BBM Pertalite, Bahlil: Sesuai Jenis Kendaraannya</t>
+        </is>
+      </c>
+      <c r="C1417" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1417" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1417" t="inlineStr">
+        <is>
+          <t>Menteri ESDM Bahlil Lahadalia merumuskan kriteria yang akan dibatasi menggunakan BBM Pertalite</t>
+        </is>
+      </c>
+      <c r="F1417" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1417" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811171307-4-758381/soal-pembatasan-bbm-pertalite-bahlil-sesuai-jenis-kendaraannya</t>
+        </is>
+      </c>
+      <c r="H1417" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/menteri-esdm-bahlil-lahadalia-datangi-kantor-menteri-keuangan-purbaya-yudhi-sadewa-selasa-1182026-1786432462005_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1417" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1418">
+      <c r="A1418" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1418" t="inlineStr">
+        <is>
+          <t>PNBP Sektor ESDM Tahun 2026 Diramal Bisa Melebihi Target</t>
+        </is>
+      </c>
+      <c r="C1418" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:25:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1418" t="inlineStr">
+        <is>
+          <t>Firda Dwi Muliawati</t>
+        </is>
+      </c>
+      <c r="E1418" t="inlineStr">
+        <is>
+          <t>PNBP sektor ESDM diramal bakal melebihi target tahun 2026</t>
+        </is>
+      </c>
+      <c r="F1418" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1418" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811191022-4-758412/pnbp-sektor-esdm-tahun-2026-diramal-bisa-melebihi-target</t>
+        </is>
+      </c>
+      <c r="H1418" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2024/07/10/gedung-kementerian-esdm-dok-esdm_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1418" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1419">
+      <c r="A1419" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1419" t="inlineStr">
+        <is>
+          <t>Momen Utusan AS Datangi Menhan Sjafrie Sjamsoeddin, Ada Apa?</t>
+        </is>
+      </c>
+      <c r="C1419" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:20:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1419" t="inlineStr">
+        <is>
+          <t>Instagram/sjafrie.sjamsoeddin</t>
+        </is>
+      </c>
+      <c r="E1419" t="inlineStr">
+        <is>
+          <t>Menhan Sjafrie Sjamsoeddin bertemu pejabat pertahanan AS Elbridge A. Colby. Keduanya membahas penguatan kerja sama pertahanan dan keamanan kawasan.</t>
+        </is>
+      </c>
+      <c r="F1419" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1419" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811174948-7-758387/momen-utusan-as-datangi-menhan-sjafrie-sjamsoeddin-ada-apa</t>
+        </is>
+      </c>
+      <c r="H1419" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/menteri-pertahanan-menhan-sjafrie-sjamsoeddin-menerima-courtesy-call-sekaligus-melaksanakan-round-table-discussion-bersama-us--1786445238426_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1419" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1420">
+      <c r="A1420" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1420" t="inlineStr">
+        <is>
+          <t>Uji Sistem! Pembatasan Pengguna BBM Pertalite Bakal Dilakukan Bertahap</t>
+        </is>
+      </c>
+      <c r="C1420" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:15:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1420" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1420" t="inlineStr">
+        <is>
+          <t>Pemerintah bakal melakukan secara bertahap pembatasan pengguanaan BBM Pertalite</t>
+        </is>
+      </c>
+      <c r="F1420" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1420" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811183732-4-758407/uji-sistem-pembatasan-pengguna-bbm-pertalite-bakal-dilakukan-bertahap</t>
+        </is>
+      </c>
+      <c r="H1420" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2024/11/18/petugas-mengisi-bahan-bakar-minyak-bbm-jenis-pertalite-untuk-kendaraan-roda-dua-pada-salah-satu-spbu-di-jakarta-senin-18112024-8_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1420" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1421">
+      <c r="A1421" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1421" t="inlineStr">
+        <is>
+          <t>KP2MI Buka Pendaftaran Pelatihan Asta Mandala SMK Go Global!</t>
+        </is>
+      </c>
+      <c r="C1421" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:11:30 +0700</t>
+        </is>
+      </c>
+      <c r="D1421" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1421" t="inlineStr">
+        <is>
+          <t>Pendaftaran Pelatihan Asta Mandala SMK Go Global dibuka 12-16 Agustus 2026. Program ini siapkan generasi muda Indonesia untuk pasar kerja internasional.</t>
+        </is>
+      </c>
+      <c r="F1421" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1421" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811190548-4-758410/kp2mi-buka-pendaftaran-pelatihan-asta-mandala-smk-go-global</t>
+        </is>
+      </c>
+      <c r="H1421" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/dok-kementerian-pelindungan-pekerja-migran-indonesia-kp2mi-1786450231375_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1421" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1422">
+      <c r="A1422" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1422" t="inlineStr">
+        <is>
+          <t>Berita Duka: Rida Mulyana Mantan Sekjen KESDM Meninggal Dunia</t>
+        </is>
+      </c>
+      <c r="C1422" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:09:29 +0700</t>
+        </is>
+      </c>
+      <c r="D1422" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1422" t="inlineStr">
+        <is>
+          <t>Rida Mulyana mantan Sekjen Kementerian ESDM meninggal dunia</t>
+        </is>
+      </c>
+      <c r="F1422" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1422" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811185928-4-758411/berita-duka-rida-mulyana-mantan-sekjen-kesdm-meninggal-dunia</t>
+        </is>
+      </c>
+      <c r="H1422" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2018/01/10/fd501455-dd1c-48fd-a774-b70915471ff1_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1422" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1423">
+      <c r="A1423" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1423" t="inlineStr">
+        <is>
+          <t>Data Baru! Utang Pemerintah Rp10.293 T, 41% dari PDB</t>
+        </is>
+      </c>
+      <c r="C1423" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 19:01:52 +0700</t>
+        </is>
+      </c>
+      <c r="D1423" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1423" t="inlineStr">
+        <is>
+          <t>Direktorat Jenderal Pengelolaan Pembiayaan dan Risiko (DJPPR) merilis data terbaru total utang pemerintah pusat, per Semester I-2026.</t>
+        </is>
+      </c>
+      <c r="F1423" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1423" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811185938-4-758409/data-baru-utang-pemerintah-rp10293-t-41-dari-pdb</t>
+        </is>
+      </c>
+      <c r="H1423" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2024/01/10/suasana-gedung-kementerian-keuangan-kemenkeu-di-jakarta-rabu-1012024-19_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1423" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1424">
+      <c r="A1424" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1424" t="inlineStr">
+        <is>
+          <t>Menko PMK Pratikno Bantah Sakit dan Mundur dari Kabinet Presiden Prabowo</t>
+        </is>
+      </c>
+      <c r="C1424" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:55:30 +0700</t>
+        </is>
+      </c>
+      <c r="D1424" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1424" t="inlineStr">
+        <is>
+          <t>Pratikno menegaskan sedang bertugas melakukan percepatan pemadaman kebakaran hutan dan lahan (karhutla) di Taman Nasional Bromo Tengger Semeru, Jawa Timur.</t>
+        </is>
+      </c>
+      <c r="F1424" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1424" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811182030-4-758406/menko-pmk-pratikno-bantah-sakit-mundur-dari-kabinet-presiden-prabowo</t>
+        </is>
+      </c>
+      <c r="H1424" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2025/12/03/menteri-koordinator-bidang-pembangunan-manusia-dan-kebudayaan-pratikno-saat-menyampaikan-keterangan-pers-perkembangan-penanggu-1764745137945_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1424" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1425">
+      <c r="A1425" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1425" t="inlineStr">
+        <is>
+          <t>Ini Dia Jenis Kendaraan yang Tidak Akan Kena Pembatasan BBM Pertalite</t>
+        </is>
+      </c>
+      <c r="C1425" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:45:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1425" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1425" t="inlineStr">
+        <is>
+          <t>Ini jenis kendaraan yang tidak akan kena pembatasan BBM Pertalite</t>
+        </is>
+      </c>
+      <c r="F1425" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1425" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811181902-4-758405/ini-dia-jenis-kendaraan-yang-tidak-akan-kena-pembatasan-bbm-pertalite</t>
+        </is>
+      </c>
+      <c r="H1425" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/menteri-esdm-bahlil-lahadalia-dan-menteri-keuangan-purbaya-yudhi-sadewa-usai-melakukan-pertemuan-di-kantor-kementerian-keuanga-1786439887620_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1425" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1426">
+      <c r="A1426" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1426" t="inlineStr">
+        <is>
+          <t>Soal Rencana Pembatasan Pertalite, Bahlil: Biar Subsidi Tepat Sasaran</t>
+        </is>
+      </c>
+      <c r="C1426" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:40:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1426" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1426" t="inlineStr">
+        <is>
+          <t>Menteri ESDM Bahlil Lahadalia menekankan bahwa pembatasan BBM Pertalite supaya subsidi tepat sasaran</t>
+        </is>
+      </c>
+      <c r="F1426" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1426" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811165958-4-758365/soal-rencana-pembatasan-pertalite-bahlil-biar-subsidi-tepat-sasaran</t>
+        </is>
+      </c>
+      <c r="H1426" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/menteri-esdm-bahlil-lahadalia-dan-menteri-keuangan-purbaya-yudhi-sadewa-usai-melakukan-pertemuan-di-kantor-kementerian-keuanga-1786439887620_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1426" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1427">
+      <c r="A1427" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1427" t="inlineStr">
+        <is>
+          <t>CNG Alternatif Pengganti LPG 3 Kg Bakal Diuji Coba Pekan Depan</t>
+        </is>
+      </c>
+      <c r="C1427" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:35:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1427" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1427" t="inlineStr">
+        <is>
+          <t>Pemerintah bakal melakukan uji coba CNG sebagai alternatif pengganti LPG 3 Kg</t>
+        </is>
+      </c>
+      <c r="F1427" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1427" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811175616-4-758394/cng-alternatif-pengganti-lpg-3-kg-bakal-diuji-coba-pekan-depan</t>
+        </is>
+      </c>
+      <c r="H1427" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/06/29/ilustrasi-cng-merah-putih-3kg-1782728074855_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1427" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1428">
+      <c r="A1428" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1428" t="inlineStr">
+        <is>
+          <t>Pembelian Pertalite Mau Dibatasi, Purbaya: Kita Incar Kalangan Atas</t>
+        </is>
+      </c>
+      <c r="C1428" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:30:17 +0700</t>
+        </is>
+      </c>
+      <c r="D1428" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1428" t="inlineStr">
+        <is>
+          <t>Rencana pemerintah untuk membatasi pembelian bahan bakar minyak (BBM) bersubsidi ditujukan supaya konsumsinya tepat sasaran.</t>
+        </is>
+      </c>
+      <c r="F1428" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1428" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811165717-4-758364/pembelian-pertalite-mau-dibatasi-purbaya-kita-incar-kalangan-atas</t>
+        </is>
+      </c>
+      <c r="H1428" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/07/21/menteri-keuangan-menkeu-purbaya-yudhi-sadewa-saat-menyampaikan-pemaparan-dalam-konferensi-pers-apbn-kita-edisi-juli-2026-di-ka-1784620747563_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1428" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1429">
+      <c r="A1429" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1429" t="inlineStr">
+        <is>
+          <t>Integrasi Satusehat-Siak, Akte Kelahiran Terbit Setelah Bayi Lahir</t>
+        </is>
+      </c>
+      <c r="C1429" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 18:15:06 +0700</t>
+        </is>
+      </c>
+      <c r="D1429" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1429" t="inlineStr">
+        <is>
+          <t>Integrasi Satusehat-Siak, Akte Kelahiran Langsung Terbit Setelah Bayi Lahir</t>
+        </is>
+      </c>
+      <c r="F1429" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1429" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811145924-8-758316/integrasi-satusehat-siak-akte-kelahiran-terbit-setelah-bayi-lahir</t>
+        </is>
+      </c>
+      <c r="H1429" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/integrasi-satusehat-siak-akte-kelahiran-langsung-terbit-setelah-bayi-lahir-1786443833062_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1429" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1430">
+      <c r="A1430" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1430" t="inlineStr">
+        <is>
+          <t>Fenomena Baru, Ada Perubahan Perilaku di Pengguna Asuransi Kendaraan</t>
+        </is>
+      </c>
+      <c r="C1430" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:56:56 +0700</t>
+        </is>
+      </c>
+      <c r="D1430" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1430" t="inlineStr">
+        <is>
+          <t>Vincent Soegianto, CEO Oona Insurance, mengungkap perubahan perilaku pengguna asuransi kendaraan, kini fokus pada perlindungan risiko personal accident.</t>
+        </is>
+      </c>
+      <c r="F1430" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1430" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811175135-4-758393/fenomena-baru-ada-perubahan-perilaku-di-pengguna-asuransi-kendaraan</t>
+        </is>
+      </c>
+      <c r="H1430" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/president-director-chief-executive-officer-ceo-oona-insurance-indonesia-vincent-c-soegianto-saat-menyampaikan-pemaparan-dalam--1786417368032_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1430" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1431">
+      <c r="A1431" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1431" t="inlineStr">
+        <is>
+          <t>Daerah di Jabar Ini Mau Disulap Jadi Pusat Mebel dan Kerajinan RI</t>
+        </is>
+      </c>
+      <c r="C1431" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:55:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1431" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1431" t="inlineStr">
+        <is>
+          <t>Daerah di Jabar ini berpotensi jadi pusat industri mebel dan kerajinan baru di Indonesia. Ini lokasinya.</t>
+        </is>
+      </c>
+      <c r="F1431" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1431" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811164429-4-758359/daerah-di-jabar-ini-mau-disulap-jadi-pusat-mebel-dan-kerajinan-ri</t>
+        </is>
+      </c>
+      <c r="H1431" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2022/02/18/pabrik-pembuatan-mebel-19_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1431" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1432">
+      <c r="A1432" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1432" t="inlineStr">
+        <is>
+          <t>Konsumsi BBM Pertalite Bakal Dibatasi, Ini Penjelasan Bahlil dan Purbaya</t>
+        </is>
+      </c>
+      <c r="C1432" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:50:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1432" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1432" t="inlineStr">
+        <is>
+          <t>Menteri Keuangan dan Menteri ESDM bahas pembatasan subsidi Pertalite untuk kelompok ekonomi atas.</t>
+        </is>
+      </c>
+      <c r="F1432" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1432" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811164705-4-758361/konsumsi-bbm-pertalite-bakal-dibatasi-ini-penjelasan-bahlil-purbaya</t>
+        </is>
+      </c>
+      <c r="H1432" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/menteri-esdm-bahlil-lahadalia-dan-menteri-keuangan-purbaya-yudhi-sadewa-usai-melakukan-pertemuan-di-kantor-kementerian-keuanga-1786439887620_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1432" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1433">
+      <c r="A1433" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1433" t="inlineStr">
+        <is>
+          <t>Industri Sepatu RI Lagi Tancap Gas-Gegara AS Jadi Dipepet 2 Negara Ini</t>
+        </is>
+      </c>
+      <c r="C1433" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:45:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1433" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1433" t="inlineStr">
+        <is>
+          <t>Industri kulit dan alas kaki tumbuh 11,30% pada kuartal II-2026, tertinggi dalam 15 kuartal.</t>
+        </is>
+      </c>
+      <c r="F1433" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1433" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811172207-4-758382/industri-sepatu-ri-lagi-tancap-gas-gegara-as-jadi-dipepet-2-negara-ini</t>
+        </is>
+      </c>
+      <c r="H1433" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2025/07/10/ilustrasi-sepatu-dok-freepik-1752130339557_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1433" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1434">
+      <c r="A1434" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1434" t="inlineStr">
+        <is>
+          <t>Trump Diancam Dibunuh, Diam-Diam Kabur dari Turki Naik Truk Katering</t>
+        </is>
+      </c>
+      <c r="C1434" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:35:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1434" t="inlineStr">
+        <is>
+          <t>sef</t>
+        </is>
+      </c>
+      <c r="E1434" t="inlineStr">
+        <is>
+          <t>Laporan The Washington Post mengungkap ancaman pembunuhan terhadap Trump, memaksanya dipindahkan secara rahasia ke pesawat militer saat KTT NATO.</t>
+        </is>
+      </c>
+      <c r="F1434" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1434" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811141820-4-758288/trump-diancam-dibunuh-diam-diam-kabur-dari-turki-naik-truk-katering</t>
+        </is>
+      </c>
+      <c r="H1434" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/pesawat-air-force-one-jenis-vc-25a-mendarat-di-pangkalan-angkatan-udara-nellis-nevada-21-agustus-2012-vc-25a-adalah-versi-modi-1786429713376_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1434" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1435">
+      <c r="A1435" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1435" t="inlineStr">
+        <is>
+          <t>Bahlil Pastikan Kendaraan Roda Dua Tak Kena Pembatasan BBM Pertalite</t>
+        </is>
+      </c>
+      <c r="C1435" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1435" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1435" t="inlineStr">
+        <is>
+          <t>Menteri ESDM Bahlil memastikan tidak ada pembatasan pembelian BBM subsidi Pertalite untuk sepeda motor.</t>
+        </is>
+      </c>
+      <c r="F1435" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1435" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811162912-4-758352/bahlil-pastikan-kendaraan-roda-dua-tak-kena-pembatasan-bbm-pertalite</t>
+        </is>
+      </c>
+      <c r="H1435" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/menteri-esdm-bahlil-lahadalia-dan-menteri-keuangan-purbaya-yudhi-sadewa-usai-melakukan-pertemuan-di-kantor-kementerian-keuanga-1786439887710_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1435" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1436">
+      <c r="A1436" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1436" t="inlineStr">
+        <is>
+          <t>Ban Murah Ini Marak Dijual Bebas di Pinggir Jalan, Horor Kalau Dipakai</t>
+        </is>
+      </c>
+      <c r="C1436" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:23:29 +0700</t>
+        </is>
+      </c>
+      <c r="D1436" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia/Tri Susilo</t>
+        </is>
+      </c>
+      <c r="E1436" t="inlineStr">
+        <is>
+          <t>Ban motor ini makin diminati karena harganya murah meriah. Ini penampakannya.</t>
+        </is>
+      </c>
+      <c r="F1436" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1436" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811164640-7-758360/ban-murah-ini-marak-dijual-bebas-di-pinggir-jalan-horor-kalau-dipakai</t>
+        </is>
+      </c>
+      <c r="H1436" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/seorang-pekerja-menyelesaikan-pengerikan-ulang-ban-motor-bekas-vulkanisir-di-kawasan-beji-depok-jawa-barat-selasa-1182026-1786442591491_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1436" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1437">
+      <c r="A1437" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1437" t="inlineStr">
+        <is>
+          <t>Purbaya Soal Kondisi Anggaran Subsidi BBM: Aman!</t>
+        </is>
+      </c>
+      <c r="C1437" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:21:35 +0700</t>
+        </is>
+      </c>
+      <c r="D1437" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1437" t="inlineStr">
+        <is>
+          <t>Menteri Keuangan Purbaya Yudhi Sadewa memastikan anggaran subsidi BBM aman meski harga minyak fluktuatif.</t>
+        </is>
+      </c>
+      <c r="F1437" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1437" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811171439-4-758380/purbaya-soal-kondisi-anggaran-subsidi-bbm-aman</t>
+        </is>
+      </c>
+      <c r="H1437" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/menteri-esdm-bahlil-lahadalia-dan-menteri-keuangan-purbaya-yudhi-sadewa-usai-melakukan-pertemuan-di-kantor-kementerian-keuanga-1786439887710_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1437" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1438">
+      <c r="A1438" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1438" t="inlineStr">
+        <is>
+          <t>Gempa Guncang Kolombia M 7,4 - Tak Ada Pajak Rumah Kontrakan di 2027</t>
+        </is>
+      </c>
+      <c r="C1438" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:20:41 +0700</t>
+        </is>
+      </c>
+      <c r="D1438" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1438" t="inlineStr">
+        <is>
+          <t>Gempa Guncang Kolombia M 7,4 - Tak Ada Pajak Rumah Kontrakan di 2027</t>
+        </is>
+      </c>
+      <c r="F1438" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1438" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811145923-8-758314/gempa-guncang-kolombia-m-74--tak-ada-pajak-rumah-kontrakan-di-2027</t>
+        </is>
+      </c>
+      <c r="H1438" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/gempa-guncang-kolombia-m-74-tak-ada-pajak-rumah-kontrakan-di-2027-1786442681748_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1438" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1439">
+      <c r="A1439" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1439" t="inlineStr">
+        <is>
+          <t>Video: IHSG 7.000: Asing Silakan Masuk, Jangan Ditopang Ritel Terus</t>
+        </is>
+      </c>
+      <c r="C1439" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:15:30 +0700</t>
+        </is>
+      </c>
+      <c r="D1439" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1439" t="inlineStr">
+        <is>
+          <t>IHSG 7.000: Asing Silakan Masuk, Jangan Ditopang Ritel Terus</t>
+        </is>
+      </c>
+      <c r="F1439" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1439" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811135109-8-758312/video-ihsg-7000-asing-silakan-masuk-jangan-ditopang-ritel-terus</t>
+        </is>
+      </c>
+      <c r="H1439" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/ihsg-7000-asing-silakan-masuk-jangan-ditopang-ritel-terus-1786442652215_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1439" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1440">
+      <c r="A1440" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1440" t="inlineStr">
+        <is>
+          <t>Kemenperin Tunjuk Biang Keladi Mamin RI Kalah Saing, Ternyata Ini</t>
+        </is>
+      </c>
+      <c r="C1440" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:15:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1440" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1440" t="inlineStr">
+        <is>
+          <t>Kemenperin ungkap tantangan bahan baku mempengaruhi daya saing industri makanan dan minuman Indonesia. Impor dan penguatan lokal jadi solusi untuk bersaing.</t>
+        </is>
+      </c>
+      <c r="F1440" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1440" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811162153-4-758348/kemenperin-tunjuk-biang-keladi-mamin-ri-kalah-saing-ternyata-ini</t>
+        </is>
+      </c>
+      <c r="H1440" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/ilustrasi-pabrik-makanan-1786441256617_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1440" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1441">
+      <c r="A1441" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1441" t="inlineStr">
+        <is>
+          <t>Kronologi Bea Cukai Bongkar Penyelundupan 8,9 Juta Batang Rokok Ilegal</t>
+        </is>
+      </c>
+      <c r="C1441" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:10:04 +0700</t>
+        </is>
+      </c>
+      <c r="D1441" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1441" t="inlineStr">
+        <is>
+          <t>Direktorat Jenderal Bea Cukai menggagalkan penyelundupan 8,96 juta batang rokok ilegal senilai Rp13,30 miliar. Penindakan berawal dari informasi masyarakat.</t>
+        </is>
+      </c>
+      <c r="F1441" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1441" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811160522-4-758337/kronologi-bea-cukai-bongkar-penyelundupan-89-juta-batang-rokok-ilegal</t>
+        </is>
+      </c>
+      <c r="H1441" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/direktur-jenderal-bea-dan-cukai-indonesia-djaka-budi-utama-saat-melihat-barang-bukti-rokok-ilegal-dalam-konferensi-pers-penind-1786435165633_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1441" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1442">
+      <c r="A1442" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1442" t="inlineStr">
+        <is>
+          <t>Pelaku Industri Energi, Regulator, dan Perbankan Berkumpul Bahas Energi</t>
+        </is>
+      </c>
+      <c r="C1442" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 17:00:37 +0700</t>
+        </is>
+      </c>
+      <c r="D1442" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1442" t="inlineStr">
+        <is>
+          <t>Pelaku Industri Energi, Regulator, dan Perbankan Berkumpul Bahas 'Jurus' Jaga Ketahanan Energi Indonesia</t>
+        </is>
+      </c>
+      <c r="F1442" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1442" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811132133-8-758277/pelaku-industri-energi-regulator-perbankan-berkumpul-bahas-energi</t>
+        </is>
+      </c>
+      <c r="H1442" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/pelaku-industri-energi-regulator-perbankan-berkumpul-bahas-jurus-jaga-ketahanan-energi-indonesia-1786431304333_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1442" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1443">
+      <c r="A1443" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1443" t="inlineStr">
+        <is>
+          <t>Api Membara, Kilang Minyak Terbakar Hebat Usai Drone Jatuh</t>
+        </is>
+      </c>
+      <c r="C1443" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 16:55:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1443" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1443" t="inlineStr">
+        <is>
+          <t>Api berkobar di dalam tangki penyimpanan sementara petugas pemadam kebakaran berupaya mengendalikan kobaran api, di sebuah kilang minyak di Zawiya, Libya.</t>
+        </is>
+      </c>
+      <c r="F1443" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1443" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811121210-7-758227/api-membara-kilang-minyak-terbakar-hebat-usai-drone-jatuh</t>
+        </is>
+      </c>
+      <c r="H1443" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/api-berkobar-di-dalam-tangki-penyimpanan-sementara-petugas-pemadam-kebakaran-berupaya-mengendalikan-kobaran-api-di-sebuah-kila-1786420591759_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1443" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1444">
+      <c r="A1444" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1444" t="inlineStr">
+        <is>
+          <t>Bea Cukai Gagalkan 8,96 Juta Rokok Ilegal, Negara Nyaris Rugi Rp8,6 M</t>
+        </is>
+      </c>
+      <c r="C1444" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 16:50:47 +0700</t>
+        </is>
+      </c>
+      <c r="D1444" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1444" t="inlineStr">
+        <is>
+          <t>Bea Cukai gagalkan pengiriman 8,96 juta batang rokok ilegal di Tanjung Priok. Barang senilai Rp13,31 miliar itu berpotensi rugikan negara Rp8,67 miliar.</t>
+        </is>
+      </c>
+      <c r="F1444" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1444" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811152245-7-758321/bea-cukai-gagalkan-896-juta-rokok-ilegal-negara-nyaris-rugi-rp86-m</t>
+        </is>
+      </c>
+      <c r="H1444" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/direktur-jenderal-bea-dan-cukai-indonesia-djaka-budi-utama-saat-melihat-barang-bukti-rokok-ilegal-dalam-konferensi-pers-penind-1786435165695_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1444" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1445">
+      <c r="A1445" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1445" t="inlineStr">
+        <is>
+          <t>PLN dan Komunitas Rappo Makassar 'Sulap' 10,5 Ton Sampah Jadi Furnitur</t>
+        </is>
+      </c>
+      <c r="C1445" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 16:45:23 +0700</t>
+        </is>
+      </c>
+      <c r="D1445" t="inlineStr">
+        <is>
+          <t>Khoirul Anam</t>
+        </is>
+      </c>
+      <c r="E1445" t="inlineStr">
+        <is>
+          <t>Masyarakat Pesisir Untia, Makassar, bersama Rappo, mengolah sampah plastik menjadi furnitur. Program ini mendukung ekonomi sirkular dan pemberdayaan masyarakat.</t>
+        </is>
+      </c>
+      <c r="F1445" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1445" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811163503-4-758355/pln-dan-komunitas-rappo-makassar-sulap-105-ton-sampah-jadi-furnitur</t>
+        </is>
+      </c>
+      <c r="H1445" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/bersama-komunitas-pemberdayaan-rappo-masyarakat-makassar-ubah-sampah-jadi-furniturkhoirul-anam-1786441486273_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1445" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1446">
+      <c r="A1446" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1446" t="inlineStr">
+        <is>
+          <t>China Siap-Siap Masuk Madura, Bangun Komplek Pabrik di Sini</t>
+        </is>
+      </c>
+      <c r="C1446" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 16:45:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1446" t="inlineStr">
+        <is>
+          <t>Ferry Sandi</t>
+        </is>
+      </c>
+      <c r="E1446" t="inlineStr">
+        <is>
+          <t>China berinvestasi besar di Madura. Lokasinya di sini.</t>
+        </is>
+      </c>
+      <c r="F1446" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1446" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811154847-4-758335/china-siap-siap-masuk-madura-bangun-komplek-pabrik-di-sini</t>
+        </is>
+      </c>
+      <c r="H1446" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/pulau-madura-dok-detikcom-1786427513459_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1446" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1447">
+      <c r="A1447" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1447" t="inlineStr">
+        <is>
+          <t>Pembatasan Pembelian Pertalite Mulai Kapan? Ini Kata Purbaya</t>
+        </is>
+      </c>
+      <c r="C1447" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 16:37:44 +0700</t>
+        </is>
+      </c>
+      <c r="D1447" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1447" t="inlineStr">
+        <is>
+          <t>Pemerintah tengah menyusun kebijakan baru yang ditujukan untuk membatasi konsumsi bahan bakar minyak (BBM) jenis pertalite.</t>
+        </is>
+      </c>
+      <c r="F1447" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1447" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811163638-4-758354/pembatasan-pembelian-pertalite-mulai-kapan-ini-kata-purbaya</t>
+        </is>
+      </c>
+      <c r="H1447" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/menteri-esdm-bahlil-lahadalia-dan-menteri-keuangan-purbaya-yudhi-sadewa-usai-melakukan-pertemuan-di-kantor-kementerian-keuanga-1786439887710_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1447" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1448">
+      <c r="A1448" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1448" t="inlineStr">
+        <is>
+          <t>Amran Mau Bagi-Bagi Alsintan Gratis untuk Buruh Tani, Caranya Begini</t>
+        </is>
+      </c>
+      <c r="C1448" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 16:35:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1448" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1448" t="inlineStr">
+        <is>
+          <t>Mentan Amran mau bagi-bagi alat pertanian gratis untuk buruh tani di Indonesia. Caranya begini.</t>
+        </is>
+      </c>
+      <c r="F1448" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1448" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811150425-4-758315/amran-mau-bagi-bagi-alsintan-gratis-untuk-buruh-tani-caranya-begini</t>
+        </is>
+      </c>
+      <c r="H1448" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/menteri-pertanian-mentan-amran-sulaiman-saat-dalam-kunjungannya-ke-gresik-jawa-timur-juga-mengecek-langsung-lahan-pertanian-ya-1786435312407_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1448" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1449">
+      <c r="A1449" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1449" t="inlineStr">
+        <is>
+          <t>Pemerintah Bakal Batasi Penggunaan BBM Pertalite Untuk Golongan Ini</t>
+        </is>
+      </c>
+      <c r="C1449" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 16:31:55 +0700</t>
+        </is>
+      </c>
+      <c r="D1449" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1449" t="inlineStr">
+        <is>
+          <t>Pemerintah berencana membatasi BBM subsidi Pertalite untuk desil 9 dan 10</t>
+        </is>
+      </c>
+      <c r="F1449" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1449" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811162629-4-758351/pemerintah-bakal-batasi-penggunaan-bbm-pertalite-untuk-golongan-ini</t>
+        </is>
+      </c>
+      <c r="H1449" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/menteri-esdm-bahlil-lahadalia-dan-menteri-keuangan-purbaya-yudhi-sadewa-usai-melakukan-pertemuan-di-kantor-kementerian-keuanga-1786439887710_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1449" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1450">
+      <c r="A1450" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1450" t="inlineStr">
+        <is>
+          <t>'Jurus' Bank DBS Indonesia Dukung Pertumbuhan Sektor ERI</t>
+        </is>
+      </c>
+      <c r="C1450" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 16:23:12 +0700</t>
+        </is>
+      </c>
+      <c r="D1450" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1450" t="inlineStr">
+        <is>
+          <t>'Jurus' Bank DBS Indonesia Dukung Pertumbuhan Sektor Energi, Sumber Daya, dan Infrastruktur (ERI)</t>
+        </is>
+      </c>
+      <c r="F1450" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1450" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811132134-8-758267/jurus-bank-dbs-indonesia-dukung-pertumbuhan-sektor-eri</t>
+        </is>
+      </c>
+      <c r="H1450" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/jurus-bank-dbs-indonesia-dukung-pertumbuhan-sektor-energi-sumber-daya-infrastruktur-eri-1786431277947_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1450" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1451">
+      <c r="A1451" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1451" t="inlineStr">
+        <is>
+          <t>Bahlil-Purbaya Rapat, Bahas Rencana Pembatasan Pengguna BBM Pertalite!</t>
+        </is>
+      </c>
+      <c r="C1451" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 16:20:57 +0700</t>
+        </is>
+      </c>
+      <c r="D1451" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1451" t="inlineStr">
+        <is>
+          <t>Menteri Keuangan Purbaya Yudhi Sadewa dan Menteri ESDM Bahlil merencang pembatasan penggunaan BBM jenis Pertalite untuk desil 9 dan 10</t>
+        </is>
+      </c>
+      <c r="F1451" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1451" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811153506-4-758345/bahlil-purbaya-rapat-bahas-rencana-pembatasan-pengguna-bbm-pertalite</t>
+        </is>
+      </c>
+      <c r="H1451" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/menteri-esdm-bahlil-lahadalia-dan-menteri-keuangan-purbaya-yudhi-sadewa-usai-melakukan-pertemuan-di-kantor-kementerian-keuanga-1786439887620_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1451" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1452">
+      <c r="A1452" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1452" t="inlineStr">
+        <is>
+          <t>Bom Mobil Meledak, Kepala Intelijen Militer Tewas</t>
+        </is>
+      </c>
+      <c r="C1452" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 16:15:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1452" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1452" t="inlineStr">
+        <is>
+          <t>Mayor Jenderal Fawzi al-Mansouri, kepala intelijen militer Libya timur, tewas dalam serangan bom mobil di Benghazi. Situasi politik Libya semakin tegang.</t>
+        </is>
+      </c>
+      <c r="F1452" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1452" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811145033-4-758305/bom-mobil-meledak-kepala-intelijen-militer-tewas</t>
+        </is>
+      </c>
+      <c r="H1452" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2020/11/11/ilustrasi-bom_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1452" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1453">
+      <c r="A1453" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1453" t="inlineStr">
+        <is>
+          <t>Bea Cukai Gagalkan Penyelundupan 8,96 Juta Rokok Ilegal via Kereta</t>
+        </is>
+      </c>
+      <c r="C1453" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 16:05:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1453" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1453" t="inlineStr">
+        <is>
+          <t>BC Tanjung Priok gagalkan pengiriman 8,96 juta batang rokok ilegal tanpa pita cukai. Nilai barang diperkirakan Rp13,30 miliar.</t>
+        </is>
+      </c>
+      <c r="F1453" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1453" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811150848-4-758319/bea-cukai-gagalkan-penyelundupan-896-juta-rokok-ilegal-via-kereta</t>
+        </is>
+      </c>
+      <c r="H1453" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/direktur-jenderal-bea-dan-cukai-indonesia-djaka-budi-utama-saat-menyampaikan-konferensi-pers-penindakan-rokok-ilegal-kpu-bea-d-1786433777101_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1453" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1454">
+      <c r="A1454" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1454" t="inlineStr">
+        <is>
+          <t>Masjid Istiqlal Investasikan Dana Amal, Trump Tagih Kompensasi Iran</t>
+        </is>
+      </c>
+      <c r="C1454" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 15:45:34 +0700</t>
+        </is>
+      </c>
+      <c r="D1454" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1454" t="inlineStr">
+        <is>
+          <t>Masjid Istiqlal Investasikan Dana Amal, Trump Tagih Kompensasi Iran</t>
+        </is>
+      </c>
+      <c r="F1454" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1454" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811132256-8-758268/masjid-istiqlal-investasikan-dana-amal-trump-tagih-kompensasi-iran</t>
+        </is>
+      </c>
+      <c r="H1454" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/masjid-istiqlal-investasikan-dana-amal-trump-tagih-kompensasi-iran-1786434754535_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1454" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1455">
+      <c r="A1455" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1455" t="inlineStr">
+        <is>
+          <t>Wamendag Keluarkan Jurus Ini Kejar Target Ekspor RI US$315 Miliar</t>
+        </is>
+      </c>
+      <c r="C1455" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 15:45:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1455" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1455" t="inlineStr">
+        <is>
+          <t>Kementerian Perdagangan targetkan ekspor Indonesia mencapai US$315 miliar pada 2026. Wamendag Roro siap keluarkan jurus ini.</t>
+        </is>
+      </c>
+      <c r="F1455" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1455" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811134000-4-758274/wamendag-keluarkan-jurus-ini-kejar-target-ekspor-ri-us-315-miliar</t>
+        </is>
+      </c>
+      <c r="H1455" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/wakil-menteri-perdagangan-wamendag-dyah-roro-esti-widya-putri-dalam-acara-indonesia-fb-trade-promotion-forum-di-auditorium-kem-1786425998018_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1455" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1456">
+      <c r="A1456" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1456" t="inlineStr">
+        <is>
+          <t>Update Terbaru Perang Iran, Trump Sebut AS Kuasai 100% Selat Hormuz</t>
+        </is>
+      </c>
+      <c r="C1456" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 15:40:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1456" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1456" t="inlineStr">
+        <is>
+          <t>Presiden Trump klaim AS menguasai 100% Selat Hormuz, menyebut posisi AS sebagai "tembok baja". Sanksi Iran dan harga minyak melonjak akibat ketegangan ini.</t>
+        </is>
+      </c>
+      <c r="F1456" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1456" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811150937-4-758320/update-terbaru-perang-iran-trump-sebut-as-kuasai-100-selat-hormuz</t>
+        </is>
+      </c>
+      <c r="H1456" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/06/18/g7-summit-1781764542605_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1456" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1457">
+      <c r="A1457" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1457" t="inlineStr">
+        <is>
+          <t>Pertamina Tuntaskan Docking 12 Kapal, Distribusi Energi RI Makin Andal</t>
+        </is>
+      </c>
+      <c r="C1457" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 15:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1457" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1457" t="inlineStr">
+        <is>
+          <t>Pertamina rampungkan proses docking terhadap 12 kapal</t>
+        </is>
+      </c>
+      <c r="F1457" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1457" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811132351-4-758269/pertamina-tuntaskan-docking-12-kapal-distribusi-energi-ri-makin-andal</t>
+        </is>
+      </c>
+      <c r="H1457" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/pertamina-rampungkan-proses-docking-kapal-1786429678221_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1457" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1458">
+      <c r="A1458" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1458" t="inlineStr">
+        <is>
+          <t>Airlangga Bakal Perluas Pembiayaan Buat UMKM, Naik Jadi Rp2.000 T</t>
+        </is>
+      </c>
+      <c r="C1458" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 15:25:15 +0700</t>
+        </is>
+      </c>
+      <c r="D1458" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1458" t="inlineStr">
+        <is>
+          <t>Menko Airlangga menaikkan target pembiayaan UMKM dari Rp1.500 triliun menjadi Rp2.000 triliun untuk memperluas akses dan mendorong digitalisasi.</t>
+        </is>
+      </c>
+      <c r="F1458" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1458" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811141424-4-758285/airlangga-bakal-perluas-pembiayaan-buat-umkm-naik-jadi-rp2000-t</t>
+        </is>
+      </c>
+      <c r="H1458" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/menko-perekonomian-airlangga-hartarto-dalam-acara-umkm-finance-summit-2026-dengan-tema-penguatan-akses-pembiayaan-dan-ekosiste-1786418467181_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1458" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1459">
+      <c r="A1459" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1459" t="inlineStr">
+        <is>
+          <t>APPI Curhat Soal Penggunaan Jasa Debt Collector, Ini Alasannya!</t>
+        </is>
+      </c>
+      <c r="C1459" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 15:11:51 +0700</t>
+        </is>
+      </c>
+      <c r="D1459" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1459" t="inlineStr">
+        <is>
+          <t>Ketua APPI Suwandi Wiratno menjelaskan tantangan multifinance, termasuk penggunaan debt collector untuk pemulihan pembiayaan. Kualitas pembiayaan harus dijaga.</t>
+        </is>
+      </c>
+      <c r="F1459" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1459" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811150829-4-758318/appi-curhat-soal-penggunaan-jasa-debt-collector-ini-alasannya</t>
+        </is>
+      </c>
+      <c r="H1459" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/ketua-umum-asosiasi-perusahaan-pembiayaan-indonesia-appi-suwandi-wiratno-saat-menyampaikan-pemaparan-dalam-multifinance-ceo-ga-1786416630643_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1459" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1460">
+      <c r="A1460" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1460" t="inlineStr">
+        <is>
+          <t>Pertamina Gandeng Dukcapil Perkuat Data Penerima LPG Subsidi</t>
+        </is>
+      </c>
+      <c r="C1460" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 15:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1460" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1460" t="inlineStr">
+        <is>
+          <t>Pertamina dan Ditjen Dukcapil menandatangani PKS untuk pemanfaatan data kependudukan mendukung penyaluran energi bersubsidi</t>
+        </is>
+      </c>
+      <c r="F1460" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1460" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811141801-4-758287/pertamina-gandeng-dukcapil-perkuat-data-penerima-lpg-subsidi</t>
+        </is>
+      </c>
+      <c r="H1460" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2018/05/21/bd9283be-cc65-40eb-b64e-9364804a54bd_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1460" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1461">
+      <c r="A1461" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1461" t="inlineStr">
+        <is>
+          <t>Mensesneg Sebut Ojol Tetap Dapat Bonus Hari Raya Walau Berstatus UMKM</t>
+        </is>
+      </c>
+      <c r="C1461" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:57:30 +0700</t>
+        </is>
+      </c>
+      <c r="D1461" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1461" t="inlineStr">
+        <is>
+          <t>Menteri Sekretaris Negara Prasetyo Hadi memastikan pengendara transportasi online tetap menerima Bantuan Hari Raya meski statusnya berubah menjadi UMKM.</t>
+        </is>
+      </c>
+      <c r="F1461" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1461" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811140851-4-758284/mensesneg-sebut-ojol-tetap-dapat-bonus-hari-raya-walau-berstatus-umkm</t>
+        </is>
+      </c>
+      <c r="H1461" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/01/15/menteri-sekretaris-negara-mensesneg-ri-prasetyo-hadi-saat-doorstop-di-kawasan-istana-negara-jakarta-kamis-1512026-cnbc-indones-1768443750862_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1461" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1462">
+      <c r="A1462" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1462" t="inlineStr">
+        <is>
+          <t>Timur Tengah Ditarget Jadi Pasar Produk Mamin Halal RI, Ini Alasannya</t>
+        </is>
+      </c>
+      <c r="C1462" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:55:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1462" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1462" t="inlineStr">
+        <is>
+          <t>Kemendag targetkan pasar Timur Tengah untuk ekspor produk makanan halal Indonesia. Ini alasannya.</t>
+        </is>
+      </c>
+      <c r="F1462" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1462" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811141746-4-758290/timur-tengah-ditarget-jadi-pasar-produk-mamin-halal-ri-ini-alasannya</t>
+        </is>
+      </c>
+      <c r="H1462" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2025/08/07/suasana-area-booth-makanan-dan-minuman-dalam-acara-lps-financial-festival-2025-di-dyandra-convention-center-surabaya-jawa-timu-1754550427584_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1462" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1463">
+      <c r="A1463" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1463" t="inlineStr">
+        <is>
+          <t>Mobil China di RI Makin Ganas: BYD Salip Honda, Jaecoo-Geely Mengancam</t>
+        </is>
+      </c>
+      <c r="C1463" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:53:24 +0700</t>
+        </is>
+      </c>
+      <c r="D1463" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1463" t="inlineStr">
+        <is>
+          <t>Persaingan pasar mobil Indonesia berubah, dengan BYD menembus lima besar penjualan. Penjualan kendaraan tumbuh 18,3% di 2026.</t>
+        </is>
+      </c>
+      <c r="F1463" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1463" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811144110-4-758301/mobil-china-di-ri-makin-ganas-byd-salip-honda-jaecoo-geely-mengancam</t>
+        </is>
+      </c>
+      <c r="H1463" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/01/pengunjung-melihat-byd-atto-1-dalam-ajang-pameran-gaikindo-indonesia-international-auto-show-giias-2026-yang-berlangsung-di-in-1785582470761_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1463" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1464">
+      <c r="A1464" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1464" t="inlineStr">
+        <is>
+          <t>Video: Tanggapi Pakta Pertahanan Mekah, Iran Tegaskan Tak Khawatir</t>
+        </is>
+      </c>
+      <c r="C1464" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:48:24 +0700</t>
+        </is>
+      </c>
+      <c r="D1464" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1464" t="inlineStr">
+        <is>
+          <t>Tanggapi Pakta Pertahanan Mekah, Iran Tegaskan Tak Khawatir</t>
+        </is>
+      </c>
+      <c r="F1464" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1464" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811131951-8-758264/video-tanggapi-pakta-pertahanan-mekah-iran-tegaskan-tak-khawatir</t>
+        </is>
+      </c>
+      <c r="H1464" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/tanggapi-pakta-pertahanan-mekah-iran-tegaskan-tak-khawatir-1786434398636_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1464" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1465">
+      <c r="A1465" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1465" t="inlineStr">
+        <is>
+          <t>Lengkap! Ini Rincian Bantuan Prabowo ke Pemda Buat Bayar Gaji PNS-PPPK</t>
+        </is>
+      </c>
+      <c r="C1465" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:45:05 +0700</t>
+        </is>
+      </c>
+      <c r="D1465" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1465" t="inlineStr">
+        <is>
+          <t>Seluruh bantuan itu ia telah ditransfer ke pemda yang mengalami tekanan fiskal sejak 7 Agustus 2026.</t>
+        </is>
+      </c>
+      <c r="F1465" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1465" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811133536-4-758272/lengkap-ini-rincian-bantuan-prabowo-ke-pemda-buat-bayar-gaji-pns-pppk</t>
+        </is>
+      </c>
+      <c r="H1465" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/05/purbaya-yudhi-sadewa-menteri-keuangan-nufransa-wira-sakti-plt-direktur-jenderal-perimbangan-keuangan-dan-ubaidillah-amin-staf--1785916718720_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1465" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1466">
+      <c r="A1466" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1466" t="inlineStr">
+        <is>
+          <t>APPI Ungkap Risiko Multifinance Masuk ke Ekosistem Kendaraan Listrik</t>
+        </is>
+      </c>
+      <c r="C1466" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:38:36 +0700</t>
+        </is>
+      </c>
+      <c r="D1466" t="inlineStr">
+        <is>
+          <t>Teti Purwanti</t>
+        </is>
+      </c>
+      <c r="E1466" t="inlineStr">
+        <is>
+          <t>Suwandi Wiratno menyatakan market share pembiayaan kendaraan listrik mencapai 25%. Namun, industri harus hati-hati terhadap risiko harga jual dan kerusakan.</t>
+        </is>
+      </c>
+      <c r="F1466" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1466" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811143353-4-758297/appi-ungkap-risiko-multifinance-masuk-ke-ekosistem-kendaraan-listrik</t>
+        </is>
+      </c>
+      <c r="H1466" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/ketua-umum-asosiasi-perusahaan-pembiayaan-indonesia-appi-suwandi-wiratno-saat-menyampaikan-pemaparan-dalam-multifinance-ceo-ga-1786416630157_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1466" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1467">
+      <c r="A1467" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1467" t="inlineStr">
+        <is>
+          <t>Negara di Tepi Jurang Krisis, Investor Berpesta-Rakyat Masih Merana</t>
+        </is>
+      </c>
+      <c r="C1467" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:35:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1467" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1467" t="inlineStr">
+        <is>
+          <t>Reformasi ekonomi Presiden Nigeria Bola Tinubu membawa hasil bagi investor, namun jutaan warga menghadapi lonjakan biaya hidup, memperlebar kesenjangan sosial.</t>
+        </is>
+      </c>
+      <c r="F1467" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1467" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811142514-4-758292/negara-di-tepi-jurang-krisis-investor-berpesta-rakyat-masih-merana</t>
+        </is>
+      </c>
+      <c r="H1467" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/01/29/warga-beristirahat-di-dalam-tempat-penampungan-darurat-sementara-pihak-berwenang-membakar-bangunan-yang-tersisa-di-komunitas-t-1769650235005_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1467" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1468">
+      <c r="A1468" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1468" t="inlineStr">
+        <is>
+          <t>Bahlil Tiba-Tiba ke Kantor Purbaya, Bahas Apa?</t>
+        </is>
+      </c>
+      <c r="C1468" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:32:53 +0700</t>
+        </is>
+      </c>
+      <c r="D1468" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1468" t="inlineStr">
+        <is>
+          <t>Menteri ESDM Bahlil Lahadalia menyambangi kantor Kementerian Keuangan (Kemenkeu) RI</t>
+        </is>
+      </c>
+      <c r="F1468" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1468" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811143131-4-758295/bahlil-tiba-tiba-ke-kantor-purbaya-bahas-apa</t>
+        </is>
+      </c>
+      <c r="H1468" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/menteri-esdm-bahlil-lahadalia-datangi-kantor-menteri-keuangan-purbaya-yudhi-sadewa-selasa-1182026-1786432462005_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1468" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1469">
+      <c r="A1469" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1469" t="inlineStr">
+        <is>
+          <t>Penjualan Mobil Juli Naik 33%, Purbaya Benar-Daya Beli Warga RI Kuat?</t>
+        </is>
+      </c>
+      <c r="C1469" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:27:29 +0700</t>
+        </is>
+      </c>
+      <c r="D1469" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1469" t="inlineStr">
+        <is>
+          <t>Pasar mobil Indonesia bangkit dengan penjualan Juli 2026 naik 33%. Pertumbuhan ini didorong oleh perbaikan ekonomi dan daya beli masyarakat yang meningkat.</t>
+        </is>
+      </c>
+      <c r="F1469" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1469" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811141732-4-758289/penjualan-mobil-juli-naik-33-purbaya-benar-daya-beli-warga-ri-kuat</t>
+        </is>
+      </c>
+      <c r="H1469" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/04/menteri-keuangan-menkeu-purbaya-yudhi-sadewa-menjajal-menaiki-hyundai-palisade-hybrid-yang-dipamerkan-dalam-gaikindo-indonesia-1785815867621_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1469" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1470">
+      <c r="A1470" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1470" t="inlineStr">
+        <is>
+          <t>Cadangan Emas RI Top 4 di Dunia, Segini Produksinya</t>
+        </is>
+      </c>
+      <c r="C1470" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:25:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1470" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1470" t="inlineStr">
+        <is>
+          <t>Indonesia menempati peringkat keempat dunia dengan cadangan emas 3.600 ton pada 2025, menurut USGS.</t>
+        </is>
+      </c>
+      <c r="F1470" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1470" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811131601-4-758262/cadangan-emas-ri-top-4-di-dunia-segini-produksinya</t>
+        </is>
+      </c>
+      <c r="H1470" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2025/05/23/ilustrasi-bijih-emas-1747992108650_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1470" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1471">
+      <c r="A1471" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1471" t="inlineStr">
+        <is>
+          <t>RI Siaga Darurat Kebakaran! Awan Hujan Tipis-Asap Mulai Menyeberang</t>
+        </is>
+      </c>
+      <c r="C1471" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:20:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1471" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1471" t="inlineStr">
+        <is>
+          <t>Kebakaran hutan dan lahan di Indonesia mencapai 48.889 ha. BNPB fokus pada penanganan darat dan operasi modifikasi cuaca untuk mencegah karhutla.</t>
+        </is>
+      </c>
+      <c r="F1471" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1471" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811132457-4-758281/ri-siaga-darurat-kebakaran-awan-hujan-tipis-asap-mulai-menyeberang</t>
+        </is>
+      </c>
+      <c r="H1471" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/upaya-petugas-gabungan-dalam-memadamkan-api-yang-membakar-kawasan-bukit-di-dusun-waililan-negeri-bula-kecamatan-bula-kabupaten-1786423840520_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1471" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1472">
+      <c r="A1472" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1472" t="inlineStr">
+        <is>
+          <t>Pusingnya Warga RI: Uang Sekolah-Sembako Mahal, Jadi "Malas" Beli Baju</t>
+        </is>
+      </c>
+      <c r="C1472" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:15:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1472" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1472" t="inlineStr">
+        <is>
+          <t>Industri tekstil Indonesia menghadapi tantangan akibat pelemahan konsumsi masyarakat. Daya beli tertekan oleh kenaikan harga kebutuhan pokok.</t>
+        </is>
+      </c>
+      <c r="F1472" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1472" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811113338-4-758202/pusingnya-warga-ri-uang-sekolah-sembako-mahal-jadi-malas-beli-baju</t>
+        </is>
+      </c>
+      <c r="H1472" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2024/06/10/ilustrasi-pabrik-tekstil_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1472" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1473">
+      <c r="A1473" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1473" t="inlineStr">
+        <is>
+          <t>Usai Libur Panjang, BI Prediksi Belanja Masyarakat Mulai Melambat</t>
+        </is>
+      </c>
+      <c r="C1473" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:10:04 +0700</t>
+        </is>
+      </c>
+      <c r="D1473" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1473" t="inlineStr">
+        <is>
+          <t>BI memprediksi penjualan eceran Juli 2026 terkontraksi 0,3% mtm, lebih baik dari tahun lalu. Beberapa kelompok barang menunjukkan pertumbuhan.</t>
+        </is>
+      </c>
+      <c r="F1473" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1473" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811131214-4-758263/usai-libur-panjang-bi-prediksi-belanja-masyarakat-mulai-melambat</t>
+        </is>
+      </c>
+      <c r="H1473" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/03/26/pengunjung-melihat-produk-yang-dijual-pada-salah-satu-tenan-di-pusat-perbelanjaan-kota-kasablanka-jakarta-kamis-2632026-1774522727003_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1473" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1474">
+      <c r="A1474" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1474" t="inlineStr">
+        <is>
+          <t>Jaksa Agung ST Burhanuddin Lantik 34 Pejabat Kejaksaan, Beri Pesan Ini</t>
+        </is>
+      </c>
+      <c r="C1474" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:02:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1474" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1474" t="inlineStr">
+        <is>
+          <t>Jaksa Agung Sanitiar Burhanuddin melantik 34 pejabat baru di Kejaksaan Agung, menekankan integritas dan tanggung jawab dalam penegakan hukum.</t>
+        </is>
+      </c>
+      <c r="F1474" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1474" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811135259-4-758279/jaksa-agung-st-burhanuddin-lantik-34-pejabat-kejaksaan-beri-pesan-ini</t>
+        </is>
+      </c>
+      <c r="H1474" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/jaksa-agung-republik-indonesia-sanitiar-burhanuddin-melantik-dan-memimpin-prosesi-pengambilan-sumpah-jabatan-kepala-kejaksaan--1786430784710_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1474" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1475">
+      <c r="A1475" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1475" t="inlineStr">
+        <is>
+          <t>Video Detik-Detik "Gempa Terkuat Abad 21" Guncang Kolombia, 138 Tewas</t>
+        </is>
+      </c>
+      <c r="C1475" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 14:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1475" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1475" t="inlineStr">
+        <is>
+          <t>Gempa magnitudo 7,4 mengguncang Kolombia, menewaskan 138 orang dan melukai 570. Sejumlah video memperlihatkan bagaimana saat gempa terjadi.</t>
+        </is>
+      </c>
+      <c r="F1475" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1475" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811125746-4-758249/video-detik-detik-gempa-terkuat-abad-21-guncang-kolombia-138-tewas</t>
+        </is>
+      </c>
+      <c r="H1475" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/suasana-pasca-gempa-bumi-di-cali-kolombia-senin-1082026-reuterschristian-escobarmora-1786405793769_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1475" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1476">
+      <c r="A1476" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1476" t="inlineStr">
+        <is>
+          <t>Madura Siap-Siap Berubah Total, Proyek Besar Ini Mau Dibangun</t>
+        </is>
+      </c>
+      <c r="C1476" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 13:50:19 +0700</t>
+        </is>
+      </c>
+      <c r="D1476" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1476" t="inlineStr">
+        <is>
+          <t>Pengembangan kawasan industri di Bangkalan ini akan menjadi penentu perubahan di Pulau Madura.</t>
+        </is>
+      </c>
+      <c r="F1476" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1476" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811125019-4-758246/madura-siap-siap-berubah-total-proyek-besar-ini-mau-dibangun</t>
+        </is>
+      </c>
+      <c r="H1476" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/pulau-madura-dok-detikcom-1786427513459_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1476" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1477">
+      <c r="A1477" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1477" t="inlineStr">
+        <is>
+          <t>Hashim Kukuhkan 20 Ormas Baru, Siap Kawal Program Pemerintahan Prabowo</t>
+        </is>
+      </c>
+      <c r="C1477" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 13:45:40 +0700</t>
+        </is>
+      </c>
+      <c r="D1477" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1477" t="inlineStr">
+        <is>
+          <t>Ketua Dewan Pembina FORMAS, Hashim Djojohadikusumo, kukuhkan 20 ormas baru untuk perkuat peran masyarakat sipil dalam mendukung program pemerintah.</t>
+        </is>
+      </c>
+      <c r="F1477" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1477" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811124245-4-758245/hashim-kukuhkan-20-ormas-baru-siap-kawal-program-pemerintahan-prabowo</t>
+        </is>
+      </c>
+      <c r="H1477" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/02/03/sesi-dialog-dengan-utusan-khusus-presiden-bidang-iklim-dan-energi-hashim-s-djojohadikusumo-menyampaikan-sambutan-dalam-acara-e-1770093260245_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1477" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1478">
+      <c r="A1478" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1478" t="inlineStr">
+        <is>
+          <t>Prabowo Usulkan Destry Damayanti Jadi Calon Tunggal Gubernur BI</t>
+        </is>
+      </c>
+      <c r="C1478" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 13:40:45 +0700</t>
+        </is>
+      </c>
+      <c r="D1478" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1478" t="inlineStr">
+        <is>
+          <t>Prabowo Usulkan Destry Damayanti Jadi Calon Tunggal Gubernur BI</t>
+        </is>
+      </c>
+      <c r="F1478" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1478" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811105426-8-758192/prabowo-usulkan-destry-damayanti-jadi-calon-tunggal-gubernur-bi</t>
+        </is>
+      </c>
+      <c r="H1478" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/prabowo-usulkan-destry-damayanti-jadi-calon-tunggal-gubernur-bi-1786429413389_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1478" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1479">
+      <c r="A1479" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1479" t="inlineStr">
+        <is>
+          <t>Pemerintah Minta UMKM RI Belajar dari India</t>
+        </is>
+      </c>
+      <c r="C1479" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 13:35:02 +0700</t>
+        </is>
+      </c>
+      <c r="D1479" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1479" t="inlineStr">
+        <is>
+          <t>Pemerintah Indonesia menganggap pengembangan usaha mikro, kecil, dan menengah (UMKM) di tanah air harus belajar dari India</t>
+        </is>
+      </c>
+      <c r="F1479" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1479" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811124140-4-758237/pemerintah-minta-umkm-ri-belajar-dari-india</t>
+        </is>
+      </c>
+      <c r="H1479" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/06/aimenteri-koordinator-bidang-perekonomian-airlangga-hartarto-pada-konferensi-pers-di-jakarta-rabu-582026-1785971442706_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1479" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1480">
+      <c r="A1480" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1480" t="inlineStr">
+        <is>
+          <t>Mayday Mayday! Mesin Pesawat Boeing 737 Terbakar Usai Tabrak Burung</t>
+        </is>
+      </c>
+      <c r="C1480" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 13:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1480" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1480" t="inlineStr">
+        <is>
+          <t>Pesawat Boeing 737 American Airlines melakukan pendaratan darurat setelah menabrak burung. Tidak ada korban, penyelidikan FAA sedang berlangsung.</t>
+        </is>
+      </c>
+      <c r="F1480" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1480" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811124235-4-758238/mayday-mayday-mesin-pesawat-boeing-737-terbakar-usai-tabrak-burung</t>
+        </is>
+      </c>
+      <c r="H1480" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2021/03/03/ilustrasi-kecelakaan-pesawat-istockphotokesu01_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1480" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1481">
+      <c r="A1481" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1481" t="inlineStr">
+        <is>
+          <t>Kabar Baik! BI Ramal Tekanan Inflasi Mulai Mereda September</t>
+        </is>
+      </c>
+      <c r="C1481" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 13:25:45 +0700</t>
+        </is>
+      </c>
+      <c r="D1481" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1481" t="inlineStr">
+        <is>
+          <t>Bank Indonesia memperkirakan inflasi mereda pada September 2026. Penjualan eceran dipengaruhi normalisasi pasca HUT RI, dengan IEP menurun.</t>
+        </is>
+      </c>
+      <c r="F1481" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1481" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811124144-4-758236/kabar-baik-bi-ramal-tekanan-inflasi-mulai-mereda-september</t>
+        </is>
+      </c>
+      <c r="H1481" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/04/22/pekerja-menata-minyak-goreng-di-kawasan-pasar-pondok-labu-jakarta-selatan-rabu-2242026-1776852494383_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1481" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1482">
+      <c r="A1482" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1482" t="inlineStr">
+        <is>
+          <t>40% Bisnis di RI Pakai AI-Pendapatan Naik, Begini Penjelasan Airlangga</t>
+        </is>
+      </c>
+      <c r="C1482" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 13:20:02 +0700</t>
+        </is>
+      </c>
+      <c r="D1482" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1482" t="inlineStr">
+        <is>
+          <t>Banyak pengusaha atau pelaku bisnis di Indonesia yang sudah mengadopsi artificial Intelligence/AI untuk kemudahan usaha.</t>
+        </is>
+      </c>
+      <c r="F1482" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1482" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811122802-4-758234/40-bisnis-di-ri-pakai-ai-pendapatan-naik-begini-penjelasan-airlangga</t>
+        </is>
+      </c>
+      <c r="H1482" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/menko-perekonomian-airlangga-hartarto-dalam-acara-umkm-finance-summit-2026-dengan-tema-penguatan-akses-pembiayaan-dan-ekosiste-1786418467181_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1482" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1483">
+      <c r="A1483" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1483" t="inlineStr">
+        <is>
+          <t>Penampakan Kabut Asap Kebakaran Hutan Kepung Palembang, Matahari Kabur</t>
+        </is>
+      </c>
+      <c r="C1483" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 13:10:05 +0700</t>
+        </is>
+      </c>
+      <c r="D1483" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1483" t="inlineStr">
+        <is>
+          <t>Masyarakat juga diimbau untuk mengurangi aktivitas luar ruangan dan memakai masker ketika berada di luar, khususnya pada malam hari.</t>
+        </is>
+      </c>
+      <c r="F1483" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1483" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811124446-7-758239/penampakan-kabut-asap-kebakaran-hutan-kepung-palembang-matahari-kabur</t>
+        </is>
+      </c>
+      <c r="H1483" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/kabut-asap-akibat-kebakaran-hutan-di-palembang-provinsi-sumatera-selatan-selasa-1182026-reutersabriansyah-liberto-1786425753336_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1483" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1484">
+      <c r="A1484" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1484" t="inlineStr">
+        <is>
+          <t>Potret TKP Eks Anggota Dewan Tembak Leher Pejabat Pemda Gegara Utang</t>
+        </is>
+      </c>
+      <c r="C1484" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 13:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1484" t="inlineStr">
+        <is>
+          <t>Reuters</t>
+        </is>
+      </c>
+      <c r="E1484" t="inlineStr">
+        <is>
+          <t>Pelaku penembakan mengatakan ia melakukan serangan itu karena perselisihan yang sudah lama terjadi terkait uang.</t>
+        </is>
+      </c>
+      <c r="F1484" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1484" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811073749-7-758129/potret-tkp-eks-anggota-dewan-tembak-leher-pejabat-pemda-gegara-utang</t>
+        </is>
+      </c>
+      <c r="H1484" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/petugas-memeriksa-lokasi-penembakan-setelah-mantan-anggota-parlemen-chalong-riewrang-diduga-menembak-thongchai-yenprasert-pres-1786408168079_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1484" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1485">
+      <c r="A1485" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1485" t="inlineStr">
+        <is>
+          <t>China Kini Jadi "OPEC" Baru? Penguasa dan Pemain Pasar Minyak Dunia</t>
+        </is>
+      </c>
+      <c r="C1485" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:55:37 +0700</t>
+        </is>
+      </c>
+      <c r="D1485" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1485" t="inlineStr">
+        <is>
+          <t>China Kini Jadi "OPEC" Baru? Penguasa dan Pemain Pasar Minyak Dunia</t>
+        </is>
+      </c>
+      <c r="F1485" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1485" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811105425-8-758191/china-kini-jadi-opec-baru-penguasa-pemain-pasar-minyak-dunia</t>
+        </is>
+      </c>
+      <c r="H1485" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/china-kini-jadi-opec-baru-penguasa-pemain-pasar-minyak-dunia-1786423383489_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1485" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1486">
+      <c r="A1486" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1486" t="inlineStr">
+        <is>
+          <t>RI Kalah Lawan Thailand, Vietnam-Singapura, Wamendag Kasih Pesan Tegas</t>
+        </is>
+      </c>
+      <c r="C1486" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:55:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1486" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1486" t="inlineStr">
+        <is>
+          <t>Wamendag Roro mengungkap posisi Indonesia dalam ekspor makanan dan minuman di ASEAN. Tapi, RI masih tertinggal dari Thailand dan perlu tingkatkan daya saing.</t>
+        </is>
+      </c>
+      <c r="F1486" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1486" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811120825-4-758224/ri-kalah-lawan-thailand-vietnam-singapura-wamendag-kasih-pesan-tegas</t>
+        </is>
+      </c>
+      <c r="H1486" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/wakil-menteri-perdagangan-wamendag-dyah-roro-esti-widya-putri-dalam-acara-indonesia-fb-trade-promotion-forum-di-auditorium-kem-1786425998101_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1486" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1487">
+      <c r="A1487" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1487" t="inlineStr">
+        <is>
+          <t>RI Sudah Punya BBM Bioetanol, Cek Segini Harganya di SPBU</t>
+        </is>
+      </c>
+      <c r="C1487" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:50:05 +0700</t>
+        </is>
+      </c>
+      <c r="D1487" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1487" t="inlineStr">
+        <is>
+          <t>Presiden Prabowo Subianto dorong pengembangan bioetanol di Indonesia, menargetkan penerapan E10 dan E20.</t>
+        </is>
+      </c>
+      <c r="F1487" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1487" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811102243-4-758181/ri-sudah-punya-bbm-bioetanol-cek-segini-harganya-di-spbu</t>
+        </is>
+      </c>
+      <c r="H1487" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2023/07/24/bbm-pertamax-green-ron-95-pt-pertamina-persero-di-spbu-pertamina-mt-haryono-jakarta-selatan-senin-2472023-4_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1487" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1488">
+      <c r="A1488" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1488" t="inlineStr">
+        <is>
+          <t>Video: Amerika Siapkan 'Tombol Pembunuh' - Banjir Terjang Filipina</t>
+        </is>
+      </c>
+      <c r="C1488" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:45:16 +0700</t>
+        </is>
+      </c>
+      <c r="D1488" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1488" t="inlineStr">
+        <is>
+          <t>Amerika Siapkan 'Tombol Pembunuh' - Banjir Terjang Filipina</t>
+        </is>
+      </c>
+      <c r="F1488" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1488" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811105423-8-758190/video-amerika-siapkan-tombol-pembunuh--banjir-terjang-filipina</t>
+        </is>
+      </c>
+      <c r="H1488" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/amerika-siapkan-tombol-pembunuh-banjir-terjang-filipina-1786423353528_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1488" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1489">
+      <c r="A1489" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1489" t="inlineStr">
+        <is>
+          <t>Waspada Akhir Tahun, Harga-Harga Diperkirakan Naik Lagi</t>
+        </is>
+      </c>
+      <c r="C1489" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:45:09 +0700</t>
+        </is>
+      </c>
+      <c r="D1489" t="inlineStr">
+        <is>
+          <t>Robertus Andrianto</t>
+        </is>
+      </c>
+      <c r="E1489" t="inlineStr">
+        <is>
+          <t>BI memprediksi kenaikan harga barang eceran pada Desember 2026, yang dapat memengaruhi inflasi, seiring dengan meningkatnya ekspektasi penjualan.</t>
+        </is>
+      </c>
+      <c r="F1489" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1489" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811120611-4-758223/waspada-akhir-tahun-harga-harga-diperkirakan-naik-lagi</t>
+        </is>
+      </c>
+      <c r="H1489" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/04/14/los-sayur-mayur-di-pasar-santa-jakarta-selatan-selasa-144-cnbc-indonesiahadijah-alaydrus-1776148728988_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1489" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1490">
+      <c r="A1490" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1490" t="inlineStr">
+        <is>
+          <t>Wow! Cadangan Emas RI No.4 Terbesar Dunia, Segini Jumlahnya</t>
+        </is>
+      </c>
+      <c r="C1490" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:35:05 +0700</t>
+        </is>
+      </c>
+      <c r="D1490" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1490" t="inlineStr">
+        <is>
+          <t>Indonesia menempati peringkat ke-4 terbesar dunia untuk cadangan emas dengan jumlah 3.600 ton.</t>
+        </is>
+      </c>
+      <c r="F1490" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1490" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811113243-4-758201/wow-cadangan-emas-ri-no4-terbesar-dunia-segini-jumlahnya</t>
+        </is>
+      </c>
+      <c r="H1490" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/03/04/penyebab-harga-emas-naik-saat-isu-perang-kebijakan-bank-sentral-meningkatkan-cadangan-emasfoto-freepikcomwirestock-1773018322135_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1490" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1491">
+      <c r="A1491" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1491" t="inlineStr">
+        <is>
+          <t>Garap Proyek Tambang Baru, Freeport Bakal Kocek Rp 71,2 Triliun</t>
+        </is>
+      </c>
+      <c r="C1491" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:30:05 +0700</t>
+        </is>
+      </c>
+      <c r="D1491" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1491" t="inlineStr">
+        <is>
+          <t>PT Freeport Indonesia mengembangkan tambang bawah tanah Kucing Liar yang ditargetkan beroperasi pada 2029.</t>
+        </is>
+      </c>
+      <c r="F1491" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1491" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811101202-4-758175/garap-proyek-tambang-baru-freeport-bakal-kocek-rp-712-triliun</t>
+        </is>
+      </c>
+      <c r="H1491" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/04/12/area-tambang-terbuka-grasberg-dan-tambang-bawah-tanah-deep-mill-level-zone-dmlz-pt-freeport-indonesia-ptfi-pt-freeport-indones-1775944307191_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1491" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1492">
+      <c r="A1492" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1492" t="inlineStr">
+        <is>
+          <t>Video: "Investasi Berdampak" Bikin Dana Hibah Efektif Atasi Isu Sosial</t>
+        </is>
+      </c>
+      <c r="C1492" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:27:44 +0700</t>
+        </is>
+      </c>
+      <c r="D1492" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1492" t="inlineStr">
+        <is>
+          <t>"Investasi Berdampak" Bikin Dana Hibah Efektif Atasi Isu Kesehatan, Pendidikan - UMKM di RI</t>
+        </is>
+      </c>
+      <c r="F1492" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1492" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260810154928-8-758000/video-investasi-berdampak-bikin-dana-hibah-efektif-atasi-isu-sosial</t>
+        </is>
+      </c>
+      <c r="H1492" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/investasi-berdampak-bikin-dana-hibah-efektif-atasi-isu-kesehatan-pendidikan-umkm-di-ri-1786424302671_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1492" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1493">
+      <c r="A1493" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1493" t="inlineStr">
+        <is>
+          <t>Panas Mendidih Bawa Petaka, RI Kebakaran dari Sumatra-Papua Ribuan Ha</t>
+        </is>
+      </c>
+      <c r="C1493" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:21:12 +0700</t>
+        </is>
+      </c>
+      <c r="D1493" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1493" t="inlineStr">
+        <is>
+          <t>Kebakaran hutan dan lahan (karhutla) terjadi di sejumlah wilayah di Indonesia pada periode 8-10 Agustus 2026.</t>
+        </is>
+      </c>
+      <c r="F1493" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1493" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811115418-7-758211/panas-mendidih-bawa-petaka-ri-kebakaran-dari-sumatra-papua-ribuan-ha</t>
+        </is>
+      </c>
+      <c r="H1493" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/petugas-berupaya-memadamkan-api-yang-membakar-bukit-pindul-dukuh-girisono-rt-03-rw-05-desa-gunung-gajah-kecamatan-bayat-kabupa-1786423989900_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1493" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1494">
+      <c r="A1494" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1494" t="inlineStr">
+        <is>
+          <t>Investor China, Korea hingga Jepang Berebut Masuk Madura, Ada Apa?</t>
+        </is>
+      </c>
+      <c r="C1494" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:10:26 +0700</t>
+        </is>
+      </c>
+      <c r="D1494" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1494" t="inlineStr">
+        <is>
+          <t>Kawasan Industri di Madura ini mulai menarik investor global, termasuk dari China, Korea, dan Jepang. Ada apa?</t>
+        </is>
+      </c>
+      <c r="F1494" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1494" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811113118-4-758204/investor-china-korea-hingga-jepang-berebut-masuk-madura-ada-apa</t>
+        </is>
+      </c>
+      <c r="H1494" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/pulau-madura-dok-istimewa-1786423646408_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1494" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1495">
+      <c r="A1495" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1495" t="inlineStr">
+        <is>
+          <t>Demo Pemuda Menuju Parlemen, Polisi Tembak Gas Air Mata dan Meriam Air</t>
+        </is>
+      </c>
+      <c r="C1495" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 12:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1495" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1495" t="inlineStr">
+        <is>
+          <t>Ribuan pemuda bentrok dengan polisi saat melakukan protes menuju parlemen. Polisi menembakki dengan gas air mata dan meriam air.</t>
+        </is>
+      </c>
+      <c r="F1495" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1495" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811075052-4-758136/demo-pemuda-menuju-parlemen-polisi-tembak-gas-air-mata-meriam-air</t>
+        </is>
+      </c>
+      <c r="H1495" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/07/20/ricuh-pendukung-partai-kecoa-saat-demonstrasi-menuntut-pengunduran-diri-menteri-pendidikan-dharmendra-pradhan-karena-kebocoran-1784551944594_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1495" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1496">
+      <c r="A1496" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1496" t="inlineStr">
+        <is>
+          <t>Prabowo Pantau Ketat BBM B50, Cek Segini Harganya di SPBU Pertamina</t>
+        </is>
+      </c>
+      <c r="C1496" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:55:05 +0700</t>
+        </is>
+      </c>
+      <c r="D1496" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1496" t="inlineStr">
+        <is>
+          <t>Presiden Prabowo memanggil Dirut Pertamina untuk membahas implementasi program BBM biodiesel B50.</t>
+        </is>
+      </c>
+      <c r="F1496" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1496" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811104334-4-758186/prabowo-pantau-ketat-bbm-b50-cek-segini-harganya-di-spbu-pertamina</t>
+        </is>
+      </c>
+      <c r="H1496" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/07/09/presiden-ri-prabowo-subianto-resmi-meluncurkan-mandatori-biodiesel-b50-yakni-bahan-bakar-minyak-jenis-solar-yang-dicampur-baha-1783599161264_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1496" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1497">
+      <c r="A1497" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1497" t="inlineStr">
+        <is>
+          <t>Kejadian Aneh di RI, Pabrik Tekstil Lama Bertumbangan-Muncul yang Baru</t>
+        </is>
+      </c>
+      <c r="C1497" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:50:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1497" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1497" t="inlineStr">
+        <is>
+          <t>Industri tekstil Indonesia diproyeksikan tumbuh 5% pada 2026, namun menghadapi paradoks akibat investasi baru dan tekanan dari produk impor murah.</t>
+        </is>
+      </c>
+      <c r="F1497" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1497" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811111940-4-758198/kejadian-aneh-di-ri-pabrik-tekstil-lama-bertumbangan-muncul-yang-baru</t>
+        </is>
+      </c>
+      <c r="H1497" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2022/10/20/ilustrasi-buruh-pabrik-tekstil-5_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1497" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1498">
+      <c r="A1498" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1498" t="inlineStr">
+        <is>
+          <t>Ada 'Bensin' Baru, Singapura Naikkan Proyeksi Ekonomi 2026</t>
+        </is>
+      </c>
+      <c r="C1498" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:48:25 +0700</t>
+        </is>
+      </c>
+      <c r="D1498" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1498" t="inlineStr">
+        <is>
+          <t>Pemerintah Singapura menaikkan proyeksi pertumbuhan ekonomi 2026 menjadi 4,5%-5,5% berkat sektor AI dan ekspor. Inflasi tetap menjadi perhatian.</t>
+        </is>
+      </c>
+      <c r="F1498" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1498" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811114230-4-758208/ada-bensin-baru-singapura-naikkan-proyeksi-ekonomi-2026</t>
+        </is>
+      </c>
+      <c r="H1498" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2022/06/30/warga-yang-memakai-masker-wajah-melewati-cakrawala-kota-selama-wabah-penyakit-coronavirus-covid-19-di-singapura-reutersedgar-s_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1498" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1499">
+      <c r="A1499" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1499" t="inlineStr">
+        <is>
+          <t>Siap-Siap Pabrik Baterai EV ke-2 RI Segera Beroperasi, Ini Pemiliknya</t>
+        </is>
+      </c>
+      <c r="C1499" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:35:05 +0700</t>
+        </is>
+      </c>
+      <c r="D1499" t="inlineStr">
+        <is>
+          <t>Firda Dwi Muliawati</t>
+        </is>
+      </c>
+      <c r="E1499" t="inlineStr">
+        <is>
+          <t>Indonesia segera memiliki pabrik baterai kendaraan listrik terbesar kedua di Karawang, Jawa Barat.</t>
+        </is>
+      </c>
+      <c r="F1499" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1499" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811101636-4-758178/siap-siap-pabrik-baterai-ev-ke-2-ri-segera-beroperasi-ini-pemiliknya</t>
+        </is>
+      </c>
+      <c r="H1499" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2025/06/12/baterai-mobil-flp-lithium-ferro-phosphate-1749716117484_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1499" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1500">
+      <c r="A1500" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1500" t="inlineStr">
+        <is>
+          <t>Belajar AI dan Investment Banking, Ini Cara DBS Siapkan Generasi Penerus</t>
+        </is>
+      </c>
+      <c r="C1500" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:31:52 +0700</t>
+        </is>
+      </c>
+      <c r="D1500" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1500" t="inlineStr">
+        <is>
+          <t>Bank DBS Indonesia luncurkan program DBS NextGen Excursion 2026 untuk anak nasabah, fokus pada AI dan kepemimpinan, memperluas wawasan global dan jejaring.</t>
+        </is>
+      </c>
+      <c r="F1500" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1500" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811132716-4-758270/belajar-ai-investment-banking-ini-cara-dbs-siapkan-generasi-penerus</t>
+        </is>
+      </c>
+      <c r="H1500" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2025/08/15/bank-dbs-indonesia-1755229660984_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1500" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1501">
+      <c r="A1501" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1501" t="inlineStr">
+        <is>
+          <t>Video: Menko Perekonomian Tengah Mengkaji Insentif Dampak El Nino</t>
+        </is>
+      </c>
+      <c r="C1501" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:21:04 +0700</t>
+        </is>
+      </c>
+      <c r="D1501" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1501" t="inlineStr">
+        <is>
+          <t>Airlangga Hartarto masih meninjau insentif sektor pangan sebagai bentuk untuk mitigasi dampak El Nino.</t>
+        </is>
+      </c>
+      <c r="F1501" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1501" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811100804-8-758171/video-menko-perekonomian-tengah-mengkaji-insentif-dampak-el-nino</t>
+        </is>
+      </c>
+      <c r="H1501" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/11/menko-perekonomian-tengah-mengkaji-insentif-dampak-el-nino-1786417754864_169.png?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1501" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1502">
+      <c r="A1502" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1502" t="inlineStr">
+        <is>
+          <t>Viral Klaim Barang Pribadi Kena Pajak 2027, Ini Penjelasan DJP</t>
+        </is>
+      </c>
+      <c r="C1502" t="inlineStr">
+        <is>
+          <t>Tue, 11 Aug 2026 11:20:55 +0700</t>
+        </is>
+      </c>
+      <c r="D1502" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1502" t="inlineStr">
+        <is>
+          <t>DJP membantah berbagai barang pribadi akan dikenai pajak mulai tahun 2027.</t>
+        </is>
+      </c>
+      <c r="F1502" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1502" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260811110155-4-758189/viral-klaim-barang-pribadi-kena-pajak-2027-ini-penjelasan-djp</t>
+        </is>
+      </c>
+      <c r="H1502" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2022/08/04/tanah-rumah-warisan-bebas-pajak-lho-tapi-ada-syaratnya_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1502" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I1397"/>
+  <autoFilter ref="A1:I1502"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>